<commit_message>
Atualizacao de arquivos - 28/02/2026 13:12:35,62
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7631074-5B3A-46E7-B758-81F1D81D5395}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4646C255-73DE-4858-8388-A8AB6406C629}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2811" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3183" uniqueCount="603">
   <si>
     <t>ID</t>
   </si>
@@ -1702,6 +1702,216 @@
   </si>
   <si>
     <t>Foi feito a troca dos filtros , mas ficou pingando o ponto de água na parede(mangueira) com a manipulação do aparelho. Deveria fazer um check list para tentar identificar esses problemas</t>
+  </si>
+  <si>
+    <t>Demora no atendimento, postergação de atendimento para mais de 15 dias, tivemos que comprar água em galão para suprimento residencial.Péssimo, se a próxima vez acontecer o mesmo atendimento, cancelo minhas assinaturas.</t>
+  </si>
+  <si>
+    <t>Horrível, serviço pessimo, empresa terrível. Estou sem o filtro desde a instalação. Péssima empresa</t>
+  </si>
+  <si>
+    <t>O novo que foi colocado estragou em 24 h</t>
+  </si>
+  <si>
+    <t>Antes do 3 meses, á agua já apresentou odor</t>
+  </si>
+  <si>
+    <t>O puficador ainda está com problema, o técnico informou que seria feito a troca do produto no prazo de 5 dias</t>
+  </si>
+  <si>
+    <t>Nao houve contato para confirmar a data da troca eo aparelho</t>
+  </si>
+  <si>
+    <t>O serviço de manuteção e conserto de problemas é PÉSSIMO. O problema é a falta de comunicação entre cliente, central de atendimento e pessoal da manutenção.Ficamos mais de um mês sem o filtro, pessoal da manutenção veio, mas como não há comunicação, não davam continuidade corretamente.Não é culpa nem dos técnicos, que são super atenciosos, nem do pessoal no telefone. É o sistema que é ruim mesmo</t>
+  </si>
+  <si>
+    <t>O equipamento é muito bom. No entanto o suporte de assistência é dificil de acreditar qye seja Brastemp.. Nao se consegue falar, a não ser com um chatbox da pior qualidade.- os agendamentos feitos por minha solicitação nunca acontecem. O técnico não chega.- o técnico  vem por conta própria  sem agendamento.-  quando vc pede pra ser sentido por um humano, o atendimento consegue piorar  Ou seja, pago mensalidade por um produto qye dificilmente precisa de manutenção, quando precisa é  um caos!</t>
+  </si>
+  <si>
+    <t>Inconclusiva. O técnico foi embora sem mexer no aparelho. Aparentemente, ficou de fazer a substituição.</t>
+  </si>
+  <si>
+    <t>FRQ ZONA OESTE2 SP R01</t>
+  </si>
+  <si>
+    <t>A última assistência técnica deixou a desejar.</t>
+  </si>
+  <si>
+    <t>A data disponível para agendar a visita foi muito para frente. Quando estamos com problema com o filtro, teria que ter data disponível para o dia seguinte.</t>
+  </si>
+  <si>
+    <t>Não houve, a visita é marcada e remarcada e o técnico não aparece. Continuo com o purificador sem funcionar.</t>
+  </si>
+  <si>
+    <t>FRQ OSASCO SP R02</t>
+  </si>
+  <si>
+    <t>Marquei três veze a  revisão e o técnico nao apareceu</t>
+  </si>
+  <si>
+    <t>FRQ ZONA NORTE SP R01</t>
+  </si>
+  <si>
+    <t>Não ficou correto para a intenção a tomada..</t>
+  </si>
+  <si>
+    <t>FRQ OSASCO SP R01</t>
+  </si>
+  <si>
+    <t>Parece-me que o purificador chegou ao final de sua existência!!!</t>
+  </si>
+  <si>
+    <t>Experiência boa , aparelho de muita qualidade e durabilidade , assistência muita boa tbem … porém o preço está um pouco pesado … acredito q uma melhor tarifa ainda mais para o público residencial seria o ideal</t>
+  </si>
+  <si>
+    <t>O local da instalação ficou ruim estou aguardando o técnico hoje e caso não dê para instalar na área de serviço terei que cancelar pois quando eu comprei a atendente disse que poderia pendurar na parede e o técnico quando veio instalar disse que não pode pois ele é muito pesado e acabou colocando em cima da minha pia e não ficou bom.</t>
+  </si>
+  <si>
+    <t>Antigamente vcs nos alertavam sobre o momento da manutenção e dessa vez eu que tive de ir atrás, até então já haviam se passado 7 meses da última manutenção, antigamente os técnicos higienizavam o filtro todo, inclusive o bocal de onde sai a água pra consumo, antigamente testavam a qualidade da água antes e após troca do filtro, hoje é somente troca do filtro e tchau. O técnico foi educado e concluiu o serviço mas antes de entrar não sabia a senha que forneci no agendamento da visita, tive que aguardar 15 minutos até que descobrissem a senha. Enfim, é decepcionante como decaíram.</t>
+  </si>
+  <si>
+    <t>Meu purificador está sem funcionar desde segunda-feira passada. Estou aguardando contato da brastemp com a indicação do dia da troca</t>
+  </si>
+  <si>
+    <t>FRQ SBC SP R01</t>
+  </si>
+  <si>
+    <t>Estou sem meu purificador desde dezembro, pagando nas datas, agendo com a manutenção e me tratam com descaso. Meu filtro sai agua quente, e não foi isso que contratei, se quisesse agua quente, usaria o fogão. Mesmo assim, insisti em fazer agenda para troca do aparelho e nada foi feito. Quero que me restitua os valores que paguei esses meses sem usa-lo. Isso é uma falta de respeito ao consumidor. Já estou pesquisando outro produto.</t>
+  </si>
+  <si>
+    <t>Sou cliente a muitos anos, sempre gostei... ultimamente que está sendo complicado agendar visita técnica e algumas vezes não vem... este último tecnico foi muito atencioso e prestativo</t>
+  </si>
+  <si>
+    <t>Valor mensal</t>
+  </si>
+  <si>
+    <t>Fiquei esperando e o técnico não apareceu mais uma vez.O serviço de vocês está péssimo. Estou com problemas no purificar desde novembro/25. Até o momento o problema não foi resolvido e eu precisando comprar água, pois não tenho outra forma de ter água para beber.</t>
+  </si>
+  <si>
+    <t>Com altos e baixos. Ultimamente minha experiência não está tão boa.</t>
+  </si>
+  <si>
+    <t>Vcs resgendarwm a minha visita por 3 vezes ....a última ...no último acabei não veio ninguém e eu tive que ligar ....porém o chamado dizia que já trocaram ... Aqui em casa não vieram ... Estamos muitos decepcionados com o atendimento de vcs ... Reagendaram agora para 21/03 ...e nos tomando água com gosto horrível ...</t>
+  </si>
+  <si>
+    <t>Minha avaliação é baixa,pois vcs demoraram mais de 20 dias para a substituição de um purificador que não estava gelando ,mesmo eu tendo reclamado umas 3 vêzes e dito pessoalmente ao técnico que foi lá ..obs : neste espaço da empresa tem + de 15 pessoas e tomaram água quente por muito tempo</t>
+  </si>
+  <si>
+    <t>O filtro apresenta um problema e o técnico fala que não tem problema</t>
+  </si>
+  <si>
+    <t>Uma eternidade para trocar o aparelho que deu defeito</t>
+  </si>
+  <si>
+    <t>Demorou muito para ter a manutenção preventiva. Além disso, na primeira manutenção marcada, o técnico não apareceu. E não recebi nenhum comunicado. A Brastemp também não verificou se eu havia recebido o atendimento.Após algum tempo, tive q abrir um novo chamado, informar q eu não havia sido atendida e tentar marcar o mais breve possível. Tive que insistir, porque a atendente queria marcar só pra Maio, dizendo q não precisava trocar o elemento filtrante. Só dei essa nota, porque o equipamento é útil. Mas o atendimento está horrível.</t>
+  </si>
+  <si>
+    <t>A agua nao está gelando.  E o técnico nao consertou e nao trocou o filtro.</t>
+  </si>
+  <si>
+    <t>Meu purificador quebrou, única fonte de água potável. Não possuo gelagua com botijao de agua mineral. Enfrento dificuldade de atendimento. Só consegui agendamento para o dua seguinte.Durante a visita, fui informada de que seria substituído o equipamento, que está fora de linha. Não há peças e conserto. Até agora sem resposta e previsão sobre a substituição.Isso poderia ter sido evitado com substituição preventiva!</t>
+  </si>
+  <si>
+    <t>Me parece mto bom, mas acho um pouco cara a mensalidade</t>
+  </si>
+  <si>
+    <t>O purificador é bom, o problema é com o atendimento para agendamento que não "entende" a necessidade do cliente. Temos 2 aparelhos, inicialmente havia agendado a troca regular dos filtros , que já contava com a espera de 3 semanas. Mesmo com antecedência, fomos informados que não poderia ser realizadas no mesmo dia, primeiro iriam dia 23/02 para fazer a troca de 1 e no dia 24 do outro. Detalhe, mesma empresa mesmo local. Não faz sentido.Depois no dia 19/02, os 2 filtros apresentaram odor, impossibilitando a utilização da água. Liguei.pedindo prioridade no atendimento, liguei umas 4 vezes, falando com pessoas diferentes. IMPLOREI para anteciparem o atendimento,  não houve acordo, precisamos gastar uma.grana comprando garrafas de água para 40.pessoas diariamente, até ontem quando técnico apareceu para em.15 minutos realizar a troca dos filtros. Me informou que nem estava sabendo, que era para trocar os filtros, que por "sorte" ele estava com 2 de reserva e pôde realizar a troca.Acham norma um cliente ter que aguardar rtodo esse tempo.para um.atendimento?</t>
+  </si>
+  <si>
+    <t>não veio ninguem fazer a visita</t>
+  </si>
+  <si>
+    <t>atendimento péssimo, assim que o técnico saiu da empresa, o filtro parou de funcionar, entrei em contato informando o ocorrido e não tive nenhum suporte em relação a isso, pedi prioridade pois estava sem água e aqui na empresa temos mais de 30 funcionários, a atendente informou que não podia e que eu tinha que aguardar até o dia seguinte, pedi pro atendimento ser de manhã e a mesma disse que não teve retorno do técnico e que não tinha o que fazer. muito decepcionada com a empresa.</t>
+  </si>
+  <si>
+    <t>O horário da visita não foi respeitado. A sorte é que tinha gente em casa.Da próxima vez o técnico não será recebido fora do horário marcado.</t>
+  </si>
+  <si>
+    <t>passei três meses esperando assistência técnica</t>
+  </si>
+  <si>
+    <t>Instalação foi tudo ok O problema só foi o tamanho do produto</t>
+  </si>
+  <si>
+    <t>Ele é bom, porem, não Gela muito em ambientes como chão de fabrica</t>
+  </si>
+  <si>
+    <t>Até o momento  estou gostando  do purificador.  O único  problema é o  tamanho  dele, ocupa muito espaço</t>
+  </si>
+  <si>
+    <t>Devido ao tempo deveriam considerar um bônus por fidelidade.</t>
+  </si>
+  <si>
+    <t>É Só voc~es veriifcarem quantas chamadas aminha esposa fez para vocês que saberão porque estou dando nota zero</t>
+  </si>
+  <si>
+    <t>O técnico veio até o endereço mas foi embora sem nos atender alegando nao ter ninguém, entretanto estávamos aguardando e o mesmo foi embora sem fazer nenhuma tentativa de contato, estamos sem água gelada e com vazamento no aparelho ha mais de 30 dias! Sem nenhuma solução até hoje 26/02/2026</t>
+  </si>
+  <si>
+    <t>Prazo absurdo para a troca e colocaram um aparelho similar</t>
+  </si>
+  <si>
+    <t>FRQ BASE LESTE SP R01</t>
+  </si>
+  <si>
+    <t>O aparelho é muito bom.Estou contente.Menos a assistência técnica.</t>
+  </si>
+  <si>
+    <t>O técnico disse que o aparelho está danificado e precisa ser trocado. A Brastemp não me contatou sobre a troca do aparelho.</t>
+  </si>
+  <si>
+    <t>FRQ ZONA OESTE1 SP R01</t>
+  </si>
+  <si>
+    <t>O serviço é horrível, não consigo fazer nenhuma solicitação pelo site, no meu cadastro no site não consta minha assinatura de purificador. Para fazer qualquer solicitação tenho que entrar em contato por telefone e perder muito tempo.A visita técnica não cumpriu o horário combinado.</t>
+  </si>
+  <si>
+    <t>Gosto muito!</t>
+  </si>
+  <si>
+    <t>Aparelho é bom mas a assistência precisa melhorar.. nao cumprem agenda de manutenção. Toda vez tem que reagendar pois ninguém aparece.  Também já  solicitei a instalação do tal pressurizador interno e até hoje nem sinal..</t>
+  </si>
+  <si>
+    <t>Foi instalado porém ficou com um pouco de vazamento na conexão de agua</t>
+  </si>
+  <si>
+    <t>FRQ SBC SP R03</t>
+  </si>
+  <si>
+    <t>Tive que remarcar , não apareceu ninguém a primeira vez</t>
+  </si>
+  <si>
+    <t>Visitaram por 3 vezes consecutivos o endereço de Copacabana, apenas.Não fazem visitas nos endereços do Recreio há mais de 2 anos.</t>
+  </si>
+  <si>
+    <t>Estou com o purificador sem sair água gelada e quero a troca do aparelho . Estou muito insatisfeita!</t>
+  </si>
+  <si>
+    <t>Péssima experiencia até agora. O rapaz veio instalar e me disse que o aparelhos veio com defeito pois o sensor do dispensador de água instalado é de outro aparelho, o que faz como que ele não funcione. Me disse que ia abrir uma solicitação de reparo.Notei que além disso, ainda está vazando agua por baixo do purificador e molhando toda minha pia e a vazão da agua gelada (que é a unica que funciona) está muito fraca.Recebi o contato por WhatsApp para marcar a visita de reparo e para minha surpresa agendaram apenas para dia 16/03, ou seja, 24 dias após a instalação (quase 1 mês). UmCompleto absurdo! Para instalar é de um dia pro outro, mas para consertar o aparelho que vocês já enviaram quebrado para um cliente novo, ai leva 24 dias!O atendimento no WhatsApp não me deu sequer oportunidade de resposta e encerrou o atendimento.Com isso liguei para a central onde, ao relatar todo esse contexto, pensei que fosse melhorar, mas só piorou… a moça bem mal preparada para o atendimento e ai da me disse que só podia agendar para depois do dia 20de março, mais longe ainda.Ou seja, a Brastemp me oferece o 1° mês grátis, mas com um aparelho que não funciona e ainda vazando e me pede mais de 20 dias pra eu esperar!Realmente uma experiência péssima!</t>
+  </si>
+  <si>
+    <t>Venho por meio deste registrar minha insatisfação quanto à entrega do produto contratado e à ausência de retorno por parte da equipe de atendimento.Contratei 2 (dois) filtros, porém foi entregue apenas 1 (um). Desde então, venho tentando obter informações sobre a entrega do segundo filtro, mas não recebo qualquer posicionamento. Envio mensagens pelo WhatsApp e simplesmente não obtenho resposta. A atendente visualiza, porém não informa absolutamente nada.Gostaria de destacar que, antes da assinatura do contrato, o atendimento era imediato e as respostas eram praticamente instantâneas. No entanto, após a contratação, não consigo sequer uma previsão básica, não sei se a entrega ocorrerá na próxima semana, no próximo mês ou quando.Essa falta de informação me deixa completamente sem direcionamento. Caso eu tivesse ao menos uma previsão concreta, poderia providenciar uma solução provisória, como a utilização de um filtro temporário ou uma jarra com filtragem até a chegada do produto. Contudo, sem qualquer data estimada, torna-se extremamente difícil organizar essa situação.Solicito, com urgência, um posicionamento formal informando:Quando o segundo filtro será entregue;O motivo da não entrega conjunta;E a previsão exata ou estimada para regularização.Fico no aguardo de retorno imediato.</t>
+  </si>
+  <si>
+    <t>Instalação horrível, o técnico não sabia nada de hidráulica e deixou vazamentos e estragou a saída de água</t>
+  </si>
+  <si>
+    <t>Sou cliente do serviço de locação do purificador de água Brastemp há bastante tempo e sempre considerei um diferencial da marca a previsibilidade e a segurança no processo de manutenção semestral, com a troca regular do elemento filtrante.Fui informada, na última manutenção, de que a política foi alterada e que a substituição do filtro agora ocorre apenas se o técnico considerar que ainda há ou não vida útil remanescente. Essa mudança compromete minha percepção de segurança, qualidade e transparência do serviço contratado, especialmente porque a troca periódica sempre fez parte da proposta que justificava o valor mensal da locação.Caso essa nova política seja mantida, informo que optarei pelo cancelamento do contrato de locação, pois o modelo atual deixa de atender às minhas expectativas como consumidor.</t>
+  </si>
+  <si>
+    <t>Visita semestral foi agendada para dia 23/02 e não teve comparecimento do técnico e até o momento nenhum retorno por parte da Brastemp.</t>
+  </si>
+  <si>
+    <t>Instalador competente, contudo chegou às 13:30h, fora do horário agendado - manhã.</t>
+  </si>
+  <si>
+    <t>Fiquei mais de uma semana sem poder usar o filtro....água com gosto e cheiro podre. Nao me atenderam com a urgência esperada.</t>
+  </si>
+  <si>
+    <t>Profissional que foi até o local muito atencioso</t>
+  </si>
+  <si>
+    <t>Prazop de manutenção  horrivel</t>
   </si>
 </sst>
 </file>
@@ -2070,7 +2280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I468"/>
+  <dimension ref="A1:I530"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -15656,6 +15866,1804 @@
         <v>51</v>
       </c>
     </row>
+    <row r="469" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A469">
+        <v>468</v>
+      </c>
+      <c r="B469" t="s">
+        <v>9</v>
+      </c>
+      <c r="C469">
+        <v>8005298818</v>
+      </c>
+      <c r="D469" s="3">
+        <v>46074.697604166657</v>
+      </c>
+      <c r="E469" t="s">
+        <v>20</v>
+      </c>
+      <c r="F469" t="s">
+        <v>16</v>
+      </c>
+      <c r="G469" t="s">
+        <v>533</v>
+      </c>
+      <c r="H469" t="s">
+        <v>32</v>
+      </c>
+      <c r="I469" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="470" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A470">
+        <v>469</v>
+      </c>
+      <c r="B470" t="s">
+        <v>9</v>
+      </c>
+      <c r="C470">
+        <v>8005290120</v>
+      </c>
+      <c r="D470" s="3">
+        <v>46075.612141203703</v>
+      </c>
+      <c r="E470" t="s">
+        <v>20</v>
+      </c>
+      <c r="F470" t="s">
+        <v>16</v>
+      </c>
+      <c r="G470" t="s">
+        <v>534</v>
+      </c>
+      <c r="H470" t="s">
+        <v>18</v>
+      </c>
+      <c r="I470" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="471" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A471">
+        <v>470</v>
+      </c>
+      <c r="B471" t="s">
+        <v>9</v>
+      </c>
+      <c r="C471">
+        <v>8005310412</v>
+      </c>
+      <c r="D471" s="3">
+        <v>46076.404421296298</v>
+      </c>
+      <c r="E471" t="s">
+        <v>262</v>
+      </c>
+      <c r="F471" t="s">
+        <v>11</v>
+      </c>
+      <c r="G471" t="s">
+        <v>535</v>
+      </c>
+      <c r="H471" t="s">
+        <v>35</v>
+      </c>
+      <c r="I471" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="472" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A472">
+        <v>471</v>
+      </c>
+      <c r="B472" t="s">
+        <v>9</v>
+      </c>
+      <c r="C472">
+        <v>8005312399</v>
+      </c>
+      <c r="D472" s="3">
+        <v>46076.443124999998</v>
+      </c>
+      <c r="E472" t="s">
+        <v>65</v>
+      </c>
+      <c r="F472" t="s">
+        <v>16</v>
+      </c>
+      <c r="G472" t="s">
+        <v>536</v>
+      </c>
+      <c r="H472" t="s">
+        <v>35</v>
+      </c>
+      <c r="I472" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="473" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A473">
+        <v>472</v>
+      </c>
+      <c r="B473" t="s">
+        <v>9</v>
+      </c>
+      <c r="C473">
+        <v>8005313226</v>
+      </c>
+      <c r="D473" s="3">
+        <v>46076.509652777779</v>
+      </c>
+      <c r="E473" t="s">
+        <v>20</v>
+      </c>
+      <c r="F473" t="s">
+        <v>16</v>
+      </c>
+      <c r="G473" t="s">
+        <v>537</v>
+      </c>
+      <c r="H473" t="s">
+        <v>35</v>
+      </c>
+      <c r="I473" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="474" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A474">
+        <v>473</v>
+      </c>
+      <c r="B474" t="s">
+        <v>9</v>
+      </c>
+      <c r="C474">
+        <v>8005308180</v>
+      </c>
+      <c r="D474" s="3">
+        <v>46076.573078703703</v>
+      </c>
+      <c r="E474" t="s">
+        <v>20</v>
+      </c>
+      <c r="F474" t="s">
+        <v>16</v>
+      </c>
+      <c r="G474" t="s">
+        <v>538</v>
+      </c>
+      <c r="H474" t="s">
+        <v>154</v>
+      </c>
+      <c r="I474" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="475" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A475">
+        <v>474</v>
+      </c>
+      <c r="B475" t="s">
+        <v>9</v>
+      </c>
+      <c r="C475">
+        <v>8005310689</v>
+      </c>
+      <c r="D475" s="3">
+        <v>46076.631215277783</v>
+      </c>
+      <c r="E475" t="s">
+        <v>20</v>
+      </c>
+      <c r="F475" t="s">
+        <v>16</v>
+      </c>
+      <c r="G475" t="s">
+        <v>539</v>
+      </c>
+      <c r="H475" t="s">
+        <v>32</v>
+      </c>
+      <c r="I475" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="476" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A476">
+        <v>475</v>
+      </c>
+      <c r="B476" t="s">
+        <v>9</v>
+      </c>
+      <c r="C476">
+        <v>8005285314</v>
+      </c>
+      <c r="D476" s="3">
+        <v>46076.695902777778</v>
+      </c>
+      <c r="E476" t="s">
+        <v>20</v>
+      </c>
+      <c r="F476" t="s">
+        <v>11</v>
+      </c>
+      <c r="G476" t="s">
+        <v>540</v>
+      </c>
+      <c r="H476" t="s">
+        <v>82</v>
+      </c>
+      <c r="I476" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="477" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A477">
+        <v>476</v>
+      </c>
+      <c r="B477" t="s">
+        <v>9</v>
+      </c>
+      <c r="C477">
+        <v>8005312286</v>
+      </c>
+      <c r="D477" s="3">
+        <v>46076.700821759259</v>
+      </c>
+      <c r="E477" t="s">
+        <v>98</v>
+      </c>
+      <c r="F477" t="s">
+        <v>11</v>
+      </c>
+      <c r="G477" t="s">
+        <v>541</v>
+      </c>
+      <c r="H477" t="s">
+        <v>18</v>
+      </c>
+      <c r="I477" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="478" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A478">
+        <v>477</v>
+      </c>
+      <c r="B478" t="s">
+        <v>9</v>
+      </c>
+      <c r="C478">
+        <v>346</v>
+      </c>
+      <c r="D478" s="3">
+        <v>46077.467719907407</v>
+      </c>
+      <c r="E478" t="s">
+        <v>542</v>
+      </c>
+      <c r="F478" t="s">
+        <v>16</v>
+      </c>
+      <c r="G478" t="s">
+        <v>543</v>
+      </c>
+      <c r="H478" t="s">
+        <v>18</v>
+      </c>
+      <c r="I478" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="479" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A479">
+        <v>478</v>
+      </c>
+      <c r="B479" t="s">
+        <v>9</v>
+      </c>
+      <c r="C479">
+        <v>8005289947</v>
+      </c>
+      <c r="D479" s="3">
+        <v>46077.485995370371</v>
+      </c>
+      <c r="E479" t="s">
+        <v>20</v>
+      </c>
+      <c r="F479" t="s">
+        <v>16</v>
+      </c>
+      <c r="G479" t="s">
+        <v>544</v>
+      </c>
+      <c r="H479" t="s">
+        <v>32</v>
+      </c>
+      <c r="I479" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="480" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A480">
+        <v>479</v>
+      </c>
+      <c r="B480" t="s">
+        <v>9</v>
+      </c>
+      <c r="C480">
+        <v>8005303148</v>
+      </c>
+      <c r="D480" s="3">
+        <v>46077.488657407397</v>
+      </c>
+      <c r="E480" t="s">
+        <v>53</v>
+      </c>
+      <c r="F480" t="s">
+        <v>16</v>
+      </c>
+      <c r="G480" t="s">
+        <v>545</v>
+      </c>
+      <c r="H480" t="s">
+        <v>18</v>
+      </c>
+      <c r="I480" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="481" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A481">
+        <v>480</v>
+      </c>
+      <c r="B481" t="s">
+        <v>9</v>
+      </c>
+      <c r="C481">
+        <v>333</v>
+      </c>
+      <c r="D481" s="3">
+        <v>46077.622407407413</v>
+      </c>
+      <c r="E481" t="s">
+        <v>546</v>
+      </c>
+      <c r="F481" t="s">
+        <v>11</v>
+      </c>
+      <c r="G481" t="s">
+        <v>547</v>
+      </c>
+      <c r="H481" t="s">
+        <v>18</v>
+      </c>
+      <c r="I481" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="482" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A482">
+        <v>481</v>
+      </c>
+      <c r="B482" t="s">
+        <v>61</v>
+      </c>
+      <c r="C482">
+        <v>792</v>
+      </c>
+      <c r="D482" s="3">
+        <v>46077.627071759263</v>
+      </c>
+      <c r="E482" t="s">
+        <v>548</v>
+      </c>
+      <c r="F482" t="s">
+        <v>16</v>
+      </c>
+      <c r="G482" t="s">
+        <v>549</v>
+      </c>
+      <c r="H482" t="s">
+        <v>18</v>
+      </c>
+      <c r="I482" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="483" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A483">
+        <v>482</v>
+      </c>
+      <c r="B483" t="s">
+        <v>9</v>
+      </c>
+      <c r="C483">
+        <v>585</v>
+      </c>
+      <c r="D483" s="3">
+        <v>46077.630706018521</v>
+      </c>
+      <c r="E483" t="s">
+        <v>550</v>
+      </c>
+      <c r="F483" t="s">
+        <v>11</v>
+      </c>
+      <c r="G483" t="s">
+        <v>551</v>
+      </c>
+      <c r="H483" t="s">
+        <v>35</v>
+      </c>
+      <c r="I483" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="484" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A484">
+        <v>483</v>
+      </c>
+      <c r="B484" t="s">
+        <v>9</v>
+      </c>
+      <c r="C484">
+        <v>8005298914</v>
+      </c>
+      <c r="D484" s="3">
+        <v>46077.631655092591</v>
+      </c>
+      <c r="E484" t="s">
+        <v>20</v>
+      </c>
+      <c r="F484" t="s">
+        <v>11</v>
+      </c>
+      <c r="G484" t="s">
+        <v>552</v>
+      </c>
+      <c r="H484" t="s">
+        <v>13</v>
+      </c>
+      <c r="I484" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="485" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A485">
+        <v>484</v>
+      </c>
+      <c r="B485" t="s">
+        <v>61</v>
+      </c>
+      <c r="C485">
+        <v>8005309748</v>
+      </c>
+      <c r="D485" s="3">
+        <v>46077.636701388888</v>
+      </c>
+      <c r="E485" t="s">
+        <v>20</v>
+      </c>
+      <c r="F485" t="s">
+        <v>16</v>
+      </c>
+      <c r="G485" t="s">
+        <v>553</v>
+      </c>
+      <c r="H485" t="s">
+        <v>154</v>
+      </c>
+      <c r="I485" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="486" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A486">
+        <v>485</v>
+      </c>
+      <c r="B486" t="s">
+        <v>9</v>
+      </c>
+      <c r="C486">
+        <v>3227</v>
+      </c>
+      <c r="D486" s="3">
+        <v>46077.645879629628</v>
+      </c>
+      <c r="E486" t="s">
+        <v>548</v>
+      </c>
+      <c r="F486" t="s">
+        <v>16</v>
+      </c>
+      <c r="G486" t="s">
+        <v>554</v>
+      </c>
+      <c r="H486" t="s">
+        <v>18</v>
+      </c>
+      <c r="I486" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="487" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A487">
+        <v>486</v>
+      </c>
+      <c r="B487" t="s">
+        <v>9</v>
+      </c>
+      <c r="C487">
+        <v>2718</v>
+      </c>
+      <c r="D487" s="3">
+        <v>46077.666539351849</v>
+      </c>
+      <c r="E487" t="s">
+        <v>542</v>
+      </c>
+      <c r="F487" t="s">
+        <v>11</v>
+      </c>
+      <c r="G487" t="s">
+        <v>555</v>
+      </c>
+      <c r="H487" t="s">
+        <v>154</v>
+      </c>
+      <c r="I487" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="488" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A488">
+        <v>487</v>
+      </c>
+      <c r="B488" t="s">
+        <v>9</v>
+      </c>
+      <c r="C488">
+        <v>243</v>
+      </c>
+      <c r="D488" s="3">
+        <v>46077.678518518522</v>
+      </c>
+      <c r="E488" t="s">
+        <v>556</v>
+      </c>
+      <c r="F488" t="s">
+        <v>16</v>
+      </c>
+      <c r="G488" t="s">
+        <v>557</v>
+      </c>
+      <c r="H488" t="s">
+        <v>18</v>
+      </c>
+      <c r="I488" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="489" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A489">
+        <v>488</v>
+      </c>
+      <c r="B489" t="s">
+        <v>9</v>
+      </c>
+      <c r="C489">
+        <v>8005222999</v>
+      </c>
+      <c r="D489" s="3">
+        <v>46077.684618055559</v>
+      </c>
+      <c r="E489" t="s">
+        <v>15</v>
+      </c>
+      <c r="F489" t="s">
+        <v>11</v>
+      </c>
+      <c r="G489" t="s">
+        <v>558</v>
+      </c>
+      <c r="H489" t="s">
+        <v>18</v>
+      </c>
+      <c r="I489" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="490" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A490">
+        <v>489</v>
+      </c>
+      <c r="B490" t="s">
+        <v>9</v>
+      </c>
+      <c r="C490">
+        <v>305</v>
+      </c>
+      <c r="D490" s="3">
+        <v>46077.729398148149</v>
+      </c>
+      <c r="E490" t="s">
+        <v>542</v>
+      </c>
+      <c r="F490" t="s">
+        <v>11</v>
+      </c>
+      <c r="G490" t="s">
+        <v>559</v>
+      </c>
+      <c r="H490" t="s">
+        <v>13</v>
+      </c>
+      <c r="I490" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="491" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A491">
+        <v>490</v>
+      </c>
+      <c r="B491" t="s">
+        <v>9</v>
+      </c>
+      <c r="C491">
+        <v>8005311006</v>
+      </c>
+      <c r="D491" s="3">
+        <v>46077.732361111113</v>
+      </c>
+      <c r="E491" t="s">
+        <v>53</v>
+      </c>
+      <c r="F491" t="s">
+        <v>16</v>
+      </c>
+      <c r="G491" t="s">
+        <v>560</v>
+      </c>
+      <c r="H491" t="s">
+        <v>18</v>
+      </c>
+      <c r="I491" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="492" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A492">
+        <v>491</v>
+      </c>
+      <c r="B492" t="s">
+        <v>9</v>
+      </c>
+      <c r="C492">
+        <v>8005288543</v>
+      </c>
+      <c r="D492" s="3">
+        <v>46077.754548611112</v>
+      </c>
+      <c r="E492" t="s">
+        <v>53</v>
+      </c>
+      <c r="F492" t="s">
+        <v>11</v>
+      </c>
+      <c r="G492" t="s">
+        <v>561</v>
+      </c>
+      <c r="H492" t="s">
+        <v>13</v>
+      </c>
+      <c r="I492" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="493" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A493">
+        <v>492</v>
+      </c>
+      <c r="B493" t="s">
+        <v>9</v>
+      </c>
+      <c r="C493">
+        <v>2797</v>
+      </c>
+      <c r="D493" s="3">
+        <v>46077.76966435185</v>
+      </c>
+      <c r="E493" t="s">
+        <v>556</v>
+      </c>
+      <c r="F493" t="s">
+        <v>16</v>
+      </c>
+      <c r="G493" t="s">
+        <v>562</v>
+      </c>
+      <c r="H493" t="s">
+        <v>18</v>
+      </c>
+      <c r="I493" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="494" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A494">
+        <v>493</v>
+      </c>
+      <c r="B494" t="s">
+        <v>9</v>
+      </c>
+      <c r="C494">
+        <v>8005280980</v>
+      </c>
+      <c r="D494" s="3">
+        <v>46078.316701388889</v>
+      </c>
+      <c r="E494" t="s">
+        <v>20</v>
+      </c>
+      <c r="F494" t="s">
+        <v>16</v>
+      </c>
+      <c r="G494" t="s">
+        <v>563</v>
+      </c>
+      <c r="H494" t="s">
+        <v>154</v>
+      </c>
+      <c r="I494" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="495" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A495">
+        <v>494</v>
+      </c>
+      <c r="B495" t="s">
+        <v>9</v>
+      </c>
+      <c r="C495">
+        <v>8005309338</v>
+      </c>
+      <c r="D495" s="3">
+        <v>46078.41615740741</v>
+      </c>
+      <c r="E495" t="s">
+        <v>224</v>
+      </c>
+      <c r="F495" t="s">
+        <v>16</v>
+      </c>
+      <c r="G495" t="s">
+        <v>564</v>
+      </c>
+      <c r="H495" t="s">
+        <v>18</v>
+      </c>
+      <c r="I495" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="496" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A496">
+        <v>495</v>
+      </c>
+      <c r="B496" t="s">
+        <v>9</v>
+      </c>
+      <c r="C496">
+        <v>8005292743</v>
+      </c>
+      <c r="D496" s="3">
+        <v>46078.504942129628</v>
+      </c>
+      <c r="E496" t="s">
+        <v>20</v>
+      </c>
+      <c r="F496" t="s">
+        <v>16</v>
+      </c>
+      <c r="G496" t="s">
+        <v>565</v>
+      </c>
+      <c r="H496" t="s">
+        <v>154</v>
+      </c>
+      <c r="I496" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="497" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A497">
+        <v>496</v>
+      </c>
+      <c r="B497" t="s">
+        <v>9</v>
+      </c>
+      <c r="C497">
+        <v>8005308644</v>
+      </c>
+      <c r="D497" s="3">
+        <v>46078.521979166668</v>
+      </c>
+      <c r="E497" t="s">
+        <v>53</v>
+      </c>
+      <c r="F497" t="s">
+        <v>16</v>
+      </c>
+      <c r="G497" t="s">
+        <v>566</v>
+      </c>
+      <c r="H497" t="s">
+        <v>18</v>
+      </c>
+      <c r="I497" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="498" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A498">
+        <v>497</v>
+      </c>
+      <c r="B498" t="s">
+        <v>9</v>
+      </c>
+      <c r="C498">
+        <v>8005297149</v>
+      </c>
+      <c r="D498" s="3">
+        <v>46078.53769675926</v>
+      </c>
+      <c r="E498" t="s">
+        <v>74</v>
+      </c>
+      <c r="F498" t="s">
+        <v>16</v>
+      </c>
+      <c r="G498" t="s">
+        <v>567</v>
+      </c>
+      <c r="H498" t="s">
+        <v>18</v>
+      </c>
+      <c r="I498" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="499" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A499">
+        <v>498</v>
+      </c>
+      <c r="B499" t="s">
+        <v>9</v>
+      </c>
+      <c r="C499">
+        <v>8005313678</v>
+      </c>
+      <c r="D499" s="3">
+        <v>46078.544722222221</v>
+      </c>
+      <c r="E499" t="s">
+        <v>98</v>
+      </c>
+      <c r="F499" t="s">
+        <v>16</v>
+      </c>
+      <c r="G499" t="s">
+        <v>568</v>
+      </c>
+      <c r="H499" t="s">
+        <v>154</v>
+      </c>
+      <c r="I499" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="500" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A500">
+        <v>499</v>
+      </c>
+      <c r="B500" t="s">
+        <v>9</v>
+      </c>
+      <c r="C500">
+        <v>8005285501</v>
+      </c>
+      <c r="D500" s="3">
+        <v>46078.579328703701</v>
+      </c>
+      <c r="E500" t="s">
+        <v>49</v>
+      </c>
+      <c r="F500" t="s">
+        <v>11</v>
+      </c>
+      <c r="G500" t="s">
+        <v>569</v>
+      </c>
+      <c r="H500" t="s">
+        <v>13</v>
+      </c>
+      <c r="I500" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="501" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A501">
+        <v>500</v>
+      </c>
+      <c r="B501" t="s">
+        <v>9</v>
+      </c>
+      <c r="C501">
+        <v>8005289398</v>
+      </c>
+      <c r="D501" s="3">
+        <v>46078.667118055557</v>
+      </c>
+      <c r="E501" t="s">
+        <v>20</v>
+      </c>
+      <c r="F501" t="s">
+        <v>11</v>
+      </c>
+      <c r="G501" t="s">
+        <v>570</v>
+      </c>
+      <c r="H501" t="s">
+        <v>32</v>
+      </c>
+      <c r="I501" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="502" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A502">
+        <v>501</v>
+      </c>
+      <c r="B502" t="s">
+        <v>9</v>
+      </c>
+      <c r="C502">
+        <v>705</v>
+      </c>
+      <c r="D502" s="3">
+        <v>46079.381585648152</v>
+      </c>
+      <c r="E502" t="s">
+        <v>556</v>
+      </c>
+      <c r="F502" t="s">
+        <v>16</v>
+      </c>
+      <c r="G502" t="s">
+        <v>571</v>
+      </c>
+      <c r="H502" t="s">
+        <v>18</v>
+      </c>
+      <c r="I502" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="503" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A503">
+        <v>502</v>
+      </c>
+      <c r="B503" t="s">
+        <v>61</v>
+      </c>
+      <c r="C503">
+        <v>8005312020</v>
+      </c>
+      <c r="D503" s="3">
+        <v>46079.428368055553</v>
+      </c>
+      <c r="E503" t="s">
+        <v>37</v>
+      </c>
+      <c r="F503" t="s">
+        <v>16</v>
+      </c>
+      <c r="G503" t="s">
+        <v>572</v>
+      </c>
+      <c r="H503" t="s">
+        <v>18</v>
+      </c>
+      <c r="I503" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="504" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A504">
+        <v>503</v>
+      </c>
+      <c r="B504" t="s">
+        <v>9</v>
+      </c>
+      <c r="C504">
+        <v>76</v>
+      </c>
+      <c r="D504" s="3">
+        <v>46079.474421296298</v>
+      </c>
+      <c r="E504" t="s">
+        <v>550</v>
+      </c>
+      <c r="F504" t="s">
+        <v>16</v>
+      </c>
+      <c r="G504" t="s">
+        <v>573</v>
+      </c>
+      <c r="H504" t="s">
+        <v>18</v>
+      </c>
+      <c r="I504" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="505" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A505">
+        <v>504</v>
+      </c>
+      <c r="B505" t="s">
+        <v>9</v>
+      </c>
+      <c r="C505">
+        <v>8005299894</v>
+      </c>
+      <c r="D505" s="3">
+        <v>46079.501643518517</v>
+      </c>
+      <c r="E505" t="s">
+        <v>65</v>
+      </c>
+      <c r="F505" t="s">
+        <v>11</v>
+      </c>
+      <c r="G505" t="s">
+        <v>574</v>
+      </c>
+      <c r="H505" t="s">
+        <v>32</v>
+      </c>
+      <c r="I505" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="506" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A506">
+        <v>505</v>
+      </c>
+      <c r="B506" t="s">
+        <v>61</v>
+      </c>
+      <c r="C506">
+        <v>4296</v>
+      </c>
+      <c r="D506" s="3">
+        <v>46079.508009259262</v>
+      </c>
+      <c r="E506" t="s">
+        <v>548</v>
+      </c>
+      <c r="F506" t="s">
+        <v>16</v>
+      </c>
+      <c r="G506" t="s">
+        <v>575</v>
+      </c>
+      <c r="H506" t="s">
+        <v>35</v>
+      </c>
+      <c r="I506" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="507" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A507">
+        <v>506</v>
+      </c>
+      <c r="B507" t="s">
+        <v>9</v>
+      </c>
+      <c r="C507">
+        <v>8005310487</v>
+      </c>
+      <c r="D507" s="3">
+        <v>46079.508518518523</v>
+      </c>
+      <c r="E507" t="s">
+        <v>15</v>
+      </c>
+      <c r="F507" t="s">
+        <v>11</v>
+      </c>
+      <c r="G507" t="s">
+        <v>576</v>
+      </c>
+      <c r="H507" t="s">
+        <v>35</v>
+      </c>
+      <c r="I507" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="508" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A508">
+        <v>507</v>
+      </c>
+      <c r="B508" t="s">
+        <v>9</v>
+      </c>
+      <c r="C508">
+        <v>8005292702</v>
+      </c>
+      <c r="D508" s="3">
+        <v>46079.508877314824</v>
+      </c>
+      <c r="E508" t="s">
+        <v>37</v>
+      </c>
+      <c r="F508" t="s">
+        <v>11</v>
+      </c>
+      <c r="G508" t="s">
+        <v>577</v>
+      </c>
+      <c r="H508" t="s">
+        <v>35</v>
+      </c>
+      <c r="I508" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="509" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A509">
+        <v>508</v>
+      </c>
+      <c r="B509" t="s">
+        <v>9</v>
+      </c>
+      <c r="C509">
+        <v>8005263351</v>
+      </c>
+      <c r="D509" s="3">
+        <v>46079.531041666669</v>
+      </c>
+      <c r="E509" t="s">
+        <v>41</v>
+      </c>
+      <c r="F509" t="s">
+        <v>11</v>
+      </c>
+      <c r="G509" t="s">
+        <v>578</v>
+      </c>
+      <c r="H509" t="s">
+        <v>13</v>
+      </c>
+      <c r="I509" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="510" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A510">
+        <v>509</v>
+      </c>
+      <c r="B510" t="s">
+        <v>9</v>
+      </c>
+      <c r="C510">
+        <v>3168</v>
+      </c>
+      <c r="D510" s="3">
+        <v>46079.643460648149</v>
+      </c>
+      <c r="E510" t="s">
+        <v>548</v>
+      </c>
+      <c r="F510" t="s">
+        <v>16</v>
+      </c>
+      <c r="G510" t="s">
+        <v>579</v>
+      </c>
+      <c r="H510" t="s">
+        <v>13</v>
+      </c>
+      <c r="I510" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="511" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A511">
+        <v>510</v>
+      </c>
+      <c r="B511" t="s">
+        <v>9</v>
+      </c>
+      <c r="C511">
+        <v>302</v>
+      </c>
+      <c r="D511" s="3">
+        <v>46079.687083333331</v>
+      </c>
+      <c r="E511" t="s">
+        <v>556</v>
+      </c>
+      <c r="F511" t="s">
+        <v>16</v>
+      </c>
+      <c r="G511" t="s">
+        <v>580</v>
+      </c>
+      <c r="H511" t="s">
+        <v>18</v>
+      </c>
+      <c r="I511" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="512" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A512">
+        <v>511</v>
+      </c>
+      <c r="B512" t="s">
+        <v>9</v>
+      </c>
+      <c r="C512">
+        <v>8005303918</v>
+      </c>
+      <c r="D512" s="3">
+        <v>46079.869016203702</v>
+      </c>
+      <c r="E512" t="s">
+        <v>37</v>
+      </c>
+      <c r="F512" t="s">
+        <v>16</v>
+      </c>
+      <c r="G512" t="s">
+        <v>581</v>
+      </c>
+      <c r="H512" t="s">
+        <v>154</v>
+      </c>
+      <c r="I512" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="513" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A513">
+        <v>512</v>
+      </c>
+      <c r="B513" t="s">
+        <v>9</v>
+      </c>
+      <c r="C513">
+        <v>930</v>
+      </c>
+      <c r="D513" s="3">
+        <v>46080.484571759262</v>
+      </c>
+      <c r="E513" t="s">
+        <v>582</v>
+      </c>
+      <c r="F513" t="s">
+        <v>11</v>
+      </c>
+      <c r="G513" t="s">
+        <v>583</v>
+      </c>
+      <c r="H513" t="s">
+        <v>13</v>
+      </c>
+      <c r="I513" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="514" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A514">
+        <v>513</v>
+      </c>
+      <c r="B514" t="s">
+        <v>9</v>
+      </c>
+      <c r="C514">
+        <v>8005315212</v>
+      </c>
+      <c r="D514" s="3">
+        <v>46080.491064814807</v>
+      </c>
+      <c r="E514" t="s">
+        <v>37</v>
+      </c>
+      <c r="F514" t="s">
+        <v>16</v>
+      </c>
+      <c r="G514" t="s">
+        <v>584</v>
+      </c>
+      <c r="H514" t="s">
+        <v>154</v>
+      </c>
+      <c r="I514" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="515" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A515">
+        <v>514</v>
+      </c>
+      <c r="B515" t="s">
+        <v>9</v>
+      </c>
+      <c r="C515">
+        <v>4389</v>
+      </c>
+      <c r="D515" s="3">
+        <v>46080.519525462973</v>
+      </c>
+      <c r="E515" t="s">
+        <v>585</v>
+      </c>
+      <c r="F515" t="s">
+        <v>16</v>
+      </c>
+      <c r="G515" t="s">
+        <v>586</v>
+      </c>
+      <c r="H515" t="s">
+        <v>82</v>
+      </c>
+      <c r="I515" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="516" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A516">
+        <v>515</v>
+      </c>
+      <c r="B516" t="s">
+        <v>9</v>
+      </c>
+      <c r="C516">
+        <v>8005297736</v>
+      </c>
+      <c r="D516" s="3">
+        <v>46080.535000000003</v>
+      </c>
+      <c r="E516" t="s">
+        <v>37</v>
+      </c>
+      <c r="F516" t="s">
+        <v>11</v>
+      </c>
+      <c r="G516" t="s">
+        <v>587</v>
+      </c>
+      <c r="H516" t="s">
+        <v>13</v>
+      </c>
+      <c r="I516" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="517" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A517">
+        <v>516</v>
+      </c>
+      <c r="B517" t="s">
+        <v>9</v>
+      </c>
+      <c r="C517">
+        <v>8005313321</v>
+      </c>
+      <c r="D517" s="3">
+        <v>46080.536909722221</v>
+      </c>
+      <c r="E517" t="s">
+        <v>262</v>
+      </c>
+      <c r="F517" t="s">
+        <v>11</v>
+      </c>
+      <c r="G517" t="s">
+        <v>588</v>
+      </c>
+      <c r="H517" t="s">
+        <v>18</v>
+      </c>
+      <c r="I517" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="518" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A518">
+        <v>517</v>
+      </c>
+      <c r="B518" t="s">
+        <v>61</v>
+      </c>
+      <c r="C518">
+        <v>8005306724</v>
+      </c>
+      <c r="D518" s="3">
+        <v>46080.545578703714</v>
+      </c>
+      <c r="E518" t="s">
+        <v>15</v>
+      </c>
+      <c r="F518" t="s">
+        <v>11</v>
+      </c>
+      <c r="G518" t="s">
+        <v>589</v>
+      </c>
+      <c r="H518" t="s">
+        <v>18</v>
+      </c>
+      <c r="I518" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="519" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A519">
+        <v>518</v>
+      </c>
+      <c r="B519" t="s">
+        <v>9</v>
+      </c>
+      <c r="C519">
+        <v>965</v>
+      </c>
+      <c r="D519" s="3">
+        <v>46080.555254629631</v>
+      </c>
+      <c r="E519" t="s">
+        <v>590</v>
+      </c>
+      <c r="F519" t="s">
+        <v>16</v>
+      </c>
+      <c r="G519" t="s">
+        <v>591</v>
+      </c>
+      <c r="H519" t="s">
+        <v>18</v>
+      </c>
+      <c r="I519" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="520" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A520">
+        <v>519</v>
+      </c>
+      <c r="B520" t="s">
+        <v>9</v>
+      </c>
+      <c r="C520">
+        <v>8005296092</v>
+      </c>
+      <c r="D520" s="3">
+        <v>46080.557002314818</v>
+      </c>
+      <c r="E520" t="s">
+        <v>53</v>
+      </c>
+      <c r="F520" t="s">
+        <v>16</v>
+      </c>
+      <c r="G520" t="s">
+        <v>592</v>
+      </c>
+      <c r="H520" t="s">
+        <v>32</v>
+      </c>
+      <c r="I520" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="521" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A521">
+        <v>520</v>
+      </c>
+      <c r="B521" t="s">
+        <v>9</v>
+      </c>
+      <c r="C521">
+        <v>8005312799</v>
+      </c>
+      <c r="D521" s="3">
+        <v>46080.562789351847</v>
+      </c>
+      <c r="E521" t="s">
+        <v>53</v>
+      </c>
+      <c r="F521" t="s">
+        <v>16</v>
+      </c>
+      <c r="G521" t="s">
+        <v>593</v>
+      </c>
+      <c r="H521" t="s">
+        <v>35</v>
+      </c>
+      <c r="I521" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="522" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A522">
+        <v>521</v>
+      </c>
+      <c r="B522" t="s">
+        <v>61</v>
+      </c>
+      <c r="C522">
+        <v>3382</v>
+      </c>
+      <c r="D522" s="3">
+        <v>46080.577615740738</v>
+      </c>
+      <c r="E522" t="s">
+        <v>556</v>
+      </c>
+      <c r="F522" t="s">
+        <v>16</v>
+      </c>
+      <c r="G522" t="s">
+        <v>594</v>
+      </c>
+      <c r="H522" t="s">
+        <v>35</v>
+      </c>
+      <c r="I522" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="523" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A523">
+        <v>522</v>
+      </c>
+      <c r="B523" t="s">
+        <v>61</v>
+      </c>
+      <c r="C523">
+        <v>8005312593</v>
+      </c>
+      <c r="D523" s="3">
+        <v>46080.699421296304</v>
+      </c>
+      <c r="E523" t="s">
+        <v>20</v>
+      </c>
+      <c r="F523" t="s">
+        <v>16</v>
+      </c>
+      <c r="G523" t="s">
+        <v>595</v>
+      </c>
+      <c r="H523" t="s">
+        <v>63</v>
+      </c>
+      <c r="I523" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="524" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A524">
+        <v>523</v>
+      </c>
+      <c r="B524" t="s">
+        <v>9</v>
+      </c>
+      <c r="C524">
+        <v>8005314473</v>
+      </c>
+      <c r="D524" s="3">
+        <v>46080.725173611107</v>
+      </c>
+      <c r="E524" t="s">
+        <v>20</v>
+      </c>
+      <c r="F524" t="s">
+        <v>16</v>
+      </c>
+      <c r="G524" t="s">
+        <v>596</v>
+      </c>
+      <c r="H524" t="s">
+        <v>18</v>
+      </c>
+      <c r="I524" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="525" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A525">
+        <v>524</v>
+      </c>
+      <c r="B525" t="s">
+        <v>9</v>
+      </c>
+      <c r="C525">
+        <v>8005306799</v>
+      </c>
+      <c r="D525" s="3">
+        <v>46080.731087962973</v>
+      </c>
+      <c r="E525" t="s">
+        <v>224</v>
+      </c>
+      <c r="F525" t="s">
+        <v>11</v>
+      </c>
+      <c r="G525" t="s">
+        <v>597</v>
+      </c>
+      <c r="H525" t="s">
+        <v>18</v>
+      </c>
+      <c r="I525" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="526" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A526">
+        <v>525</v>
+      </c>
+      <c r="B526" t="s">
+        <v>9</v>
+      </c>
+      <c r="C526">
+        <v>8005261486</v>
+      </c>
+      <c r="D526" s="3">
+        <v>46080.774039351847</v>
+      </c>
+      <c r="E526" t="s">
+        <v>53</v>
+      </c>
+      <c r="F526" t="s">
+        <v>16</v>
+      </c>
+      <c r="G526" t="s">
+        <v>598</v>
+      </c>
+      <c r="H526" t="s">
+        <v>18</v>
+      </c>
+      <c r="I526" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="527" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A527">
+        <v>526</v>
+      </c>
+      <c r="B527" t="s">
+        <v>9</v>
+      </c>
+      <c r="C527">
+        <v>236</v>
+      </c>
+      <c r="D527" s="3">
+        <v>46080.781064814822</v>
+      </c>
+      <c r="E527" t="s">
+        <v>550</v>
+      </c>
+      <c r="F527" t="s">
+        <v>16</v>
+      </c>
+      <c r="G527" t="s">
+        <v>599</v>
+      </c>
+      <c r="H527" t="s">
+        <v>18</v>
+      </c>
+      <c r="I527" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="528" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A528">
+        <v>527</v>
+      </c>
+      <c r="B528" t="s">
+        <v>9</v>
+      </c>
+      <c r="C528">
+        <v>146</v>
+      </c>
+      <c r="D528" s="3">
+        <v>46080.838101851848</v>
+      </c>
+      <c r="E528" t="s">
+        <v>548</v>
+      </c>
+      <c r="F528" t="s">
+        <v>16</v>
+      </c>
+      <c r="G528" t="s">
+        <v>600</v>
+      </c>
+      <c r="H528" t="s">
+        <v>35</v>
+      </c>
+      <c r="I528" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="529" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A529">
+        <v>528</v>
+      </c>
+      <c r="B529" t="s">
+        <v>9</v>
+      </c>
+      <c r="C529">
+        <v>8005261322</v>
+      </c>
+      <c r="D529" s="3">
+        <v>46081.43246527778</v>
+      </c>
+      <c r="E529" t="s">
+        <v>41</v>
+      </c>
+      <c r="F529" t="s">
+        <v>11</v>
+      </c>
+      <c r="G529" t="s">
+        <v>601</v>
+      </c>
+      <c r="H529" t="s">
+        <v>18</v>
+      </c>
+      <c r="I529" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="530" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A530">
+        <v>529</v>
+      </c>
+      <c r="B530" t="s">
+        <v>9</v>
+      </c>
+      <c r="C530">
+        <v>699</v>
+      </c>
+      <c r="D530" s="3">
+        <v>46081.469490740739</v>
+      </c>
+      <c r="E530" t="s">
+        <v>546</v>
+      </c>
+      <c r="F530" t="s">
+        <v>16</v>
+      </c>
+      <c r="G530" t="s">
+        <v>602</v>
+      </c>
+      <c r="H530" t="s">
+        <v>32</v>
+      </c>
+      <c r="I530" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/03/2026 14:53:19,20
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4646C255-73DE-4858-8388-A8AB6406C629}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9B756BA-C28F-4004-A26C-D0CF641248BE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3183" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="606">
   <si>
     <t>ID</t>
   </si>
@@ -1912,6 +1912,15 @@
   </si>
   <si>
     <t>Prazop de manutenção  horrivel</t>
+  </si>
+  <si>
+    <t>Não foi resolvido. A máquina não gela. Não tem peça de reposição. Continua sem solução. Quero trocar por outro modelo, imediatamente.</t>
+  </si>
+  <si>
+    <t>Esperei tanto pela troca do filtro e o o mesmo vem com defeito. A brastemp deveria testar seus produtos novos, isso deixa o cliente decepcionado. Agora ... mais uns dias pra nova troca!!?? Nao posso crucificar o técnico.  Mas tenho que dar nota baixa.</t>
+  </si>
+  <si>
+    <t>O rapaz estalou o aparelho mais ainda não usei porque ficou faltando uma peça o conector (alongador) ainda não vieram colocar e o dia da cobrança está rolando espero que eu possa usar e ter um desconto nos dias que não estou usando.Estalaram dia 24/02/26Colocar alongador 03/03/26Fico no aguardo.</t>
   </si>
 </sst>
 </file>
@@ -2280,7 +2289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I530"/>
+  <dimension ref="A1:I533"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -17664,6 +17673,93 @@
         <v>33</v>
       </c>
     </row>
+    <row r="531" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A531">
+        <v>530</v>
+      </c>
+      <c r="B531" t="s">
+        <v>61</v>
+      </c>
+      <c r="C531">
+        <v>8005312278</v>
+      </c>
+      <c r="D531" s="3">
+        <v>46081.469490740739</v>
+      </c>
+      <c r="E531" t="s">
+        <v>53</v>
+      </c>
+      <c r="F531" t="s">
+        <v>16</v>
+      </c>
+      <c r="G531" t="s">
+        <v>605</v>
+      </c>
+      <c r="H531" t="s">
+        <v>18</v>
+      </c>
+      <c r="I531" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="532" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A532">
+        <v>531</v>
+      </c>
+      <c r="B532" t="s">
+        <v>9</v>
+      </c>
+      <c r="C532">
+        <v>8005311935</v>
+      </c>
+      <c r="D532" s="3">
+        <v>46081.469490740739</v>
+      </c>
+      <c r="E532" t="s">
+        <v>53</v>
+      </c>
+      <c r="F532" t="s">
+        <v>16</v>
+      </c>
+      <c r="G532" t="s">
+        <v>603</v>
+      </c>
+      <c r="H532" t="s">
+        <v>35</v>
+      </c>
+      <c r="I532" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="533" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A533">
+        <v>532</v>
+      </c>
+      <c r="B533" t="s">
+        <v>9</v>
+      </c>
+      <c r="C533">
+        <v>8005299947</v>
+      </c>
+      <c r="D533" s="3">
+        <v>46081.469490740739</v>
+      </c>
+      <c r="E533" t="s">
+        <v>37</v>
+      </c>
+      <c r="F533" t="s">
+        <v>11</v>
+      </c>
+      <c r="G533" t="s">
+        <v>604</v>
+      </c>
+      <c r="H533" t="s">
+        <v>35</v>
+      </c>
+      <c r="I533" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/03/2026 10:55:12,39
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9B756BA-C28F-4004-A26C-D0CF641248BE}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04F45B61-AE6F-495D-AF0A-0A483857EF16}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$533</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="678">
   <si>
     <t>ID</t>
   </si>
@@ -1921,6 +1921,249 @@
   </si>
   <si>
     <t>O rapaz estalou o aparelho mais ainda não usei porque ficou faltando uma peça o conector (alongador) ainda não vieram colocar e o dia da cobrança está rolando espero que eu possa usar e ter um desconto nos dias que não estou usando.Estalaram dia 24/02/26Colocar alongador 03/03/26Fico no aguardo.</t>
+  </si>
+  <si>
+    <t>Muita demora do atendimento. Tive que comprar água para beber 
+Demora de um mês para o atendimento 
+Não pode demorar tanto 
+Peço urgência no atendimento</t>
+  </si>
+  <si>
+    <t>O técnico trocou o compressor, mas não resolveu. Desde que trocaram o equipamento, que estamos convivendo com o problema. Água gelada sai natural, e a natural sai morna.</t>
+  </si>
+  <si>
+    <t>O aparelho instalado dia 27 e no dia 28 já não funciona mais</t>
+  </si>
+  <si>
+    <t>Qualidade do produto</t>
+  </si>
+  <si>
+    <t>Foi muito bom no início e agora nos últimos anos a manutenção ficou um pouco a desejar. Não é feito mais a limpeza do filtro somente a troca de filtro. E a marcação que era feita de 6 em 6 meses também não é feita regularmente. Anteriormente era certinho sempre no período certo</t>
+  </si>
+  <si>
+    <t>Foram no local errado e o prazo manutenção é de 30
+Dias</t>
+  </si>
+  <si>
+    <t>CAPACIDADE</t>
+  </si>
+  <si>
+    <t>Está deixando a desejar</t>
+  </si>
+  <si>
+    <t>Meu aparelho até desde quando foi instalado nao para de pingar. Não conseguem resolver.</t>
+  </si>
+  <si>
+    <t>Muito prático.</t>
+  </si>
+  <si>
+    <t>FRQ BASE LESTE SP R02</t>
+  </si>
+  <si>
+    <t>Pedi para trocar a vela porque esta com gosto ruim e nao foi trocada.</t>
+  </si>
+  <si>
+    <t>água muito gostosa, poderia ser um pouco mais barata.</t>
+  </si>
+  <si>
+    <t>O técnico foi super eficiente mas o filtro não funciona na agua gelada</t>
+  </si>
+  <si>
+    <t>Atendendimento SAC é pessimo, visita tecnica é otima</t>
+  </si>
+  <si>
+    <t>Água com cheiro estranho e gosto diferente do normal. Estamos utilizando apenas para limpeza, pois não está potável pelo que referimos.</t>
+  </si>
+  <si>
+    <t>O técnico diagnosticou e resolveu o problema. A questão é que o purificador foi trocado 2 vezes por equipamento "novo", saído da caixa, e os dois apresentaram problema. Ou seja, o trabalho do técnico foi perfeito, mas o equipamento estava com problema, dois equipamentos com problema. A Brastemp precisa melhorar o controle de qualidade dos purificadores.</t>
+  </si>
+  <si>
+    <t>O serviço de assistência da Brastemp vem piorando a cada ano infelizmente.
+Apesar de gostar do purificador.</t>
+  </si>
+  <si>
+    <t>Produto é excelente, porém a logística para as manutenções preventivas é extremamente deficiente, ou seja, não existe uma programação e já reclamei a respeito disso, pois minha última manutenção SEMESTRAL foi em março de 2025 e para realização da próxima (que deveria ser semestral) seria em setembro de 2025 nunca ocorreu.
+A partir deste momento eu que tive que ir atrás para programar a próxima e somente agora - MARÇO/2026 que ocorrreu a Preventiva.
+Quando o técnico chegou, não ficou mais de 5 minutos, analisou a água e disse que não era necessário fazer nada !!!!!!! Foi quando solicitei a troca do filtro, pois este estava no Purificador a mais de 1,5 anos !!! Somente aí que fez a troca.</t>
+  </si>
+  <si>
+    <t>Purificador com defeito mesmo após a visita técnica e ainda não trocaram o produto</t>
+  </si>
+  <si>
+    <t>O purificador em si é muito bom, mas a Assitencia a manutenção deixa muito a desejar. Marcam e não aparecem, demorou mais de 6 meses e ainda veio em um dia sem comunicar previamente.</t>
+  </si>
+  <si>
+    <t>Estou sem água há 5 dias no purificador e o técnico não trouxe o sensor na M P ,e o próximo  agendamento via sistema só  daqui 16 dias. ABSURDO,  termos de ficar comprando água em mercado a preço muito superior a mensalidade do nosso plano. Uma empresa deste porte ,não  atender o cliente  de imediato, reparando ou até mesmo substituindo o aparelho porque o técnico não  trouxe o sensor correto! Vamos ficar 21 dias sem água, produto excencial pro ser humano, que honra os pagamentos de uma parceria. Não  basta ser educados, têm de ser eficientes.</t>
+  </si>
+  <si>
+    <t>Muito bom o purificador de água Brastemp porém acho o custo muito alto</t>
+  </si>
+  <si>
+    <t>O purificador é muito bom mas falta uma bateria nele pra quando há falta de luz</t>
+  </si>
+  <si>
+    <t>pela segunda vez, não resolveu o problema! O serviço está péssimo!</t>
+  </si>
+  <si>
+    <t>A VISITA AGENDADA PARA O DIA 28/02/2026 NÃO ACONTECEU.</t>
+  </si>
+  <si>
+    <t>Os botões do purificador depois que abriu e fechou estão muito duros, não era dessa forma</t>
+  </si>
+  <si>
+    <t>O técnico não veio em minha residência. estou muito insatisfeito com a Brastemp.</t>
+  </si>
+  <si>
+    <t>A manutenção feita no dia de hoje, a atendente sequer abrir o filtro internamente.  Apenas retirou uma amostra de água e mediu acredito ser o ph da água ou a qualidade da mesma com algumas gotinhas. Não houve troca do elemento filtrante. Gostsria de um retorno por parte da empresa.</t>
+  </si>
+  <si>
+    <t>Tenho o purificador de água Brastemp, e sempre que preciso de assistência técnica, o prazo para mandarem um técnico é muito longo.
+Nesta última visita, informaram que iriam CANCELAR a visita do técnico.
+Somente mantiveram a vinda do mesmo, pois informei que estaria CANCELANDO O CONTRATO.
+Muito INSATISFEITA.
+AMELIA SALIM GERIOS</t>
+  </si>
+  <si>
+    <t>Foi entregua na voltagem errada!</t>
+  </si>
+  <si>
+    <t>O técnico não resolveu o problema e ainda deu informações incorretas. O filtro não esfria mais (nem um pouco) e também baixou significativamente a vazão da água; porém o técnico disse q isto é normal. Também não trocou o filtro. Se estes pontos não for solucionado logo, cancelaremos o serviço.</t>
+  </si>
+  <si>
+    <t>O técnico não compareceu no dia agendado, por isso não dei nota 10!</t>
+  </si>
+  <si>
+    <t>Meu purificador não está gelando. Ja foi feita visita técnica sem resolução</t>
+  </si>
+  <si>
+    <t>O purificador em si é bom. O problema é sempre a a falta de datas para agendar a manutenção preventiva. Mais de um mês de espera é absurdo.</t>
+  </si>
+  <si>
+    <t>Dificuldade muito grande na hora de marcar uma visita de manutenção. Fiquei mais de 5 meses sem assistência.</t>
+  </si>
+  <si>
+    <t>Muito aborrecida com as ligações frequentes da Brastemp durante minhas férias.</t>
+  </si>
+  <si>
+    <t>Após a aquisição pela Culligan, o purificador não é mais o mesmo. O filtro que a Culligan está adotando é infinitamente inferior aos que a Whirpool utilizava. Já foram 2 problemas sequentes que não só eu como vários amigos que usam estão também sentindo. Nunca tivemos problemas com a Whripool, pois a qualidade oferecida era muito superior. Por precaução tive até que tomar medicamento pois a água estava totalmente impura. Em breve vou me mudar e não creio que eu continuarei com o purificador, pois se é para ter um filtro qualquer, eu mesma compro um purificador e troco o filtro.</t>
+  </si>
+  <si>
+    <t>Boa qualidade</t>
+  </si>
+  <si>
+    <t>Marcamos pela manhã mas chegaram depois de meio-dia. Fizeram rapidamente.</t>
+  </si>
+  <si>
+    <t>O técnico ja veio duas vezes a minha casa e nao trocou o aparelho. Agua nao está gelando</t>
+  </si>
+  <si>
+    <t>O técnico foi muito competente, atencioso e profissional. Trouxe a peça que precisava trocar, explicou o processo, limpou tudo com muito cuidado desmontando a máquina, sem pressa. Atendimento excepcional do Mateus!! Se a Culligan tivesse os técnicos com a mesma competência dele, seria outra empresa muito mais organizada, profissional e humana! Parabéns Mateus! Você merece tudo de melhor!</t>
+  </si>
+  <si>
+    <t>A água é de qualidade, gosto muito, porém existem algumas questões que não são nada favorável. fiquei com o mesmo purificador por muitos anos e não foi feito higienização nele. Consegui a troca por um novo e  dia 26/02 vieram fazer a troca acredite se quiser, permaneceram com a mangueira de anos atrás e não testaram o volume da água. ontem dia 04/03 voltou outro rapaz pra regular a saída da água que estava muito forte e informou que já estava pedindo uma nova mangueira. "Assim espero"</t>
+  </si>
+  <si>
+    <t>o técnico orientou p ligar e solicitar a substituição do aparelho todo, ligamos no numero orientado e não tem essa opção.</t>
+  </si>
+  <si>
+    <t>Não recebi visita nenhuma. Isso sempre acontece</t>
+  </si>
+  <si>
+    <t>Mais uma vez continuo sem funcionamento do purificador. Aparelho recém trocado com defeito. Sofrendo com este problema desde novembro/25.
+Se continuar assim, vou cancelar o serviço.</t>
+  </si>
+  <si>
+    <t>Nao gela muito no verão Ou ambiente quente</t>
+  </si>
+  <si>
+    <t>Atendimento para manutencao e solucao de problema muito lento, prazos para visita tecnica de 1 mes. 
+Isso significa ficar sem agua por 1 mes.</t>
+  </si>
+  <si>
+    <t>Horrível no mesmo dia o purificador deu problema</t>
+  </si>
+  <si>
+    <t>O técnico esteve ontem aqui e não trocou o filtro motivo não tinha.
+Estou pensando seriamente em cancelar minha assinatura.</t>
+  </si>
+  <si>
+    <t>Boa experiência. Contudo o preço do suprimento - gás CO2 - é alto. Adicionalmente, a agenda para assistência técnica é sempre para datas muito à frente.</t>
+  </si>
+  <si>
+    <t>Minha última experiência não foi muito boa,  mas agora está resolvida</t>
+  </si>
+  <si>
+    <t>Sou cliente há 16 anos .Vieram ontem trocaram o elemento filtrante como normalmente acontecia nas manutenções anteriores e hoje lançaram um boleto em meu nome no valor de $101,08 com vencimento para 30/03 e a central de atendimento 4004-4006 não sabe dizer ao que se refere o boleto e disseram que eu que tenho que enviar um boleto questionando ao que se refere o boleto . Pessimo atendimento</t>
+  </si>
+  <si>
+    <t>Aparelho já está defasado , prestador de serviço não foi no dia programado</t>
+  </si>
+  <si>
+    <t>O agendamento da visita técnica demora muito.</t>
+  </si>
+  <si>
+    <t>O seu técnico solicitou a troca do equipamento por um novo.
+Reforço a solicitação, pois estamos sem água filtrada já a vários dias.
+Hoje dia 05 de março, ainda não foi trocado.
+Estou no aguardo, conforme foi prometido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Supply</t>
+  </si>
+  <si>
+    <t>Agora, ok.</t>
+  </si>
+  <si>
+    <t>Atendimento normal</t>
+  </si>
+  <si>
+    <t>O equipamento apresenta defeito a mais de 1 mês, o técnico verificou que purificador aquecia de forma irregular (acima de 50 graus), na desmontagem o técnico quebrou a lateral do purificador, porém não foi autorizado a substituição do aparelho e vão substituir a peça danificada, a lateral tem que ser substituída também, vou aguardar esse concerto com muita atenção. Não fiquei satisfeito com o desfecho do atendimento.</t>
+  </si>
+  <si>
+    <t>Tive muitos aborrecimentos para conseguir o agendamento da minha manutenção, que pago assinatura mensal. Após diversas tentativas sem sucesso, entrei no Reclame Aqui, foi quando obtive uma devolutiva, que entrariam em contato comigo. No entanto, a pessoa já chegou foi lá em casa, sem agendamento. Por sorte, tinha uma pessoa em casa para atender. Outro ponto é a dificuldade para comprar o gás. Sinceramente, não recomendo.</t>
+  </si>
+  <si>
+    <t>Demora no agendamento para serviços</t>
+  </si>
+  <si>
+    <t>abri o chamado por que o purificador ESTAVA AQUECENDO , e comentei que eles vieram poucos dias antes para arrumar por que estava saindo pouca  água, porém a atendente só colocou o chamado pq estava saindo pouca água.
+E como não solucionou  por que isso aconteceu depois do primeiro tecnico sair, falei que era recorrencia e pedi URGENCIA. 
+ALém de não atender a URGENCIA, veio com chamado errado</t>
+  </si>
+  <si>
+    <t>A brastemp fica ligando, mandando mensagem, insistindo para fazer a manutenção do purificador.
+Agendamos a manutenção e ninguém aparece, vem em um outro dia, sem agendamento. E o pior sem nenhuma satisfação.
+E.muito descaso com.o cliente</t>
+  </si>
+  <si>
+    <t>Em relação ao purificador, não tenho nenhuma reclamação quanto ao seu funcionamento. Contudo, em relação ao técnico Neylon Silverio Silva, que tem nos atendido, registro minha insatisfação com sua postura durante as visitas. O profissional tem demonstrado um comportamento pouco cordial, além de não prestar esclarecimentos de forma adequada sobre a manutenção realizada e, em alguns momentos, apresentar respostas inadequadas durante o atendimento.</t>
+  </si>
+  <si>
+    <t>O rapaz veio aqui, trocou o filtro e não esperou. Não tenho mais água gelada no meu filtro</t>
+  </si>
+  <si>
+    <t>É a segunda vez que peço a troca do equipamento, através do WhatsApp,  devido ao barulho, mas não o fizeram. Os valores da locação nao param de subir. Ontem o liquido que vcs fazem o teste da água indicou pureza em 2 torneiras diferentes. é no minimo pra se pensar se está correto.</t>
+  </si>
+  <si>
+    <t>Temos contrato há muitos anos, só peço que seja dada a devida atenção para a data de manutenção dos equipamentos, antes do prazo do vencimento pelo fato de ter gerado descontentamento por parte dos clientes sobre isso, para registro gostaria apenas que fosse ajustado esse item e que realmente eu não precisasse ter que lembrá-los e sim receber um e-mail ou mensagem informando que o vencimento da manutenção será dia x e que antes do dia x, virá um técnico para executar a manutenção.</t>
+  </si>
+  <si>
+    <t>Marcado das 8h as 13h
+O técnico chegou 13h45.
+Deixou toda a pia suja e os restos da instalação.</t>
+  </si>
+  <si>
+    <t>O produto é muito bom mas o atendimento ao consumidor é muito ruim, vieram sem agendamento e sem consultar. Quando liguei para reclamar o atende-se me tratou mal, não justificou a visita, e disse que não podia fazer nada. O atendimento ao consumidor piorou muito. Vai continuar assim?
+Não estou disposta a pagar para ser mal atendida.</t>
+  </si>
+  <si>
+    <t>Não trocaram a vela  água continua com gosto ruim</t>
+  </si>
+  <si>
+    <t>Estou completamente insatisfeito com a Brastemp, pois estou a mais de 20 dias sem purificador, já liguei 5 vezes e não resolvem o problema.
+a penúltima vez falaram que na quarta feira, 05/03/26, viriam trocar o purificador de agua e não apareceu ninguém.
+No dia 2 apareceu um técnico e resolveu o problema, foi ele sair e quando voltei na cozinha esta cheia de agua.
+Os atendentes são nota 10 mas o procedimento nota zéro.</t>
   </si>
 </sst>
 </file>
@@ -2289,7 +2532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I533"/>
+  <dimension ref="A1:I601"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2298,7 +2541,7 @@
     <col min="4" max="4" width="33.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.140625" customWidth="1"/>
+    <col min="7" max="7" width="50.42578125" customWidth="1"/>
     <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
   </cols>
@@ -17760,6 +18003,1978 @@
         <v>39</v>
       </c>
     </row>
+    <row r="534" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A534">
+        <v>8857814</v>
+      </c>
+      <c r="B534" t="s">
+        <v>9</v>
+      </c>
+      <c r="C534">
+        <v>8005294783</v>
+      </c>
+      <c r="D534" s="3">
+        <v>46082.429363425923</v>
+      </c>
+      <c r="E534" t="s">
+        <v>20</v>
+      </c>
+      <c r="F534" t="s">
+        <v>16</v>
+      </c>
+      <c r="G534" t="s">
+        <v>606</v>
+      </c>
+      <c r="H534" t="s">
+        <v>32</v>
+      </c>
+      <c r="I534" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="535" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A535">
+        <v>8881701</v>
+      </c>
+      <c r="B535" t="s">
+        <v>9</v>
+      </c>
+      <c r="C535">
+        <v>8005316005</v>
+      </c>
+      <c r="D535" s="3">
+        <v>46083.448148148149</v>
+      </c>
+      <c r="E535" t="s">
+        <v>166</v>
+      </c>
+      <c r="F535" t="s">
+        <v>16</v>
+      </c>
+      <c r="G535" t="s">
+        <v>607</v>
+      </c>
+      <c r="H535" t="s">
+        <v>18</v>
+      </c>
+      <c r="I535" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="536" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A536">
+        <v>8881896</v>
+      </c>
+      <c r="B536" t="s">
+        <v>61</v>
+      </c>
+      <c r="C536">
+        <v>4323</v>
+      </c>
+      <c r="D536" s="3">
+        <v>46083.467465277783</v>
+      </c>
+      <c r="E536" t="s">
+        <v>582</v>
+      </c>
+      <c r="F536" t="s">
+        <v>16</v>
+      </c>
+      <c r="G536" t="s">
+        <v>608</v>
+      </c>
+      <c r="H536" t="s">
+        <v>609</v>
+      </c>
+      <c r="I536" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="537" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A537">
+        <v>8881808</v>
+      </c>
+      <c r="B537" t="s">
+        <v>9</v>
+      </c>
+      <c r="C537">
+        <v>8005301972</v>
+      </c>
+      <c r="D537" s="3">
+        <v>46083.522858796299</v>
+      </c>
+      <c r="E537" t="s">
+        <v>20</v>
+      </c>
+      <c r="F537" t="s">
+        <v>11</v>
+      </c>
+      <c r="G537" t="s">
+        <v>610</v>
+      </c>
+      <c r="H537" t="s">
+        <v>32</v>
+      </c>
+      <c r="I537" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="538" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A538">
+        <v>8881685</v>
+      </c>
+      <c r="B538" t="s">
+        <v>9</v>
+      </c>
+      <c r="C538">
+        <v>8005310505</v>
+      </c>
+      <c r="D538" s="3">
+        <v>46083.526979166672</v>
+      </c>
+      <c r="E538" t="s">
+        <v>20</v>
+      </c>
+      <c r="F538" t="s">
+        <v>16</v>
+      </c>
+      <c r="G538" t="s">
+        <v>611</v>
+      </c>
+      <c r="H538" t="s">
+        <v>612</v>
+      </c>
+      <c r="I538" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="539" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A539">
+        <v>8881804</v>
+      </c>
+      <c r="B539" t="s">
+        <v>9</v>
+      </c>
+      <c r="C539">
+        <v>8005301255</v>
+      </c>
+      <c r="D539" s="3">
+        <v>46083.526990740742</v>
+      </c>
+      <c r="E539" t="s">
+        <v>20</v>
+      </c>
+      <c r="F539" t="s">
+        <v>11</v>
+      </c>
+      <c r="G539" t="s">
+        <v>613</v>
+      </c>
+      <c r="H539" t="s">
+        <v>13</v>
+      </c>
+      <c r="I539" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="540" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A540">
+        <v>8881771</v>
+      </c>
+      <c r="B540" t="s">
+        <v>9</v>
+      </c>
+      <c r="C540">
+        <v>8005315377</v>
+      </c>
+      <c r="D540" s="3">
+        <v>46083.537141203713</v>
+      </c>
+      <c r="E540" t="s">
+        <v>53</v>
+      </c>
+      <c r="F540" t="s">
+        <v>16</v>
+      </c>
+      <c r="G540" t="s">
+        <v>614</v>
+      </c>
+      <c r="H540" t="s">
+        <v>609</v>
+      </c>
+      <c r="I540" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="541" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A541">
+        <v>8881671</v>
+      </c>
+      <c r="B541" t="s">
+        <v>9</v>
+      </c>
+      <c r="C541">
+        <v>8005293339</v>
+      </c>
+      <c r="D541" s="3">
+        <v>46083.552881944437</v>
+      </c>
+      <c r="E541" t="s">
+        <v>49</v>
+      </c>
+      <c r="F541" t="s">
+        <v>11</v>
+      </c>
+      <c r="G541" t="s">
+        <v>615</v>
+      </c>
+      <c r="H541" t="s">
+        <v>13</v>
+      </c>
+      <c r="I541" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="542" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A542">
+        <v>8867237</v>
+      </c>
+      <c r="B542" t="s">
+        <v>9</v>
+      </c>
+      <c r="C542">
+        <v>4509</v>
+      </c>
+      <c r="D542" s="3">
+        <v>46083.849236111113</v>
+      </c>
+      <c r="E542" t="s">
+        <v>616</v>
+      </c>
+      <c r="F542" t="s">
+        <v>16</v>
+      </c>
+      <c r="G542" t="s">
+        <v>617</v>
+      </c>
+      <c r="H542" t="s">
+        <v>609</v>
+      </c>
+      <c r="I542" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="543" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A543">
+        <v>8866898</v>
+      </c>
+      <c r="B543" t="s">
+        <v>9</v>
+      </c>
+      <c r="C543">
+        <v>8005293411</v>
+      </c>
+      <c r="D543" s="3">
+        <v>46084.344571759262</v>
+      </c>
+      <c r="E543" t="s">
+        <v>20</v>
+      </c>
+      <c r="F543" t="s">
+        <v>11</v>
+      </c>
+      <c r="G543" t="s">
+        <v>618</v>
+      </c>
+      <c r="H543" t="s">
+        <v>13</v>
+      </c>
+      <c r="I543" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="544" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A544">
+        <v>8889614</v>
+      </c>
+      <c r="B544" t="s">
+        <v>9</v>
+      </c>
+      <c r="C544">
+        <v>8005315380</v>
+      </c>
+      <c r="D544" s="3">
+        <v>46084.407060185193</v>
+      </c>
+      <c r="E544" t="s">
+        <v>262</v>
+      </c>
+      <c r="F544" t="s">
+        <v>16</v>
+      </c>
+      <c r="G544" t="s">
+        <v>619</v>
+      </c>
+      <c r="H544" t="s">
+        <v>609</v>
+      </c>
+      <c r="I544" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="545" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A545">
+        <v>8889585</v>
+      </c>
+      <c r="B545" t="s">
+        <v>9</v>
+      </c>
+      <c r="C545">
+        <v>8005311603</v>
+      </c>
+      <c r="D545" s="3">
+        <v>46084.412083333344</v>
+      </c>
+      <c r="E545" t="s">
+        <v>53</v>
+      </c>
+      <c r="F545" t="s">
+        <v>16</v>
+      </c>
+      <c r="G545" t="s">
+        <v>620</v>
+      </c>
+      <c r="H545" t="s">
+        <v>82</v>
+      </c>
+      <c r="I545" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="546" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A546">
+        <v>8889620</v>
+      </c>
+      <c r="B546" t="s">
+        <v>61</v>
+      </c>
+      <c r="C546">
+        <v>8005316687</v>
+      </c>
+      <c r="D546" s="3">
+        <v>46084.447187500002</v>
+      </c>
+      <c r="E546" t="s">
+        <v>262</v>
+      </c>
+      <c r="F546" t="s">
+        <v>16</v>
+      </c>
+      <c r="G546" t="s">
+        <v>621</v>
+      </c>
+      <c r="H546" t="s">
+        <v>609</v>
+      </c>
+      <c r="I546" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="547" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A547">
+        <v>8889373</v>
+      </c>
+      <c r="B547" t="s">
+        <v>9</v>
+      </c>
+      <c r="C547">
+        <v>8005313566</v>
+      </c>
+      <c r="D547" s="3">
+        <v>46084.459664351853</v>
+      </c>
+      <c r="E547" t="s">
+        <v>262</v>
+      </c>
+      <c r="F547" t="s">
+        <v>16</v>
+      </c>
+      <c r="G547" t="s">
+        <v>622</v>
+      </c>
+      <c r="H547" t="s">
+        <v>609</v>
+      </c>
+      <c r="I547" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="548" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A548">
+        <v>8889520</v>
+      </c>
+      <c r="B548" t="s">
+        <v>9</v>
+      </c>
+      <c r="C548">
+        <v>8005318555</v>
+      </c>
+      <c r="D548" s="3">
+        <v>46084.477372685193</v>
+      </c>
+      <c r="E548" t="s">
+        <v>15</v>
+      </c>
+      <c r="F548" t="s">
+        <v>11</v>
+      </c>
+      <c r="G548" t="s">
+        <v>623</v>
+      </c>
+      <c r="H548" t="s">
+        <v>13</v>
+      </c>
+      <c r="I548" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="549" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A549">
+        <v>8889417</v>
+      </c>
+      <c r="B549" t="s">
+        <v>9</v>
+      </c>
+      <c r="C549">
+        <v>8005275070</v>
+      </c>
+      <c r="D549" s="3">
+        <v>46084.482824074083</v>
+      </c>
+      <c r="E549" t="s">
+        <v>15</v>
+      </c>
+      <c r="F549" t="s">
+        <v>16</v>
+      </c>
+      <c r="G549" t="s">
+        <v>624</v>
+      </c>
+      <c r="H549" t="s">
+        <v>32</v>
+      </c>
+      <c r="I549" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="550" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A550">
+        <v>8889594</v>
+      </c>
+      <c r="B550" t="s">
+        <v>9</v>
+      </c>
+      <c r="C550">
+        <v>8005315327</v>
+      </c>
+      <c r="D550" s="3">
+        <v>46084.521504629629</v>
+      </c>
+      <c r="E550" t="s">
+        <v>37</v>
+      </c>
+      <c r="F550" t="s">
+        <v>16</v>
+      </c>
+      <c r="G550" t="s">
+        <v>625</v>
+      </c>
+      <c r="H550" t="s">
+        <v>609</v>
+      </c>
+      <c r="I550" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="551" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A551">
+        <v>8889318</v>
+      </c>
+      <c r="B551" t="s">
+        <v>9</v>
+      </c>
+      <c r="C551">
+        <v>8005273189</v>
+      </c>
+      <c r="D551" s="3">
+        <v>46084.525937500002</v>
+      </c>
+      <c r="E551" t="s">
+        <v>166</v>
+      </c>
+      <c r="F551" t="s">
+        <v>11</v>
+      </c>
+      <c r="G551" t="s">
+        <v>626</v>
+      </c>
+      <c r="H551" t="s">
+        <v>18</v>
+      </c>
+      <c r="I551" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="552" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A552">
+        <v>8889670</v>
+      </c>
+      <c r="B552" t="s">
+        <v>9</v>
+      </c>
+      <c r="C552">
+        <v>766</v>
+      </c>
+      <c r="D552" s="3">
+        <v>46084.528923611113</v>
+      </c>
+      <c r="E552" t="s">
+        <v>616</v>
+      </c>
+      <c r="F552" t="s">
+        <v>16</v>
+      </c>
+      <c r="G552" t="s">
+        <v>627</v>
+      </c>
+      <c r="H552" t="s">
+        <v>32</v>
+      </c>
+      <c r="I552" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="553" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A553">
+        <v>8889305</v>
+      </c>
+      <c r="B553" t="s">
+        <v>9</v>
+      </c>
+      <c r="C553">
+        <v>8005300988</v>
+      </c>
+      <c r="D553" s="3">
+        <v>46084.529224537036</v>
+      </c>
+      <c r="E553" t="s">
+        <v>20</v>
+      </c>
+      <c r="F553" t="s">
+        <v>11</v>
+      </c>
+      <c r="G553" t="s">
+        <v>628</v>
+      </c>
+      <c r="H553" t="s">
+        <v>13</v>
+      </c>
+      <c r="I553" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="554" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A554">
+        <v>8889325</v>
+      </c>
+      <c r="B554" t="s">
+        <v>9</v>
+      </c>
+      <c r="C554">
+        <v>8005285916</v>
+      </c>
+      <c r="D554" s="3">
+        <v>46084.532233796293</v>
+      </c>
+      <c r="E554" t="s">
+        <v>37</v>
+      </c>
+      <c r="F554" t="s">
+        <v>11</v>
+      </c>
+      <c r="G554" t="s">
+        <v>629</v>
+      </c>
+      <c r="H554" t="s">
+        <v>609</v>
+      </c>
+      <c r="I554" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="555" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A555">
+        <v>8889523</v>
+      </c>
+      <c r="B555" t="s">
+        <v>9</v>
+      </c>
+      <c r="C555">
+        <v>8005312588</v>
+      </c>
+      <c r="D555" s="3">
+        <v>46084.533506944441</v>
+      </c>
+      <c r="E555" t="s">
+        <v>20</v>
+      </c>
+      <c r="F555" t="s">
+        <v>16</v>
+      </c>
+      <c r="G555" t="s">
+        <v>630</v>
+      </c>
+      <c r="H555" t="s">
+        <v>18</v>
+      </c>
+      <c r="I555" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="556" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A556">
+        <v>8866885</v>
+      </c>
+      <c r="B556" t="s">
+        <v>9</v>
+      </c>
+      <c r="C556">
+        <v>8005315881</v>
+      </c>
+      <c r="D556" s="3">
+        <v>46084.537268518521</v>
+      </c>
+      <c r="E556" t="s">
+        <v>37</v>
+      </c>
+      <c r="F556" t="s">
+        <v>16</v>
+      </c>
+      <c r="G556" t="s">
+        <v>631</v>
+      </c>
+      <c r="H556" t="s">
+        <v>18</v>
+      </c>
+      <c r="I556" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="557" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A557">
+        <v>8889435</v>
+      </c>
+      <c r="B557" t="s">
+        <v>9</v>
+      </c>
+      <c r="C557">
+        <v>8005313227</v>
+      </c>
+      <c r="D557" s="3">
+        <v>46084.541030092587</v>
+      </c>
+      <c r="E557" t="s">
+        <v>15</v>
+      </c>
+      <c r="F557" t="s">
+        <v>11</v>
+      </c>
+      <c r="G557" t="s">
+        <v>632</v>
+      </c>
+      <c r="H557" t="s">
+        <v>609</v>
+      </c>
+      <c r="I557" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="558" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A558">
+        <v>8889483</v>
+      </c>
+      <c r="B558" t="s">
+        <v>9</v>
+      </c>
+      <c r="C558">
+        <v>8005318074</v>
+      </c>
+      <c r="D558" s="3">
+        <v>46084.549884259257</v>
+      </c>
+      <c r="E558" t="s">
+        <v>98</v>
+      </c>
+      <c r="F558" t="s">
+        <v>16</v>
+      </c>
+      <c r="G558" t="s">
+        <v>633</v>
+      </c>
+      <c r="H558" t="s">
+        <v>18</v>
+      </c>
+      <c r="I558" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="559" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A559">
+        <v>8889478</v>
+      </c>
+      <c r="B559" t="s">
+        <v>9</v>
+      </c>
+      <c r="C559">
+        <v>8005216489</v>
+      </c>
+      <c r="D559" s="3">
+        <v>46084.659699074073</v>
+      </c>
+      <c r="E559" t="s">
+        <v>20</v>
+      </c>
+      <c r="F559" t="s">
+        <v>16</v>
+      </c>
+      <c r="G559" t="s">
+        <v>634</v>
+      </c>
+      <c r="H559" t="s">
+        <v>18</v>
+      </c>
+      <c r="I559" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="560" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A560">
+        <v>8889672</v>
+      </c>
+      <c r="B560" t="s">
+        <v>9</v>
+      </c>
+      <c r="C560">
+        <v>763</v>
+      </c>
+      <c r="D560" s="3">
+        <v>46084.823425925933</v>
+      </c>
+      <c r="E560" t="s">
+        <v>582</v>
+      </c>
+      <c r="F560" t="s">
+        <v>16</v>
+      </c>
+      <c r="G560" t="s">
+        <v>635</v>
+      </c>
+      <c r="H560" t="s">
+        <v>32</v>
+      </c>
+      <c r="I560" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="561" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A561">
+        <v>8897786</v>
+      </c>
+      <c r="B561" t="s">
+        <v>9</v>
+      </c>
+      <c r="C561">
+        <v>8005296274</v>
+      </c>
+      <c r="D561" s="3">
+        <v>46085.445289351846</v>
+      </c>
+      <c r="E561" t="s">
+        <v>15</v>
+      </c>
+      <c r="F561" t="s">
+        <v>16</v>
+      </c>
+      <c r="G561" t="s">
+        <v>636</v>
+      </c>
+      <c r="H561" t="s">
+        <v>609</v>
+      </c>
+      <c r="I561" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="562" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A562">
+        <v>8897778</v>
+      </c>
+      <c r="B562" t="s">
+        <v>9</v>
+      </c>
+      <c r="C562">
+        <v>8005300942</v>
+      </c>
+      <c r="D562" s="3">
+        <v>46085.492719907408</v>
+      </c>
+      <c r="E562" t="s">
+        <v>20</v>
+      </c>
+      <c r="F562" t="s">
+        <v>16</v>
+      </c>
+      <c r="G562" t="s">
+        <v>637</v>
+      </c>
+      <c r="H562" t="s">
+        <v>18</v>
+      </c>
+      <c r="I562" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="563" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A563">
+        <v>8897772</v>
+      </c>
+      <c r="B563" t="s">
+        <v>9</v>
+      </c>
+      <c r="C563">
+        <v>8005298782</v>
+      </c>
+      <c r="D563" s="3">
+        <v>46085.502141203702</v>
+      </c>
+      <c r="E563" t="s">
+        <v>15</v>
+      </c>
+      <c r="F563" t="s">
+        <v>11</v>
+      </c>
+      <c r="G563" t="s">
+        <v>638</v>
+      </c>
+      <c r="H563" t="s">
+        <v>18</v>
+      </c>
+      <c r="I563" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="564" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A564">
+        <v>8897755</v>
+      </c>
+      <c r="B564" t="s">
+        <v>9</v>
+      </c>
+      <c r="C564">
+        <v>8005319211</v>
+      </c>
+      <c r="D564" s="3">
+        <v>46085.549247685187</v>
+      </c>
+      <c r="E564" t="s">
+        <v>49</v>
+      </c>
+      <c r="F564" t="s">
+        <v>16</v>
+      </c>
+      <c r="G564" t="s">
+        <v>639</v>
+      </c>
+      <c r="H564" t="s">
+        <v>18</v>
+      </c>
+      <c r="I564" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="565" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A565">
+        <v>8897660</v>
+      </c>
+      <c r="B565" t="s">
+        <v>9</v>
+      </c>
+      <c r="C565">
+        <v>8005274723</v>
+      </c>
+      <c r="D565" s="3">
+        <v>46085.563356481478</v>
+      </c>
+      <c r="E565" t="s">
+        <v>53</v>
+      </c>
+      <c r="F565" t="s">
+        <v>16</v>
+      </c>
+      <c r="G565" t="s">
+        <v>640</v>
+      </c>
+      <c r="H565" t="s">
+        <v>18</v>
+      </c>
+      <c r="I565" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="566" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A566">
+        <v>8897704</v>
+      </c>
+      <c r="B566" t="s">
+        <v>9</v>
+      </c>
+      <c r="C566">
+        <v>8005230638</v>
+      </c>
+      <c r="D566" s="3">
+        <v>46085.565555555557</v>
+      </c>
+      <c r="E566" t="s">
+        <v>53</v>
+      </c>
+      <c r="F566" t="s">
+        <v>16</v>
+      </c>
+      <c r="G566" t="s">
+        <v>641</v>
+      </c>
+      <c r="H566" t="s">
+        <v>13</v>
+      </c>
+      <c r="I566" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="567" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A567">
+        <v>8897681</v>
+      </c>
+      <c r="B567" t="s">
+        <v>9</v>
+      </c>
+      <c r="C567">
+        <v>8005317028</v>
+      </c>
+      <c r="D567" s="3">
+        <v>46085.573159722233</v>
+      </c>
+      <c r="E567" t="s">
+        <v>20</v>
+      </c>
+      <c r="F567" t="s">
+        <v>11</v>
+      </c>
+      <c r="G567" t="s">
+        <v>642</v>
+      </c>
+      <c r="H567" t="s">
+        <v>82</v>
+      </c>
+      <c r="I567" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="568" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A568">
+        <v>8897572</v>
+      </c>
+      <c r="B568" t="s">
+        <v>9</v>
+      </c>
+      <c r="C568">
+        <v>8005317759</v>
+      </c>
+      <c r="D568" s="3">
+        <v>46085.588171296287</v>
+      </c>
+      <c r="E568" t="s">
+        <v>20</v>
+      </c>
+      <c r="F568" t="s">
+        <v>16</v>
+      </c>
+      <c r="G568" t="s">
+        <v>643</v>
+      </c>
+      <c r="H568" t="s">
+        <v>609</v>
+      </c>
+      <c r="I568" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="569" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A569">
+        <v>8897639</v>
+      </c>
+      <c r="B569" t="s">
+        <v>9</v>
+      </c>
+      <c r="C569">
+        <v>8005293744</v>
+      </c>
+      <c r="D569" s="3">
+        <v>46085.601979166669</v>
+      </c>
+      <c r="E569" t="s">
+        <v>15</v>
+      </c>
+      <c r="F569" t="s">
+        <v>11</v>
+      </c>
+      <c r="G569" t="s">
+        <v>644</v>
+      </c>
+      <c r="H569" t="s">
+        <v>13</v>
+      </c>
+      <c r="I569" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="570" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A570">
+        <v>8897519</v>
+      </c>
+      <c r="B570" t="s">
+        <v>9</v>
+      </c>
+      <c r="C570">
+        <v>8005300381</v>
+      </c>
+      <c r="D570" s="3">
+        <v>46085.608657407407</v>
+      </c>
+      <c r="E570" t="s">
+        <v>53</v>
+      </c>
+      <c r="F570" t="s">
+        <v>16</v>
+      </c>
+      <c r="G570" t="s">
+        <v>645</v>
+      </c>
+      <c r="H570" t="s">
+        <v>18</v>
+      </c>
+      <c r="I570" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="571" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A571">
+        <v>8897606</v>
+      </c>
+      <c r="B571" t="s">
+        <v>9</v>
+      </c>
+      <c r="C571">
+        <v>8005320072</v>
+      </c>
+      <c r="D571" s="3">
+        <v>46085.75304398148</v>
+      </c>
+      <c r="E571" t="s">
+        <v>74</v>
+      </c>
+      <c r="F571" t="s">
+        <v>16</v>
+      </c>
+      <c r="G571" t="s">
+        <v>646</v>
+      </c>
+      <c r="H571" t="s">
+        <v>18</v>
+      </c>
+      <c r="I571" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="572" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A572">
+        <v>8903836</v>
+      </c>
+      <c r="B572" t="s">
+        <v>9</v>
+      </c>
+      <c r="C572">
+        <v>6199</v>
+      </c>
+      <c r="D572" s="3">
+        <v>46086.425416666672</v>
+      </c>
+      <c r="E572" t="s">
+        <v>585</v>
+      </c>
+      <c r="F572" t="s">
+        <v>11</v>
+      </c>
+      <c r="G572" t="s">
+        <v>647</v>
+      </c>
+      <c r="H572" t="s">
+        <v>13</v>
+      </c>
+      <c r="I572" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="573" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A573">
+        <v>8903588</v>
+      </c>
+      <c r="B573" t="s">
+        <v>9</v>
+      </c>
+      <c r="C573">
+        <v>8005317771</v>
+      </c>
+      <c r="D573" s="3">
+        <v>46086.439131944448</v>
+      </c>
+      <c r="E573" t="s">
+        <v>20</v>
+      </c>
+      <c r="F573" t="s">
+        <v>11</v>
+      </c>
+      <c r="G573" t="s">
+        <v>648</v>
+      </c>
+      <c r="H573" t="s">
+        <v>18</v>
+      </c>
+      <c r="I573" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="574" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A574">
+        <v>8881537</v>
+      </c>
+      <c r="B574" t="s">
+        <v>9</v>
+      </c>
+      <c r="C574">
+        <v>8005314920</v>
+      </c>
+      <c r="D574" s="3">
+        <v>46086.441296296303</v>
+      </c>
+      <c r="E574" t="s">
+        <v>49</v>
+      </c>
+      <c r="F574" t="s">
+        <v>16</v>
+      </c>
+      <c r="G574" t="s">
+        <v>649</v>
+      </c>
+      <c r="H574" t="s">
+        <v>82</v>
+      </c>
+      <c r="I574" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="575" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A575">
+        <v>8903598</v>
+      </c>
+      <c r="B575" t="s">
+        <v>9</v>
+      </c>
+      <c r="C575">
+        <v>8005315929</v>
+      </c>
+      <c r="D575" s="3">
+        <v>46086.4534375</v>
+      </c>
+      <c r="E575" t="s">
+        <v>98</v>
+      </c>
+      <c r="F575" t="s">
+        <v>16</v>
+      </c>
+      <c r="G575" t="s">
+        <v>650</v>
+      </c>
+      <c r="H575" t="s">
+        <v>18</v>
+      </c>
+      <c r="I575" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="576" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A576">
+        <v>8903502</v>
+      </c>
+      <c r="B576" t="s">
+        <v>9</v>
+      </c>
+      <c r="C576">
+        <v>8005314219</v>
+      </c>
+      <c r="D576" s="3">
+        <v>46086.489861111113</v>
+      </c>
+      <c r="E576" t="s">
+        <v>53</v>
+      </c>
+      <c r="F576" t="s">
+        <v>16</v>
+      </c>
+      <c r="G576" t="s">
+        <v>651</v>
+      </c>
+      <c r="H576" t="s">
+        <v>609</v>
+      </c>
+      <c r="I576" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="577" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A577">
+        <v>8903614</v>
+      </c>
+      <c r="B577" t="s">
+        <v>9</v>
+      </c>
+      <c r="C577">
+        <v>8005310486</v>
+      </c>
+      <c r="D577" s="3">
+        <v>46086.515879629631</v>
+      </c>
+      <c r="E577" t="s">
+        <v>15</v>
+      </c>
+      <c r="F577" t="s">
+        <v>11</v>
+      </c>
+      <c r="G577" t="s">
+        <v>652</v>
+      </c>
+      <c r="H577" t="s">
+        <v>609</v>
+      </c>
+      <c r="I577" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="578" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A578">
+        <v>8903637</v>
+      </c>
+      <c r="B578" t="s">
+        <v>9</v>
+      </c>
+      <c r="C578">
+        <v>8005302812</v>
+      </c>
+      <c r="D578" s="3">
+        <v>46086.516284722216</v>
+      </c>
+      <c r="E578" t="s">
+        <v>15</v>
+      </c>
+      <c r="F578" t="s">
+        <v>16</v>
+      </c>
+      <c r="G578" t="s">
+        <v>653</v>
+      </c>
+      <c r="H578" t="s">
+        <v>612</v>
+      </c>
+      <c r="I578" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="579" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A579">
+        <v>8903858</v>
+      </c>
+      <c r="B579" t="s">
+        <v>61</v>
+      </c>
+      <c r="C579">
+        <v>6642</v>
+      </c>
+      <c r="D579" s="3">
+        <v>46086.517245370371</v>
+      </c>
+      <c r="E579" t="s">
+        <v>548</v>
+      </c>
+      <c r="F579" t="s">
+        <v>16</v>
+      </c>
+      <c r="G579" t="s">
+        <v>654</v>
+      </c>
+      <c r="H579" t="s">
+        <v>609</v>
+      </c>
+      <c r="I579" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="580" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A580">
+        <v>8903461</v>
+      </c>
+      <c r="B580" t="s">
+        <v>9</v>
+      </c>
+      <c r="C580">
+        <v>8005315100</v>
+      </c>
+      <c r="D580" s="3">
+        <v>46086.522731481477</v>
+      </c>
+      <c r="E580" t="s">
+        <v>53</v>
+      </c>
+      <c r="F580" t="s">
+        <v>16</v>
+      </c>
+      <c r="G580" t="s">
+        <v>655</v>
+      </c>
+      <c r="H580" t="s">
+        <v>154</v>
+      </c>
+      <c r="I580" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="581" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A581">
+        <v>8903606</v>
+      </c>
+      <c r="B581" t="s">
+        <v>9</v>
+      </c>
+      <c r="C581">
+        <v>8005302803</v>
+      </c>
+      <c r="D581" s="3">
+        <v>46086.523252314822</v>
+      </c>
+      <c r="E581" t="s">
+        <v>15</v>
+      </c>
+      <c r="F581" t="s">
+        <v>11</v>
+      </c>
+      <c r="G581" t="s">
+        <v>656</v>
+      </c>
+      <c r="H581" t="s">
+        <v>13</v>
+      </c>
+      <c r="I581" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="582" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A582">
+        <v>8903644</v>
+      </c>
+      <c r="B582" t="s">
+        <v>9</v>
+      </c>
+      <c r="C582">
+        <v>8005285985</v>
+      </c>
+      <c r="D582" s="3">
+        <v>46086.526412037027</v>
+      </c>
+      <c r="E582" t="s">
+        <v>20</v>
+      </c>
+      <c r="F582" t="s">
+        <v>11</v>
+      </c>
+      <c r="G582" t="s">
+        <v>657</v>
+      </c>
+      <c r="H582" t="s">
+        <v>13</v>
+      </c>
+      <c r="I582" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="583" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A583">
+        <v>8903848</v>
+      </c>
+      <c r="B583" t="s">
+        <v>9</v>
+      </c>
+      <c r="C583">
+        <v>6547</v>
+      </c>
+      <c r="D583" s="3">
+        <v>46086.529328703713</v>
+      </c>
+      <c r="E583" t="s">
+        <v>542</v>
+      </c>
+      <c r="F583" t="s">
+        <v>16</v>
+      </c>
+      <c r="G583" t="s">
+        <v>658</v>
+      </c>
+      <c r="H583" t="s">
+        <v>13</v>
+      </c>
+      <c r="I583" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="584" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A584">
+        <v>8903597</v>
+      </c>
+      <c r="B584" t="s">
+        <v>9</v>
+      </c>
+      <c r="C584">
+        <v>8005307475</v>
+      </c>
+      <c r="D584" s="3">
+        <v>46086.529942129629</v>
+      </c>
+      <c r="E584" t="s">
+        <v>49</v>
+      </c>
+      <c r="F584" t="s">
+        <v>16</v>
+      </c>
+      <c r="G584" t="s">
+        <v>659</v>
+      </c>
+      <c r="H584" t="s">
+        <v>609</v>
+      </c>
+      <c r="I584" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="585" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A585">
+        <v>8903838</v>
+      </c>
+      <c r="B585" t="s">
+        <v>9</v>
+      </c>
+      <c r="C585">
+        <v>6244</v>
+      </c>
+      <c r="D585" s="3">
+        <v>46086.531284722223</v>
+      </c>
+      <c r="E585" t="s">
+        <v>585</v>
+      </c>
+      <c r="F585" t="s">
+        <v>16</v>
+      </c>
+      <c r="G585" t="s">
+        <v>660</v>
+      </c>
+      <c r="H585" t="s">
+        <v>32</v>
+      </c>
+      <c r="I585" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="586" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A586">
+        <v>8903571</v>
+      </c>
+      <c r="B586" t="s">
+        <v>9</v>
+      </c>
+      <c r="C586">
+        <v>8005320280</v>
+      </c>
+      <c r="D586" s="3">
+        <v>46086.533946759257</v>
+      </c>
+      <c r="E586" t="s">
+        <v>20</v>
+      </c>
+      <c r="F586" t="s">
+        <v>11</v>
+      </c>
+      <c r="G586" t="s">
+        <v>661</v>
+      </c>
+      <c r="H586" t="s">
+        <v>662</v>
+      </c>
+      <c r="I586" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="587" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A587">
+        <v>8903450</v>
+      </c>
+      <c r="B587" t="s">
+        <v>9</v>
+      </c>
+      <c r="C587">
+        <v>8005313137</v>
+      </c>
+      <c r="D587" s="3">
+        <v>46086.536574074067</v>
+      </c>
+      <c r="E587" t="s">
+        <v>20</v>
+      </c>
+      <c r="F587" t="s">
+        <v>11</v>
+      </c>
+      <c r="G587" t="s">
+        <v>663</v>
+      </c>
+      <c r="H587" t="s">
+        <v>13</v>
+      </c>
+      <c r="I587" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="588" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A588">
+        <v>8903657</v>
+      </c>
+      <c r="B588" t="s">
+        <v>9</v>
+      </c>
+      <c r="C588">
+        <v>8005314061</v>
+      </c>
+      <c r="D588" s="3">
+        <v>46086.538773148153</v>
+      </c>
+      <c r="E588" t="s">
+        <v>20</v>
+      </c>
+      <c r="F588" t="s">
+        <v>11</v>
+      </c>
+      <c r="G588" t="s">
+        <v>664</v>
+      </c>
+      <c r="H588" t="s">
+        <v>13</v>
+      </c>
+      <c r="I588" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="589" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A589">
+        <v>8881894</v>
+      </c>
+      <c r="B589" t="s">
+        <v>9</v>
+      </c>
+      <c r="C589">
+        <v>4270</v>
+      </c>
+      <c r="D589" s="3">
+        <v>46086.552106481482</v>
+      </c>
+      <c r="E589" t="s">
+        <v>582</v>
+      </c>
+      <c r="F589" t="s">
+        <v>16</v>
+      </c>
+      <c r="G589" t="s">
+        <v>665</v>
+      </c>
+      <c r="H589" t="s">
+        <v>609</v>
+      </c>
+      <c r="I589" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="590" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A590">
+        <v>8903712</v>
+      </c>
+      <c r="B590" t="s">
+        <v>9</v>
+      </c>
+      <c r="C590">
+        <v>8005269435</v>
+      </c>
+      <c r="D590" s="3">
+        <v>46086.61818287037</v>
+      </c>
+      <c r="E590" t="s">
+        <v>65</v>
+      </c>
+      <c r="F590" t="s">
+        <v>16</v>
+      </c>
+      <c r="G590" t="s">
+        <v>666</v>
+      </c>
+      <c r="H590" t="s">
+        <v>18</v>
+      </c>
+      <c r="I590" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="591" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A591">
+        <v>8903551</v>
+      </c>
+      <c r="B591" t="s">
+        <v>9</v>
+      </c>
+      <c r="C591">
+        <v>8005316747</v>
+      </c>
+      <c r="D591" s="3">
+        <v>46086.742546296293</v>
+      </c>
+      <c r="E591" t="s">
+        <v>53</v>
+      </c>
+      <c r="F591" t="s">
+        <v>16</v>
+      </c>
+      <c r="G591" t="s">
+        <v>667</v>
+      </c>
+      <c r="H591" t="s">
+        <v>612</v>
+      </c>
+      <c r="I591" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="592" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A592">
+        <v>8915306</v>
+      </c>
+      <c r="B592" t="s">
+        <v>9</v>
+      </c>
+      <c r="C592">
+        <v>2480</v>
+      </c>
+      <c r="D592" s="3">
+        <v>46087.417326388888</v>
+      </c>
+      <c r="E592" t="s">
+        <v>616</v>
+      </c>
+      <c r="F592" t="s">
+        <v>16</v>
+      </c>
+      <c r="G592" t="s">
+        <v>668</v>
+      </c>
+      <c r="H592" t="s">
+        <v>82</v>
+      </c>
+      <c r="I592" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="593" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A593">
+        <v>8903783</v>
+      </c>
+      <c r="B593" t="s">
+        <v>9</v>
+      </c>
+      <c r="C593">
+        <v>2414</v>
+      </c>
+      <c r="D593" s="3">
+        <v>46087.418634259258</v>
+      </c>
+      <c r="E593" t="s">
+        <v>582</v>
+      </c>
+      <c r="F593" t="s">
+        <v>16</v>
+      </c>
+      <c r="G593" t="s">
+        <v>669</v>
+      </c>
+      <c r="H593" t="s">
+        <v>18</v>
+      </c>
+      <c r="I593" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="594" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A594">
+        <v>8915198</v>
+      </c>
+      <c r="B594" t="s">
+        <v>9</v>
+      </c>
+      <c r="C594">
+        <v>8005322462</v>
+      </c>
+      <c r="D594" s="3">
+        <v>46087.42287037037</v>
+      </c>
+      <c r="E594" t="s">
+        <v>125</v>
+      </c>
+      <c r="F594" t="s">
+        <v>16</v>
+      </c>
+      <c r="G594" t="s">
+        <v>670</v>
+      </c>
+      <c r="H594" t="s">
+        <v>18</v>
+      </c>
+      <c r="I594" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="595" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A595">
+        <v>8889589</v>
+      </c>
+      <c r="B595" t="s">
+        <v>9</v>
+      </c>
+      <c r="C595">
+        <v>8005302653</v>
+      </c>
+      <c r="D595" s="3">
+        <v>46087.436655092592</v>
+      </c>
+      <c r="E595" t="s">
+        <v>20</v>
+      </c>
+      <c r="F595" t="s">
+        <v>16</v>
+      </c>
+      <c r="G595" t="s">
+        <v>671</v>
+      </c>
+      <c r="H595" t="s">
+        <v>18</v>
+      </c>
+      <c r="I595" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="596" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A596">
+        <v>8915325</v>
+      </c>
+      <c r="B596" t="s">
+        <v>9</v>
+      </c>
+      <c r="C596">
+        <v>3424</v>
+      </c>
+      <c r="D596" s="3">
+        <v>46087.457384259258</v>
+      </c>
+      <c r="E596" t="s">
+        <v>556</v>
+      </c>
+      <c r="F596" t="s">
+        <v>16</v>
+      </c>
+      <c r="G596" t="s">
+        <v>672</v>
+      </c>
+      <c r="H596" t="s">
+        <v>609</v>
+      </c>
+      <c r="I596" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="597" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A597">
+        <v>8915108</v>
+      </c>
+      <c r="B597" t="s">
+        <v>9</v>
+      </c>
+      <c r="C597">
+        <v>8005300671</v>
+      </c>
+      <c r="D597" s="3">
+        <v>46087.52039351852</v>
+      </c>
+      <c r="E597" t="s">
+        <v>20</v>
+      </c>
+      <c r="F597" t="s">
+        <v>11</v>
+      </c>
+      <c r="G597" t="s">
+        <v>673</v>
+      </c>
+      <c r="H597" t="s">
+        <v>32</v>
+      </c>
+      <c r="I597" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="598" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A598">
+        <v>8915259</v>
+      </c>
+      <c r="B598" t="s">
+        <v>9</v>
+      </c>
+      <c r="C598">
+        <v>8005278922</v>
+      </c>
+      <c r="D598" s="3">
+        <v>46087.600127314807</v>
+      </c>
+      <c r="E598" t="s">
+        <v>65</v>
+      </c>
+      <c r="F598" t="s">
+        <v>16</v>
+      </c>
+      <c r="G598" t="s">
+        <v>674</v>
+      </c>
+      <c r="H598" t="s">
+        <v>18</v>
+      </c>
+      <c r="I598" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="599" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A599">
+        <v>8915275</v>
+      </c>
+      <c r="B599" t="s">
+        <v>9</v>
+      </c>
+      <c r="C599">
+        <v>8005312840</v>
+      </c>
+      <c r="D599" s="3">
+        <v>46087.63244212963</v>
+      </c>
+      <c r="E599" t="s">
+        <v>65</v>
+      </c>
+      <c r="F599" t="s">
+        <v>16</v>
+      </c>
+      <c r="G599" t="s">
+        <v>675</v>
+      </c>
+      <c r="H599" t="s">
+        <v>18</v>
+      </c>
+      <c r="I599" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="600" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A600">
+        <v>8915042</v>
+      </c>
+      <c r="B600" t="s">
+        <v>9</v>
+      </c>
+      <c r="C600">
+        <v>8005302150</v>
+      </c>
+      <c r="D600" s="3">
+        <v>46087.636504629627</v>
+      </c>
+      <c r="E600" t="s">
+        <v>20</v>
+      </c>
+      <c r="F600" t="s">
+        <v>16</v>
+      </c>
+      <c r="G600" t="s">
+        <v>676</v>
+      </c>
+      <c r="H600" t="s">
+        <v>18</v>
+      </c>
+      <c r="I600" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="601" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A601">
+        <v>8889308</v>
+      </c>
+      <c r="B601" t="s">
+        <v>9</v>
+      </c>
+      <c r="C601">
+        <v>8005313688</v>
+      </c>
+      <c r="D601" s="3">
+        <v>46088.342916666668</v>
+      </c>
+      <c r="E601" t="s">
+        <v>464</v>
+      </c>
+      <c r="F601" t="s">
+        <v>16</v>
+      </c>
+      <c r="G601" t="s">
+        <v>677</v>
+      </c>
+      <c r="H601" t="s">
+        <v>18</v>
+      </c>
+      <c r="I601" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/03/2026 11:44:35,02
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04F45B61-AE6F-495D-AF0A-0A483857EF16}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B66DE297-29AD-46BB-A098-3E6D6B802E92}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$533</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$601</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="676">
   <si>
     <t>ID</t>
   </si>
@@ -1945,9 +1945,6 @@
 Dias</t>
   </si>
   <si>
-    <t>CAPACIDADE</t>
-  </si>
-  <si>
     <t>Está deixando a desejar</t>
   </si>
   <si>
@@ -2106,9 +2103,6 @@
 Reforço a solicitação, pois estamos sem água filtrada já a vários dias.
 Hoje dia 05 de março, ainda não foi trocado.
 Estou no aguardo, conforme foi prometido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Supply</t>
   </si>
   <si>
     <t>Agora, ok.</t>
@@ -18142,7 +18136,7 @@
         <v>611</v>
       </c>
       <c r="H538" t="s">
-        <v>612</v>
+        <v>32</v>
       </c>
       <c r="I538" t="s">
         <v>354</v>
@@ -18168,7 +18162,7 @@
         <v>11</v>
       </c>
       <c r="G539" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H539" t="s">
         <v>13</v>
@@ -18197,7 +18191,7 @@
         <v>16</v>
       </c>
       <c r="G540" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="H540" t="s">
         <v>609</v>
@@ -18226,7 +18220,7 @@
         <v>11</v>
       </c>
       <c r="G541" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="H541" t="s">
         <v>13</v>
@@ -18249,13 +18243,13 @@
         <v>46083.849236111113</v>
       </c>
       <c r="E542" t="s">
+        <v>615</v>
+      </c>
+      <c r="F542" t="s">
+        <v>16</v>
+      </c>
+      <c r="G542" t="s">
         <v>616</v>
-      </c>
-      <c r="F542" t="s">
-        <v>16</v>
-      </c>
-      <c r="G542" t="s">
-        <v>617</v>
       </c>
       <c r="H542" t="s">
         <v>609</v>
@@ -18284,7 +18278,7 @@
         <v>11</v>
       </c>
       <c r="G543" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H543" t="s">
         <v>13</v>
@@ -18313,7 +18307,7 @@
         <v>16</v>
       </c>
       <c r="G544" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="H544" t="s">
         <v>609</v>
@@ -18342,7 +18336,7 @@
         <v>16</v>
       </c>
       <c r="G545" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="H545" t="s">
         <v>82</v>
@@ -18371,7 +18365,7 @@
         <v>16</v>
       </c>
       <c r="G546" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="H546" t="s">
         <v>609</v>
@@ -18400,7 +18394,7 @@
         <v>16</v>
       </c>
       <c r="G547" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="H547" t="s">
         <v>609</v>
@@ -18429,7 +18423,7 @@
         <v>11</v>
       </c>
       <c r="G548" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H548" t="s">
         <v>13</v>
@@ -18458,7 +18452,7 @@
         <v>16</v>
       </c>
       <c r="G549" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="H549" t="s">
         <v>32</v>
@@ -18487,7 +18481,7 @@
         <v>16</v>
       </c>
       <c r="G550" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="H550" t="s">
         <v>609</v>
@@ -18516,7 +18510,7 @@
         <v>11</v>
       </c>
       <c r="G551" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H551" t="s">
         <v>18</v>
@@ -18539,13 +18533,13 @@
         <v>46084.528923611113</v>
       </c>
       <c r="E552" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F552" t="s">
         <v>16</v>
       </c>
       <c r="G552" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="H552" t="s">
         <v>32</v>
@@ -18574,7 +18568,7 @@
         <v>11</v>
       </c>
       <c r="G553" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="H553" t="s">
         <v>13</v>
@@ -18603,7 +18597,7 @@
         <v>11</v>
       </c>
       <c r="G554" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H554" t="s">
         <v>609</v>
@@ -18632,7 +18626,7 @@
         <v>16</v>
       </c>
       <c r="G555" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="H555" t="s">
         <v>18</v>
@@ -18661,7 +18655,7 @@
         <v>16</v>
       </c>
       <c r="G556" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H556" t="s">
         <v>18</v>
@@ -18690,7 +18684,7 @@
         <v>11</v>
       </c>
       <c r="G557" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H557" t="s">
         <v>609</v>
@@ -18719,7 +18713,7 @@
         <v>16</v>
       </c>
       <c r="G558" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H558" t="s">
         <v>18</v>
@@ -18748,7 +18742,7 @@
         <v>16</v>
       </c>
       <c r="G559" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H559" t="s">
         <v>18</v>
@@ -18777,7 +18771,7 @@
         <v>16</v>
       </c>
       <c r="G560" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H560" t="s">
         <v>32</v>
@@ -18806,7 +18800,7 @@
         <v>16</v>
       </c>
       <c r="G561" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H561" t="s">
         <v>609</v>
@@ -18835,7 +18829,7 @@
         <v>16</v>
       </c>
       <c r="G562" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="H562" t="s">
         <v>18</v>
@@ -18864,7 +18858,7 @@
         <v>11</v>
       </c>
       <c r="G563" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H563" t="s">
         <v>18</v>
@@ -18893,7 +18887,7 @@
         <v>16</v>
       </c>
       <c r="G564" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="H564" t="s">
         <v>18</v>
@@ -18922,7 +18916,7 @@
         <v>16</v>
       </c>
       <c r="G565" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="H565" t="s">
         <v>18</v>
@@ -18951,7 +18945,7 @@
         <v>16</v>
       </c>
       <c r="G566" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="H566" t="s">
         <v>13</v>
@@ -18980,7 +18974,7 @@
         <v>11</v>
       </c>
       <c r="G567" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H567" t="s">
         <v>82</v>
@@ -19009,7 +19003,7 @@
         <v>16</v>
       </c>
       <c r="G568" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="H568" t="s">
         <v>609</v>
@@ -19038,7 +19032,7 @@
         <v>11</v>
       </c>
       <c r="G569" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="H569" t="s">
         <v>13</v>
@@ -19067,7 +19061,7 @@
         <v>16</v>
       </c>
       <c r="G570" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="H570" t="s">
         <v>18</v>
@@ -19096,7 +19090,7 @@
         <v>16</v>
       </c>
       <c r="G571" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="H571" t="s">
         <v>18</v>
@@ -19125,7 +19119,7 @@
         <v>11</v>
       </c>
       <c r="G572" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="H572" t="s">
         <v>13</v>
@@ -19154,7 +19148,7 @@
         <v>11</v>
       </c>
       <c r="G573" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="H573" t="s">
         <v>18</v>
@@ -19183,7 +19177,7 @@
         <v>16</v>
       </c>
       <c r="G574" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="H574" t="s">
         <v>82</v>
@@ -19212,7 +19206,7 @@
         <v>16</v>
       </c>
       <c r="G575" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H575" t="s">
         <v>18</v>
@@ -19241,7 +19235,7 @@
         <v>16</v>
       </c>
       <c r="G576" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H576" t="s">
         <v>609</v>
@@ -19270,7 +19264,7 @@
         <v>11</v>
       </c>
       <c r="G577" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="H577" t="s">
         <v>609</v>
@@ -19299,10 +19293,10 @@
         <v>16</v>
       </c>
       <c r="G578" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H578" t="s">
-        <v>612</v>
+        <v>32</v>
       </c>
       <c r="I578" t="s">
         <v>354</v>
@@ -19328,7 +19322,7 @@
         <v>16</v>
       </c>
       <c r="G579" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H579" t="s">
         <v>609</v>
@@ -19357,7 +19351,7 @@
         <v>16</v>
       </c>
       <c r="G580" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H580" t="s">
         <v>154</v>
@@ -19386,7 +19380,7 @@
         <v>11</v>
       </c>
       <c r="G581" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H581" t="s">
         <v>13</v>
@@ -19415,7 +19409,7 @@
         <v>11</v>
       </c>
       <c r="G582" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="H582" t="s">
         <v>13</v>
@@ -19444,7 +19438,7 @@
         <v>16</v>
       </c>
       <c r="G583" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="H583" t="s">
         <v>13</v>
@@ -19473,7 +19467,7 @@
         <v>16</v>
       </c>
       <c r="G584" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H584" t="s">
         <v>609</v>
@@ -19502,7 +19496,7 @@
         <v>16</v>
       </c>
       <c r="G585" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H585" t="s">
         <v>32</v>
@@ -19531,10 +19525,10 @@
         <v>11</v>
       </c>
       <c r="G586" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H586" t="s">
-        <v>662</v>
+        <v>154</v>
       </c>
       <c r="I586" t="s">
         <v>179</v>
@@ -19560,7 +19554,7 @@
         <v>11</v>
       </c>
       <c r="G587" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="H587" t="s">
         <v>13</v>
@@ -19589,7 +19583,7 @@
         <v>11</v>
       </c>
       <c r="G588" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="H588" t="s">
         <v>13</v>
@@ -19618,7 +19612,7 @@
         <v>16</v>
       </c>
       <c r="G589" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="H589" t="s">
         <v>609</v>
@@ -19647,7 +19641,7 @@
         <v>16</v>
       </c>
       <c r="G590" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="H590" t="s">
         <v>18</v>
@@ -19676,10 +19670,10 @@
         <v>16</v>
       </c>
       <c r="G591" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="H591" t="s">
-        <v>612</v>
+        <v>32</v>
       </c>
       <c r="I591" t="s">
         <v>354</v>
@@ -19699,13 +19693,13 @@
         <v>46087.417326388888</v>
       </c>
       <c r="E592" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F592" t="s">
         <v>16</v>
       </c>
       <c r="G592" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="H592" t="s">
         <v>82</v>
@@ -19734,7 +19728,7 @@
         <v>16</v>
       </c>
       <c r="G593" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="H593" t="s">
         <v>18</v>
@@ -19763,7 +19757,7 @@
         <v>16</v>
       </c>
       <c r="G594" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="H594" t="s">
         <v>18</v>
@@ -19792,7 +19786,7 @@
         <v>16</v>
       </c>
       <c r="G595" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="H595" t="s">
         <v>18</v>
@@ -19821,7 +19815,7 @@
         <v>16</v>
       </c>
       <c r="G596" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="H596" t="s">
         <v>609</v>
@@ -19850,7 +19844,7 @@
         <v>11</v>
       </c>
       <c r="G597" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="H597" t="s">
         <v>32</v>
@@ -19879,7 +19873,7 @@
         <v>16</v>
       </c>
       <c r="G598" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="H598" t="s">
         <v>18</v>
@@ -19908,7 +19902,7 @@
         <v>16</v>
       </c>
       <c r="G599" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="H599" t="s">
         <v>18</v>
@@ -19937,7 +19931,7 @@
         <v>16</v>
       </c>
       <c r="G600" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="H600" t="s">
         <v>18</v>
@@ -19966,7 +19960,7 @@
         <v>16</v>
       </c>
       <c r="G601" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="H601" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 13/03/2026 11:00:27,44
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B66DE297-29AD-46BB-A098-3E6D6B802E92}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7C36A5-444B-45FD-A0DA-5557A4825CD7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="676">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3951" uniqueCount="740">
   <si>
     <t>ID</t>
   </si>
@@ -2158,6 +2158,198 @@
 a penúltima vez falaram que na quarta feira, 05/03/26, viriam trocar o purificador de agua e não apareceu ninguém.
 No dia 2 apareceu um técnico e resolveu o problema, foi ele sair e quando voltei na cozinha esta cheia de agua.
 Os atendentes são nota 10 mas o procedimento nota zéro.</t>
+  </si>
+  <si>
+    <t>Gostaria que se atentassem ao agendamento das visitas, pois marcamos para o sábado e o técnico sem avisar apareceu na sexta feira pois disse que não haveria expediente no sábado de carnaval.</t>
+  </si>
+  <si>
+    <t>Brazoavel não enche uma garrafa de 310 ml</t>
+  </si>
+  <si>
+    <t>Perguntamos para o instalador se estava tudo em ordem e o mesmo informou que sim, mas impossível pegar água no filtro devido a pressão que foi deixada no mesmo. Acreditamos que esteja sem redutor no filtro.</t>
+  </si>
+  <si>
+    <t>liga ninguém atende. Estamos a quase 1 ano sem o cilindro de gás. Solicitei o envio da fatura uma vez, tive que implorar. não recomendo.</t>
+  </si>
+  <si>
+    <t>FRQ BASE LESTE SP</t>
+  </si>
+  <si>
+    <t>Já agendei a visita 4x e nunca vieram. Agendei 3x para sábado, uma das vezes tentaram vir na sexta (não podia atender, por isso agendei no sábado) e nas outras, simplesmente ninguem sequer apareceu. Aí na última agora, tentei agendar na sexta, visto que de sábado estava impossível, ninguem apareceu também. Não está fazendo sentido algum eu manter o serviço, visto que não tenho a manutenção preventiva, a troca do filtro.</t>
+  </si>
+  <si>
+    <t>Técnico não cumpriu agenda</t>
+  </si>
+  <si>
+    <t>Agendei duas vezes a manutenção periódica e o técnico não foi, para piorar a última manutenção realizada, foi em 07/2025 ou seja, passou muito o prazo.</t>
+  </si>
+  <si>
+    <t>FRQ OSASCO SP</t>
+  </si>
+  <si>
+    <t>Simplesmente não trocaram o filtro, a incompetencia de voces é admirável. O Contrato esta cancelado já retirei o pagamento.</t>
+  </si>
+  <si>
+    <t>O técnico foi bom. Mas, vocês enviaram um purificador inferior ao meu. Por favor, verificar o meu pagamento mensal, pois esse purificador enviado é de nível inferior ao que eu tinha</t>
+  </si>
+  <si>
+    <t>Foi aberto chamado 2 vezes e em nenhuma delas o problema foi resolvido, sendo que o caso é somente colocar um pressurizador do purificador, pois a saìda da agua está muito fraca. O ultimo técnico informou que estaria colocando uma observação na ordem de serviço, mas até agora não recebi nenhuma posição ára resolver o problema.</t>
+  </si>
+  <si>
+    <t>Não resolveu o problema é tempo da visita técnica muito demorada, sabendo que o pedido de vocês fornece água</t>
+  </si>
+  <si>
+    <t>Gosto muito , porém ultimamente o atendimento de manutenção está terrível</t>
+  </si>
+  <si>
+    <t>A água sempre está boa, o filtro nunca precisa trocar. É eterno.</t>
+  </si>
+  <si>
+    <t>O produto é bom.</t>
+  </si>
+  <si>
+    <t>Serviço muito ruim, só chega troca o filtro e nem olha , além de ser caro não compensa</t>
+  </si>
+  <si>
+    <t>Após 2 a e 7 meses de manutenção e pagando, o que acham que posso dizer?? Qual as desculpas que acham poder me fornecer x dês desconto por ter pagode ser utilizar os benefícios cabíveis.</t>
+  </si>
+  <si>
+    <t>De forma geral, estou satisfeito com o produto. O único porém é que, como eu estava presente nessa última visita, só então pude saber que o elemento filtrante não é trocado a cada visita periódica de 6 meses. O que acho errado, pois, várias vezes o filtro ficou com cheiro ruim pouco tempo após uma visita e o site diz que o problema é das algas da Sabesp. Mas agora já sei que é porque o filtro não é trocado. Daqui em diante, vou sempre pedir a troca do elemento filtrante.</t>
+  </si>
+  <si>
+    <t>São muitos anos de uma boa parceria.</t>
+  </si>
+  <si>
+    <t>A visita seria para retirar o aparelho e não para trocar ...Muito desinformação, a Brastemp de hoje não é a mesma. Comparada a 1ª e 2ª  vez que foi assinante. As condições de aparelho que INSTALARAM  é um nojo. MOFADO POR DENTRO, VAZANDO, OXIDANDO, ESQUENTADO ...TIVE QUE LIGAR NOVAMENTE PARA VIR RETIRAR O APARELHO.O PROBLEMA NÃO SÃO OS TÉCNICOS SÃO EXCELENTES, EDUCADOS..</t>
+  </si>
+  <si>
+    <t>Sou cliente a 18 anos neste período houve inúmeras mudanças e piorou no atendimento emergencial fiquei do dia 20 de fevereiro até dia 5 de março sem águapotável e mesmo assim o técnico não tinha uma peça e disse que se houver problemas solicite assistência técnica portanto novos tempos</t>
+  </si>
+  <si>
+    <t>Falta de estoque/pecas</t>
+  </si>
+  <si>
+    <t>o Técnico veio sem Pro -pé e sem lavar as mãos da rua para fazer a manutenção do aparelho Brastemp ! Estou pensando seriamente em trocar o aparelho de filtro de água Brastemp .</t>
+  </si>
+  <si>
+    <t>FRQ ZONA OESTE1 SP</t>
+  </si>
+  <si>
+    <t>A utilização do purificador é boa, entretanto a comunicação via remota é sofrível</t>
+  </si>
+  <si>
+    <t>FRQ GUARULHOS SP</t>
+  </si>
+  <si>
+    <t>Bom dia.Então recebi a visita técnica, foi trocado o filtro de água.Mas depois eu percebi que tinha um vazamento de água, eu mesmo abri o aparelho e tinha uma mangueira meia desconecta da, consegui conectar a mesma e parou o vazamento.Quero dizer que na hora da troca o técnico não percebeu que tinha desconectado a mesma.</t>
+  </si>
+  <si>
+    <t>O filtro está com vazamento e precisa ser trocado</t>
+  </si>
+  <si>
+    <t>Venho há muito tempo informando que a água com gás está ruim. Já foram 2 técnicos falando que estava com defeito e teria que trocar o aparelho. Nunca ninguém foi trocar! Pedi agora para trocar o plano e o técnico que foi falou que não tem defeito. Atualmente não é isso que solicitei!!!! Cansei da Brastemp</t>
+  </si>
+  <si>
+    <t>Eficiente</t>
+  </si>
+  <si>
+    <t>Estou bem com o purificador. Muito bom</t>
+  </si>
+  <si>
+    <t>atende as necessidades, porem quando falta energia eletrica, ficamos sem agua, precisam dar uma solução,</t>
+  </si>
+  <si>
+    <t>Difícil agendar manutenção</t>
+  </si>
+  <si>
+    <t>Só não dou 10 pq o agendamento de vcs demora mt</t>
+  </si>
+  <si>
+    <t>Apareceram na minha casa sem terem marcado comigo antes</t>
+  </si>
+  <si>
+    <t>É boa , aja vista q tenho o purificador a mts anos .  O funcionário q veio aqui foi mt correto, mas chegou parte manhã e eu escolhi horário parte da tarde . Isso vcs precisam melhorar qto as marcações q escolhemos pra fazer jus essas prioridades. Por várias vezes , marquei e não veio ninguém. Fiquei esperando e isso é uma grande falha. Precisam melhorar nessa logística . Outra coisa : o q tinha q ser trocado , o termostato de temperatura não foi trocado pq , conforme o funcionário, ele não  tinha a peça e agora tenho q remarcar pra vir outro funcionário com a peça .. …. Pq já não vem com as peças necessárias pra troca ? Acho isso ineficiente por parte da Brastemp . Espero q a Culligan não repita isso .</t>
+  </si>
+  <si>
+    <t>o conserto demoru para ser feito mais de vinte dias e a brastemp não da desconto pelo serviço que não prestou nesses dias que o purificador ficou quebrado.Absurdo cobrar por um serviço que naõ prestou, issoporque sou cliente a mais de 15 anos, imagina se não fosse.</t>
+  </si>
+  <si>
+    <t>NÃO RECEBI ESTA MANUTENÇÃO.  NÃO FOI FEITO NENHUM REVISÃO.</t>
+  </si>
+  <si>
+    <t>FRQ ZONA OESTE2 SP</t>
+  </si>
+  <si>
+    <t>Este ano tive graves problemas com a assistência técnica.Fique praticamente 60 dias com problemas no purificador.Só resolvido nesta semana / dia 09/03.Espero que a nova gestão seja assertiva</t>
+  </si>
+  <si>
+    <t>tenha ĥa mtos anos.</t>
+  </si>
+  <si>
+    <t>A cobrança agora é pela empresa Culligan?O período entre as revisões passou do aceitavel</t>
+  </si>
+  <si>
+    <t>O atendimento da Brastemp é péssimo. Sempre é absurdamente demorado e na maioria das vezes não resolve o problema. Fiquei mais de um mês sem poder tomar a água do aparelho, que estava com gosto e cheiro ruins, e não houve jeito de agendar uma visita técnica imediada. Além disso, o técnico (muito profissional e competente) veio em um dia diferente do marcado - por sorte eu estava em casa.</t>
+  </si>
+  <si>
+    <t>Satisfeito, porém a assistência técnica  não  tem sido realizada  conforme  combinado cada 6 meses.</t>
+  </si>
+  <si>
+    <t>Estou a quase 3 meses solicitando a troca porque não está gelando e nada, quase 8 anos com vcs e esse é o tratamento que recebo</t>
+  </si>
+  <si>
+    <t>Voces sao pessimos! O atendimento é horrivel, desligam a ligação, uma tremenda falta de consideração. Nao respeitam prazos.</t>
+  </si>
+  <si>
+    <t>FRQ ZONA NORTE SP</t>
+  </si>
+  <si>
+    <t>Tivemos a visita, o técnico já tinha conhecimento que estávamos sem água, pois o painel eletronico está com avarias (isso foi mencionado na solicitação técnica). Infelizmente ele veio com painel eletrônico do modelo atual, sendo que tenho instalado em minha residência o modelo antigo Active, segundo o técnico não mais fabricado. Disse que Letícia entraria em contato, mas aconselhava solicitar um novo modelo de purificador, ele tbm disse que o barulho do aparelho estava anormal. Até o momento ninguém entrou em contato.</t>
+  </si>
+  <si>
+    <t>Não aconteceu visita técnica. O atendente ao menos continuou com o agendamento. Aguardando contato da Brastemp.Cel 11 96317-4904</t>
+  </si>
+  <si>
+    <t>Muitas dificuldades com a agua gelada, o sensor queima muito</t>
+  </si>
+  <si>
+    <t>Bom dia!O horário do agendamento eletrônico da visita técnica não condiz com a visita do técnico. A marcação do período do atendimento não funciona. Anteriormente a visita semestral era monitorada e comunicada ao cliente pela Brastemp. Agora não tenho recebido tal comunicado.</t>
+  </si>
+  <si>
+    <t>Boa, porém algumas vezes apresenta problemas, porém o técnico vem e resolve</t>
+  </si>
+  <si>
+    <t>Atendimento foi rápido.</t>
+  </si>
+  <si>
+    <t>Purificar muito bom, já tenho há anos</t>
+  </si>
+  <si>
+    <t>O técnico fez a visita semestral para. Atração do filtro ,mas deixou vazando água no mesmo. Liguei para um atendimento de emergência e só consegui amanhã de tarde uma nova visita.</t>
+  </si>
+  <si>
+    <t>Problemas reiterados</t>
+  </si>
+  <si>
+    <t>Marquei para o horário da tarde, pois quero sempre pessoalmente acompanhar o serviço, mas o técnico chegou próximo às 11:50 h. Muito embora estivesse uma pessoa em minha casa,  no horário da manhã,  o horário da manhã é comum que as pessoas da casa estejam ausente. Como meu irmão chegou de viagem em minha casa, possibilitou o técnico realizar o serviço. Solicito que da próxima vez, chegue no horário correto, pois corre o risco de não ter uma pessoa em casa.</t>
+  </si>
+  <si>
+    <t>Péssima assistência técnica, estou com o purificador quebrado e fazem visitas a toa e não resolvem o problema, cuja solução é trocar o purificador</t>
+  </si>
+  <si>
+    <t>O equipamento e o serviço são excelentes. O custo mensal acho um pouco elevado.</t>
+  </si>
+  <si>
+    <t>O produto eu nao tenho o que reclamar, todavia o serviço se manutenção (que pra mim é o mais importante) ficou a desejar. Tive problema com a qualidade da agua em meu comercio por falta de manutenção periódica. Infelizmente não tenho como me programar para agendar às manutenções pois tem contrato em mais de um estabelecimento. E para minha surpresa, comecei a ter reclamação de colaboradores pela qualidade da agua e quando chamei o tecnico, descobri que a troca do elemento filtrante estava vencida a mais de 3 meses!Algo que contratei pela comodidade, agora tenho que me preocupar em agendar as manutenções.</t>
+  </si>
+  <si>
+    <t>Não vieram fazer a substituição do filtro Estou desde fevereiro sem água gelada Já vieram 2 técnicos e não resolveram e já solicitei a troca que foi agendada para dia 11/03 e nada ninguém apareceu</t>
+  </si>
+  <si>
+    <t>problemas com a troca do aparelho, já solicitado embvisitas tecnicas anteriores e não efetivado</t>
+  </si>
+  <si>
+    <t>Não foi trocado filtro da água. O técnico fez o teste na água e disse que a qualidade estava boa. Eu perguntei do filtro e ele falou que só é trocado a cada 3 anos!?!De qualquer forma vou me mudar em Maio e vou adquirir uma geladeira com água e gelo na porta, daí vou devolver o filtro.</t>
   </si>
 </sst>
 </file>
@@ -2526,7 +2718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I601"/>
+  <dimension ref="A1:I658"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -17999,7 +18191,7 @@
     </row>
     <row r="534" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A534">
-        <v>8857814</v>
+        <v>533</v>
       </c>
       <c r="B534" t="s">
         <v>9</v>
@@ -18028,7 +18220,7 @@
     </row>
     <row r="535" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A535">
-        <v>8881701</v>
+        <v>534</v>
       </c>
       <c r="B535" t="s">
         <v>9</v>
@@ -18057,7 +18249,7 @@
     </row>
     <row r="536" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A536">
-        <v>8881896</v>
+        <v>535</v>
       </c>
       <c r="B536" t="s">
         <v>61</v>
@@ -18086,7 +18278,7 @@
     </row>
     <row r="537" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A537">
-        <v>8881808</v>
+        <v>536</v>
       </c>
       <c r="B537" t="s">
         <v>9</v>
@@ -18115,7 +18307,7 @@
     </row>
     <row r="538" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A538">
-        <v>8881685</v>
+        <v>537</v>
       </c>
       <c r="B538" t="s">
         <v>9</v>
@@ -18144,7 +18336,7 @@
     </row>
     <row r="539" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A539">
-        <v>8881804</v>
+        <v>538</v>
       </c>
       <c r="B539" t="s">
         <v>9</v>
@@ -18173,7 +18365,7 @@
     </row>
     <row r="540" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A540">
-        <v>8881771</v>
+        <v>539</v>
       </c>
       <c r="B540" t="s">
         <v>9</v>
@@ -18202,7 +18394,7 @@
     </row>
     <row r="541" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A541">
-        <v>8881671</v>
+        <v>540</v>
       </c>
       <c r="B541" t="s">
         <v>9</v>
@@ -18231,7 +18423,7 @@
     </row>
     <row r="542" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A542">
-        <v>8867237</v>
+        <v>541</v>
       </c>
       <c r="B542" t="s">
         <v>9</v>
@@ -18260,7 +18452,7 @@
     </row>
     <row r="543" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A543">
-        <v>8866898</v>
+        <v>542</v>
       </c>
       <c r="B543" t="s">
         <v>9</v>
@@ -18289,7 +18481,7 @@
     </row>
     <row r="544" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A544">
-        <v>8889614</v>
+        <v>543</v>
       </c>
       <c r="B544" t="s">
         <v>9</v>
@@ -18318,7 +18510,7 @@
     </row>
     <row r="545" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A545">
-        <v>8889585</v>
+        <v>544</v>
       </c>
       <c r="B545" t="s">
         <v>9</v>
@@ -18347,7 +18539,7 @@
     </row>
     <row r="546" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A546">
-        <v>8889620</v>
+        <v>545</v>
       </c>
       <c r="B546" t="s">
         <v>61</v>
@@ -18376,7 +18568,7 @@
     </row>
     <row r="547" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A547">
-        <v>8889373</v>
+        <v>546</v>
       </c>
       <c r="B547" t="s">
         <v>9</v>
@@ -18405,7 +18597,7 @@
     </row>
     <row r="548" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A548">
-        <v>8889520</v>
+        <v>547</v>
       </c>
       <c r="B548" t="s">
         <v>9</v>
@@ -18434,7 +18626,7 @@
     </row>
     <row r="549" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A549">
-        <v>8889417</v>
+        <v>548</v>
       </c>
       <c r="B549" t="s">
         <v>9</v>
@@ -18463,7 +18655,7 @@
     </row>
     <row r="550" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A550">
-        <v>8889594</v>
+        <v>549</v>
       </c>
       <c r="B550" t="s">
         <v>9</v>
@@ -18492,7 +18684,7 @@
     </row>
     <row r="551" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A551">
-        <v>8889318</v>
+        <v>550</v>
       </c>
       <c r="B551" t="s">
         <v>9</v>
@@ -18521,7 +18713,7 @@
     </row>
     <row r="552" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A552">
-        <v>8889670</v>
+        <v>551</v>
       </c>
       <c r="B552" t="s">
         <v>9</v>
@@ -18550,7 +18742,7 @@
     </row>
     <row r="553" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A553">
-        <v>8889305</v>
+        <v>552</v>
       </c>
       <c r="B553" t="s">
         <v>9</v>
@@ -18579,7 +18771,7 @@
     </row>
     <row r="554" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A554">
-        <v>8889325</v>
+        <v>553</v>
       </c>
       <c r="B554" t="s">
         <v>9</v>
@@ -18608,7 +18800,7 @@
     </row>
     <row r="555" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A555">
-        <v>8889523</v>
+        <v>554</v>
       </c>
       <c r="B555" t="s">
         <v>9</v>
@@ -18637,7 +18829,7 @@
     </row>
     <row r="556" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A556">
-        <v>8866885</v>
+        <v>555</v>
       </c>
       <c r="B556" t="s">
         <v>9</v>
@@ -18666,7 +18858,7 @@
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A557">
-        <v>8889435</v>
+        <v>556</v>
       </c>
       <c r="B557" t="s">
         <v>9</v>
@@ -18695,7 +18887,7 @@
     </row>
     <row r="558" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A558">
-        <v>8889483</v>
+        <v>557</v>
       </c>
       <c r="B558" t="s">
         <v>9</v>
@@ -18724,7 +18916,7 @@
     </row>
     <row r="559" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A559">
-        <v>8889478</v>
+        <v>558</v>
       </c>
       <c r="B559" t="s">
         <v>9</v>
@@ -18753,7 +18945,7 @@
     </row>
     <row r="560" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A560">
-        <v>8889672</v>
+        <v>559</v>
       </c>
       <c r="B560" t="s">
         <v>9</v>
@@ -18782,7 +18974,7 @@
     </row>
     <row r="561" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A561">
-        <v>8897786</v>
+        <v>560</v>
       </c>
       <c r="B561" t="s">
         <v>9</v>
@@ -18811,7 +19003,7 @@
     </row>
     <row r="562" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A562">
-        <v>8897778</v>
+        <v>561</v>
       </c>
       <c r="B562" t="s">
         <v>9</v>
@@ -18840,7 +19032,7 @@
     </row>
     <row r="563" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A563">
-        <v>8897772</v>
+        <v>562</v>
       </c>
       <c r="B563" t="s">
         <v>9</v>
@@ -18869,7 +19061,7 @@
     </row>
     <row r="564" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A564">
-        <v>8897755</v>
+        <v>563</v>
       </c>
       <c r="B564" t="s">
         <v>9</v>
@@ -18898,7 +19090,7 @@
     </row>
     <row r="565" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A565">
-        <v>8897660</v>
+        <v>564</v>
       </c>
       <c r="B565" t="s">
         <v>9</v>
@@ -18927,7 +19119,7 @@
     </row>
     <row r="566" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A566">
-        <v>8897704</v>
+        <v>565</v>
       </c>
       <c r="B566" t="s">
         <v>9</v>
@@ -18956,7 +19148,7 @@
     </row>
     <row r="567" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A567">
-        <v>8897681</v>
+        <v>566</v>
       </c>
       <c r="B567" t="s">
         <v>9</v>
@@ -18985,7 +19177,7 @@
     </row>
     <row r="568" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A568">
-        <v>8897572</v>
+        <v>567</v>
       </c>
       <c r="B568" t="s">
         <v>9</v>
@@ -19014,7 +19206,7 @@
     </row>
     <row r="569" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A569">
-        <v>8897639</v>
+        <v>568</v>
       </c>
       <c r="B569" t="s">
         <v>9</v>
@@ -19043,7 +19235,7 @@
     </row>
     <row r="570" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A570">
-        <v>8897519</v>
+        <v>569</v>
       </c>
       <c r="B570" t="s">
         <v>9</v>
@@ -19072,7 +19264,7 @@
     </row>
     <row r="571" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A571">
-        <v>8897606</v>
+        <v>570</v>
       </c>
       <c r="B571" t="s">
         <v>9</v>
@@ -19101,7 +19293,7 @@
     </row>
     <row r="572" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A572">
-        <v>8903836</v>
+        <v>571</v>
       </c>
       <c r="B572" t="s">
         <v>9</v>
@@ -19130,7 +19322,7 @@
     </row>
     <row r="573" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A573">
-        <v>8903588</v>
+        <v>572</v>
       </c>
       <c r="B573" t="s">
         <v>9</v>
@@ -19159,7 +19351,7 @@
     </row>
     <row r="574" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A574">
-        <v>8881537</v>
+        <v>573</v>
       </c>
       <c r="B574" t="s">
         <v>9</v>
@@ -19188,7 +19380,7 @@
     </row>
     <row r="575" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A575">
-        <v>8903598</v>
+        <v>574</v>
       </c>
       <c r="B575" t="s">
         <v>9</v>
@@ -19217,7 +19409,7 @@
     </row>
     <row r="576" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A576">
-        <v>8903502</v>
+        <v>575</v>
       </c>
       <c r="B576" t="s">
         <v>9</v>
@@ -19246,7 +19438,7 @@
     </row>
     <row r="577" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A577">
-        <v>8903614</v>
+        <v>576</v>
       </c>
       <c r="B577" t="s">
         <v>9</v>
@@ -19275,7 +19467,7 @@
     </row>
     <row r="578" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A578">
-        <v>8903637</v>
+        <v>577</v>
       </c>
       <c r="B578" t="s">
         <v>9</v>
@@ -19304,7 +19496,7 @@
     </row>
     <row r="579" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A579">
-        <v>8903858</v>
+        <v>578</v>
       </c>
       <c r="B579" t="s">
         <v>61</v>
@@ -19333,7 +19525,7 @@
     </row>
     <row r="580" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A580">
-        <v>8903461</v>
+        <v>579</v>
       </c>
       <c r="B580" t="s">
         <v>9</v>
@@ -19362,7 +19554,7 @@
     </row>
     <row r="581" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A581">
-        <v>8903606</v>
+        <v>580</v>
       </c>
       <c r="B581" t="s">
         <v>9</v>
@@ -19391,7 +19583,7 @@
     </row>
     <row r="582" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A582">
-        <v>8903644</v>
+        <v>581</v>
       </c>
       <c r="B582" t="s">
         <v>9</v>
@@ -19420,7 +19612,7 @@
     </row>
     <row r="583" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A583">
-        <v>8903848</v>
+        <v>582</v>
       </c>
       <c r="B583" t="s">
         <v>9</v>
@@ -19449,7 +19641,7 @@
     </row>
     <row r="584" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A584">
-        <v>8903597</v>
+        <v>583</v>
       </c>
       <c r="B584" t="s">
         <v>9</v>
@@ -19478,7 +19670,7 @@
     </row>
     <row r="585" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A585">
-        <v>8903838</v>
+        <v>584</v>
       </c>
       <c r="B585" t="s">
         <v>9</v>
@@ -19507,7 +19699,7 @@
     </row>
     <row r="586" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A586">
-        <v>8903571</v>
+        <v>585</v>
       </c>
       <c r="B586" t="s">
         <v>9</v>
@@ -19536,7 +19728,7 @@
     </row>
     <row r="587" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A587">
-        <v>8903450</v>
+        <v>586</v>
       </c>
       <c r="B587" t="s">
         <v>9</v>
@@ -19565,7 +19757,7 @@
     </row>
     <row r="588" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A588">
-        <v>8903657</v>
+        <v>587</v>
       </c>
       <c r="B588" t="s">
         <v>9</v>
@@ -19594,7 +19786,7 @@
     </row>
     <row r="589" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A589">
-        <v>8881894</v>
+        <v>588</v>
       </c>
       <c r="B589" t="s">
         <v>9</v>
@@ -19623,7 +19815,7 @@
     </row>
     <row r="590" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A590">
-        <v>8903712</v>
+        <v>589</v>
       </c>
       <c r="B590" t="s">
         <v>9</v>
@@ -19652,7 +19844,7 @@
     </row>
     <row r="591" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A591">
-        <v>8903551</v>
+        <v>590</v>
       </c>
       <c r="B591" t="s">
         <v>9</v>
@@ -19681,7 +19873,7 @@
     </row>
     <row r="592" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A592">
-        <v>8915306</v>
+        <v>591</v>
       </c>
       <c r="B592" t="s">
         <v>9</v>
@@ -19710,7 +19902,7 @@
     </row>
     <row r="593" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A593">
-        <v>8903783</v>
+        <v>592</v>
       </c>
       <c r="B593" t="s">
         <v>9</v>
@@ -19739,7 +19931,7 @@
     </row>
     <row r="594" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A594">
-        <v>8915198</v>
+        <v>593</v>
       </c>
       <c r="B594" t="s">
         <v>9</v>
@@ -19768,7 +19960,7 @@
     </row>
     <row r="595" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A595">
-        <v>8889589</v>
+        <v>594</v>
       </c>
       <c r="B595" t="s">
         <v>9</v>
@@ -19797,7 +19989,7 @@
     </row>
     <row r="596" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A596">
-        <v>8915325</v>
+        <v>595</v>
       </c>
       <c r="B596" t="s">
         <v>9</v>
@@ -19826,7 +20018,7 @@
     </row>
     <row r="597" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A597">
-        <v>8915108</v>
+        <v>596</v>
       </c>
       <c r="B597" t="s">
         <v>9</v>
@@ -19855,7 +20047,7 @@
     </row>
     <row r="598" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A598">
-        <v>8915259</v>
+        <v>597</v>
       </c>
       <c r="B598" t="s">
         <v>9</v>
@@ -19884,7 +20076,7 @@
     </row>
     <row r="599" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A599">
-        <v>8915275</v>
+        <v>598</v>
       </c>
       <c r="B599" t="s">
         <v>9</v>
@@ -19913,7 +20105,7 @@
     </row>
     <row r="600" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A600">
-        <v>8915042</v>
+        <v>599</v>
       </c>
       <c r="B600" t="s">
         <v>9</v>
@@ -19942,7 +20134,7 @@
     </row>
     <row r="601" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A601">
-        <v>8889308</v>
+        <v>600</v>
       </c>
       <c r="B601" t="s">
         <v>9</v>
@@ -19967,6 +20159,1659 @@
       </c>
       <c r="I601" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="602" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A602">
+        <v>601</v>
+      </c>
+      <c r="B602" t="s">
+        <v>9</v>
+      </c>
+      <c r="C602">
+        <v>4690</v>
+      </c>
+      <c r="D602" s="3">
+        <v>46089.48265046296</v>
+      </c>
+      <c r="E602" t="s">
+        <v>582</v>
+      </c>
+      <c r="F602" t="s">
+        <v>11</v>
+      </c>
+      <c r="G602" t="s">
+        <v>676</v>
+      </c>
+      <c r="H602" t="s">
+        <v>18</v>
+      </c>
+      <c r="I602" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="603" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A603">
+        <v>602</v>
+      </c>
+      <c r="B603" t="s">
+        <v>9</v>
+      </c>
+      <c r="C603">
+        <v>8005280262</v>
+      </c>
+      <c r="D603" s="3">
+        <v>46090.374479166669</v>
+      </c>
+      <c r="E603" t="s">
+        <v>15</v>
+      </c>
+      <c r="F603" t="s">
+        <v>11</v>
+      </c>
+      <c r="G603" t="s">
+        <v>677</v>
+      </c>
+      <c r="H603" t="s">
+        <v>609</v>
+      </c>
+      <c r="I603" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="604" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A604">
+        <v>603</v>
+      </c>
+      <c r="B604" t="s">
+        <v>9</v>
+      </c>
+      <c r="C604">
+        <v>8005290999</v>
+      </c>
+      <c r="D604" s="3">
+        <v>46090.414444444446</v>
+      </c>
+      <c r="E604" t="s">
+        <v>20</v>
+      </c>
+      <c r="F604" t="s">
+        <v>16</v>
+      </c>
+      <c r="G604" t="s">
+        <v>678</v>
+      </c>
+      <c r="H604" t="s">
+        <v>609</v>
+      </c>
+      <c r="I604" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="605" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A605">
+        <v>604</v>
+      </c>
+      <c r="B605" t="s">
+        <v>9</v>
+      </c>
+      <c r="C605">
+        <v>2862</v>
+      </c>
+      <c r="D605" s="3">
+        <v>46090.431203703702</v>
+      </c>
+      <c r="E605" t="s">
+        <v>556</v>
+      </c>
+      <c r="F605" t="s">
+        <v>16</v>
+      </c>
+      <c r="G605" t="s">
+        <v>679</v>
+      </c>
+      <c r="H605" t="s">
+        <v>82</v>
+      </c>
+      <c r="I605" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="606" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A606">
+        <v>605</v>
+      </c>
+      <c r="B606" t="s">
+        <v>9</v>
+      </c>
+      <c r="C606">
+        <v>3195</v>
+      </c>
+      <c r="D606" s="3">
+        <v>46090.435601851852</v>
+      </c>
+      <c r="E606" t="s">
+        <v>680</v>
+      </c>
+      <c r="F606" t="s">
+        <v>16</v>
+      </c>
+      <c r="G606" t="s">
+        <v>681</v>
+      </c>
+      <c r="H606" t="s">
+        <v>18</v>
+      </c>
+      <c r="I606" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="607" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A607">
+        <v>606</v>
+      </c>
+      <c r="B607" t="s">
+        <v>9</v>
+      </c>
+      <c r="C607">
+        <v>8005302123</v>
+      </c>
+      <c r="D607" s="3">
+        <v>46090.438113425917</v>
+      </c>
+      <c r="E607" t="s">
+        <v>20</v>
+      </c>
+      <c r="F607" t="s">
+        <v>16</v>
+      </c>
+      <c r="G607" t="s">
+        <v>683</v>
+      </c>
+      <c r="H607" t="s">
+        <v>18</v>
+      </c>
+      <c r="I607" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="608" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A608">
+        <v>607</v>
+      </c>
+      <c r="B608" t="s">
+        <v>9</v>
+      </c>
+      <c r="C608">
+        <v>6921</v>
+      </c>
+      <c r="D608" s="3">
+        <v>46090.448009259257</v>
+      </c>
+      <c r="E608" t="s">
+        <v>684</v>
+      </c>
+      <c r="F608" t="s">
+        <v>16</v>
+      </c>
+      <c r="G608" t="s">
+        <v>685</v>
+      </c>
+      <c r="H608" t="s">
+        <v>18</v>
+      </c>
+      <c r="I608" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="609" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A609">
+        <v>608</v>
+      </c>
+      <c r="B609" t="s">
+        <v>9</v>
+      </c>
+      <c r="C609">
+        <v>8005317883</v>
+      </c>
+      <c r="D609" s="3">
+        <v>46090.464548611111</v>
+      </c>
+      <c r="E609" t="s">
+        <v>53</v>
+      </c>
+      <c r="F609" t="s">
+        <v>11</v>
+      </c>
+      <c r="G609" t="s">
+        <v>686</v>
+      </c>
+      <c r="H609" t="s">
+        <v>609</v>
+      </c>
+      <c r="I609" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="610" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A610">
+        <v>609</v>
+      </c>
+      <c r="B610" t="s">
+        <v>9</v>
+      </c>
+      <c r="C610">
+        <v>8005318458</v>
+      </c>
+      <c r="D610" s="3">
+        <v>46090.466226851851</v>
+      </c>
+      <c r="E610" t="s">
+        <v>20</v>
+      </c>
+      <c r="F610" t="s">
+        <v>11</v>
+      </c>
+      <c r="G610" t="s">
+        <v>157</v>
+      </c>
+      <c r="H610" t="s">
+        <v>13</v>
+      </c>
+      <c r="I610" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="611" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A611">
+        <v>610</v>
+      </c>
+      <c r="B611" t="s">
+        <v>9</v>
+      </c>
+      <c r="C611">
+        <v>8005305336</v>
+      </c>
+      <c r="D611" s="3">
+        <v>46090.480879629627</v>
+      </c>
+      <c r="E611" t="s">
+        <v>20</v>
+      </c>
+      <c r="F611" t="s">
+        <v>16</v>
+      </c>
+      <c r="G611" t="s">
+        <v>687</v>
+      </c>
+      <c r="H611" t="s">
+        <v>18</v>
+      </c>
+      <c r="I611" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="612" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A612">
+        <v>611</v>
+      </c>
+      <c r="B612" t="s">
+        <v>9</v>
+      </c>
+      <c r="C612">
+        <v>8005306795</v>
+      </c>
+      <c r="D612" s="3">
+        <v>46090.497893518521</v>
+      </c>
+      <c r="E612" t="s">
+        <v>20</v>
+      </c>
+      <c r="F612" t="s">
+        <v>16</v>
+      </c>
+      <c r="G612" t="s">
+        <v>688</v>
+      </c>
+      <c r="H612" t="s">
+        <v>18</v>
+      </c>
+      <c r="I612" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="613" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A613">
+        <v>612</v>
+      </c>
+      <c r="B613" t="s">
+        <v>9</v>
+      </c>
+      <c r="C613">
+        <v>5338</v>
+      </c>
+      <c r="D613" s="3">
+        <v>46090.501446759263</v>
+      </c>
+      <c r="E613" t="s">
+        <v>680</v>
+      </c>
+      <c r="F613" t="s">
+        <v>16</v>
+      </c>
+      <c r="G613" t="s">
+        <v>689</v>
+      </c>
+      <c r="H613" t="s">
+        <v>13</v>
+      </c>
+      <c r="I613" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="614" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A614">
+        <v>613</v>
+      </c>
+      <c r="B614" t="s">
+        <v>9</v>
+      </c>
+      <c r="C614">
+        <v>8005302146</v>
+      </c>
+      <c r="D614" s="3">
+        <v>46090.511261574073</v>
+      </c>
+      <c r="E614" t="s">
+        <v>49</v>
+      </c>
+      <c r="F614" t="s">
+        <v>16</v>
+      </c>
+      <c r="G614" t="s">
+        <v>690</v>
+      </c>
+      <c r="H614" t="s">
+        <v>18</v>
+      </c>
+      <c r="I614" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="615" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A615">
+        <v>614</v>
+      </c>
+      <c r="B615" t="s">
+        <v>9</v>
+      </c>
+      <c r="C615">
+        <v>8005310015</v>
+      </c>
+      <c r="D615" s="3">
+        <v>46090.513726851852</v>
+      </c>
+      <c r="E615" t="s">
+        <v>20</v>
+      </c>
+      <c r="F615" t="s">
+        <v>11</v>
+      </c>
+      <c r="G615" t="s">
+        <v>691</v>
+      </c>
+      <c r="H615" t="s">
+        <v>13</v>
+      </c>
+      <c r="I615" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="616" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A616">
+        <v>615</v>
+      </c>
+      <c r="B616" t="s">
+        <v>9</v>
+      </c>
+      <c r="C616">
+        <v>8005302395</v>
+      </c>
+      <c r="D616" s="3">
+        <v>46090.618726851862</v>
+      </c>
+      <c r="E616" t="s">
+        <v>125</v>
+      </c>
+      <c r="F616" t="s">
+        <v>16</v>
+      </c>
+      <c r="G616" t="s">
+        <v>692</v>
+      </c>
+      <c r="H616" t="s">
+        <v>18</v>
+      </c>
+      <c r="I616" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="617" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A617">
+        <v>616</v>
+      </c>
+      <c r="B617" t="s">
+        <v>9</v>
+      </c>
+      <c r="C617">
+        <v>8005303304</v>
+      </c>
+      <c r="D617" s="3">
+        <v>46090.629212962973</v>
+      </c>
+      <c r="E617" t="s">
+        <v>20</v>
+      </c>
+      <c r="F617" t="s">
+        <v>16</v>
+      </c>
+      <c r="G617" t="s">
+        <v>693</v>
+      </c>
+      <c r="H617" t="s">
+        <v>13</v>
+      </c>
+      <c r="I617" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="618" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A618">
+        <v>617</v>
+      </c>
+      <c r="B618" t="s">
+        <v>9</v>
+      </c>
+      <c r="C618">
+        <v>8005317407</v>
+      </c>
+      <c r="D618" s="3">
+        <v>46090.641018518523</v>
+      </c>
+      <c r="E618" t="s">
+        <v>20</v>
+      </c>
+      <c r="F618" t="s">
+        <v>11</v>
+      </c>
+      <c r="G618" t="s">
+        <v>694</v>
+      </c>
+      <c r="H618" t="s">
+        <v>18</v>
+      </c>
+      <c r="I618" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="619" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A619">
+        <v>618</v>
+      </c>
+      <c r="B619" t="s">
+        <v>9</v>
+      </c>
+      <c r="C619">
+        <v>8005301539</v>
+      </c>
+      <c r="D619" s="3">
+        <v>46090.943391203713</v>
+      </c>
+      <c r="E619" t="s">
+        <v>20</v>
+      </c>
+      <c r="F619" t="s">
+        <v>11</v>
+      </c>
+      <c r="G619" t="s">
+        <v>695</v>
+      </c>
+      <c r="H619" t="s">
+        <v>13</v>
+      </c>
+      <c r="I619" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="620" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A620">
+        <v>619</v>
+      </c>
+      <c r="B620" t="s">
+        <v>9</v>
+      </c>
+      <c r="C620">
+        <v>6340</v>
+      </c>
+      <c r="D620" s="3">
+        <v>46091.385729166657</v>
+      </c>
+      <c r="E620" t="s">
+        <v>585</v>
+      </c>
+      <c r="F620" t="s">
+        <v>16</v>
+      </c>
+      <c r="G620" t="s">
+        <v>696</v>
+      </c>
+      <c r="H620" t="s">
+        <v>609</v>
+      </c>
+      <c r="I620" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="621" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A621">
+        <v>620</v>
+      </c>
+      <c r="B621" t="s">
+        <v>9</v>
+      </c>
+      <c r="C621">
+        <v>8005320373</v>
+      </c>
+      <c r="D621" s="3">
+        <v>46091.404930555553</v>
+      </c>
+      <c r="E621" t="s">
+        <v>74</v>
+      </c>
+      <c r="F621" t="s">
+        <v>11</v>
+      </c>
+      <c r="G621" t="s">
+        <v>697</v>
+      </c>
+      <c r="H621" t="s">
+        <v>154</v>
+      </c>
+      <c r="I621" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="622" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A622">
+        <v>621</v>
+      </c>
+      <c r="B622" t="s">
+        <v>9</v>
+      </c>
+      <c r="C622">
+        <v>8005302363</v>
+      </c>
+      <c r="D622" s="3">
+        <v>46091.437696759262</v>
+      </c>
+      <c r="E622" t="s">
+        <v>20</v>
+      </c>
+      <c r="F622" t="s">
+        <v>16</v>
+      </c>
+      <c r="G622" t="s">
+        <v>699</v>
+      </c>
+      <c r="H622" t="s">
+        <v>18</v>
+      </c>
+      <c r="I622" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="623" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A623">
+        <v>622</v>
+      </c>
+      <c r="B623" t="s">
+        <v>9</v>
+      </c>
+      <c r="C623">
+        <v>1177</v>
+      </c>
+      <c r="D623" s="3">
+        <v>46091.450520833343</v>
+      </c>
+      <c r="E623" t="s">
+        <v>700</v>
+      </c>
+      <c r="F623" t="s">
+        <v>11</v>
+      </c>
+      <c r="G623" t="s">
+        <v>701</v>
+      </c>
+      <c r="H623" t="s">
+        <v>82</v>
+      </c>
+      <c r="I623" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="624" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A624">
+        <v>623</v>
+      </c>
+      <c r="B624" t="s">
+        <v>9</v>
+      </c>
+      <c r="C624">
+        <v>6174</v>
+      </c>
+      <c r="D624" s="3">
+        <v>46091.474988425929</v>
+      </c>
+      <c r="E624" t="s">
+        <v>702</v>
+      </c>
+      <c r="F624" t="s">
+        <v>16</v>
+      </c>
+      <c r="G624" t="s">
+        <v>703</v>
+      </c>
+      <c r="H624" t="s">
+        <v>609</v>
+      </c>
+      <c r="I624" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="625" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A625">
+        <v>624</v>
+      </c>
+      <c r="B625" t="s">
+        <v>9</v>
+      </c>
+      <c r="C625">
+        <v>8005251852</v>
+      </c>
+      <c r="D625" s="3">
+        <v>46091.514664351853</v>
+      </c>
+      <c r="E625" t="s">
+        <v>37</v>
+      </c>
+      <c r="F625" t="s">
+        <v>16</v>
+      </c>
+      <c r="G625" t="s">
+        <v>704</v>
+      </c>
+      <c r="H625" t="s">
+        <v>609</v>
+      </c>
+      <c r="I625" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="626" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A626">
+        <v>625</v>
+      </c>
+      <c r="B626" t="s">
+        <v>9</v>
+      </c>
+      <c r="C626">
+        <v>8005321370</v>
+      </c>
+      <c r="D626" s="3">
+        <v>46091.51902777778</v>
+      </c>
+      <c r="E626" t="s">
+        <v>53</v>
+      </c>
+      <c r="F626" t="s">
+        <v>16</v>
+      </c>
+      <c r="G626" t="s">
+        <v>705</v>
+      </c>
+      <c r="H626" t="s">
+        <v>609</v>
+      </c>
+      <c r="I626" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="627" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A627">
+        <v>626</v>
+      </c>
+      <c r="B627" t="s">
+        <v>9</v>
+      </c>
+      <c r="C627">
+        <v>8005301779</v>
+      </c>
+      <c r="D627" s="3">
+        <v>46091.530266203707</v>
+      </c>
+      <c r="E627" t="s">
+        <v>20</v>
+      </c>
+      <c r="F627" t="s">
+        <v>11</v>
+      </c>
+      <c r="G627" t="s">
+        <v>706</v>
+      </c>
+      <c r="H627" t="s">
+        <v>13</v>
+      </c>
+      <c r="I627" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="628" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A628">
+        <v>627</v>
+      </c>
+      <c r="B628" t="s">
+        <v>9</v>
+      </c>
+      <c r="C628">
+        <v>8005322861</v>
+      </c>
+      <c r="D628" s="3">
+        <v>46091.538831018523</v>
+      </c>
+      <c r="E628" t="s">
+        <v>20</v>
+      </c>
+      <c r="F628" t="s">
+        <v>11</v>
+      </c>
+      <c r="G628" t="s">
+        <v>707</v>
+      </c>
+      <c r="H628" t="s">
+        <v>13</v>
+      </c>
+      <c r="I628" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="629" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A629">
+        <v>628</v>
+      </c>
+      <c r="B629" t="s">
+        <v>9</v>
+      </c>
+      <c r="C629">
+        <v>8005293029</v>
+      </c>
+      <c r="D629" s="3">
+        <v>46091.549664351849</v>
+      </c>
+      <c r="E629" t="s">
+        <v>15</v>
+      </c>
+      <c r="F629" t="s">
+        <v>11</v>
+      </c>
+      <c r="G629" t="s">
+        <v>708</v>
+      </c>
+      <c r="H629" t="s">
+        <v>609</v>
+      </c>
+      <c r="I629" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="630" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A630">
+        <v>629</v>
+      </c>
+      <c r="B630" t="s">
+        <v>9</v>
+      </c>
+      <c r="C630">
+        <v>8005315721</v>
+      </c>
+      <c r="D630" s="3">
+        <v>46091.556435185194</v>
+      </c>
+      <c r="E630" t="s">
+        <v>65</v>
+      </c>
+      <c r="F630" t="s">
+        <v>11</v>
+      </c>
+      <c r="G630" t="s">
+        <v>709</v>
+      </c>
+      <c r="H630" t="s">
+        <v>13</v>
+      </c>
+      <c r="I630" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="631" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A631">
+        <v>630</v>
+      </c>
+      <c r="B631" t="s">
+        <v>9</v>
+      </c>
+      <c r="C631">
+        <v>8005319591</v>
+      </c>
+      <c r="D631" s="3">
+        <v>46091.558333333327</v>
+      </c>
+      <c r="E631" t="s">
+        <v>53</v>
+      </c>
+      <c r="F631" t="s">
+        <v>11</v>
+      </c>
+      <c r="G631" t="s">
+        <v>710</v>
+      </c>
+      <c r="H631" t="s">
+        <v>32</v>
+      </c>
+      <c r="I631" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="632" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A632">
+        <v>631</v>
+      </c>
+      <c r="B632" t="s">
+        <v>9</v>
+      </c>
+      <c r="C632">
+        <v>8005298116</v>
+      </c>
+      <c r="D632" s="3">
+        <v>46091.586550925917</v>
+      </c>
+      <c r="E632" t="s">
+        <v>49</v>
+      </c>
+      <c r="F632" t="s">
+        <v>16</v>
+      </c>
+      <c r="G632" t="s">
+        <v>711</v>
+      </c>
+      <c r="H632" t="s">
+        <v>18</v>
+      </c>
+      <c r="I632" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="633" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A633">
+        <v>632</v>
+      </c>
+      <c r="B633" t="s">
+        <v>9</v>
+      </c>
+      <c r="C633">
+        <v>8005301315</v>
+      </c>
+      <c r="D633" s="3">
+        <v>46091.607893518521</v>
+      </c>
+      <c r="E633" t="s">
+        <v>20</v>
+      </c>
+      <c r="F633" t="s">
+        <v>11</v>
+      </c>
+      <c r="G633" t="s">
+        <v>712</v>
+      </c>
+      <c r="H633" t="s">
+        <v>18</v>
+      </c>
+      <c r="I633" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="634" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A634">
+        <v>633</v>
+      </c>
+      <c r="B634" t="s">
+        <v>9</v>
+      </c>
+      <c r="C634">
+        <v>6457</v>
+      </c>
+      <c r="D634" s="3">
+        <v>46091.610069444447</v>
+      </c>
+      <c r="E634" t="s">
+        <v>684</v>
+      </c>
+      <c r="F634" t="s">
+        <v>16</v>
+      </c>
+      <c r="G634" t="s">
+        <v>713</v>
+      </c>
+      <c r="H634" t="s">
+        <v>32</v>
+      </c>
+      <c r="I634" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="635" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A635">
+        <v>634</v>
+      </c>
+      <c r="B635" t="s">
+        <v>9</v>
+      </c>
+      <c r="C635">
+        <v>8005321855</v>
+      </c>
+      <c r="D635" s="3">
+        <v>46091.631493055553</v>
+      </c>
+      <c r="E635" t="s">
+        <v>98</v>
+      </c>
+      <c r="F635" t="s">
+        <v>16</v>
+      </c>
+      <c r="G635" t="s">
+        <v>714</v>
+      </c>
+      <c r="H635" t="s">
+        <v>18</v>
+      </c>
+      <c r="I635" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="636" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A636">
+        <v>635</v>
+      </c>
+      <c r="B636" t="s">
+        <v>9</v>
+      </c>
+      <c r="C636">
+        <v>6778</v>
+      </c>
+      <c r="D636" s="3">
+        <v>46091.738668981481</v>
+      </c>
+      <c r="E636" t="s">
+        <v>715</v>
+      </c>
+      <c r="F636" t="s">
+        <v>16</v>
+      </c>
+      <c r="G636" t="s">
+        <v>716</v>
+      </c>
+      <c r="H636" t="s">
+        <v>32</v>
+      </c>
+      <c r="I636" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="637" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A637">
+        <v>636</v>
+      </c>
+      <c r="B637" t="s">
+        <v>9</v>
+      </c>
+      <c r="C637">
+        <v>1184</v>
+      </c>
+      <c r="D637" s="3">
+        <v>46091.75209490741</v>
+      </c>
+      <c r="E637" t="s">
+        <v>700</v>
+      </c>
+      <c r="F637" t="s">
+        <v>11</v>
+      </c>
+      <c r="G637" t="s">
+        <v>717</v>
+      </c>
+      <c r="H637" t="s">
+        <v>13</v>
+      </c>
+      <c r="I637" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="638" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A638">
+        <v>637</v>
+      </c>
+      <c r="B638" t="s">
+        <v>9</v>
+      </c>
+      <c r="C638">
+        <v>7769</v>
+      </c>
+      <c r="D638" s="3">
+        <v>46092.369247685187</v>
+      </c>
+      <c r="E638" t="s">
+        <v>702</v>
+      </c>
+      <c r="F638" t="s">
+        <v>16</v>
+      </c>
+      <c r="G638" t="s">
+        <v>718</v>
+      </c>
+      <c r="H638" t="s">
+        <v>13</v>
+      </c>
+      <c r="I638" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="639" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A639">
+        <v>638</v>
+      </c>
+      <c r="B639" t="s">
+        <v>9</v>
+      </c>
+      <c r="C639">
+        <v>7799</v>
+      </c>
+      <c r="D639" s="3">
+        <v>46092.406168981477</v>
+      </c>
+      <c r="E639" t="s">
+        <v>700</v>
+      </c>
+      <c r="F639" t="s">
+        <v>16</v>
+      </c>
+      <c r="G639" t="s">
+        <v>719</v>
+      </c>
+      <c r="H639" t="s">
+        <v>32</v>
+      </c>
+      <c r="I639" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="640" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A640">
+        <v>639</v>
+      </c>
+      <c r="B640" t="s">
+        <v>9</v>
+      </c>
+      <c r="C640">
+        <v>8005305762</v>
+      </c>
+      <c r="D640" s="3">
+        <v>46092.413298611107</v>
+      </c>
+      <c r="E640" t="s">
+        <v>15</v>
+      </c>
+      <c r="F640" t="s">
+        <v>11</v>
+      </c>
+      <c r="G640" t="s">
+        <v>720</v>
+      </c>
+      <c r="H640" t="s">
+        <v>32</v>
+      </c>
+      <c r="I640" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="641" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A641">
+        <v>640</v>
+      </c>
+      <c r="B641" t="s">
+        <v>9</v>
+      </c>
+      <c r="C641">
+        <v>6757</v>
+      </c>
+      <c r="D641" s="3">
+        <v>46092.501481481479</v>
+      </c>
+      <c r="E641" t="s">
+        <v>684</v>
+      </c>
+      <c r="F641" t="s">
+        <v>16</v>
+      </c>
+      <c r="G641" t="s">
+        <v>721</v>
+      </c>
+      <c r="H641" t="s">
+        <v>154</v>
+      </c>
+      <c r="I641" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="642" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A642">
+        <v>641</v>
+      </c>
+      <c r="B642" t="s">
+        <v>9</v>
+      </c>
+      <c r="C642">
+        <v>8005293642</v>
+      </c>
+      <c r="D642" s="3">
+        <v>46092.503784722219</v>
+      </c>
+      <c r="E642" t="s">
+        <v>53</v>
+      </c>
+      <c r="F642" t="s">
+        <v>16</v>
+      </c>
+      <c r="G642" t="s">
+        <v>722</v>
+      </c>
+      <c r="H642" t="s">
+        <v>82</v>
+      </c>
+      <c r="I642" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="643" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A643">
+        <v>642</v>
+      </c>
+      <c r="B643" t="s">
+        <v>9</v>
+      </c>
+      <c r="C643">
+        <v>8126</v>
+      </c>
+      <c r="D643" s="3">
+        <v>46092.664965277778</v>
+      </c>
+      <c r="E643" t="s">
+        <v>723</v>
+      </c>
+      <c r="F643" t="s">
+        <v>16</v>
+      </c>
+      <c r="G643" t="s">
+        <v>724</v>
+      </c>
+      <c r="H643" t="s">
+        <v>154</v>
+      </c>
+      <c r="I643" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="644" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A644">
+        <v>643</v>
+      </c>
+      <c r="B644" t="s">
+        <v>9</v>
+      </c>
+      <c r="C644">
+        <v>8105</v>
+      </c>
+      <c r="D644" s="3">
+        <v>46093.390613425923</v>
+      </c>
+      <c r="E644" t="s">
+        <v>700</v>
+      </c>
+      <c r="F644" t="s">
+        <v>16</v>
+      </c>
+      <c r="G644" t="s">
+        <v>725</v>
+      </c>
+      <c r="H644" t="s">
+        <v>18</v>
+      </c>
+      <c r="I644" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="645" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A645">
+        <v>644</v>
+      </c>
+      <c r="B645" t="s">
+        <v>9</v>
+      </c>
+      <c r="C645">
+        <v>8005319082</v>
+      </c>
+      <c r="D645" s="3">
+        <v>46093.392071759263</v>
+      </c>
+      <c r="E645" t="s">
+        <v>20</v>
+      </c>
+      <c r="F645" t="s">
+        <v>11</v>
+      </c>
+      <c r="G645" t="s">
+        <v>726</v>
+      </c>
+      <c r="H645" t="s">
+        <v>609</v>
+      </c>
+      <c r="I645" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="646" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A646">
+        <v>645</v>
+      </c>
+      <c r="B646" t="s">
+        <v>9</v>
+      </c>
+      <c r="C646">
+        <v>8005299181</v>
+      </c>
+      <c r="D646" s="3">
+        <v>46093.398761574077</v>
+      </c>
+      <c r="E646" t="s">
+        <v>20</v>
+      </c>
+      <c r="F646" t="s">
+        <v>11</v>
+      </c>
+      <c r="G646" t="s">
+        <v>727</v>
+      </c>
+      <c r="H646" t="s">
+        <v>18</v>
+      </c>
+      <c r="I646" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="647" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A647">
+        <v>646</v>
+      </c>
+      <c r="B647" t="s">
+        <v>9</v>
+      </c>
+      <c r="C647">
+        <v>8005325479</v>
+      </c>
+      <c r="D647" s="3">
+        <v>46093.47314814815</v>
+      </c>
+      <c r="E647" t="s">
+        <v>10</v>
+      </c>
+      <c r="F647" t="s">
+        <v>11</v>
+      </c>
+      <c r="G647" t="s">
+        <v>728</v>
+      </c>
+      <c r="H647" t="s">
+        <v>13</v>
+      </c>
+      <c r="I647" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="648" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A648">
+        <v>647</v>
+      </c>
+      <c r="B648" t="s">
+        <v>9</v>
+      </c>
+      <c r="C648">
+        <v>8005317001</v>
+      </c>
+      <c r="D648" s="3">
+        <v>46093.485486111109</v>
+      </c>
+      <c r="E648" t="s">
+        <v>53</v>
+      </c>
+      <c r="F648" t="s">
+        <v>11</v>
+      </c>
+      <c r="G648" t="s">
+        <v>729</v>
+      </c>
+      <c r="H648" t="s">
+        <v>13</v>
+      </c>
+      <c r="I648" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="649" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A649">
+        <v>648</v>
+      </c>
+      <c r="B649" t="s">
+        <v>9</v>
+      </c>
+      <c r="C649">
+        <v>8005319559</v>
+      </c>
+      <c r="D649" s="3">
+        <v>46093.509328703702</v>
+      </c>
+      <c r="E649" t="s">
+        <v>20</v>
+      </c>
+      <c r="F649" t="s">
+        <v>11</v>
+      </c>
+      <c r="G649" t="s">
+        <v>730</v>
+      </c>
+      <c r="H649" t="s">
+        <v>13</v>
+      </c>
+      <c r="I649" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="650" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A650">
+        <v>649</v>
+      </c>
+      <c r="B650" t="s">
+        <v>9</v>
+      </c>
+      <c r="C650">
+        <v>8005318026</v>
+      </c>
+      <c r="D650" s="3">
+        <v>46093.519386574073</v>
+      </c>
+      <c r="E650" t="s">
+        <v>53</v>
+      </c>
+      <c r="F650" t="s">
+        <v>16</v>
+      </c>
+      <c r="G650" t="s">
+        <v>731</v>
+      </c>
+      <c r="H650" t="s">
+        <v>18</v>
+      </c>
+      <c r="I650" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="651" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A651">
+        <v>650</v>
+      </c>
+      <c r="B651" t="s">
+        <v>9</v>
+      </c>
+      <c r="C651">
+        <v>8005317952</v>
+      </c>
+      <c r="D651" s="3">
+        <v>46093.519537037027</v>
+      </c>
+      <c r="E651" t="s">
+        <v>53</v>
+      </c>
+      <c r="F651" t="s">
+        <v>16</v>
+      </c>
+      <c r="G651" t="s">
+        <v>732</v>
+      </c>
+      <c r="H651" t="s">
+        <v>18</v>
+      </c>
+      <c r="I651" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="652" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A652">
+        <v>651</v>
+      </c>
+      <c r="B652" t="s">
+        <v>9</v>
+      </c>
+      <c r="C652">
+        <v>8005317803</v>
+      </c>
+      <c r="D652" s="3">
+        <v>46093.531793981478</v>
+      </c>
+      <c r="E652" t="s">
+        <v>98</v>
+      </c>
+      <c r="F652" t="s">
+        <v>11</v>
+      </c>
+      <c r="G652" t="s">
+        <v>733</v>
+      </c>
+      <c r="H652" t="s">
+        <v>18</v>
+      </c>
+      <c r="I652" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="653" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A653">
+        <v>652</v>
+      </c>
+      <c r="B653" t="s">
+        <v>9</v>
+      </c>
+      <c r="C653">
+        <v>8005321193</v>
+      </c>
+      <c r="D653" s="3">
+        <v>46093.547118055547</v>
+      </c>
+      <c r="E653" t="s">
+        <v>20</v>
+      </c>
+      <c r="F653" t="s">
+        <v>16</v>
+      </c>
+      <c r="G653" t="s">
+        <v>734</v>
+      </c>
+      <c r="H653" t="s">
+        <v>18</v>
+      </c>
+      <c r="I653" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="654" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A654">
+        <v>653</v>
+      </c>
+      <c r="B654" t="s">
+        <v>9</v>
+      </c>
+      <c r="C654">
+        <v>8005315972</v>
+      </c>
+      <c r="D654" s="3">
+        <v>46093.549259259264</v>
+      </c>
+      <c r="E654" t="s">
+        <v>41</v>
+      </c>
+      <c r="F654" t="s">
+        <v>11</v>
+      </c>
+      <c r="G654" t="s">
+        <v>735</v>
+      </c>
+      <c r="H654" t="s">
+        <v>13</v>
+      </c>
+      <c r="I654" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="655" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A655">
+        <v>654</v>
+      </c>
+      <c r="B655" t="s">
+        <v>9</v>
+      </c>
+      <c r="C655">
+        <v>8279</v>
+      </c>
+      <c r="D655" s="3">
+        <v>46093.549525462957</v>
+      </c>
+      <c r="E655" t="s">
+        <v>684</v>
+      </c>
+      <c r="F655" t="s">
+        <v>11</v>
+      </c>
+      <c r="G655" t="s">
+        <v>736</v>
+      </c>
+      <c r="H655" t="s">
+        <v>32</v>
+      </c>
+      <c r="I655" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="656" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A656">
+        <v>655</v>
+      </c>
+      <c r="B656" t="s">
+        <v>9</v>
+      </c>
+      <c r="C656">
+        <v>8005320601</v>
+      </c>
+      <c r="D656" s="3">
+        <v>46093.659178240741</v>
+      </c>
+      <c r="E656" t="s">
+        <v>20</v>
+      </c>
+      <c r="F656" t="s">
+        <v>16</v>
+      </c>
+      <c r="G656" t="s">
+        <v>737</v>
+      </c>
+      <c r="H656" t="s">
+        <v>18</v>
+      </c>
+      <c r="I656" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="657" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A657">
+        <v>656</v>
+      </c>
+      <c r="B657" t="s">
+        <v>9</v>
+      </c>
+      <c r="C657">
+        <v>8005324803</v>
+      </c>
+      <c r="D657" s="3">
+        <v>46093.717881944453</v>
+      </c>
+      <c r="E657" t="s">
+        <v>20</v>
+      </c>
+      <c r="F657" t="s">
+        <v>16</v>
+      </c>
+      <c r="G657" t="s">
+        <v>738</v>
+      </c>
+      <c r="H657" t="s">
+        <v>154</v>
+      </c>
+      <c r="I657" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="658" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A658">
+        <v>657</v>
+      </c>
+      <c r="B658" t="s">
+        <v>9</v>
+      </c>
+      <c r="C658">
+        <v>8005302493</v>
+      </c>
+      <c r="D658" s="3">
+        <v>46093.760439814818</v>
+      </c>
+      <c r="E658" t="s">
+        <v>10</v>
+      </c>
+      <c r="F658" t="s">
+        <v>11</v>
+      </c>
+      <c r="G658" t="s">
+        <v>739</v>
+      </c>
+      <c r="H658" t="s">
+        <v>18</v>
+      </c>
+      <c r="I658" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/03/2026 11:45:45,42
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="133" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7C36A5-444B-45FD-A0DA-5557A4825CD7}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B7558BD-58BD-47C8-BE93-785F38886D54}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3951" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4131" uniqueCount="771">
   <si>
     <t>ID</t>
   </si>
@@ -2350,6 +2350,99 @@
   </si>
   <si>
     <t>Não foi trocado filtro da água. O técnico fez o teste na água e disse que a qualidade estava boa. Eu perguntei do filtro e ele falou que só é trocado a cada 3 anos!?!De qualquer forma vou me mudar em Maio e vou adquirir uma geladeira com água e gelo na porta, daí vou devolver o filtro.</t>
+  </si>
+  <si>
+    <t>FRQ SBC SP</t>
+  </si>
+  <si>
+    <t>Demora para disponibilidade do técnico, despreparo na vinda, abertura como manutenção preventiva, quando na realidade precisava de peça.</t>
+  </si>
+  <si>
+    <t>Excelente</t>
+  </si>
+  <si>
+    <t>Nota não foi 10, porque do horário estipulado (13h às 18h) chegou exatamente às 18h!!! ou seja, tivemos que ficar esperando a tarde toda, para ele chegar no último minuto!Precisa melhorar isso...</t>
+  </si>
+  <si>
+    <t>Muito bom.</t>
+  </si>
+  <si>
+    <t>Eu gosto do produto mas quanto as datas para a troca do filtro eu acho muito ruim . Elas são muito longe.</t>
+  </si>
+  <si>
+    <t>A parte de atendimento fica a desejar</t>
+  </si>
+  <si>
+    <t>O aparelho é muito bom mas, na hora que precisamos de uma visita técnica, para que se faça algum conserto, é uma dificuldade!!!</t>
+  </si>
+  <si>
+    <t>Sou cliente há muitos anos e gosto muito de ter água boa e manutenção facilita a vida corrida, sem precisar se preocupar se tudo está funcionando bem.</t>
+  </si>
+  <si>
+    <t>Vcs tentam marcar visitas através de WhatsApp digital. Quando respondo, a máquina não entende. Ligam de novo sucessivamente e sempre acontece a mesma coisa. No fim, vcs enviam técnico SEM avisar… Por acaso, minha funcionária conseguiu me achar e eu autorizei, mas gostaria de ser consultada antes.Vcs precisam aprimorar urgentemente o WhattsApp digital.Obrigada</t>
+  </si>
+  <si>
+    <t>O problema não foi resolvido.Att:</t>
+  </si>
+  <si>
+    <t>Muito bom.Tudo ótimo mas esta ficando muito custoso para mim.Sou aposentado.</t>
+  </si>
+  <si>
+    <t>Existem dois pontos negativos que desejo criticar que são as seguintes: de que não estão mais avisando o cliente sobre a troca do refil pós 6 meses, e não encaminharam nenhum comprovante de visita técnica por e-mail até o presente momento.E o outro ponto negativo (que eu acho muito esquisito), é do refil não vir com um lacre de segurança, apenas dentro de um saquinho plástico simples. Quem me garante que este refil é novo? Então, fica a sugestão, para que passem a lacrar ou embalar de uma forma segura onde mostrará para o cliente que o refil é totalmente novo e seguro de fábrica. Digo isso, porque comprei um refil da IBBL pela internet e o refil deles, vem com uma embalagem lacrada, com nome da marca tudo aparentemente certinho, e gostei do modo. Já o da Brastemp, o técnico retira da bolsa onde outros refis estão juntos na bolsa, não confere (devido a rapidez e a pressa) e que pode colocar o de outro cliente usado no meu purificador e infelizmente não temos como saber não é verdade?Então, fica a sugestão de voltarem a encaminhar mensagem de aviso de troca de refil e também, passarem a lacrar (embalar melhor) o refil, onde o técnico retirará esta embalagem na frente do cliente, que passará confiabilidade no produto.Grata.</t>
+  </si>
+  <si>
+    <t>Falta na assistência de urgência pois , ficou com defeito na substituição do refil e não tenho pronto atendimento para correção.</t>
+  </si>
+  <si>
+    <t>Há anos temos a "assinatura" e nunca houve qualquer problema. No entanto, o purificador deixou de funcionar desde o início de janeiro, os técnicos, nas diversas visitas foram bastante atenciosos, mas estava "presos" a definições e decisões da central que atrasou tudo, inclusive o cadastro da necessidade de troca do aparelho, que demorou mais de um mês, e demora no envio, mais um mês!!! Além disso, houve dano ao móvel por vazamento do aparelho, conforme registrado em fotos, mas aparentemente "como não havia vazamento no momento da visita", realizada muito tempo depois, o reembolso não foi autorizado.Portanto, fica difícil continuar  recomendando um aparelho e assinatura que eu mesmo estou pensando em cancelar!!!</t>
+  </si>
+  <si>
+    <t>O técnico chegou meio-dia, um horário difícil para parar a cozinha. Ao contrário das outras visitas, o técnico não estava uniformizado.</t>
+  </si>
+  <si>
+    <t>Estou altamente insatisfeito. Estou desde 13/02 reclamado de vazamento e mal funcionamento. Já recebi 2 visitas técnicas. A 1a não resolveu, a 2a pediu a troca do purificador mas até o momento não tenho nenhuma informação de quando ele será trocado. Enquanto isso, continuo com vazamento e sem água gelada . Péssima experiência.</t>
+  </si>
+  <si>
+    <t>NÃO É A PRIMEIRA VEZ QUE AGENDO NUMA DATA E HORÁRIO E O TÉCNICO APARECE EM OUTRO DIA TOTALMENTE DIFERENTE.A VISITA ESTAVA AGENDADA PARA DIA 31/03, MAS O QUE ACONTECEU FOI ANTECIPADA SEM QUALQUER CONSULTA.DE QUE ADIANTA A LIGAÇÃO PARA AGENDAMENTO SE NÃO É FEITO CONFORME O COMBINADO. ESPERO QUE NÃO HAJA NOVAMENTE ESTE O OCORRIDO. É UMA TOTAL FALTA DE RESPEITO COM O CLIENTE, CLIENTE ESTE QUE PAGA SEMPRE, SEMPRE E SEMPRE EM DIA.</t>
+  </si>
+  <si>
+    <t>O prestador de serviço não trocou o filtro que está com mal cheiro a água.Apenas veio passear aqui, inclusive o fluxo de água está pouco ele disse que teria que abrir outro chamado.</t>
+  </si>
+  <si>
+    <t>O aparelho não gela a água. Pasmem! A água sai morna. Tentei chamar o técnico e a demora é absurda. Não gostei.</t>
+  </si>
+  <si>
+    <t>Para melhorar é necessário que após o vencimento dos 6 meses quem tem o aparelho seja avisado da manutenção preventiva. Mesmo que não haja o agendamento a comunicação é dificil por telefone.</t>
+  </si>
+  <si>
+    <t>Muito boa. A única reslava é que não consigo falar sobre uma possibilidade de melhora no valor do contrato, pois acho que está pesado. A última vez que falei com o responsável via e-mail, não gostei do atendimento, parecia que estava falando com uma máquina e não com um ser humano. Fui mal atendido. Se dependesse do que tive como retorno via e-mail, não indicaria pra ninguém e nem eu mesmo continuaria cliente da empresa.Vale lembrar que das perguntas abaixo, não condiz com a realidade, pois as visitas técnicas não foram mediante minha solicitação e sim por agendamento de manutenção preventiva e não corretiva. Coloquei como satisfeito, mas não foi eu quem solicitei a visita, é automático da Brastemp.</t>
+  </si>
+  <si>
+    <t>Estou com problema no filtro já tem mais de uma semana, tivemos duas visitas técnicas que disseram que deveria trocar o filtro e não deram continuidade na troca. Já abri chamados e sigo esperando resposta</t>
+  </si>
+  <si>
+    <t>Bom dia, Essa é a minha segunda assinatura. A instalação dessa segunda poderia ter sido melhor- pois o local de instalação não foi ideal- por falta do material- mangueira de instalação- segundo o técnico- mesmo sendo menos de 2 metros do local da agua.</t>
+  </si>
+  <si>
+    <t>A manutenção do purificador foi mal feita, tive que reclamar do técnico que ainda voltou com ma vontade.</t>
+  </si>
+  <si>
+    <t>Tenho o purificador a muitos anos, desde o dia 09/02 ocorreu um problema fiquei mais de 20 dias sem o filtro, saindo água quente, e constataram q foi o sensor q está c problema até hoje não vieram arrumar</t>
+  </si>
+  <si>
+    <t>Os filtros do aparelho eram trocados a cada seis meses conforme contrato em época com a Brastemp. Agora este período foi extendido, conforme o técnico, que ao meu ver compromete a qualidade da água.</t>
+  </si>
+  <si>
+    <t>Durante algum tempo não tive problema com o aparelho, a cerca de 2 mês meu aparelho começou a vazar e não sai água gelada. O técnico já abriu um chamado no último sábado porém ninguém entrou em contato para dizer quando vão instalar o novo.</t>
+  </si>
+  <si>
+    <t>Infelizmente o purificador já não está mais atendendo minhas expectativas. Em grande parte em razão da água que chega no meu apartamento: prédio antigo e encanamento também. Com isto o purificador não é suficiente para melhorar a qualidade da água. Houve também a questão de erro na data da visita. Fiz questão de ligar no 4004-4006, para ressaltar o meu pedido específico que era a instalação de um MIB GEO. Fiz a ligação dia 02/03/26 protocolo 8005320119, onde foi agendado a data 18/03/26 período da tarde. Recebi e-mail em 12/03 de que o técnico iria fazer o atendimento no período da manhã. Felizmente tenho suporte do Paulo da assistência em Curitiba, onde conseguimos combinar um horário que eu poderia chegar no apto. Uma confusão total entre o dia realmente agendado e o da visita, e também minha solicitação da instalação do Mib gel não constava no meu pedido. Terei que agendar outra visita, ou melhor cancelar minha assinatura de anos e buscar outro aparelho? Reforço que o atendimento do técnico Allan e do Paulo (escritório) foram impecáveis.</t>
+  </si>
+  <si>
+    <t>Ainda a situação não foi resolvida. Cada tecnico fala uma coisa. Péssimo.Continui com o problema. Pagando por um serviço que desde nov/25 não vem sido ofertado.</t>
+  </si>
+  <si>
+    <t>Estou preocupada com a troca de filtro, faz hj 20 dias q o.filtro foi trocado e já está c a.agua podre. N dá pra.entender.Será q n estão tratando c rigor os filtros pra serem reutilizados</t>
   </si>
 </sst>
 </file>
@@ -2718,7 +2811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I658"/>
+  <dimension ref="A1:I688"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -21814,6 +21907,876 @@
         <v>51</v>
       </c>
     </row>
+    <row r="659" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A659">
+        <v>658</v>
+      </c>
+      <c r="B659" t="s">
+        <v>9</v>
+      </c>
+      <c r="C659">
+        <v>2688</v>
+      </c>
+      <c r="D659" s="3">
+        <v>46094.476805555554</v>
+      </c>
+      <c r="E659" t="s">
+        <v>740</v>
+      </c>
+      <c r="F659" t="s">
+        <v>16</v>
+      </c>
+      <c r="G659" t="s">
+        <v>741</v>
+      </c>
+      <c r="H659" t="s">
+        <v>32</v>
+      </c>
+      <c r="I659" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="660" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A660">
+        <v>659</v>
+      </c>
+      <c r="B660" t="s">
+        <v>9</v>
+      </c>
+      <c r="C660">
+        <v>8005318604</v>
+      </c>
+      <c r="D660" s="3">
+        <v>46094.489629629628</v>
+      </c>
+      <c r="E660" t="s">
+        <v>53</v>
+      </c>
+      <c r="F660" t="s">
+        <v>11</v>
+      </c>
+      <c r="G660" t="s">
+        <v>742</v>
+      </c>
+      <c r="H660" t="s">
+        <v>13</v>
+      </c>
+      <c r="I660" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="661" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A661">
+        <v>660</v>
+      </c>
+      <c r="B661" t="s">
+        <v>9</v>
+      </c>
+      <c r="C661">
+        <v>8005274455</v>
+      </c>
+      <c r="D661" s="3">
+        <v>46094.533182870371</v>
+      </c>
+      <c r="E661" t="s">
+        <v>15</v>
+      </c>
+      <c r="F661" t="s">
+        <v>11</v>
+      </c>
+      <c r="G661" t="s">
+        <v>743</v>
+      </c>
+      <c r="H661" t="s">
+        <v>18</v>
+      </c>
+      <c r="I661" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="662" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A662">
+        <v>661</v>
+      </c>
+      <c r="B662" t="s">
+        <v>9</v>
+      </c>
+      <c r="C662">
+        <v>8005315273</v>
+      </c>
+      <c r="D662" s="3">
+        <v>46094.53628472222</v>
+      </c>
+      <c r="E662" t="s">
+        <v>20</v>
+      </c>
+      <c r="F662" t="s">
+        <v>11</v>
+      </c>
+      <c r="G662" t="s">
+        <v>744</v>
+      </c>
+      <c r="H662" t="s">
+        <v>13</v>
+      </c>
+      <c r="I662" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="663" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A663">
+        <v>662</v>
+      </c>
+      <c r="B663" t="s">
+        <v>9</v>
+      </c>
+      <c r="C663">
+        <v>8005319496</v>
+      </c>
+      <c r="D663" s="3">
+        <v>46094.538310185184</v>
+      </c>
+      <c r="E663" t="s">
+        <v>98</v>
+      </c>
+      <c r="F663" t="s">
+        <v>11</v>
+      </c>
+      <c r="G663" t="s">
+        <v>745</v>
+      </c>
+      <c r="H663" t="s">
+        <v>32</v>
+      </c>
+      <c r="I663" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="664" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A664">
+        <v>663</v>
+      </c>
+      <c r="B664" t="s">
+        <v>9</v>
+      </c>
+      <c r="C664">
+        <v>8005298239</v>
+      </c>
+      <c r="D664" s="3">
+        <v>46094.580474537041</v>
+      </c>
+      <c r="E664" t="s">
+        <v>15</v>
+      </c>
+      <c r="F664" t="s">
+        <v>16</v>
+      </c>
+      <c r="G664" t="s">
+        <v>746</v>
+      </c>
+      <c r="H664" t="s">
+        <v>13</v>
+      </c>
+      <c r="I664" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="665" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A665">
+        <v>664</v>
+      </c>
+      <c r="B665" t="s">
+        <v>9</v>
+      </c>
+      <c r="C665">
+        <v>8005319290</v>
+      </c>
+      <c r="D665" s="3">
+        <v>46094.612013888887</v>
+      </c>
+      <c r="E665" t="s">
+        <v>53</v>
+      </c>
+      <c r="F665" t="s">
+        <v>11</v>
+      </c>
+      <c r="G665" t="s">
+        <v>747</v>
+      </c>
+      <c r="H665" t="s">
+        <v>13</v>
+      </c>
+      <c r="I665" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="666" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A666">
+        <v>665</v>
+      </c>
+      <c r="B666" t="s">
+        <v>9</v>
+      </c>
+      <c r="C666">
+        <v>17</v>
+      </c>
+      <c r="D666" s="3">
+        <v>46094.639421296299</v>
+      </c>
+      <c r="E666" t="s">
+        <v>700</v>
+      </c>
+      <c r="F666" t="s">
+        <v>11</v>
+      </c>
+      <c r="G666" t="s">
+        <v>748</v>
+      </c>
+      <c r="H666" t="s">
+        <v>13</v>
+      </c>
+      <c r="I666" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="667" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A667">
+        <v>666</v>
+      </c>
+      <c r="B667" t="s">
+        <v>9</v>
+      </c>
+      <c r="C667">
+        <v>8005306207</v>
+      </c>
+      <c r="D667" s="3">
+        <v>46095.063576388886</v>
+      </c>
+      <c r="E667" t="s">
+        <v>20</v>
+      </c>
+      <c r="F667" t="s">
+        <v>11</v>
+      </c>
+      <c r="G667" t="s">
+        <v>749</v>
+      </c>
+      <c r="H667" t="s">
+        <v>82</v>
+      </c>
+      <c r="I667" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="668" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A668">
+        <v>667</v>
+      </c>
+      <c r="B668" t="s">
+        <v>9</v>
+      </c>
+      <c r="C668">
+        <v>8005324971</v>
+      </c>
+      <c r="D668" s="3">
+        <v>46095.496469907404</v>
+      </c>
+      <c r="E668" t="s">
+        <v>74</v>
+      </c>
+      <c r="F668" t="s">
+        <v>16</v>
+      </c>
+      <c r="G668" t="s">
+        <v>750</v>
+      </c>
+      <c r="H668" t="s">
+        <v>18</v>
+      </c>
+      <c r="I668" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="669" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A669">
+        <v>668</v>
+      </c>
+      <c r="B669" t="s">
+        <v>9</v>
+      </c>
+      <c r="C669">
+        <v>8005302489</v>
+      </c>
+      <c r="D669" s="3">
+        <v>46095.574907407405</v>
+      </c>
+      <c r="E669" t="s">
+        <v>20</v>
+      </c>
+      <c r="F669" t="s">
+        <v>11</v>
+      </c>
+      <c r="G669" t="s">
+        <v>751</v>
+      </c>
+      <c r="H669" t="s">
+        <v>13</v>
+      </c>
+      <c r="I669" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="670" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A670">
+        <v>669</v>
+      </c>
+      <c r="B670" t="s">
+        <v>9</v>
+      </c>
+      <c r="C670">
+        <v>8932</v>
+      </c>
+      <c r="D670" s="3">
+        <v>46095.971944444442</v>
+      </c>
+      <c r="E670" t="s">
+        <v>680</v>
+      </c>
+      <c r="F670" t="s">
+        <v>11</v>
+      </c>
+      <c r="G670" t="s">
+        <v>752</v>
+      </c>
+      <c r="H670" t="s">
+        <v>18</v>
+      </c>
+      <c r="I670" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="671" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A671">
+        <v>670</v>
+      </c>
+      <c r="B671" t="s">
+        <v>9</v>
+      </c>
+      <c r="C671">
+        <v>6555</v>
+      </c>
+      <c r="D671" s="3">
+        <v>46096.352141203701</v>
+      </c>
+      <c r="E671" t="s">
+        <v>684</v>
+      </c>
+      <c r="F671" t="s">
+        <v>16</v>
+      </c>
+      <c r="G671" t="s">
+        <v>753</v>
+      </c>
+      <c r="H671" t="s">
+        <v>32</v>
+      </c>
+      <c r="I671" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="672" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A672">
+        <v>671</v>
+      </c>
+      <c r="B672" t="s">
+        <v>9</v>
+      </c>
+      <c r="C672">
+        <v>8005307680</v>
+      </c>
+      <c r="D672" s="3">
+        <v>46096.581712962965</v>
+      </c>
+      <c r="E672" t="s">
+        <v>98</v>
+      </c>
+      <c r="F672" t="s">
+        <v>16</v>
+      </c>
+      <c r="G672" t="s">
+        <v>754</v>
+      </c>
+      <c r="H672" t="s">
+        <v>154</v>
+      </c>
+      <c r="I672" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="673" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A673">
+        <v>672</v>
+      </c>
+      <c r="B673" t="s">
+        <v>9</v>
+      </c>
+      <c r="C673">
+        <v>8005319055</v>
+      </c>
+      <c r="D673" s="3">
+        <v>46096.889074074075</v>
+      </c>
+      <c r="E673" t="s">
+        <v>41</v>
+      </c>
+      <c r="F673" t="s">
+        <v>11</v>
+      </c>
+      <c r="G673" t="s">
+        <v>755</v>
+      </c>
+      <c r="H673" t="s">
+        <v>18</v>
+      </c>
+      <c r="I673" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="674" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A674">
+        <v>673</v>
+      </c>
+      <c r="B674" t="s">
+        <v>9</v>
+      </c>
+      <c r="C674">
+        <v>8005320296</v>
+      </c>
+      <c r="D674" s="3">
+        <v>46096.898159722223</v>
+      </c>
+      <c r="E674" t="s">
+        <v>53</v>
+      </c>
+      <c r="F674" t="s">
+        <v>16</v>
+      </c>
+      <c r="G674" t="s">
+        <v>756</v>
+      </c>
+      <c r="H674" t="s">
+        <v>18</v>
+      </c>
+      <c r="I674" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="675" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A675">
+        <v>674</v>
+      </c>
+      <c r="B675" t="s">
+        <v>9</v>
+      </c>
+      <c r="C675">
+        <v>8005315946</v>
+      </c>
+      <c r="D675" s="3">
+        <v>46097.409108796295</v>
+      </c>
+      <c r="E675" t="s">
+        <v>262</v>
+      </c>
+      <c r="F675" t="s">
+        <v>16</v>
+      </c>
+      <c r="G675" t="s">
+        <v>757</v>
+      </c>
+      <c r="H675" t="s">
+        <v>18</v>
+      </c>
+      <c r="I675" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="676" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A676">
+        <v>675</v>
+      </c>
+      <c r="B676" t="s">
+        <v>9</v>
+      </c>
+      <c r="C676">
+        <v>8005300478</v>
+      </c>
+      <c r="D676" s="3">
+        <v>46097.415034722224</v>
+      </c>
+      <c r="E676" t="s">
+        <v>20</v>
+      </c>
+      <c r="F676" t="s">
+        <v>16</v>
+      </c>
+      <c r="G676" t="s">
+        <v>758</v>
+      </c>
+      <c r="H676" t="s">
+        <v>18</v>
+      </c>
+      <c r="I676" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="677" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A677">
+        <v>676</v>
+      </c>
+      <c r="B677" t="s">
+        <v>61</v>
+      </c>
+      <c r="C677">
+        <v>8005327883</v>
+      </c>
+      <c r="D677" s="3">
+        <v>46097.432037037041</v>
+      </c>
+      <c r="E677" t="s">
+        <v>125</v>
+      </c>
+      <c r="F677" t="s">
+        <v>16</v>
+      </c>
+      <c r="G677" t="s">
+        <v>759</v>
+      </c>
+      <c r="H677" t="s">
+        <v>35</v>
+      </c>
+      <c r="I677" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="678" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A678">
+        <v>677</v>
+      </c>
+      <c r="B678" t="s">
+        <v>9</v>
+      </c>
+      <c r="C678">
+        <v>8005279493</v>
+      </c>
+      <c r="D678" s="3">
+        <v>46097.434421296297</v>
+      </c>
+      <c r="E678" t="s">
+        <v>41</v>
+      </c>
+      <c r="F678" t="s">
+        <v>11</v>
+      </c>
+      <c r="G678" t="s">
+        <v>760</v>
+      </c>
+      <c r="H678" t="s">
+        <v>82</v>
+      </c>
+      <c r="I678" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="679" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A679">
+        <v>678</v>
+      </c>
+      <c r="B679" t="s">
+        <v>9</v>
+      </c>
+      <c r="C679">
+        <v>8005304869</v>
+      </c>
+      <c r="D679" s="3">
+        <v>46097.445601851854</v>
+      </c>
+      <c r="E679" t="s">
+        <v>10</v>
+      </c>
+      <c r="F679" t="s">
+        <v>11</v>
+      </c>
+      <c r="G679" t="s">
+        <v>761</v>
+      </c>
+      <c r="H679" t="s">
+        <v>82</v>
+      </c>
+      <c r="I679" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="680" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A680">
+        <v>679</v>
+      </c>
+      <c r="B680" t="s">
+        <v>9</v>
+      </c>
+      <c r="C680">
+        <v>8005328284</v>
+      </c>
+      <c r="D680" s="3">
+        <v>46097.50104166667</v>
+      </c>
+      <c r="E680" t="s">
+        <v>15</v>
+      </c>
+      <c r="F680" t="s">
+        <v>16</v>
+      </c>
+      <c r="G680" t="s">
+        <v>762</v>
+      </c>
+      <c r="H680" t="s">
+        <v>154</v>
+      </c>
+      <c r="I680" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="681" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A681">
+        <v>680</v>
+      </c>
+      <c r="B681" t="s">
+        <v>61</v>
+      </c>
+      <c r="C681">
+        <v>8005324456</v>
+      </c>
+      <c r="D681" s="3">
+        <v>46097.501585648148</v>
+      </c>
+      <c r="E681" t="s">
+        <v>70</v>
+      </c>
+      <c r="F681" t="s">
+        <v>11</v>
+      </c>
+      <c r="G681" t="s">
+        <v>763</v>
+      </c>
+      <c r="H681" t="s">
+        <v>18</v>
+      </c>
+      <c r="I681" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="682" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A682">
+        <v>681</v>
+      </c>
+      <c r="B682" t="s">
+        <v>9</v>
+      </c>
+      <c r="C682">
+        <v>8005328861</v>
+      </c>
+      <c r="D682" s="3">
+        <v>46097.509004629632</v>
+      </c>
+      <c r="E682" t="s">
+        <v>224</v>
+      </c>
+      <c r="F682" t="s">
+        <v>16</v>
+      </c>
+      <c r="G682" t="s">
+        <v>764</v>
+      </c>
+      <c r="H682" t="s">
+        <v>18</v>
+      </c>
+      <c r="I682" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="683" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A683">
+        <v>682</v>
+      </c>
+      <c r="B683" t="s">
+        <v>9</v>
+      </c>
+      <c r="C683">
+        <v>2899</v>
+      </c>
+      <c r="D683" s="3">
+        <v>46097.565729166665</v>
+      </c>
+      <c r="E683" t="s">
+        <v>740</v>
+      </c>
+      <c r="F683" t="s">
+        <v>16</v>
+      </c>
+      <c r="G683" t="s">
+        <v>765</v>
+      </c>
+      <c r="H683" t="s">
+        <v>18</v>
+      </c>
+      <c r="I683" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="684" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A684">
+        <v>683</v>
+      </c>
+      <c r="B684" t="s">
+        <v>9</v>
+      </c>
+      <c r="C684">
+        <v>8005329401</v>
+      </c>
+      <c r="D684" s="3">
+        <v>46097.570844907408</v>
+      </c>
+      <c r="E684" t="s">
+        <v>125</v>
+      </c>
+      <c r="F684" t="s">
+        <v>16</v>
+      </c>
+      <c r="G684" t="s">
+        <v>766</v>
+      </c>
+      <c r="H684" t="s">
+        <v>18</v>
+      </c>
+      <c r="I684" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="685" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A685">
+        <v>684</v>
+      </c>
+      <c r="B685" t="s">
+        <v>9</v>
+      </c>
+      <c r="C685">
+        <v>6573</v>
+      </c>
+      <c r="D685" s="3">
+        <v>46097.624849537038</v>
+      </c>
+      <c r="E685" t="s">
+        <v>684</v>
+      </c>
+      <c r="F685" t="s">
+        <v>16</v>
+      </c>
+      <c r="G685" t="s">
+        <v>767</v>
+      </c>
+      <c r="H685" t="s">
+        <v>35</v>
+      </c>
+      <c r="I685" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="686" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A686">
+        <v>685</v>
+      </c>
+      <c r="B686" t="s">
+        <v>9</v>
+      </c>
+      <c r="C686">
+        <v>8005320119</v>
+      </c>
+      <c r="D686" s="3">
+        <v>46097.643877314818</v>
+      </c>
+      <c r="E686" t="s">
+        <v>41</v>
+      </c>
+      <c r="F686" t="s">
+        <v>16</v>
+      </c>
+      <c r="G686" t="s">
+        <v>768</v>
+      </c>
+      <c r="H686" t="s">
+        <v>35</v>
+      </c>
+      <c r="I686" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="687" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A687">
+        <v>686</v>
+      </c>
+      <c r="B687" t="s">
+        <v>9</v>
+      </c>
+      <c r="C687">
+        <v>8005323827</v>
+      </c>
+      <c r="D687" s="3">
+        <v>46097.738692129627</v>
+      </c>
+      <c r="E687" t="s">
+        <v>53</v>
+      </c>
+      <c r="F687" t="s">
+        <v>16</v>
+      </c>
+      <c r="G687" t="s">
+        <v>769</v>
+      </c>
+      <c r="H687" t="s">
+        <v>18</v>
+      </c>
+      <c r="I687" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="688" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A688">
+        <v>687</v>
+      </c>
+      <c r="B688" t="s">
+        <v>9</v>
+      </c>
+      <c r="C688">
+        <v>8005311180</v>
+      </c>
+      <c r="D688" s="3">
+        <v>46097.832511574074</v>
+      </c>
+      <c r="E688" t="s">
+        <v>65</v>
+      </c>
+      <c r="F688" t="s">
+        <v>11</v>
+      </c>
+      <c r="G688" t="s">
+        <v>770</v>
+      </c>
+      <c r="H688" t="s">
+        <v>35</v>
+      </c>
+      <c r="I688" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/03/2026 14:46:44,59
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B7558BD-58BD-47C8-BE93-785F38886D54}"/>
+  <xr:revisionPtr revIDLastSave="145" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77E92B67-14B5-4097-89C9-E32AF04D40B2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$601</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$688</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4131" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4131" uniqueCount="769">
   <si>
     <t>ID</t>
   </si>
@@ -2178,9 +2178,6 @@
     <t>Já agendei a visita 4x e nunca vieram. Agendei 3x para sábado, uma das vezes tentaram vir na sexta (não podia atender, por isso agendei no sábado) e nas outras, simplesmente ninguem sequer apareceu. Aí na última agora, tentei agendar na sexta, visto que de sábado estava impossível, ninguem apareceu também. Não está fazendo sentido algum eu manter o serviço, visto que não tenho a manutenção preventiva, a troca do filtro.</t>
   </si>
   <si>
-    <t>Técnico não cumpriu agenda</t>
-  </si>
-  <si>
     <t>Agendei duas vezes a manutenção periódica e o técnico não foi, para piorar a última manutenção realizada, foi em 07/2025 ou seja, passou muito o prazo.</t>
   </si>
   <si>
@@ -2224,9 +2221,6 @@
   </si>
   <si>
     <t>Sou cliente a 18 anos neste período houve inúmeras mudanças e piorou no atendimento emergencial fiquei do dia 20 de fevereiro até dia 5 de março sem águapotável e mesmo assim o técnico não tinha uma peça e disse que se houver problemas solicite assistência técnica portanto novos tempos</t>
-  </si>
-  <si>
-    <t>Falta de estoque/pecas</t>
   </si>
   <si>
     <t>o Técnico veio sem Pro -pé e sem lavar as mãos da rua para fazer a manutenção do aparelho Brastemp ! Estou pensando seriamente em trocar o aparelho de filtro de água Brastemp .</t>
@@ -20396,7 +20390,7 @@
         <v>18</v>
       </c>
       <c r="I606" t="s">
-        <v>682</v>
+        <v>29</v>
       </c>
     </row>
     <row r="607" spans="1:9" x14ac:dyDescent="0.25">
@@ -20419,13 +20413,13 @@
         <v>16</v>
       </c>
       <c r="G607" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H607" t="s">
         <v>18</v>
       </c>
       <c r="I607" t="s">
-        <v>682</v>
+        <v>29</v>
       </c>
     </row>
     <row r="608" spans="1:9" x14ac:dyDescent="0.25">
@@ -20442,13 +20436,13 @@
         <v>46090.448009259257</v>
       </c>
       <c r="E608" t="s">
+        <v>683</v>
+      </c>
+      <c r="F608" t="s">
+        <v>16</v>
+      </c>
+      <c r="G608" t="s">
         <v>684</v>
-      </c>
-      <c r="F608" t="s">
-        <v>16</v>
-      </c>
-      <c r="G608" t="s">
-        <v>685</v>
       </c>
       <c r="H608" t="s">
         <v>18</v>
@@ -20477,7 +20471,7 @@
         <v>11</v>
       </c>
       <c r="G609" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H609" t="s">
         <v>609</v>
@@ -20535,7 +20529,7 @@
         <v>16</v>
       </c>
       <c r="G611" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H611" t="s">
         <v>18</v>
@@ -20564,7 +20558,7 @@
         <v>16</v>
       </c>
       <c r="G612" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H612" t="s">
         <v>18</v>
@@ -20593,7 +20587,7 @@
         <v>16</v>
       </c>
       <c r="G613" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H613" t="s">
         <v>13</v>
@@ -20622,7 +20616,7 @@
         <v>16</v>
       </c>
       <c r="G614" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H614" t="s">
         <v>18</v>
@@ -20651,7 +20645,7 @@
         <v>11</v>
       </c>
       <c r="G615" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H615" t="s">
         <v>13</v>
@@ -20680,7 +20674,7 @@
         <v>16</v>
       </c>
       <c r="G616" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H616" t="s">
         <v>18</v>
@@ -20709,7 +20703,7 @@
         <v>16</v>
       </c>
       <c r="G617" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H617" t="s">
         <v>13</v>
@@ -20738,7 +20732,7 @@
         <v>11</v>
       </c>
       <c r="G618" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H618" t="s">
         <v>18</v>
@@ -20767,7 +20761,7 @@
         <v>11</v>
       </c>
       <c r="G619" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="H619" t="s">
         <v>13</v>
@@ -20796,7 +20790,7 @@
         <v>16</v>
       </c>
       <c r="G620" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H620" t="s">
         <v>609</v>
@@ -20825,13 +20819,13 @@
         <v>11</v>
       </c>
       <c r="G621" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H621" t="s">
         <v>154</v>
       </c>
       <c r="I621" t="s">
-        <v>698</v>
+        <v>179</v>
       </c>
     </row>
     <row r="622" spans="1:9" x14ac:dyDescent="0.25">
@@ -20854,7 +20848,7 @@
         <v>16</v>
       </c>
       <c r="G622" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="H622" t="s">
         <v>18</v>
@@ -20877,13 +20871,13 @@
         <v>46091.450520833343</v>
       </c>
       <c r="E623" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F623" t="s">
         <v>11</v>
       </c>
       <c r="G623" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="H623" t="s">
         <v>82</v>
@@ -20906,13 +20900,13 @@
         <v>46091.474988425929</v>
       </c>
       <c r="E624" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="F624" t="s">
         <v>16</v>
       </c>
       <c r="G624" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="H624" t="s">
         <v>609</v>
@@ -20941,7 +20935,7 @@
         <v>16</v>
       </c>
       <c r="G625" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="H625" t="s">
         <v>609</v>
@@ -20970,7 +20964,7 @@
         <v>16</v>
       </c>
       <c r="G626" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="H626" t="s">
         <v>609</v>
@@ -20999,7 +20993,7 @@
         <v>11</v>
       </c>
       <c r="G627" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="H627" t="s">
         <v>13</v>
@@ -21028,7 +21022,7 @@
         <v>11</v>
       </c>
       <c r="G628" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="H628" t="s">
         <v>13</v>
@@ -21057,7 +21051,7 @@
         <v>11</v>
       </c>
       <c r="G629" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="H629" t="s">
         <v>609</v>
@@ -21086,7 +21080,7 @@
         <v>11</v>
       </c>
       <c r="G630" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="H630" t="s">
         <v>13</v>
@@ -21115,7 +21109,7 @@
         <v>11</v>
       </c>
       <c r="G631" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="H631" t="s">
         <v>32</v>
@@ -21144,7 +21138,7 @@
         <v>16</v>
       </c>
       <c r="G632" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="H632" t="s">
         <v>18</v>
@@ -21173,13 +21167,13 @@
         <v>11</v>
       </c>
       <c r="G633" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="H633" t="s">
         <v>18</v>
       </c>
       <c r="I633" t="s">
-        <v>682</v>
+        <v>29</v>
       </c>
     </row>
     <row r="634" spans="1:9" x14ac:dyDescent="0.25">
@@ -21196,13 +21190,13 @@
         <v>46091.610069444447</v>
       </c>
       <c r="E634" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F634" t="s">
         <v>16</v>
       </c>
       <c r="G634" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="H634" t="s">
         <v>32</v>
@@ -21231,13 +21225,13 @@
         <v>16</v>
       </c>
       <c r="G635" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="H635" t="s">
         <v>18</v>
       </c>
       <c r="I635" t="s">
-        <v>682</v>
+        <v>29</v>
       </c>
     </row>
     <row r="636" spans="1:9" x14ac:dyDescent="0.25">
@@ -21254,13 +21248,13 @@
         <v>46091.738668981481</v>
       </c>
       <c r="E636" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="F636" t="s">
         <v>16</v>
       </c>
       <c r="G636" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="H636" t="s">
         <v>32</v>
@@ -21283,13 +21277,13 @@
         <v>46091.75209490741</v>
       </c>
       <c r="E637" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F637" t="s">
         <v>11</v>
       </c>
       <c r="G637" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="H637" t="s">
         <v>13</v>
@@ -21312,13 +21306,13 @@
         <v>46092.369247685187</v>
       </c>
       <c r="E638" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="F638" t="s">
         <v>16</v>
       </c>
       <c r="G638" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="H638" t="s">
         <v>13</v>
@@ -21341,13 +21335,13 @@
         <v>46092.406168981477</v>
       </c>
       <c r="E639" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F639" t="s">
         <v>16</v>
       </c>
       <c r="G639" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="H639" t="s">
         <v>32</v>
@@ -21376,7 +21370,7 @@
         <v>11</v>
       </c>
       <c r="G640" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="H640" t="s">
         <v>32</v>
@@ -21399,13 +21393,13 @@
         <v>46092.501481481479</v>
       </c>
       <c r="E641" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F641" t="s">
         <v>16</v>
       </c>
       <c r="G641" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="H641" t="s">
         <v>154</v>
@@ -21434,7 +21428,7 @@
         <v>16</v>
       </c>
       <c r="G642" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="H642" t="s">
         <v>82</v>
@@ -21457,13 +21451,13 @@
         <v>46092.664965277778</v>
       </c>
       <c r="E643" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="F643" t="s">
         <v>16</v>
       </c>
       <c r="G643" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="H643" t="s">
         <v>154</v>
@@ -21486,19 +21480,19 @@
         <v>46093.390613425923</v>
       </c>
       <c r="E644" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F644" t="s">
         <v>16</v>
       </c>
       <c r="G644" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="H644" t="s">
         <v>18</v>
       </c>
       <c r="I644" t="s">
-        <v>682</v>
+        <v>29</v>
       </c>
     </row>
     <row r="645" spans="1:9" x14ac:dyDescent="0.25">
@@ -21521,7 +21515,7 @@
         <v>11</v>
       </c>
       <c r="G645" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="H645" t="s">
         <v>609</v>
@@ -21550,7 +21544,7 @@
         <v>11</v>
       </c>
       <c r="G646" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="H646" t="s">
         <v>18</v>
@@ -21579,7 +21573,7 @@
         <v>11</v>
       </c>
       <c r="G647" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="H647" t="s">
         <v>13</v>
@@ -21608,7 +21602,7 @@
         <v>11</v>
       </c>
       <c r="G648" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="H648" t="s">
         <v>13</v>
@@ -21637,7 +21631,7 @@
         <v>11</v>
       </c>
       <c r="G649" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="H649" t="s">
         <v>13</v>
@@ -21666,7 +21660,7 @@
         <v>16</v>
       </c>
       <c r="G650" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="H650" t="s">
         <v>18</v>
@@ -21695,7 +21689,7 @@
         <v>16</v>
       </c>
       <c r="G651" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="H651" t="s">
         <v>18</v>
@@ -21724,7 +21718,7 @@
         <v>11</v>
       </c>
       <c r="G652" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="H652" t="s">
         <v>18</v>
@@ -21753,7 +21747,7 @@
         <v>16</v>
       </c>
       <c r="G653" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="H653" t="s">
         <v>18</v>
@@ -21782,7 +21776,7 @@
         <v>11</v>
       </c>
       <c r="G654" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="H654" t="s">
         <v>13</v>
@@ -21805,13 +21799,13 @@
         <v>46093.549525462957</v>
       </c>
       <c r="E655" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F655" t="s">
         <v>11</v>
       </c>
       <c r="G655" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="H655" t="s">
         <v>32</v>
@@ -21840,7 +21834,7 @@
         <v>16</v>
       </c>
       <c r="G656" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="H656" t="s">
         <v>18</v>
@@ -21869,7 +21863,7 @@
         <v>16</v>
       </c>
       <c r="G657" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="H657" t="s">
         <v>154</v>
@@ -21898,7 +21892,7 @@
         <v>11</v>
       </c>
       <c r="G658" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="H658" t="s">
         <v>18</v>
@@ -21921,13 +21915,13 @@
         <v>46094.476805555554</v>
       </c>
       <c r="E659" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="F659" t="s">
         <v>16</v>
       </c>
       <c r="G659" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="H659" t="s">
         <v>32</v>
@@ -21956,7 +21950,7 @@
         <v>11</v>
       </c>
       <c r="G660" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="H660" t="s">
         <v>13</v>
@@ -21985,7 +21979,7 @@
         <v>11</v>
       </c>
       <c r="G661" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="H661" t="s">
         <v>18</v>
@@ -22014,7 +22008,7 @@
         <v>11</v>
       </c>
       <c r="G662" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="H662" t="s">
         <v>13</v>
@@ -22043,7 +22037,7 @@
         <v>11</v>
       </c>
       <c r="G663" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="H663" t="s">
         <v>32</v>
@@ -22072,7 +22066,7 @@
         <v>16</v>
       </c>
       <c r="G664" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="H664" t="s">
         <v>13</v>
@@ -22101,7 +22095,7 @@
         <v>11</v>
       </c>
       <c r="G665" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="H665" t="s">
         <v>13</v>
@@ -22124,13 +22118,13 @@
         <v>46094.639421296299</v>
       </c>
       <c r="E666" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F666" t="s">
         <v>11</v>
       </c>
       <c r="G666" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="H666" t="s">
         <v>13</v>
@@ -22159,7 +22153,7 @@
         <v>11</v>
       </c>
       <c r="G667" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="H667" t="s">
         <v>82</v>
@@ -22188,7 +22182,7 @@
         <v>16</v>
       </c>
       <c r="G668" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="H668" t="s">
         <v>18</v>
@@ -22217,7 +22211,7 @@
         <v>11</v>
       </c>
       <c r="G669" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="H669" t="s">
         <v>13</v>
@@ -22246,7 +22240,7 @@
         <v>11</v>
       </c>
       <c r="G670" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="H670" t="s">
         <v>18</v>
@@ -22269,13 +22263,13 @@
         <v>46096.352141203701</v>
       </c>
       <c r="E671" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F671" t="s">
         <v>16</v>
       </c>
       <c r="G671" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="H671" t="s">
         <v>32</v>
@@ -22304,7 +22298,7 @@
         <v>16</v>
       </c>
       <c r="G672" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="H672" t="s">
         <v>154</v>
@@ -22333,7 +22327,7 @@
         <v>11</v>
       </c>
       <c r="G673" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="H673" t="s">
         <v>18</v>
@@ -22362,7 +22356,7 @@
         <v>16</v>
       </c>
       <c r="G674" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="H674" t="s">
         <v>18</v>
@@ -22391,7 +22385,7 @@
         <v>16</v>
       </c>
       <c r="G675" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="H675" t="s">
         <v>18</v>
@@ -22420,7 +22414,7 @@
         <v>16</v>
       </c>
       <c r="G676" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="H676" t="s">
         <v>18</v>
@@ -22449,7 +22443,7 @@
         <v>16</v>
       </c>
       <c r="G677" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="H677" t="s">
         <v>35</v>
@@ -22478,7 +22472,7 @@
         <v>11</v>
       </c>
       <c r="G678" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="H678" t="s">
         <v>82</v>
@@ -22507,7 +22501,7 @@
         <v>11</v>
       </c>
       <c r="G679" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="H679" t="s">
         <v>82</v>
@@ -22536,7 +22530,7 @@
         <v>16</v>
       </c>
       <c r="G680" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="H680" t="s">
         <v>154</v>
@@ -22565,7 +22559,7 @@
         <v>11</v>
       </c>
       <c r="G681" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="H681" t="s">
         <v>18</v>
@@ -22594,7 +22588,7 @@
         <v>16</v>
       </c>
       <c r="G682" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="H682" t="s">
         <v>18</v>
@@ -22617,13 +22611,13 @@
         <v>46097.565729166665</v>
       </c>
       <c r="E683" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="F683" t="s">
         <v>16</v>
       </c>
       <c r="G683" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="H683" t="s">
         <v>18</v>
@@ -22652,7 +22646,7 @@
         <v>16</v>
       </c>
       <c r="G684" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="H684" t="s">
         <v>18</v>
@@ -22675,13 +22669,13 @@
         <v>46097.624849537038</v>
       </c>
       <c r="E685" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F685" t="s">
         <v>16</v>
       </c>
       <c r="G685" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="H685" t="s">
         <v>35</v>
@@ -22710,7 +22704,7 @@
         <v>16</v>
       </c>
       <c r="G686" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="H686" t="s">
         <v>35</v>
@@ -22739,7 +22733,7 @@
         <v>16</v>
       </c>
       <c r="G687" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="H687" t="s">
         <v>18</v>
@@ -22768,7 +22762,7 @@
         <v>11</v>
       </c>
       <c r="G688" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="H688" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 27/03/2026 11:21:23,42
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="172" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{882787C0-5AFA-497F-85CA-C3FB7621E1F1}"/>
+  <xr:revisionPtr revIDLastSave="184" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A03CA44-C790-4455-9EBB-69AC8B5C142D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$739</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$783</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4437" uniqueCount="819">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4701" uniqueCount="863">
   <si>
     <t>ID</t>
   </si>
@@ -2587,6 +2587,138 @@
   </si>
   <si>
     <t>Eu já conhecia o Filtro Brastemp de outra empresa que trabalhei, era Ótimo!  Tinha manutenções mensais e nem precisava agendar, agora passou para de 6 em 6 meses, e nós precisamos ficar chamando para agendar.</t>
+  </si>
+  <si>
+    <t>Nao resolveu o problema. Continua vazadno e voces nao trocam a porcariado filtro</t>
+  </si>
+  <si>
+    <t>A assistência técnica é mto boa, o purificador tb, mas vcs deveriam ter um preço diferenciado para o número de pessoas. Aqui em casa, já fomos 4, depois duas pessoas, agora que meu marido faleceu, só eu e continuo pagando a mesma coisa: R$ 94,03.</t>
+  </si>
+  <si>
+    <t>Porque fiz a solicitação da substituição do filtro, pois estava com problema frequente na vazão de agua. O técnico disse que a sugestão era instalar um pressurizador, que resolveria esse problema, conversou com o Supervisor , que disse que o dia seguinte, faria essa instalação.Mas até hoje não houve o retorno do técnico com a solução do problema.POr tanto o problema persiste.</t>
+  </si>
+  <si>
+    <t>O purificador de água continuou apresentando problemas. Não esta funcionando, ao pressionarmos o botão de acionamento de água ele dispara nos obrigando a desligá-lo na tomada para que para de sair água.</t>
+  </si>
+  <si>
+    <t>Foi agendado mas não foi cumprido tive que reagendar manutenção feita em 10 minutos muito ruim a atenção em todos os sentidos o contrato diz manutenção a cada 6 meses e não cumprem</t>
+  </si>
+  <si>
+    <t>troquei o equipamento e de cara congelou .. a visita do tecnico foi muito demorada ...</t>
+  </si>
+  <si>
+    <t>gosto do produto, mas quando tem algum defeito, nunca encontro uma data próxima para agendar a visita técnica.</t>
+  </si>
+  <si>
+    <t>Muita demora na resolução da troca do equipamento</t>
+  </si>
+  <si>
+    <t>No dia 21/03/2026, às 08h20min, recebi contato da central da Brastemp, informando que o técnico chegaria à minha residência em aproximadamente 30 minutos (com o mesmo em linha).Entretanto, se passaram 4h, desde o referido contato, e o técnico não compareceu, nem houve qualquer atualização sobre o atendimento.Liguei desde cedo e me informaram que estaria a caminho e era para aguardar até 13h00min (Os protocolos de atendimento são : 8005335082, 8005335064 e 8005335117.Gostaria de ressaltar que esta já é a 5ª solicitação de visita técnica para manutenção do purificador, sendo que, nas quatro ocasiões anteriores, também não houve comparecimento do profissional.Diante disso, gostaria, de forma respeitosa, solicitar a não cobrança da mensalidade referente a este mês e o ressarcimento dos 5 meses anteriores, em razão da ausência no cumprimento dos procedimentos acordados em contrato.Entendo que imprevistos podem ocorrer, porém, diante das falhas recorrentes na prestação do serviço, acredito ser justo reavaliar as cobranças destes períodos.</t>
+  </si>
+  <si>
+    <t>Esta se tornando muito caro.É  possível uma redução do preço</t>
+  </si>
+  <si>
+    <t>Sem atendimento nos prazos! Trocaram meu filtro e não colocaram a pressurização.</t>
+  </si>
+  <si>
+    <t>Não quero pagar este valor mensal mais</t>
+  </si>
+  <si>
+    <t>Sou assinante do serviço desde praticamente o início da prestação pela Brastemp.Se me perguntassem um tempo atrás, com certeza daria um 10.Mas, infelizmente, estou com o filtro inoperante há cerca de 20 dias. Liguei várias vezes para a central de atendimento mas a visita só foi realizada na última sexta-feira, quando o técnico identificou o problema.Agora estou aguardando o agendamento do retorno técnico para troca da peça e resolução da pendência.</t>
+  </si>
+  <si>
+    <t>Já utilizo há um certo tempo, mas o que mais me incomoda é a demora em ser atendida quando do registro da ocorrência. Outro detalhe o purificador não gela bem, penso que seja da própria fabricação, já era para ter comunicado esse fato, que eu já tinha percebido há algum tempo</t>
+  </si>
+  <si>
+    <t>Manutenção ruim</t>
+  </si>
+  <si>
+    <t>Valor alto</t>
+  </si>
+  <si>
+    <t>mais uma vez aconteceu comigo, marcamos dia e período e o técnico não apareceu, fiquei preso em casa esperando. Me ligaram e programaram para o mesmo dia até 18h, voltei para casa e esperei, ninguém fez contato.</t>
+  </si>
+  <si>
+    <t>o técnico não compareceu</t>
+  </si>
+  <si>
+    <t>Bom dia Quatro agendamentos que foi marcado mais não compareceram no dia 20/03/26 em Niterói e 03 no dia 23/03/26 em Copacabana e ate agora nem um contato</t>
+  </si>
+  <si>
+    <t>Não resolveram meu problema pela 3 vez não trouxeram o pressurizador</t>
+  </si>
+  <si>
+    <t>O equipamento é muito bom, por isso sou cliente a quase 20anos.Faço ressalva na visita técnica, que pode melhorar na comunicação e especificidade do horário. É complicado para quem trabalha e não tem gente para receber o técnico</t>
+  </si>
+  <si>
+    <t>Enfim, trocaram o meu purificador mas o aparelho está com defeito. Quando o condensador liga, parece que vai dar um curto, tenho até medo que pegue fogo. Liguei ontem para registrar e acionar um técnico mas o atendente me disse que não tinha data disponível no momento. Legal isso neh??</t>
+  </si>
+  <si>
+    <t>O purificador é de boa qualidade, mas a manutenção  e rede de atendimento é péssima , cheia de erros na agenda e atendimento ruim, para trocar o elemento filtrante demoraram mais de 2 meses , erraram o endereço  e depois não  queriam vir , ficaram jogando a data pra mais duas semanas e assim se seguiu!</t>
+  </si>
+  <si>
+    <t>Equipamento muito bom....prático, mas apresentou defeito após cerca de 4 anos de uso ...e estou encontrando dificuldades para substituição.....</t>
+  </si>
+  <si>
+    <t>não esta bom atendimento estou quase a mes sem agua gelada pediram para trocar o filtro mas ate agora nada</t>
+  </si>
+  <si>
+    <t>A minha maquina veio com defeito e vazou todo o gás ! O técnico não resolveu o problema e ainda na consigo agendar a troca pq tenho que esperar um dia pra entrar no sistema</t>
+  </si>
+  <si>
+    <t>Não indicaria por causa do atendimento falho.Meu filtro deu problema logo após a vista técnica de manutenção.Solicitei nova visita técnica e foi agendado para 15 dias achei um absurdo a demora mas agendei.Quando chegou o dia percebi que o técnico não ia vim, então tive que entrar em contato 3 vezes e brigar para conseguir que o técnico viesse, o técnico veio bem mais tarde do previsto e chegou e não tinha as ferramentas para o determinado problema que quando agendei deixei bem claro qual era o problema.Muita desorganização, péssimo, brinca com o cliente.O filtro é bom, graças a Deus é difícil dar problema, mas quando da problema é muito difícil o suporte.</t>
+  </si>
+  <si>
+    <t>NÃO ME FOI ENTREGUE LAUDO/COMPROVANTE DA LIMPEZA DO FILTRO PARA ARQUIVAMENTO DA NUTRICIONISTA DA EMPRESA</t>
+  </si>
+  <si>
+    <t>Pedi a vista pq estou achando o gosto da água estranho e o técnico não mexeu em nada, dizendo que a qualidade está ok</t>
+  </si>
+  <si>
+    <t>Péssima, pago mensalidade e só preciso de 2 visitas ao ano e nunca aparecem</t>
+  </si>
+  <si>
+    <t>bom dia minha esperiencia com a empresa é pessima e digo pq.estou com meu purificador desde que chegou na caixa com nota e tudo com problema ao acionamento da agua com gaz contatando o tecnico foi constatado que é necessario a troca ai começa o problema liga somente fala com a maquina e quando atende são pessoas mal educadas não endente ou são pagas pra não entender resumo vindo outro tecnico mesma sujestão troca do aparelho isso depois de consultar seu superior que no viva voz falou faça alguma coisa ai se não der troca e ponto ....sendo assim liguei pro cartão de credito pedindo a suspensão da assinatura até que alguém resolva esse problema resolvido volto ao normal se não irei com a Patrulha do consumidor nessa empresa...</t>
+  </si>
+  <si>
+    <t>Estou marcando esta visita desde novembro/2025. É marcado e simplesmente o técnico não vem.</t>
+  </si>
+  <si>
+    <t>Decepção!!!</t>
+  </si>
+  <si>
+    <t>Manutenção não durou 30 minutos, e o filtro agora esta vazando agua.</t>
+  </si>
+  <si>
+    <t>Olá, Bom dia! Como estão?Escrevo para relatar uma experiência bem desconfortável que tivemos com o filtro.A Máquina foi instalada há uma semana e na mesma data apresentou problema com um ruído excessivo e a água não gelava. Solicitamos um técnico que veio ao local e informou que seria necessário a troca de uma peça e isso demoraria mais uma semana.Estamos com uma equipe sem água, causando insalubridade. Em toda a minha experiência de facilities cuidando de mais de 10 empresas, é a primeira vez que vejo um filtro quebrado sendo instalado. Isso não é um padrão Brastemp e a nossa imagem ficou afetada perante a empresa. Garantindo a lei do consumidor, o aparelho deverei ter sido substituido e não remanejado em seu primeiro uso por peças novas. Ficamos com a impressão de uma máquina usada e sem zelo.Ciente do compromisso Brastemp com o cliente, aguardamos breve retorno com troca por um produto novo.Obrigada.Aline SoaresGerente administrativo</t>
+  </si>
+  <si>
+    <t>Apesar dos transtornos da demora da execução, o serviço foi feito.O tecnico muito prestativo e resolveu o problema.</t>
+  </si>
+  <si>
+    <t>Houve dificuldade em solucionar o problema, onde só encontraram solução após a terceira visita e com isso ficamos muito tempo com o purificador sem ser utilizado.</t>
+  </si>
+  <si>
+    <t>Não sei avaliar...falou que nao tinha problema...estou avaliando ainda</t>
+  </si>
+  <si>
+    <t>problema não resolvido.</t>
+  </si>
+  <si>
+    <t>Tecnico cordial e profissional!</t>
+  </si>
+  <si>
+    <t>Atendimento horrível.</t>
+  </si>
+  <si>
+    <t>Olá, Boa tarde! Como estão?Escrevo para relatar uma experiência bem desconfortável que tivemos com o filtro.A Máquina foi instalada há uma semana e na mesma data apresentou problema com um ruído excessivo e a água não gelava. Solicitamos um técnico que veio ao local e informou que seria necessário a troca de uma peça e isso demoraria mais uma semana.Estamos com uma equipe sem água, causando insalubridade. Em toda a minha experiência de facilities cuidando de mais de 10 empresas, é a primeira vez que vejo um filtro quebrado sendo instalado. Isso não é um padrão Brastemp e a nossa imagem ficou afetada perante a empresa. Garantindo a lei do consumidor, o aparelho deverei ter sido substituido e não remanejado em seu primeiro uso por peças novas. Ficamos com a impressão de uma máquina usada e sem zelo.Ciente do compromisso Brastemp com o cliente, aguardamos breve retorno com troca por um produto novo.Obrigada.Aline SoaresGerente administrativo</t>
+  </si>
+  <si>
+    <t>Estou insatisfeita com o atendimento ao suporte de clientes, muito dificil marcar OS de manutenção</t>
+  </si>
+  <si>
+    <t>Indisponibilidade para agendamento de visita técnica em prazo razoável. Tive que esperar 1 mes para ser atendido em um problema técnico no equipamento! Muito ruim!</t>
   </si>
 </sst>
 </file>
@@ -2955,7 +3087,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I739"/>
+  <dimension ref="A1:I783"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -3717,7 +3849,7 @@
         <v>61</v>
       </c>
       <c r="H26" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
       <c r="I26" t="s">
         <v>177</v>
@@ -24398,6 +24530,1282 @@
       </c>
       <c r="I739" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="740" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A740">
+        <v>739</v>
+      </c>
+      <c r="B740" t="s">
+        <v>9</v>
+      </c>
+      <c r="C740">
+        <v>8714</v>
+      </c>
+      <c r="D740" s="3">
+        <v>46102.621527777781</v>
+      </c>
+      <c r="E740" t="s">
+        <v>695</v>
+      </c>
+      <c r="F740" t="s">
+        <v>16</v>
+      </c>
+      <c r="G740" t="s">
+        <v>819</v>
+      </c>
+      <c r="H740" t="s">
+        <v>18</v>
+      </c>
+      <c r="I740" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="741" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A741">
+        <v>740</v>
+      </c>
+      <c r="B741" t="s">
+        <v>9</v>
+      </c>
+      <c r="C741">
+        <v>8005315728</v>
+      </c>
+      <c r="D741" s="3">
+        <v>46103.620648148149</v>
+      </c>
+      <c r="E741" t="s">
+        <v>48</v>
+      </c>
+      <c r="F741" t="s">
+        <v>16</v>
+      </c>
+      <c r="G741" t="s">
+        <v>820</v>
+      </c>
+      <c r="H741" t="s">
+        <v>13</v>
+      </c>
+      <c r="I741" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="742" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A742">
+        <v>741</v>
+      </c>
+      <c r="B742" t="s">
+        <v>9</v>
+      </c>
+      <c r="C742">
+        <v>9637</v>
+      </c>
+      <c r="D742" s="3">
+        <v>46103.692395833335</v>
+      </c>
+      <c r="E742" t="s">
+        <v>695</v>
+      </c>
+      <c r="F742" t="s">
+        <v>16</v>
+      </c>
+      <c r="G742" t="s">
+        <v>821</v>
+      </c>
+      <c r="H742" t="s">
+        <v>18</v>
+      </c>
+      <c r="I742" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="743" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A743">
+        <v>742</v>
+      </c>
+      <c r="B743" t="s">
+        <v>9</v>
+      </c>
+      <c r="C743">
+        <v>10859</v>
+      </c>
+      <c r="D743" s="3">
+        <v>46104.444074074076</v>
+      </c>
+      <c r="E743" t="s">
+        <v>695</v>
+      </c>
+      <c r="F743" t="s">
+        <v>16</v>
+      </c>
+      <c r="G743" t="s">
+        <v>822</v>
+      </c>
+      <c r="H743" t="s">
+        <v>34</v>
+      </c>
+      <c r="I743" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="744" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A744">
+        <v>743</v>
+      </c>
+      <c r="B744" t="s">
+        <v>9</v>
+      </c>
+      <c r="C744">
+        <v>8005302532</v>
+      </c>
+      <c r="D744" s="3">
+        <v>46104.461828703701</v>
+      </c>
+      <c r="E744" t="s">
+        <v>48</v>
+      </c>
+      <c r="F744" t="s">
+        <v>16</v>
+      </c>
+      <c r="G744" t="s">
+        <v>823</v>
+      </c>
+      <c r="H744" t="s">
+        <v>18</v>
+      </c>
+      <c r="I744" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="745" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A745">
+        <v>744</v>
+      </c>
+      <c r="B745" t="s">
+        <v>9</v>
+      </c>
+      <c r="C745">
+        <v>10256</v>
+      </c>
+      <c r="D745" s="3">
+        <v>46104.501087962963</v>
+      </c>
+      <c r="E745" t="s">
+        <v>695</v>
+      </c>
+      <c r="F745" t="s">
+        <v>11</v>
+      </c>
+      <c r="G745" t="s">
+        <v>824</v>
+      </c>
+      <c r="H745" t="s">
+        <v>34</v>
+      </c>
+      <c r="I745" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="746" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A746">
+        <v>745</v>
+      </c>
+      <c r="B746" t="s">
+        <v>9</v>
+      </c>
+      <c r="C746">
+        <v>8005329112</v>
+      </c>
+      <c r="D746" s="3">
+        <v>46104.503483796296</v>
+      </c>
+      <c r="E746" t="s">
+        <v>20</v>
+      </c>
+      <c r="F746" t="s">
+        <v>11</v>
+      </c>
+      <c r="G746" t="s">
+        <v>825</v>
+      </c>
+      <c r="H746" t="s">
+        <v>31</v>
+      </c>
+      <c r="I746" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="747" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A747">
+        <v>746</v>
+      </c>
+      <c r="B747" t="s">
+        <v>9</v>
+      </c>
+      <c r="C747">
+        <v>8005318286</v>
+      </c>
+      <c r="D747" s="3">
+        <v>46104.504166666666</v>
+      </c>
+      <c r="E747" t="s">
+        <v>20</v>
+      </c>
+      <c r="F747" t="s">
+        <v>11</v>
+      </c>
+      <c r="G747" t="s">
+        <v>826</v>
+      </c>
+      <c r="H747" t="s">
+        <v>31</v>
+      </c>
+      <c r="I747" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="748" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A748">
+        <v>747</v>
+      </c>
+      <c r="B748" t="s">
+        <v>9</v>
+      </c>
+      <c r="C748">
+        <v>8005301558</v>
+      </c>
+      <c r="D748" s="3">
+        <v>46104.506030092591</v>
+      </c>
+      <c r="E748" t="s">
+        <v>52</v>
+      </c>
+      <c r="F748" t="s">
+        <v>16</v>
+      </c>
+      <c r="G748" t="s">
+        <v>827</v>
+      </c>
+      <c r="H748" t="s">
+        <v>18</v>
+      </c>
+      <c r="I748" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="749" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A749">
+        <v>748</v>
+      </c>
+      <c r="B749" t="s">
+        <v>9</v>
+      </c>
+      <c r="C749">
+        <v>8005330864</v>
+      </c>
+      <c r="D749" s="3">
+        <v>46104.509189814817</v>
+      </c>
+      <c r="E749" t="s">
+        <v>260</v>
+      </c>
+      <c r="F749" t="s">
+        <v>11</v>
+      </c>
+      <c r="G749" t="s">
+        <v>828</v>
+      </c>
+      <c r="H749" t="s">
+        <v>13</v>
+      </c>
+      <c r="I749" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="750" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A750">
+        <v>749</v>
+      </c>
+      <c r="B750" t="s">
+        <v>9</v>
+      </c>
+      <c r="C750">
+        <v>8005321879</v>
+      </c>
+      <c r="D750" s="3">
+        <v>46104.519861111112</v>
+      </c>
+      <c r="E750" t="s">
+        <v>52</v>
+      </c>
+      <c r="F750" t="s">
+        <v>16</v>
+      </c>
+      <c r="G750" t="s">
+        <v>829</v>
+      </c>
+      <c r="H750" t="s">
+        <v>18</v>
+      </c>
+      <c r="I750" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="751" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A751">
+        <v>750</v>
+      </c>
+      <c r="B751" t="s">
+        <v>9</v>
+      </c>
+      <c r="C751">
+        <v>8005287388</v>
+      </c>
+      <c r="D751" s="3">
+        <v>46104.543414351851</v>
+      </c>
+      <c r="E751" t="s">
+        <v>15</v>
+      </c>
+      <c r="F751" t="s">
+        <v>16</v>
+      </c>
+      <c r="G751" t="s">
+        <v>830</v>
+      </c>
+      <c r="H751" t="s">
+        <v>13</v>
+      </c>
+      <c r="I751" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="752" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A752">
+        <v>751</v>
+      </c>
+      <c r="B752" t="s">
+        <v>9</v>
+      </c>
+      <c r="C752">
+        <v>8826</v>
+      </c>
+      <c r="D752" s="3">
+        <v>46104.54991898148</v>
+      </c>
+      <c r="E752" t="s">
+        <v>735</v>
+      </c>
+      <c r="F752" t="s">
+        <v>16</v>
+      </c>
+      <c r="G752" t="s">
+        <v>831</v>
+      </c>
+      <c r="H752" t="s">
+        <v>18</v>
+      </c>
+      <c r="I752" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="753" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A753">
+        <v>752</v>
+      </c>
+      <c r="B753" t="s">
+        <v>9</v>
+      </c>
+      <c r="C753">
+        <v>8005330590</v>
+      </c>
+      <c r="D753" s="3">
+        <v>46104.560335648152</v>
+      </c>
+      <c r="E753" t="s">
+        <v>63</v>
+      </c>
+      <c r="F753" t="s">
+        <v>11</v>
+      </c>
+      <c r="G753" t="s">
+        <v>832</v>
+      </c>
+      <c r="H753" t="s">
+        <v>31</v>
+      </c>
+      <c r="I753" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="754" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A754">
+        <v>753</v>
+      </c>
+      <c r="B754" t="s">
+        <v>9</v>
+      </c>
+      <c r="C754">
+        <v>8005305603</v>
+      </c>
+      <c r="D754" s="3">
+        <v>46104.570439814815</v>
+      </c>
+      <c r="E754" t="s">
+        <v>36</v>
+      </c>
+      <c r="F754" t="s">
+        <v>11</v>
+      </c>
+      <c r="G754" t="s">
+        <v>833</v>
+      </c>
+      <c r="H754" t="s">
+        <v>18</v>
+      </c>
+      <c r="I754" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="755" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A755">
+        <v>754</v>
+      </c>
+      <c r="B755" t="s">
+        <v>9</v>
+      </c>
+      <c r="C755">
+        <v>8005326412</v>
+      </c>
+      <c r="D755" s="3">
+        <v>46104.647233796299</v>
+      </c>
+      <c r="E755" t="s">
+        <v>20</v>
+      </c>
+      <c r="F755" t="s">
+        <v>11</v>
+      </c>
+      <c r="G755" t="s">
+        <v>834</v>
+      </c>
+      <c r="H755" t="s">
+        <v>13</v>
+      </c>
+      <c r="I755" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="756" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A756">
+        <v>755</v>
+      </c>
+      <c r="B756" t="s">
+        <v>9</v>
+      </c>
+      <c r="C756">
+        <v>8005331661</v>
+      </c>
+      <c r="D756" s="3">
+        <v>46104.891342592593</v>
+      </c>
+      <c r="E756" t="s">
+        <v>20</v>
+      </c>
+      <c r="F756" t="s">
+        <v>16</v>
+      </c>
+      <c r="G756" t="s">
+        <v>835</v>
+      </c>
+      <c r="H756" t="s">
+        <v>18</v>
+      </c>
+      <c r="I756" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="757" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A757">
+        <v>756</v>
+      </c>
+      <c r="B757" t="s">
+        <v>9</v>
+      </c>
+      <c r="C757">
+        <v>8005334069</v>
+      </c>
+      <c r="D757" s="3">
+        <v>46105.402685185189</v>
+      </c>
+      <c r="E757" t="s">
+        <v>96</v>
+      </c>
+      <c r="F757" t="s">
+        <v>16</v>
+      </c>
+      <c r="G757" t="s">
+        <v>836</v>
+      </c>
+      <c r="H757" t="s">
+        <v>18</v>
+      </c>
+      <c r="I757" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="758" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A758">
+        <v>757</v>
+      </c>
+      <c r="B758" t="s">
+        <v>9</v>
+      </c>
+      <c r="C758">
+        <v>8005333005</v>
+      </c>
+      <c r="D758" s="3">
+        <v>46105.418217592596</v>
+      </c>
+      <c r="E758" t="s">
+        <v>52</v>
+      </c>
+      <c r="F758" t="s">
+        <v>16</v>
+      </c>
+      <c r="G758" t="s">
+        <v>837</v>
+      </c>
+      <c r="H758" t="s">
+        <v>18</v>
+      </c>
+      <c r="I758" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="759" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A759">
+        <v>758</v>
+      </c>
+      <c r="B759" t="s">
+        <v>9</v>
+      </c>
+      <c r="C759">
+        <v>5472</v>
+      </c>
+      <c r="D759" s="3">
+        <v>46105.504745370374</v>
+      </c>
+      <c r="E759" t="s">
+        <v>735</v>
+      </c>
+      <c r="F759" t="s">
+        <v>16</v>
+      </c>
+      <c r="G759" t="s">
+        <v>838</v>
+      </c>
+      <c r="H759" t="s">
+        <v>18</v>
+      </c>
+      <c r="I759" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="760" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A760">
+        <v>759</v>
+      </c>
+      <c r="B760" t="s">
+        <v>9</v>
+      </c>
+      <c r="C760">
+        <v>8005287475</v>
+      </c>
+      <c r="D760" s="3">
+        <v>46105.521944444445</v>
+      </c>
+      <c r="E760" t="s">
+        <v>222</v>
+      </c>
+      <c r="F760" t="s">
+        <v>11</v>
+      </c>
+      <c r="G760" t="s">
+        <v>839</v>
+      </c>
+      <c r="H760" t="s">
+        <v>31</v>
+      </c>
+      <c r="I760" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="761" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A761">
+        <v>760</v>
+      </c>
+      <c r="B761" t="s">
+        <v>9</v>
+      </c>
+      <c r="C761">
+        <v>8842</v>
+      </c>
+      <c r="D761" s="3">
+        <v>46105.540034722224</v>
+      </c>
+      <c r="E761" t="s">
+        <v>735</v>
+      </c>
+      <c r="F761" t="s">
+        <v>16</v>
+      </c>
+      <c r="G761" t="s">
+        <v>840</v>
+      </c>
+      <c r="H761" t="s">
+        <v>34</v>
+      </c>
+      <c r="I761" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="762" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A762">
+        <v>761</v>
+      </c>
+      <c r="B762" t="s">
+        <v>9</v>
+      </c>
+      <c r="C762">
+        <v>10536</v>
+      </c>
+      <c r="D762" s="3">
+        <v>46105.60355324074</v>
+      </c>
+      <c r="E762" t="s">
+        <v>680</v>
+      </c>
+      <c r="F762" t="s">
+        <v>16</v>
+      </c>
+      <c r="G762" t="s">
+        <v>841</v>
+      </c>
+      <c r="H762" t="s">
+        <v>31</v>
+      </c>
+      <c r="I762" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="763" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A763">
+        <v>762</v>
+      </c>
+      <c r="B763" t="s">
+        <v>9</v>
+      </c>
+      <c r="C763">
+        <v>10351</v>
+      </c>
+      <c r="D763" s="3">
+        <v>46105.623518518521</v>
+      </c>
+      <c r="E763" t="s">
+        <v>697</v>
+      </c>
+      <c r="F763" t="s">
+        <v>11</v>
+      </c>
+      <c r="G763" t="s">
+        <v>842</v>
+      </c>
+      <c r="H763" t="s">
+        <v>34</v>
+      </c>
+      <c r="I763" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="764" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A764">
+        <v>763</v>
+      </c>
+      <c r="B764" t="s">
+        <v>9</v>
+      </c>
+      <c r="C764">
+        <v>10662</v>
+      </c>
+      <c r="D764" s="3">
+        <v>46105.638287037036</v>
+      </c>
+      <c r="E764" t="s">
+        <v>710</v>
+      </c>
+      <c r="F764" t="s">
+        <v>16</v>
+      </c>
+      <c r="G764" t="s">
+        <v>843</v>
+      </c>
+      <c r="H764" t="s">
+        <v>152</v>
+      </c>
+      <c r="I764" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="765" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A765">
+        <v>764</v>
+      </c>
+      <c r="B765" t="s">
+        <v>9</v>
+      </c>
+      <c r="C765">
+        <v>10843</v>
+      </c>
+      <c r="D765" s="3">
+        <v>46106.421979166669</v>
+      </c>
+      <c r="E765" t="s">
+        <v>695</v>
+      </c>
+      <c r="F765" t="s">
+        <v>16</v>
+      </c>
+      <c r="G765" t="s">
+        <v>844</v>
+      </c>
+      <c r="H765" t="s">
+        <v>34</v>
+      </c>
+      <c r="I765" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="766" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A766">
+        <v>765</v>
+      </c>
+      <c r="B766" t="s">
+        <v>9</v>
+      </c>
+      <c r="C766">
+        <v>8696</v>
+      </c>
+      <c r="D766" s="3">
+        <v>46106.451365740744</v>
+      </c>
+      <c r="E766" t="s">
+        <v>680</v>
+      </c>
+      <c r="F766" t="s">
+        <v>16</v>
+      </c>
+      <c r="G766" t="s">
+        <v>845</v>
+      </c>
+      <c r="H766" t="s">
+        <v>31</v>
+      </c>
+      <c r="I766" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="767" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A767">
+        <v>766</v>
+      </c>
+      <c r="B767" t="s">
+        <v>9</v>
+      </c>
+      <c r="C767">
+        <v>10970</v>
+      </c>
+      <c r="D767" s="3">
+        <v>46106.463831018518</v>
+      </c>
+      <c r="E767" t="s">
+        <v>677</v>
+      </c>
+      <c r="F767" t="s">
+        <v>11</v>
+      </c>
+      <c r="G767" t="s">
+        <v>846</v>
+      </c>
+      <c r="H767" t="s">
+        <v>18</v>
+      </c>
+      <c r="I767" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="768" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A768">
+        <v>767</v>
+      </c>
+      <c r="B768" t="s">
+        <v>9</v>
+      </c>
+      <c r="C768">
+        <v>8005321423</v>
+      </c>
+      <c r="D768" s="3">
+        <v>46106.50371527778</v>
+      </c>
+      <c r="E768" t="s">
+        <v>20</v>
+      </c>
+      <c r="F768" t="s">
+        <v>11</v>
+      </c>
+      <c r="G768" t="s">
+        <v>847</v>
+      </c>
+      <c r="H768" t="s">
+        <v>18</v>
+      </c>
+      <c r="I768" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="769" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A769">
+        <v>768</v>
+      </c>
+      <c r="B769" t="s">
+        <v>9</v>
+      </c>
+      <c r="C769">
+        <v>8005326958</v>
+      </c>
+      <c r="D769" s="3">
+        <v>46106.806064814817</v>
+      </c>
+      <c r="E769" t="s">
+        <v>20</v>
+      </c>
+      <c r="F769" t="s">
+        <v>16</v>
+      </c>
+      <c r="G769" t="s">
+        <v>848</v>
+      </c>
+      <c r="H769" t="s">
+        <v>18</v>
+      </c>
+      <c r="I769" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="770" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A770">
+        <v>769</v>
+      </c>
+      <c r="B770" t="s">
+        <v>9</v>
+      </c>
+      <c r="C770">
+        <v>9676</v>
+      </c>
+      <c r="D770" s="3">
+        <v>46107.376805555556</v>
+      </c>
+      <c r="E770" t="s">
+        <v>680</v>
+      </c>
+      <c r="F770" t="s">
+        <v>16</v>
+      </c>
+      <c r="G770" t="s">
+        <v>849</v>
+      </c>
+      <c r="H770" t="s">
+        <v>80</v>
+      </c>
+      <c r="I770" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="771" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A771">
+        <v>770</v>
+      </c>
+      <c r="B771" t="s">
+        <v>9</v>
+      </c>
+      <c r="C771">
+        <v>8005298624</v>
+      </c>
+      <c r="D771" s="3">
+        <v>46107.392581018517</v>
+      </c>
+      <c r="E771" t="s">
+        <v>52</v>
+      </c>
+      <c r="F771" t="s">
+        <v>11</v>
+      </c>
+      <c r="G771" t="s">
+        <v>850</v>
+      </c>
+      <c r="H771" t="s">
+        <v>18</v>
+      </c>
+      <c r="I771" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="772" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A772">
+        <v>771</v>
+      </c>
+      <c r="B772" t="s">
+        <v>9</v>
+      </c>
+      <c r="C772">
+        <v>10124</v>
+      </c>
+      <c r="D772" s="3">
+        <v>46107.429212962961</v>
+      </c>
+      <c r="E772" t="s">
+        <v>718</v>
+      </c>
+      <c r="F772" t="s">
+        <v>16</v>
+      </c>
+      <c r="G772" t="s">
+        <v>851</v>
+      </c>
+      <c r="H772" t="s">
+        <v>13</v>
+      </c>
+      <c r="I772" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="773" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A773">
+        <v>772</v>
+      </c>
+      <c r="B773" t="s">
+        <v>9</v>
+      </c>
+      <c r="C773">
+        <v>8005327925</v>
+      </c>
+      <c r="D773" s="3">
+        <v>46107.43236111111</v>
+      </c>
+      <c r="E773" t="s">
+        <v>96</v>
+      </c>
+      <c r="F773" t="s">
+        <v>16</v>
+      </c>
+      <c r="G773" t="s">
+        <v>852</v>
+      </c>
+      <c r="H773" t="s">
+        <v>18</v>
+      </c>
+      <c r="I773" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="774" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A774">
+        <v>773</v>
+      </c>
+      <c r="B774" t="s">
+        <v>60</v>
+      </c>
+      <c r="C774">
+        <v>8005331968</v>
+      </c>
+      <c r="D774" s="3">
+        <v>46107.459340277775</v>
+      </c>
+      <c r="E774" t="s">
+        <v>20</v>
+      </c>
+      <c r="F774" t="s">
+        <v>16</v>
+      </c>
+      <c r="G774" t="s">
+        <v>853</v>
+      </c>
+      <c r="H774" t="s">
+        <v>34</v>
+      </c>
+      <c r="I774" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="775" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A775">
+        <v>774</v>
+      </c>
+      <c r="B775" t="s">
+        <v>9</v>
+      </c>
+      <c r="C775">
+        <v>6947</v>
+      </c>
+      <c r="D775" s="3">
+        <v>46107.477037037039</v>
+      </c>
+      <c r="E775" t="s">
+        <v>677</v>
+      </c>
+      <c r="F775" t="s">
+        <v>11</v>
+      </c>
+      <c r="G775" t="s">
+        <v>854</v>
+      </c>
+      <c r="H775" t="s">
+        <v>13</v>
+      </c>
+      <c r="I775" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="776" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A776">
+        <v>775</v>
+      </c>
+      <c r="B776" t="s">
+        <v>9</v>
+      </c>
+      <c r="C776">
+        <v>8005331623</v>
+      </c>
+      <c r="D776" s="3">
+        <v>46107.493391203701</v>
+      </c>
+      <c r="E776" t="s">
+        <v>20</v>
+      </c>
+      <c r="F776" t="s">
+        <v>11</v>
+      </c>
+      <c r="G776" t="s">
+        <v>855</v>
+      </c>
+      <c r="H776" t="s">
+        <v>18</v>
+      </c>
+      <c r="I776" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="777" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A777">
+        <v>776</v>
+      </c>
+      <c r="B777" t="s">
+        <v>9</v>
+      </c>
+      <c r="C777">
+        <v>11397</v>
+      </c>
+      <c r="D777" s="3">
+        <v>46107.496307870373</v>
+      </c>
+      <c r="E777" t="s">
+        <v>718</v>
+      </c>
+      <c r="F777" t="s">
+        <v>11</v>
+      </c>
+      <c r="G777" t="s">
+        <v>856</v>
+      </c>
+      <c r="H777" t="s">
+        <v>13</v>
+      </c>
+      <c r="I777" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="778" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A778">
+        <v>777</v>
+      </c>
+      <c r="B778" t="s">
+        <v>9</v>
+      </c>
+      <c r="C778">
+        <v>8005330271</v>
+      </c>
+      <c r="D778" s="3">
+        <v>46107.500810185185</v>
+      </c>
+      <c r="E778" t="s">
+        <v>36</v>
+      </c>
+      <c r="F778" t="s">
+        <v>16</v>
+      </c>
+      <c r="G778" t="s">
+        <v>857</v>
+      </c>
+      <c r="H778" t="s">
+        <v>18</v>
+      </c>
+      <c r="I778" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="779" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A779">
+        <v>778</v>
+      </c>
+      <c r="B779" t="s">
+        <v>9</v>
+      </c>
+      <c r="C779">
+        <v>8005323511</v>
+      </c>
+      <c r="D779" s="3">
+        <v>46107.505462962959</v>
+      </c>
+      <c r="E779" t="s">
+        <v>20</v>
+      </c>
+      <c r="F779" t="s">
+        <v>11</v>
+      </c>
+      <c r="G779" t="s">
+        <v>858</v>
+      </c>
+      <c r="H779" t="s">
+        <v>13</v>
+      </c>
+      <c r="I779" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="780" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A780">
+        <v>779</v>
+      </c>
+      <c r="B780" t="s">
+        <v>9</v>
+      </c>
+      <c r="C780">
+        <v>11658</v>
+      </c>
+      <c r="D780" s="3">
+        <v>46107.579282407409</v>
+      </c>
+      <c r="E780" t="s">
+        <v>718</v>
+      </c>
+      <c r="F780" t="s">
+        <v>16</v>
+      </c>
+      <c r="G780" t="s">
+        <v>859</v>
+      </c>
+      <c r="H780" t="s">
+        <v>13</v>
+      </c>
+      <c r="I780" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="781" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A781">
+        <v>780</v>
+      </c>
+      <c r="B781" t="s">
+        <v>9</v>
+      </c>
+      <c r="C781">
+        <v>8005334164</v>
+      </c>
+      <c r="D781" s="3">
+        <v>46107.594594907408</v>
+      </c>
+      <c r="E781" t="s">
+        <v>20</v>
+      </c>
+      <c r="F781" t="s">
+        <v>16</v>
+      </c>
+      <c r="G781" t="s">
+        <v>860</v>
+      </c>
+      <c r="H781" t="s">
+        <v>18</v>
+      </c>
+      <c r="I781" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="782" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A782">
+        <v>781</v>
+      </c>
+      <c r="B782" t="s">
+        <v>9</v>
+      </c>
+      <c r="C782">
+        <v>8005334675</v>
+      </c>
+      <c r="D782" s="3">
+        <v>46107.624386574076</v>
+      </c>
+      <c r="E782" t="s">
+        <v>222</v>
+      </c>
+      <c r="F782" t="s">
+        <v>16</v>
+      </c>
+      <c r="G782" t="s">
+        <v>861</v>
+      </c>
+      <c r="H782" t="s">
+        <v>31</v>
+      </c>
+      <c r="I782" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="783" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A783">
+        <v>782</v>
+      </c>
+      <c r="B783" t="s">
+        <v>9</v>
+      </c>
+      <c r="C783">
+        <v>8005310467</v>
+      </c>
+      <c r="D783" s="3">
+        <v>46108.412627314814</v>
+      </c>
+      <c r="E783" t="s">
+        <v>48</v>
+      </c>
+      <c r="F783" t="s">
+        <v>16</v>
+      </c>
+      <c r="G783" t="s">
+        <v>862</v>
+      </c>
+      <c r="H783" t="s">
+        <v>31</v>
+      </c>
+      <c r="I783" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/04/2026 16:59:03,49
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="184" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A03CA44-C790-4455-9EBB-69AC8B5C142D}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{341405C3-8B94-4FF6-BB19-52D16E22337F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4701" uniqueCount="863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4857" uniqueCount="890">
   <si>
     <t>ID</t>
   </si>
@@ -2719,6 +2719,87 @@
   </si>
   <si>
     <t>Indisponibilidade para agendamento de visita técnica em prazo razoável. Tive que esperar 1 mes para ser atendido em um problema técnico no equipamento! Muito ruim!</t>
+  </si>
+  <si>
+    <t>Cuido da manutenção de 3 filtros nos últimos tempos temos tido problemas com o não comparecimento do técnico no dia agendado.  Neste atendimento analisado já tinha vindo um técnico aqui em dezembro q sinalizou a troca do filtro por um modelo mais atual. O técnico de ontem fez a mesma coisa do outro técnico e Tb recomendou a troca do filtro.</t>
+  </si>
+  <si>
+    <t>Os técnicos vieram instalar o filtro. Após a instalação o filtro começou a vazar água por baixo, ele está perto de um móvel de madeira vai acabar estragado se não parar o vazamento.O registro que liga água no filtro é da cozinha que e nao posso desligar.Amanhã tenho uma festa aqui em casa pra 40 pessoas e preciso do filtro e da cozinha funcionando a todo vapor.Preciso URGENTE que os técnicos retornem para ver o que está acontecendo!!!!!!!!!!</t>
+  </si>
+  <si>
+    <t>Prestador de serviço rude, mal humorado, parecia que estava fazendo um favor ao trabalhar. Chutou o elevador do meu prédio porque eu pedi para ele entrar pela área de serviço, para não ter tirar a bota. A minha vontade é cancelar a assinatura do filtro Brastemp devido a esta situação.</t>
+  </si>
+  <si>
+    <t>Fiquei quase 3 meses para enviarem técnico aqui verificar um problema recorrente.Não consegui contato com a supervisão e muito menos acionando financeiro.Estamos cotando com outras empresas.</t>
+  </si>
+  <si>
+    <t>Não houve visita</t>
+  </si>
+  <si>
+    <t>Fui muito mal atendido pelo serviço de atendimento, onde me chamaram de ignorante, sou cliente a mais de 6 anos pagando todas as mensalidades em dia para ser ofendido ao solicitar Manutenção do Purificador. Vejam a ligação no servico de atendimento.</t>
+  </si>
+  <si>
+    <t>Tempo de agendamento muito longo nos casos de manutenção emergencial.</t>
+  </si>
+  <si>
+    <t>Atendimento do técnico foi bom , agora o Call Center horrível , estou a mais de 20 dias com meu filtro quebrado e até o momento nada</t>
+  </si>
+  <si>
+    <t>O purificador está com falha na saída de água, solicitei a troca e não ocorreu, estou com o filtro já tem anos</t>
+  </si>
+  <si>
+    <t>BOM DIATEM ALGUNS MESES QUE NAO ESTA LEGAL MARCAR A VISITA MAIS NAO COMPARECE NAO DA NENHUMA SITISFAÇAO MANDO MENSAGEM NAO FALA PORQUE NAO COMPARCEU MARCAR DE NOVO E O TECNICO NAO COMPARECE DE NOVO</t>
+  </si>
+  <si>
+    <t>Ficamos durante um mês inteiro sem a refrigeração do purificador de água.Muita demora na substituição do aparelho novo.Não recebi o e-mail com os boletos de pagamentos para final deste mês.Inclusive, solicito a isenção do pagamento deste aparelho que ficou sem a refrigeração no mês inteiro.Muito obrigada</t>
+  </si>
+  <si>
+    <t>O ponto fraco é o preço da mensalidade, que está extremamente caro. O restante é ótimo.</t>
+  </si>
+  <si>
+    <t>não me informou o dia da visita e não atendeu meu pedido ou minha necessidade</t>
+  </si>
+  <si>
+    <t>Quanto a troca tudo bem o técnico veio e trocou. Mas a demora da Brastemp agendar a troca foi demais. Quando o primeiro técnico veio ver o problema e solicitou a troca eu já estava sem água gelada há quase um mês. E depois disso a Brastemp demorou demais para trocar . Ficamos quase 3 meses sem água gelada. E pagando. Isso não é certo. Meu marido pede no mínimo isenção do pagt desses meses</t>
+  </si>
+  <si>
+    <t>desde o dia 03 de março  solicitei o serviço de troca do filtro e só obtive o serviço no dia 27 de março. Fiquei quase um mês  tendo que comprar água, pois a do filtro não estava em condições de beber.  Reclamei  no serviço, aliás muito difícil a comunicação entre as pessoas, que me garantiu que seria agilizada a troca e não seria cobrada a mensalidade do mês, uma vez que não obtive água e de qualidade.  E não foi o que aconteceu.  Demorou o atendimento e foi descontado o mês.</t>
+  </si>
+  <si>
+    <t>Boa tarde. A brastemp  precisa inovar os purificadores. Estou com a brastemp  desde que ela iniciou  em Campinas.  Hoje tem purificadores  que hidrogênio,  ions, e outras coisas</t>
+  </si>
+  <si>
+    <t>Consideramos o produto da troca inferior ao modelo que tínhamos anteriormente.</t>
+  </si>
+  <si>
+    <t>QUALIDADE DO PRODUTO</t>
+  </si>
+  <si>
+    <t>Acho muito. Bom</t>
+  </si>
+  <si>
+    <t>Péssima, trocaram o purificador, e me deixaram um que não gela, e visita pra tentar solucionar, só daqui 8 dias. Péssimo atendimento.</t>
+  </si>
+  <si>
+    <t>Não vieram novamente mesmo apos marcarmos pela segunda vez a visita.</t>
+  </si>
+  <si>
+    <t>Desde o ano passado tem sido um verdadeiro parto a marcação e realização das visitas semestrais.O pior é qdo está agendado e depois de ficar aguardando a visita, ela não se realiza.Falta total de consideração em avisar que a visita foi cancelada.</t>
+  </si>
+  <si>
+    <t>Queria um modelo mais moderno</t>
+  </si>
+  <si>
+    <t>Excelente, porém dificuldade em ser atendida, várias visitas não foram cumprida. O motivo falha na Brastemp por não ter passado a ordem de serviço para o técnico</t>
+  </si>
+  <si>
+    <t>Estou com dúvida em relação a troca do filtro interno.</t>
+  </si>
+  <si>
+    <t>gosto muito do Purificador e acho que vale muito ter. É a certeza de er boa água e bem tratada.</t>
+  </si>
+  <si>
+    <t>Não estou satisfeita com a equipe  me marcação  para vir ver o meu purificador remarcaram 3 vezesAchei um absurdo</t>
   </si>
 </sst>
 </file>
@@ -3087,7 +3168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I783"/>
+  <dimension ref="A1:I809"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -25808,6 +25889,760 @@
         <v>32</v>
       </c>
     </row>
+    <row r="784" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A784">
+        <v>783</v>
+      </c>
+      <c r="B784" t="s">
+        <v>9</v>
+      </c>
+      <c r="C784">
+        <v>8005331541</v>
+      </c>
+      <c r="D784" s="3">
+        <v>46108.514340277776</v>
+      </c>
+      <c r="E784" t="s">
+        <v>52</v>
+      </c>
+      <c r="F784" t="s">
+        <v>16</v>
+      </c>
+      <c r="G784" t="s">
+        <v>863</v>
+      </c>
+      <c r="H784" t="s">
+        <v>18</v>
+      </c>
+      <c r="I784" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="785" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A785">
+        <v>784</v>
+      </c>
+      <c r="B785" t="s">
+        <v>60</v>
+      </c>
+      <c r="C785">
+        <v>8005248197</v>
+      </c>
+      <c r="D785" s="3">
+        <v>46108.520648148151</v>
+      </c>
+      <c r="E785" t="s">
+        <v>222</v>
+      </c>
+      <c r="F785" t="s">
+        <v>16</v>
+      </c>
+      <c r="G785" t="s">
+        <v>864</v>
+      </c>
+      <c r="H785" t="s">
+        <v>18</v>
+      </c>
+      <c r="I785" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="786" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A786">
+        <v>785</v>
+      </c>
+      <c r="B786" t="s">
+        <v>9</v>
+      </c>
+      <c r="C786">
+        <v>8005296658</v>
+      </c>
+      <c r="D786" s="3">
+        <v>46108.528124999997</v>
+      </c>
+      <c r="E786" t="s">
+        <v>123</v>
+      </c>
+      <c r="F786" t="s">
+        <v>16</v>
+      </c>
+      <c r="G786" t="s">
+        <v>865</v>
+      </c>
+      <c r="H786" t="s">
+        <v>18</v>
+      </c>
+      <c r="I786" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="787" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A787">
+        <v>786</v>
+      </c>
+      <c r="B787" t="s">
+        <v>9</v>
+      </c>
+      <c r="C787">
+        <v>8005320053</v>
+      </c>
+      <c r="D787" s="3">
+        <v>46108.61136574074</v>
+      </c>
+      <c r="E787" t="s">
+        <v>20</v>
+      </c>
+      <c r="F787" t="s">
+        <v>16</v>
+      </c>
+      <c r="G787" t="s">
+        <v>866</v>
+      </c>
+      <c r="H787" t="s">
+        <v>31</v>
+      </c>
+      <c r="I787" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="788" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A788">
+        <v>787</v>
+      </c>
+      <c r="B788" t="s">
+        <v>9</v>
+      </c>
+      <c r="C788">
+        <v>8005315806</v>
+      </c>
+      <c r="D788" s="3">
+        <v>46108.64472222222</v>
+      </c>
+      <c r="E788" t="s">
+        <v>52</v>
+      </c>
+      <c r="F788" t="s">
+        <v>16</v>
+      </c>
+      <c r="G788" t="s">
+        <v>867</v>
+      </c>
+      <c r="H788" t="s">
+        <v>18</v>
+      </c>
+      <c r="I788" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="789" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A789">
+        <v>788</v>
+      </c>
+      <c r="B789" t="s">
+        <v>9</v>
+      </c>
+      <c r="C789">
+        <v>10842</v>
+      </c>
+      <c r="D789" s="3">
+        <v>46108.851666666669</v>
+      </c>
+      <c r="E789" t="s">
+        <v>680</v>
+      </c>
+      <c r="F789" t="s">
+        <v>16</v>
+      </c>
+      <c r="G789" t="s">
+        <v>868</v>
+      </c>
+      <c r="H789" t="s">
+        <v>80</v>
+      </c>
+      <c r="I789" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="790" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A790">
+        <v>789</v>
+      </c>
+      <c r="B790" t="s">
+        <v>9</v>
+      </c>
+      <c r="C790">
+        <v>8005329839</v>
+      </c>
+      <c r="D790" s="3">
+        <v>46109.267453703702</v>
+      </c>
+      <c r="E790" t="s">
+        <v>63</v>
+      </c>
+      <c r="F790" t="s">
+        <v>16</v>
+      </c>
+      <c r="G790" t="s">
+        <v>869</v>
+      </c>
+      <c r="H790" t="s">
+        <v>31</v>
+      </c>
+      <c r="I790" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="791" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A791">
+        <v>790</v>
+      </c>
+      <c r="B791" t="s">
+        <v>9</v>
+      </c>
+      <c r="C791">
+        <v>8125</v>
+      </c>
+      <c r="D791" s="3">
+        <v>46109.517407407409</v>
+      </c>
+      <c r="E791" t="s">
+        <v>677</v>
+      </c>
+      <c r="F791" t="s">
+        <v>16</v>
+      </c>
+      <c r="G791" t="s">
+        <v>870</v>
+      </c>
+      <c r="H791" t="s">
+        <v>80</v>
+      </c>
+      <c r="I791" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="792" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A792">
+        <v>791</v>
+      </c>
+      <c r="B792" t="s">
+        <v>9</v>
+      </c>
+      <c r="C792">
+        <v>8005335039</v>
+      </c>
+      <c r="D792" s="3">
+        <v>46111.405613425923</v>
+      </c>
+      <c r="E792" t="s">
+        <v>52</v>
+      </c>
+      <c r="F792" t="s">
+        <v>16</v>
+      </c>
+      <c r="G792" t="s">
+        <v>871</v>
+      </c>
+      <c r="H792" t="s">
+        <v>18</v>
+      </c>
+      <c r="I792" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="793" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A793">
+        <v>792</v>
+      </c>
+      <c r="B793" t="s">
+        <v>9</v>
+      </c>
+      <c r="C793">
+        <v>8005336968</v>
+      </c>
+      <c r="D793" s="3">
+        <v>46111.420694444445</v>
+      </c>
+      <c r="E793" t="s">
+        <v>52</v>
+      </c>
+      <c r="F793" t="s">
+        <v>16</v>
+      </c>
+      <c r="G793" t="s">
+        <v>872</v>
+      </c>
+      <c r="H793" t="s">
+        <v>18</v>
+      </c>
+      <c r="I793" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="794" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A794">
+        <v>793</v>
+      </c>
+      <c r="B794" t="s">
+        <v>9</v>
+      </c>
+      <c r="C794">
+        <v>8005332255</v>
+      </c>
+      <c r="D794" s="3">
+        <v>46111.490486111114</v>
+      </c>
+      <c r="E794" t="s">
+        <v>20</v>
+      </c>
+      <c r="F794" t="s">
+        <v>11</v>
+      </c>
+      <c r="G794" t="s">
+        <v>873</v>
+      </c>
+      <c r="H794" t="s">
+        <v>152</v>
+      </c>
+      <c r="I794" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="795" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A795">
+        <v>794</v>
+      </c>
+      <c r="B795" t="s">
+        <v>9</v>
+      </c>
+      <c r="C795">
+        <v>8005291352</v>
+      </c>
+      <c r="D795" s="3">
+        <v>46111.501643518517</v>
+      </c>
+      <c r="E795" t="s">
+        <v>48</v>
+      </c>
+      <c r="F795" t="s">
+        <v>11</v>
+      </c>
+      <c r="G795" t="s">
+        <v>874</v>
+      </c>
+      <c r="H795" t="s">
+        <v>13</v>
+      </c>
+      <c r="I795" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="796" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A796">
+        <v>795</v>
+      </c>
+      <c r="B796" t="s">
+        <v>9</v>
+      </c>
+      <c r="C796">
+        <v>8005335500</v>
+      </c>
+      <c r="D796" s="3">
+        <v>46111.515694444446</v>
+      </c>
+      <c r="E796" t="s">
+        <v>461</v>
+      </c>
+      <c r="F796" t="s">
+        <v>16</v>
+      </c>
+      <c r="G796" t="s">
+        <v>875</v>
+      </c>
+      <c r="H796" t="s">
+        <v>18</v>
+      </c>
+      <c r="I796" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="797" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A797">
+        <v>796</v>
+      </c>
+      <c r="B797" t="s">
+        <v>9</v>
+      </c>
+      <c r="C797">
+        <v>8005338698</v>
+      </c>
+      <c r="D797" s="3">
+        <v>46111.518703703703</v>
+      </c>
+      <c r="E797" t="s">
+        <v>48</v>
+      </c>
+      <c r="F797" t="s">
+        <v>16</v>
+      </c>
+      <c r="G797" t="s">
+        <v>876</v>
+      </c>
+      <c r="H797" t="s">
+        <v>152</v>
+      </c>
+      <c r="I797" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="798" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A798">
+        <v>797</v>
+      </c>
+      <c r="B798" t="s">
+        <v>9</v>
+      </c>
+      <c r="C798">
+        <v>8005322674</v>
+      </c>
+      <c r="D798" s="3">
+        <v>46111.522916666669</v>
+      </c>
+      <c r="E798" t="s">
+        <v>63</v>
+      </c>
+      <c r="F798" t="s">
+        <v>16</v>
+      </c>
+      <c r="G798" t="s">
+        <v>877</v>
+      </c>
+      <c r="H798" t="s">
+        <v>31</v>
+      </c>
+      <c r="I798" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="799" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A799">
+        <v>798</v>
+      </c>
+      <c r="B799" t="s">
+        <v>9</v>
+      </c>
+      <c r="C799">
+        <v>8005309955</v>
+      </c>
+      <c r="D799" s="3">
+        <v>46111.563425925924</v>
+      </c>
+      <c r="E799" t="s">
+        <v>15</v>
+      </c>
+      <c r="F799" t="s">
+        <v>11</v>
+      </c>
+      <c r="G799" t="s">
+        <v>878</v>
+      </c>
+      <c r="H799" t="s">
+        <v>34</v>
+      </c>
+      <c r="I799" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="800" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A800">
+        <v>799</v>
+      </c>
+      <c r="B800" t="s">
+        <v>9</v>
+      </c>
+      <c r="C800">
+        <v>8265</v>
+      </c>
+      <c r="D800" s="3">
+        <v>46111.610636574071</v>
+      </c>
+      <c r="E800" t="s">
+        <v>582</v>
+      </c>
+      <c r="F800" t="s">
+        <v>16</v>
+      </c>
+      <c r="G800" t="s">
+        <v>879</v>
+      </c>
+      <c r="H800" t="s">
+        <v>880</v>
+      </c>
+      <c r="I800" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="801" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A801">
+        <v>800</v>
+      </c>
+      <c r="B801" t="s">
+        <v>9</v>
+      </c>
+      <c r="C801">
+        <v>8005338018</v>
+      </c>
+      <c r="D801" s="3">
+        <v>46111.660266203704</v>
+      </c>
+      <c r="E801" t="s">
+        <v>20</v>
+      </c>
+      <c r="F801" t="s">
+        <v>11</v>
+      </c>
+      <c r="G801" t="s">
+        <v>881</v>
+      </c>
+      <c r="H801" t="s">
+        <v>13</v>
+      </c>
+      <c r="I801" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="802" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A802">
+        <v>801</v>
+      </c>
+      <c r="B802" t="s">
+        <v>9</v>
+      </c>
+      <c r="C802">
+        <v>8005336727</v>
+      </c>
+      <c r="D802" s="3">
+        <v>46112.471168981479</v>
+      </c>
+      <c r="E802" t="s">
+        <v>15</v>
+      </c>
+      <c r="F802" t="s">
+        <v>16</v>
+      </c>
+      <c r="G802" t="s">
+        <v>882</v>
+      </c>
+      <c r="H802" t="s">
+        <v>34</v>
+      </c>
+      <c r="I802" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="803" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A803">
+        <v>802</v>
+      </c>
+      <c r="B803" t="s">
+        <v>9</v>
+      </c>
+      <c r="C803">
+        <v>8005337138</v>
+      </c>
+      <c r="D803" s="3">
+        <v>46112.475416666668</v>
+      </c>
+      <c r="E803" t="s">
+        <v>36</v>
+      </c>
+      <c r="F803" t="s">
+        <v>16</v>
+      </c>
+      <c r="G803" t="s">
+        <v>883</v>
+      </c>
+      <c r="H803" t="s">
+        <v>18</v>
+      </c>
+      <c r="I803" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="804" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A804">
+        <v>803</v>
+      </c>
+      <c r="B804" t="s">
+        <v>9</v>
+      </c>
+      <c r="C804">
+        <v>8005302251</v>
+      </c>
+      <c r="D804" s="3">
+        <v>46112.559467592589</v>
+      </c>
+      <c r="E804" t="s">
+        <v>40</v>
+      </c>
+      <c r="F804" t="s">
+        <v>11</v>
+      </c>
+      <c r="G804" t="s">
+        <v>884</v>
+      </c>
+      <c r="H804" t="s">
+        <v>18</v>
+      </c>
+      <c r="I804" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="805" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A805">
+        <v>804</v>
+      </c>
+      <c r="B805" t="s">
+        <v>9</v>
+      </c>
+      <c r="C805">
+        <v>10593</v>
+      </c>
+      <c r="D805" s="3">
+        <v>46112.584629629629</v>
+      </c>
+      <c r="E805" t="s">
+        <v>695</v>
+      </c>
+      <c r="F805" t="s">
+        <v>11</v>
+      </c>
+      <c r="G805" t="s">
+        <v>885</v>
+      </c>
+      <c r="H805" t="s">
+        <v>34</v>
+      </c>
+      <c r="I805" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="806" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A806">
+        <v>805</v>
+      </c>
+      <c r="B806" t="s">
+        <v>9</v>
+      </c>
+      <c r="C806">
+        <v>8005325389</v>
+      </c>
+      <c r="D806" s="3">
+        <v>46112.586168981485</v>
+      </c>
+      <c r="E806" t="s">
+        <v>15</v>
+      </c>
+      <c r="F806" t="s">
+        <v>16</v>
+      </c>
+      <c r="G806" t="s">
+        <v>886</v>
+      </c>
+      <c r="H806" t="s">
+        <v>18</v>
+      </c>
+      <c r="I806" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="807" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A807">
+        <v>806</v>
+      </c>
+      <c r="B807" t="s">
+        <v>9</v>
+      </c>
+      <c r="C807">
+        <v>8005335610</v>
+      </c>
+      <c r="D807" s="3">
+        <v>46112.604872685188</v>
+      </c>
+      <c r="E807" t="s">
+        <v>66</v>
+      </c>
+      <c r="F807" t="s">
+        <v>11</v>
+      </c>
+      <c r="G807" t="s">
+        <v>887</v>
+      </c>
+      <c r="H807" t="s">
+        <v>34</v>
+      </c>
+      <c r="I807" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="808" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A808">
+        <v>807</v>
+      </c>
+      <c r="B808" t="s">
+        <v>9</v>
+      </c>
+      <c r="C808">
+        <v>8005340906</v>
+      </c>
+      <c r="D808" s="3">
+        <v>46112.647662037038</v>
+      </c>
+      <c r="E808" t="s">
+        <v>20</v>
+      </c>
+      <c r="F808" t="s">
+        <v>11</v>
+      </c>
+      <c r="G808" t="s">
+        <v>888</v>
+      </c>
+      <c r="H808" t="s">
+        <v>13</v>
+      </c>
+      <c r="I808" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="809" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A809">
+        <v>808</v>
+      </c>
+      <c r="B809" t="s">
+        <v>9</v>
+      </c>
+      <c r="C809">
+        <v>8005319027</v>
+      </c>
+      <c r="D809" s="3">
+        <v>46112.672569444447</v>
+      </c>
+      <c r="E809" t="s">
+        <v>52</v>
+      </c>
+      <c r="F809" t="s">
+        <v>16</v>
+      </c>
+      <c r="G809" t="s">
+        <v>889</v>
+      </c>
+      <c r="H809" t="s">
+        <v>31</v>
+      </c>
+      <c r="I809" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/04/2026 17:09:13,96
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{341405C3-8B94-4FF6-BB19-52D16E22337F}"/>
+  <xr:revisionPtr revIDLastSave="192" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C6448DE-3513-4DF0-80C8-792CBF9302B8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$783</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$809</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4857" uniqueCount="890">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4857" uniqueCount="888">
   <si>
     <t>ID</t>
   </si>
@@ -1926,9 +1926,6 @@
     <t>O aparelho instalado dia 27 e no dia 28 já não funciona mais</t>
   </si>
   <si>
-    <t>Qualidade do produto</t>
-  </si>
-  <si>
     <t>Foi muito bom no início e agora nos últimos anos a manutenção ficou um pouco a desejar. Não é feito mais a limpeza do filtro somente a troca de filtro. E a marcação que era feita de 6 em 6 meses também não é feita regularmente. Anteriormente era certinho sempre no período certo</t>
   </si>
   <si>
@@ -2770,9 +2767,6 @@
   </si>
   <si>
     <t>Consideramos o produto da troca inferior ao modelo que tínhamos anteriormente.</t>
-  </si>
-  <si>
-    <t>QUALIDADE DO PRODUTO</t>
   </si>
   <si>
     <t>Acho muito. Bom</t>
@@ -3382,7 +3376,7 @@
         <v>18</v>
       </c>
       <c r="I7" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3527,7 +3521,7 @@
         <v>18</v>
       </c>
       <c r="I12" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -3846,7 +3840,7 @@
         <v>18</v>
       </c>
       <c r="I23" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4165,7 +4159,7 @@
         <v>18</v>
       </c>
       <c r="I34" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4426,7 +4420,7 @@
         <v>18</v>
       </c>
       <c r="I43" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4803,7 +4797,7 @@
         <v>18</v>
       </c>
       <c r="I56" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -4890,7 +4884,7 @@
         <v>18</v>
       </c>
       <c r="I59" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5006,7 +5000,7 @@
         <v>18</v>
       </c>
       <c r="I63" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5151,7 +5145,7 @@
         <v>18</v>
       </c>
       <c r="I68" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5238,7 +5232,7 @@
         <v>18</v>
       </c>
       <c r="I71" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5644,7 +5638,7 @@
         <v>18</v>
       </c>
       <c r="I85" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -5702,7 +5696,7 @@
         <v>18</v>
       </c>
       <c r="I87" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -5731,7 +5725,7 @@
         <v>18</v>
       </c>
       <c r="I88" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -5760,7 +5754,7 @@
         <v>18</v>
       </c>
       <c r="I89" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6021,7 +6015,7 @@
         <v>18</v>
       </c>
       <c r="I98" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
@@ -6137,7 +6131,7 @@
         <v>18</v>
       </c>
       <c r="I102" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6311,7 +6305,7 @@
         <v>18</v>
       </c>
       <c r="I108" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6630,7 +6624,7 @@
         <v>18</v>
       </c>
       <c r="I119" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
@@ -6804,7 +6798,7 @@
         <v>18</v>
       </c>
       <c r="I125" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7094,7 +7088,7 @@
         <v>18</v>
       </c>
       <c r="I135" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7123,7 +7117,7 @@
         <v>18</v>
       </c>
       <c r="I136" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7210,7 +7204,7 @@
         <v>18</v>
       </c>
       <c r="I139" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7471,7 +7465,7 @@
         <v>18</v>
       </c>
       <c r="I148" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8341,7 +8335,7 @@
         <v>18</v>
       </c>
       <c r="I178" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8428,7 +8422,7 @@
         <v>18</v>
       </c>
       <c r="I181" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8457,7 +8451,7 @@
         <v>18</v>
       </c>
       <c r="I182" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8486,7 +8480,7 @@
         <v>18</v>
       </c>
       <c r="I183" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -8515,7 +8509,7 @@
         <v>18</v>
       </c>
       <c r="I184" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -8573,7 +8567,7 @@
         <v>18</v>
       </c>
       <c r="I186" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -8660,7 +8654,7 @@
         <v>18</v>
       </c>
       <c r="I189" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -8718,7 +8712,7 @@
         <v>18</v>
       </c>
       <c r="I191" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -8805,7 +8799,7 @@
         <v>18</v>
       </c>
       <c r="I194" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -8834,7 +8828,7 @@
         <v>18</v>
       </c>
       <c r="I195" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -8921,7 +8915,7 @@
         <v>18</v>
       </c>
       <c r="I198" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9037,7 +9031,7 @@
         <v>18</v>
       </c>
       <c r="I202" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9385,7 +9379,7 @@
         <v>18</v>
       </c>
       <c r="I214" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.25">
@@ -9617,7 +9611,7 @@
         <v>18</v>
       </c>
       <c r="I222" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -9646,7 +9640,7 @@
         <v>18</v>
       </c>
       <c r="I223" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -9791,7 +9785,7 @@
         <v>18</v>
       </c>
       <c r="I228" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -9878,7 +9872,7 @@
         <v>18</v>
       </c>
       <c r="I231" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -9994,7 +9988,7 @@
         <v>276</v>
       </c>
       <c r="I235" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10458,7 +10452,7 @@
         <v>18</v>
       </c>
       <c r="I251" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.25">
@@ -10516,7 +10510,7 @@
         <v>18</v>
       </c>
       <c r="I253" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.25">
@@ -10661,7 +10655,7 @@
         <v>18</v>
       </c>
       <c r="I258" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.25">
@@ -10777,7 +10771,7 @@
         <v>18</v>
       </c>
       <c r="I262" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="263" spans="1:9" x14ac:dyDescent="0.25">
@@ -10864,7 +10858,7 @@
         <v>18</v>
       </c>
       <c r="I265" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.25">
@@ -10922,7 +10916,7 @@
         <v>18</v>
       </c>
       <c r="I267" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="268" spans="1:9" x14ac:dyDescent="0.25">
@@ -11241,7 +11235,7 @@
         <v>18</v>
       </c>
       <c r="I278" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="279" spans="1:9" x14ac:dyDescent="0.25">
@@ -11473,7 +11467,7 @@
         <v>18</v>
       </c>
       <c r="I286" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="287" spans="1:9" x14ac:dyDescent="0.25">
@@ -11531,7 +11525,7 @@
         <v>18</v>
       </c>
       <c r="I288" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="289" spans="1:9" x14ac:dyDescent="0.25">
@@ -11705,7 +11699,7 @@
         <v>18</v>
       </c>
       <c r="I294" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.25">
@@ -11792,7 +11786,7 @@
         <v>18</v>
       </c>
       <c r="I297" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
@@ -11850,7 +11844,7 @@
         <v>18</v>
       </c>
       <c r="I299" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="300" spans="1:9" x14ac:dyDescent="0.25">
@@ -11908,7 +11902,7 @@
         <v>18</v>
       </c>
       <c r="I301" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.25">
@@ -11966,7 +11960,7 @@
         <v>18</v>
       </c>
       <c r="I303" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="304" spans="1:9" x14ac:dyDescent="0.25">
@@ -12082,7 +12076,7 @@
         <v>18</v>
       </c>
       <c r="I307" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="308" spans="1:9" x14ac:dyDescent="0.25">
@@ -12836,7 +12830,7 @@
         <v>18</v>
       </c>
       <c r="I333" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="334" spans="1:9" x14ac:dyDescent="0.25">
@@ -13416,7 +13410,7 @@
         <v>18</v>
       </c>
       <c r="I353" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="354" spans="1:9" x14ac:dyDescent="0.25">
@@ -13648,7 +13642,7 @@
         <v>18</v>
       </c>
       <c r="I361" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="362" spans="1:9" x14ac:dyDescent="0.25">
@@ -13938,7 +13932,7 @@
         <v>18</v>
       </c>
       <c r="I371" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="372" spans="1:9" x14ac:dyDescent="0.25">
@@ -14083,7 +14077,7 @@
         <v>18</v>
       </c>
       <c r="I376" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="377" spans="1:9" x14ac:dyDescent="0.25">
@@ -14721,7 +14715,7 @@
         <v>18</v>
       </c>
       <c r="I398" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="399" spans="1:9" x14ac:dyDescent="0.25">
@@ -14982,7 +14976,7 @@
         <v>18</v>
       </c>
       <c r="I407" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="408" spans="1:9" x14ac:dyDescent="0.25">
@@ -15011,7 +15005,7 @@
         <v>18</v>
       </c>
       <c r="I408" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="409" spans="1:9" x14ac:dyDescent="0.25">
@@ -15330,7 +15324,7 @@
         <v>18</v>
       </c>
       <c r="I419" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="420" spans="1:9" x14ac:dyDescent="0.25">
@@ -15359,7 +15353,7 @@
         <v>18</v>
       </c>
       <c r="I420" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="421" spans="1:9" x14ac:dyDescent="0.25">
@@ -15620,7 +15614,7 @@
         <v>18</v>
       </c>
       <c r="I429" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="430" spans="1:9" x14ac:dyDescent="0.25">
@@ -15997,7 +15991,7 @@
         <v>18</v>
       </c>
       <c r="I442" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="443" spans="1:9" x14ac:dyDescent="0.25">
@@ -16113,7 +16107,7 @@
         <v>18</v>
       </c>
       <c r="I446" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="447" spans="1:9" x14ac:dyDescent="0.25">
@@ -17099,7 +17093,7 @@
         <v>18</v>
       </c>
       <c r="I480" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="481" spans="1:9" x14ac:dyDescent="0.25">
@@ -17128,7 +17122,7 @@
         <v>18</v>
       </c>
       <c r="I481" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="482" spans="1:9" x14ac:dyDescent="0.25">
@@ -17360,7 +17354,7 @@
         <v>18</v>
       </c>
       <c r="I489" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="490" spans="1:9" x14ac:dyDescent="0.25">
@@ -17418,7 +17412,7 @@
         <v>18</v>
       </c>
       <c r="I491" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="492" spans="1:9" x14ac:dyDescent="0.25">
@@ -17476,7 +17470,7 @@
         <v>18</v>
       </c>
       <c r="I493" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="494" spans="1:9" x14ac:dyDescent="0.25">
@@ -17592,7 +17586,7 @@
         <v>18</v>
       </c>
       <c r="I497" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="498" spans="1:9" x14ac:dyDescent="0.25">
@@ -17737,7 +17731,7 @@
         <v>18</v>
       </c>
       <c r="I502" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="503" spans="1:9" x14ac:dyDescent="0.25">
@@ -17998,7 +17992,7 @@
         <v>18</v>
       </c>
       <c r="I511" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="512" spans="1:9" x14ac:dyDescent="0.25">
@@ -18172,7 +18166,7 @@
         <v>18</v>
       </c>
       <c r="I517" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="518" spans="1:9" x14ac:dyDescent="0.25">
@@ -18230,7 +18224,7 @@
         <v>18</v>
       </c>
       <c r="I519" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="520" spans="1:9" x14ac:dyDescent="0.25">
@@ -18433,7 +18427,7 @@
         <v>18</v>
       </c>
       <c r="I526" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="527" spans="1:9" x14ac:dyDescent="0.25">
@@ -18720,7 +18714,7 @@
         <v>605</v>
       </c>
       <c r="H536" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I536" t="s">
         <v>38</v>
@@ -18746,7 +18740,7 @@
         <v>11</v>
       </c>
       <c r="G537" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H537" t="s">
         <v>31</v>
@@ -18775,7 +18769,7 @@
         <v>16</v>
       </c>
       <c r="G538" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H538" t="s">
         <v>31</v>
@@ -18804,7 +18798,7 @@
         <v>11</v>
       </c>
       <c r="G539" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H539" t="s">
         <v>13</v>
@@ -18833,10 +18827,10 @@
         <v>16</v>
       </c>
       <c r="G540" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="H540" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I540" t="s">
         <v>98</v>
@@ -18862,7 +18856,7 @@
         <v>11</v>
       </c>
       <c r="G541" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="H541" t="s">
         <v>13</v>
@@ -18885,16 +18879,16 @@
         <v>46083.849236111113</v>
       </c>
       <c r="E542" t="s">
+        <v>611</v>
+      </c>
+      <c r="F542" t="s">
+        <v>16</v>
+      </c>
+      <c r="G542" t="s">
         <v>612</v>
       </c>
-      <c r="F542" t="s">
-        <v>16</v>
-      </c>
-      <c r="G542" t="s">
-        <v>613</v>
-      </c>
       <c r="H542" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I542" t="s">
         <v>65</v>
@@ -18920,7 +18914,7 @@
         <v>11</v>
       </c>
       <c r="G543" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="H543" t="s">
         <v>13</v>
@@ -18949,10 +18943,10 @@
         <v>16</v>
       </c>
       <c r="G544" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="H544" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I544" t="s">
         <v>38</v>
@@ -18978,7 +18972,7 @@
         <v>16</v>
       </c>
       <c r="G545" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="H545" t="s">
         <v>80</v>
@@ -19007,10 +19001,10 @@
         <v>16</v>
       </c>
       <c r="G546" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H546" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I546" t="s">
         <v>65</v>
@@ -19036,10 +19030,10 @@
         <v>16</v>
       </c>
       <c r="G547" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H547" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I547" t="s">
         <v>38</v>
@@ -19065,7 +19059,7 @@
         <v>11</v>
       </c>
       <c r="G548" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="H548" t="s">
         <v>13</v>
@@ -19094,7 +19088,7 @@
         <v>16</v>
       </c>
       <c r="G549" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="H549" t="s">
         <v>31</v>
@@ -19123,10 +19117,10 @@
         <v>16</v>
       </c>
       <c r="G550" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="H550" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I550" t="s">
         <v>38</v>
@@ -19152,7 +19146,7 @@
         <v>11</v>
       </c>
       <c r="G551" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="H551" t="s">
         <v>18</v>
@@ -19175,13 +19169,13 @@
         <v>46084.528923611113</v>
       </c>
       <c r="E552" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F552" t="s">
         <v>16</v>
       </c>
       <c r="G552" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H552" t="s">
         <v>31</v>
@@ -19210,7 +19204,7 @@
         <v>11</v>
       </c>
       <c r="G553" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="H553" t="s">
         <v>13</v>
@@ -19239,10 +19233,10 @@
         <v>11</v>
       </c>
       <c r="G554" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="H554" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I554" t="s">
         <v>38</v>
@@ -19268,7 +19262,7 @@
         <v>16</v>
       </c>
       <c r="G555" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H555" t="s">
         <v>18</v>
@@ -19297,13 +19291,13 @@
         <v>16</v>
       </c>
       <c r="G556" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="H556" t="s">
         <v>18</v>
       </c>
       <c r="I556" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.25">
@@ -19326,10 +19320,10 @@
         <v>11</v>
       </c>
       <c r="G557" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="H557" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I557" t="s">
         <v>38</v>
@@ -19355,13 +19349,13 @@
         <v>16</v>
       </c>
       <c r="G558" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H558" t="s">
         <v>18</v>
       </c>
       <c r="I558" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="559" spans="1:9" x14ac:dyDescent="0.25">
@@ -19384,7 +19378,7 @@
         <v>16</v>
       </c>
       <c r="G559" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="H559" t="s">
         <v>18</v>
@@ -19413,7 +19407,7 @@
         <v>16</v>
       </c>
       <c r="G560" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H560" t="s">
         <v>31</v>
@@ -19442,10 +19436,10 @@
         <v>16</v>
       </c>
       <c r="G561" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H561" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I561" t="s">
         <v>38</v>
@@ -19471,7 +19465,7 @@
         <v>16</v>
       </c>
       <c r="G562" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H562" t="s">
         <v>18</v>
@@ -19500,13 +19494,13 @@
         <v>11</v>
       </c>
       <c r="G563" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H563" t="s">
         <v>18</v>
       </c>
       <c r="I563" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="564" spans="1:9" x14ac:dyDescent="0.25">
@@ -19529,7 +19523,7 @@
         <v>16</v>
       </c>
       <c r="G564" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H564" t="s">
         <v>18</v>
@@ -19558,7 +19552,7 @@
         <v>16</v>
       </c>
       <c r="G565" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H565" t="s">
         <v>18</v>
@@ -19587,7 +19581,7 @@
         <v>16</v>
       </c>
       <c r="G566" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="H566" t="s">
         <v>13</v>
@@ -19616,7 +19610,7 @@
         <v>11</v>
       </c>
       <c r="G567" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H567" t="s">
         <v>80</v>
@@ -19645,10 +19639,10 @@
         <v>16</v>
       </c>
       <c r="G568" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="H568" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I568" t="s">
         <v>38</v>
@@ -19674,7 +19668,7 @@
         <v>11</v>
       </c>
       <c r="G569" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="H569" t="s">
         <v>13</v>
@@ -19703,7 +19697,7 @@
         <v>16</v>
       </c>
       <c r="G570" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="H570" t="s">
         <v>18</v>
@@ -19732,7 +19726,7 @@
         <v>16</v>
       </c>
       <c r="G571" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H571" t="s">
         <v>18</v>
@@ -19761,7 +19755,7 @@
         <v>11</v>
       </c>
       <c r="G572" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="H572" t="s">
         <v>13</v>
@@ -19790,7 +19784,7 @@
         <v>11</v>
       </c>
       <c r="G573" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="H573" t="s">
         <v>18</v>
@@ -19819,7 +19813,7 @@
         <v>16</v>
       </c>
       <c r="G574" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="H574" t="s">
         <v>80</v>
@@ -19848,13 +19842,13 @@
         <v>16</v>
       </c>
       <c r="G575" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="H575" t="s">
         <v>18</v>
       </c>
       <c r="I575" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="576" spans="1:9" x14ac:dyDescent="0.25">
@@ -19877,10 +19871,10 @@
         <v>16</v>
       </c>
       <c r="G576" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="H576" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I576" t="s">
         <v>38</v>
@@ -19906,10 +19900,10 @@
         <v>11</v>
       </c>
       <c r="G577" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="H577" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I577" t="s">
         <v>85</v>
@@ -19935,7 +19929,7 @@
         <v>16</v>
       </c>
       <c r="G578" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="H578" t="s">
         <v>31</v>
@@ -19964,10 +19958,10 @@
         <v>16</v>
       </c>
       <c r="G579" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H579" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I579" t="s">
         <v>38</v>
@@ -19993,7 +19987,7 @@
         <v>16</v>
       </c>
       <c r="G580" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H580" t="s">
         <v>152</v>
@@ -20022,7 +20016,7 @@
         <v>11</v>
       </c>
       <c r="G581" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="H581" t="s">
         <v>13</v>
@@ -20051,7 +20045,7 @@
         <v>11</v>
       </c>
       <c r="G582" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H582" t="s">
         <v>13</v>
@@ -20080,7 +20074,7 @@
         <v>16</v>
       </c>
       <c r="G583" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H583" t="s">
         <v>13</v>
@@ -20109,10 +20103,10 @@
         <v>16</v>
       </c>
       <c r="G584" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H584" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I584" t="s">
         <v>35</v>
@@ -20138,7 +20132,7 @@
         <v>16</v>
       </c>
       <c r="G585" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H585" t="s">
         <v>31</v>
@@ -20167,7 +20161,7 @@
         <v>11</v>
       </c>
       <c r="G586" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="H586" t="s">
         <v>152</v>
@@ -20196,7 +20190,7 @@
         <v>11</v>
       </c>
       <c r="G587" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="H587" t="s">
         <v>13</v>
@@ -20225,7 +20219,7 @@
         <v>11</v>
       </c>
       <c r="G588" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H588" t="s">
         <v>13</v>
@@ -20254,10 +20248,10 @@
         <v>16</v>
       </c>
       <c r="G589" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H589" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I589" t="s">
         <v>38</v>
@@ -20283,7 +20277,7 @@
         <v>16</v>
       </c>
       <c r="G590" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H590" t="s">
         <v>18</v>
@@ -20312,7 +20306,7 @@
         <v>16</v>
       </c>
       <c r="G591" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H591" t="s">
         <v>31</v>
@@ -20335,13 +20329,13 @@
         <v>46087.417326388888</v>
       </c>
       <c r="E592" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F592" t="s">
         <v>16</v>
       </c>
       <c r="G592" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H592" t="s">
         <v>80</v>
@@ -20370,13 +20364,13 @@
         <v>16</v>
       </c>
       <c r="G593" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="H593" t="s">
         <v>18</v>
       </c>
       <c r="I593" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="594" spans="1:9" x14ac:dyDescent="0.25">
@@ -20399,7 +20393,7 @@
         <v>16</v>
       </c>
       <c r="G594" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="H594" t="s">
         <v>18</v>
@@ -20428,7 +20422,7 @@
         <v>16</v>
       </c>
       <c r="G595" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H595" t="s">
         <v>18</v>
@@ -20457,10 +20451,10 @@
         <v>16</v>
       </c>
       <c r="G596" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H596" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I596" t="s">
         <v>220</v>
@@ -20486,7 +20480,7 @@
         <v>11</v>
       </c>
       <c r="G597" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H597" t="s">
         <v>31</v>
@@ -20515,7 +20509,7 @@
         <v>16</v>
       </c>
       <c r="G598" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H598" t="s">
         <v>18</v>
@@ -20544,7 +20538,7 @@
         <v>16</v>
       </c>
       <c r="G599" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H599" t="s">
         <v>18</v>
@@ -20573,7 +20567,7 @@
         <v>16</v>
       </c>
       <c r="G600" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H600" t="s">
         <v>18</v>
@@ -20602,7 +20596,7 @@
         <v>16</v>
       </c>
       <c r="G601" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H601" t="s">
         <v>18</v>
@@ -20631,7 +20625,7 @@
         <v>11</v>
       </c>
       <c r="G602" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H602" t="s">
         <v>18</v>
@@ -20660,10 +20654,10 @@
         <v>11</v>
       </c>
       <c r="G603" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H603" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I603" t="s">
         <v>237</v>
@@ -20689,10 +20683,10 @@
         <v>16</v>
       </c>
       <c r="G604" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H604" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I604" t="s">
         <v>237</v>
@@ -20718,7 +20712,7 @@
         <v>16</v>
       </c>
       <c r="G605" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H605" t="s">
         <v>80</v>
@@ -20741,19 +20735,19 @@
         <v>46090.435601851852</v>
       </c>
       <c r="E606" t="s">
+        <v>676</v>
+      </c>
+      <c r="F606" t="s">
+        <v>16</v>
+      </c>
+      <c r="G606" t="s">
         <v>677</v>
       </c>
-      <c r="F606" t="s">
-        <v>16</v>
-      </c>
-      <c r="G606" t="s">
-        <v>678</v>
-      </c>
       <c r="H606" t="s">
         <v>18</v>
       </c>
       <c r="I606" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="607" spans="1:9" x14ac:dyDescent="0.25">
@@ -20776,13 +20770,13 @@
         <v>16</v>
       </c>
       <c r="G607" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H607" t="s">
         <v>18</v>
       </c>
       <c r="I607" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="608" spans="1:9" x14ac:dyDescent="0.25">
@@ -20799,13 +20793,13 @@
         <v>46090.448009259257</v>
       </c>
       <c r="E608" t="s">
+        <v>679</v>
+      </c>
+      <c r="F608" t="s">
+        <v>16</v>
+      </c>
+      <c r="G608" t="s">
         <v>680</v>
-      </c>
-      <c r="F608" t="s">
-        <v>16</v>
-      </c>
-      <c r="G608" t="s">
-        <v>681</v>
       </c>
       <c r="H608" t="s">
         <v>18</v>
@@ -20834,10 +20828,10 @@
         <v>11</v>
       </c>
       <c r="G609" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H609" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I609" t="s">
         <v>35</v>
@@ -20892,7 +20886,7 @@
         <v>16</v>
       </c>
       <c r="G611" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H611" t="s">
         <v>18</v>
@@ -20921,7 +20915,7 @@
         <v>16</v>
       </c>
       <c r="G612" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H612" t="s">
         <v>18</v>
@@ -20944,13 +20938,13 @@
         <v>46090.501446759263</v>
       </c>
       <c r="E613" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F613" t="s">
         <v>16</v>
       </c>
       <c r="G613" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H613" t="s">
         <v>13</v>
@@ -20979,7 +20973,7 @@
         <v>16</v>
       </c>
       <c r="G614" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H614" t="s">
         <v>18</v>
@@ -21008,7 +21002,7 @@
         <v>11</v>
       </c>
       <c r="G615" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H615" t="s">
         <v>13</v>
@@ -21037,7 +21031,7 @@
         <v>16</v>
       </c>
       <c r="G616" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H616" t="s">
         <v>18</v>
@@ -21066,7 +21060,7 @@
         <v>16</v>
       </c>
       <c r="G617" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H617" t="s">
         <v>13</v>
@@ -21095,7 +21089,7 @@
         <v>11</v>
       </c>
       <c r="G618" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H618" t="s">
         <v>18</v>
@@ -21124,7 +21118,7 @@
         <v>11</v>
       </c>
       <c r="G619" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H619" t="s">
         <v>13</v>
@@ -21153,10 +21147,10 @@
         <v>16</v>
       </c>
       <c r="G620" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H620" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I620" t="s">
         <v>35</v>
@@ -21182,7 +21176,7 @@
         <v>11</v>
       </c>
       <c r="G621" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H621" t="s">
         <v>152</v>
@@ -21211,7 +21205,7 @@
         <v>16</v>
       </c>
       <c r="G622" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H622" t="s">
         <v>18</v>
@@ -21234,13 +21228,13 @@
         <v>46091.450520833343</v>
       </c>
       <c r="E623" t="s">
+        <v>694</v>
+      </c>
+      <c r="F623" t="s">
+        <v>11</v>
+      </c>
+      <c r="G623" t="s">
         <v>695</v>
-      </c>
-      <c r="F623" t="s">
-        <v>11</v>
-      </c>
-      <c r="G623" t="s">
-        <v>696</v>
       </c>
       <c r="H623" t="s">
         <v>80</v>
@@ -21263,16 +21257,16 @@
         <v>46091.474988425929</v>
       </c>
       <c r="E624" t="s">
+        <v>696</v>
+      </c>
+      <c r="F624" t="s">
+        <v>16</v>
+      </c>
+      <c r="G624" t="s">
         <v>697</v>
       </c>
-      <c r="F624" t="s">
-        <v>16</v>
-      </c>
-      <c r="G624" t="s">
-        <v>698</v>
-      </c>
       <c r="H624" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I624" t="s">
         <v>98</v>
@@ -21298,10 +21292,10 @@
         <v>16</v>
       </c>
       <c r="G625" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H625" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I625" t="s">
         <v>98</v>
@@ -21327,10 +21321,10 @@
         <v>16</v>
       </c>
       <c r="G626" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H626" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I626" t="s">
         <v>38</v>
@@ -21356,7 +21350,7 @@
         <v>11</v>
       </c>
       <c r="G627" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H627" t="s">
         <v>13</v>
@@ -21385,7 +21379,7 @@
         <v>11</v>
       </c>
       <c r="G628" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H628" t="s">
         <v>13</v>
@@ -21414,10 +21408,10 @@
         <v>11</v>
       </c>
       <c r="G629" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H629" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I629" t="s">
         <v>38</v>
@@ -21443,7 +21437,7 @@
         <v>11</v>
       </c>
       <c r="G630" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H630" t="s">
         <v>13</v>
@@ -21472,7 +21466,7 @@
         <v>11</v>
       </c>
       <c r="G631" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H631" t="s">
         <v>31</v>
@@ -21501,7 +21495,7 @@
         <v>16</v>
       </c>
       <c r="G632" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H632" t="s">
         <v>18</v>
@@ -21530,13 +21524,13 @@
         <v>11</v>
       </c>
       <c r="G633" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H633" t="s">
         <v>18</v>
       </c>
       <c r="I633" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="634" spans="1:9" x14ac:dyDescent="0.25">
@@ -21553,13 +21547,13 @@
         <v>46091.610069444447</v>
       </c>
       <c r="E634" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F634" t="s">
         <v>16</v>
       </c>
       <c r="G634" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H634" t="s">
         <v>31</v>
@@ -21588,13 +21582,13 @@
         <v>16</v>
       </c>
       <c r="G635" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H635" t="s">
         <v>18</v>
       </c>
       <c r="I635" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="636" spans="1:9" x14ac:dyDescent="0.25">
@@ -21611,13 +21605,13 @@
         <v>46091.738668981481</v>
       </c>
       <c r="E636" t="s">
+        <v>709</v>
+      </c>
+      <c r="F636" t="s">
+        <v>16</v>
+      </c>
+      <c r="G636" t="s">
         <v>710</v>
-      </c>
-      <c r="F636" t="s">
-        <v>16</v>
-      </c>
-      <c r="G636" t="s">
-        <v>711</v>
       </c>
       <c r="H636" t="s">
         <v>31</v>
@@ -21640,13 +21634,13 @@
         <v>46091.75209490741</v>
       </c>
       <c r="E637" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F637" t="s">
         <v>11</v>
       </c>
       <c r="G637" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="H637" t="s">
         <v>13</v>
@@ -21669,13 +21663,13 @@
         <v>46092.369247685187</v>
       </c>
       <c r="E638" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F638" t="s">
         <v>16</v>
       </c>
       <c r="G638" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="H638" t="s">
         <v>13</v>
@@ -21698,13 +21692,13 @@
         <v>46092.406168981477</v>
       </c>
       <c r="E639" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F639" t="s">
         <v>16</v>
       </c>
       <c r="G639" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="H639" t="s">
         <v>31</v>
@@ -21733,7 +21727,7 @@
         <v>11</v>
       </c>
       <c r="G640" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="H640" t="s">
         <v>31</v>
@@ -21756,13 +21750,13 @@
         <v>46092.501481481479</v>
       </c>
       <c r="E641" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F641" t="s">
         <v>16</v>
       </c>
       <c r="G641" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="H641" t="s">
         <v>152</v>
@@ -21791,7 +21785,7 @@
         <v>16</v>
       </c>
       <c r="G642" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="H642" t="s">
         <v>80</v>
@@ -21814,13 +21808,13 @@
         <v>46092.664965277778</v>
       </c>
       <c r="E643" t="s">
+        <v>717</v>
+      </c>
+      <c r="F643" t="s">
+        <v>16</v>
+      </c>
+      <c r="G643" t="s">
         <v>718</v>
-      </c>
-      <c r="F643" t="s">
-        <v>16</v>
-      </c>
-      <c r="G643" t="s">
-        <v>719</v>
       </c>
       <c r="H643" t="s">
         <v>152</v>
@@ -21843,19 +21837,19 @@
         <v>46093.390613425923</v>
       </c>
       <c r="E644" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F644" t="s">
         <v>16</v>
       </c>
       <c r="G644" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="H644" t="s">
         <v>18</v>
       </c>
       <c r="I644" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="645" spans="1:9" x14ac:dyDescent="0.25">
@@ -21878,10 +21872,10 @@
         <v>11</v>
       </c>
       <c r="G645" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H645" t="s">
-        <v>606</v>
+        <v>34</v>
       </c>
       <c r="I645" t="s">
         <v>38</v>
@@ -21907,7 +21901,7 @@
         <v>11</v>
       </c>
       <c r="G646" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="H646" t="s">
         <v>18</v>
@@ -21936,7 +21930,7 @@
         <v>11</v>
       </c>
       <c r="G647" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H647" t="s">
         <v>13</v>
@@ -21965,7 +21959,7 @@
         <v>11</v>
       </c>
       <c r="G648" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="H648" t="s">
         <v>13</v>
@@ -21994,7 +21988,7 @@
         <v>11</v>
       </c>
       <c r="G649" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="H649" t="s">
         <v>13</v>
@@ -22023,7 +22017,7 @@
         <v>16</v>
       </c>
       <c r="G650" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="H650" t="s">
         <v>18</v>
@@ -22052,7 +22046,7 @@
         <v>16</v>
       </c>
       <c r="G651" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H651" t="s">
         <v>18</v>
@@ -22081,7 +22075,7 @@
         <v>11</v>
       </c>
       <c r="G652" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="H652" t="s">
         <v>18</v>
@@ -22110,7 +22104,7 @@
         <v>16</v>
       </c>
       <c r="G653" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H653" t="s">
         <v>18</v>
@@ -22139,7 +22133,7 @@
         <v>11</v>
       </c>
       <c r="G654" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H654" t="s">
         <v>13</v>
@@ -22162,13 +22156,13 @@
         <v>46093.549525462957</v>
       </c>
       <c r="E655" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F655" t="s">
         <v>11</v>
       </c>
       <c r="G655" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="H655" t="s">
         <v>31</v>
@@ -22197,7 +22191,7 @@
         <v>16</v>
       </c>
       <c r="G656" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H656" t="s">
         <v>18</v>
@@ -22226,7 +22220,7 @@
         <v>16</v>
       </c>
       <c r="G657" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H657" t="s">
         <v>152</v>
@@ -22255,7 +22249,7 @@
         <v>11</v>
       </c>
       <c r="G658" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H658" t="s">
         <v>18</v>
@@ -22278,13 +22272,13 @@
         <v>46094.476805555554</v>
       </c>
       <c r="E659" t="s">
+        <v>734</v>
+      </c>
+      <c r="F659" t="s">
+        <v>16</v>
+      </c>
+      <c r="G659" t="s">
         <v>735</v>
-      </c>
-      <c r="F659" t="s">
-        <v>16</v>
-      </c>
-      <c r="G659" t="s">
-        <v>736</v>
       </c>
       <c r="H659" t="s">
         <v>31</v>
@@ -22313,7 +22307,7 @@
         <v>11</v>
       </c>
       <c r="G660" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H660" t="s">
         <v>13</v>
@@ -22342,7 +22336,7 @@
         <v>11</v>
       </c>
       <c r="G661" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H661" t="s">
         <v>18</v>
@@ -22371,7 +22365,7 @@
         <v>11</v>
       </c>
       <c r="G662" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H662" t="s">
         <v>13</v>
@@ -22400,7 +22394,7 @@
         <v>11</v>
       </c>
       <c r="G663" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="H663" t="s">
         <v>31</v>
@@ -22429,7 +22423,7 @@
         <v>16</v>
       </c>
       <c r="G664" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H664" t="s">
         <v>13</v>
@@ -22458,7 +22452,7 @@
         <v>11</v>
       </c>
       <c r="G665" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="H665" t="s">
         <v>13</v>
@@ -22481,13 +22475,13 @@
         <v>46094.639421296299</v>
       </c>
       <c r="E666" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F666" t="s">
         <v>11</v>
       </c>
       <c r="G666" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="H666" t="s">
         <v>13</v>
@@ -22516,7 +22510,7 @@
         <v>11</v>
       </c>
       <c r="G667" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="H667" t="s">
         <v>80</v>
@@ -22545,7 +22539,7 @@
         <v>16</v>
       </c>
       <c r="G668" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H668" t="s">
         <v>18</v>
@@ -22574,7 +22568,7 @@
         <v>11</v>
       </c>
       <c r="G669" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="H669" t="s">
         <v>13</v>
@@ -22597,13 +22591,13 @@
         <v>46095.971944444442</v>
       </c>
       <c r="E670" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F670" t="s">
         <v>11</v>
       </c>
       <c r="G670" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="H670" t="s">
         <v>18</v>
@@ -22626,13 +22620,13 @@
         <v>46096.352141203701</v>
       </c>
       <c r="E671" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F671" t="s">
         <v>16</v>
       </c>
       <c r="G671" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="H671" t="s">
         <v>31</v>
@@ -22661,7 +22655,7 @@
         <v>16</v>
       </c>
       <c r="G672" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="H672" t="s">
         <v>152</v>
@@ -22690,7 +22684,7 @@
         <v>11</v>
       </c>
       <c r="G673" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="H673" t="s">
         <v>18</v>
@@ -22719,7 +22713,7 @@
         <v>16</v>
       </c>
       <c r="G674" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="H674" t="s">
         <v>18</v>
@@ -22748,7 +22742,7 @@
         <v>16</v>
       </c>
       <c r="G675" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H675" t="s">
         <v>18</v>
@@ -22777,7 +22771,7 @@
         <v>16</v>
       </c>
       <c r="G676" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H676" t="s">
         <v>18</v>
@@ -22806,7 +22800,7 @@
         <v>16</v>
       </c>
       <c r="G677" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="H677" t="s">
         <v>34</v>
@@ -22835,7 +22829,7 @@
         <v>11</v>
       </c>
       <c r="G678" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="H678" t="s">
         <v>80</v>
@@ -22864,7 +22858,7 @@
         <v>11</v>
       </c>
       <c r="G679" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="H679" t="s">
         <v>80</v>
@@ -22893,7 +22887,7 @@
         <v>16</v>
       </c>
       <c r="G680" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="H680" t="s">
         <v>152</v>
@@ -22922,7 +22916,7 @@
         <v>11</v>
       </c>
       <c r="G681" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="H681" t="s">
         <v>18</v>
@@ -22951,7 +22945,7 @@
         <v>16</v>
       </c>
       <c r="G682" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="H682" t="s">
         <v>18</v>
@@ -22974,13 +22968,13 @@
         <v>46097.565729166665</v>
       </c>
       <c r="E683" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F683" t="s">
         <v>16</v>
       </c>
       <c r="G683" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="H683" t="s">
         <v>18</v>
@@ -23009,7 +23003,7 @@
         <v>16</v>
       </c>
       <c r="G684" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="H684" t="s">
         <v>18</v>
@@ -23032,13 +23026,13 @@
         <v>46097.624849537038</v>
       </c>
       <c r="E685" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F685" t="s">
         <v>16</v>
       </c>
       <c r="G685" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="H685" t="s">
         <v>34</v>
@@ -23067,7 +23061,7 @@
         <v>16</v>
       </c>
       <c r="G686" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="H686" t="s">
         <v>34</v>
@@ -23096,7 +23090,7 @@
         <v>16</v>
       </c>
       <c r="G687" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="H687" t="s">
         <v>18</v>
@@ -23125,7 +23119,7 @@
         <v>11</v>
       </c>
       <c r="G688" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="H688" t="s">
         <v>34</v>
@@ -23148,19 +23142,19 @@
         <v>46098.390983796293</v>
       </c>
       <c r="E689" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F689" t="s">
         <v>16</v>
       </c>
       <c r="G689" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="H689" t="s">
         <v>18</v>
       </c>
       <c r="I689" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="690" spans="1:9" x14ac:dyDescent="0.25">
@@ -23183,7 +23177,7 @@
         <v>11</v>
       </c>
       <c r="G690" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="H690" t="s">
         <v>34</v>
@@ -23212,7 +23206,7 @@
         <v>16</v>
       </c>
       <c r="G691" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="H691" t="s">
         <v>18</v>
@@ -23241,7 +23235,7 @@
         <v>16</v>
       </c>
       <c r="G692" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="H692" t="s">
         <v>34</v>
@@ -23270,7 +23264,7 @@
         <v>11</v>
       </c>
       <c r="G693" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="H693" t="s">
         <v>13</v>
@@ -23299,7 +23293,7 @@
         <v>16</v>
       </c>
       <c r="G694" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H694" t="s">
         <v>18</v>
@@ -23328,13 +23322,13 @@
         <v>16</v>
       </c>
       <c r="G695" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="H695" t="s">
         <v>18</v>
       </c>
       <c r="I695" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="696" spans="1:9" x14ac:dyDescent="0.25">
@@ -23357,7 +23351,7 @@
         <v>16</v>
       </c>
       <c r="G696" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="H696" t="s">
         <v>34</v>
@@ -23386,7 +23380,7 @@
         <v>16</v>
       </c>
       <c r="G697" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="H697" t="s">
         <v>18</v>
@@ -23415,7 +23409,7 @@
         <v>11</v>
       </c>
       <c r="G698" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="H698" t="s">
         <v>13</v>
@@ -23438,13 +23432,13 @@
         <v>46098.520150462966</v>
       </c>
       <c r="E699" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F699" t="s">
         <v>11</v>
       </c>
       <c r="G699" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="H699" t="s">
         <v>18</v>
@@ -23473,7 +23467,7 @@
         <v>16</v>
       </c>
       <c r="G700" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="H700" t="s">
         <v>18</v>
@@ -23496,13 +23490,13 @@
         <v>46098.643784722219</v>
       </c>
       <c r="E701" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F701" t="s">
         <v>11</v>
       </c>
       <c r="G701" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="H701" t="s">
         <v>13</v>
@@ -23531,7 +23525,7 @@
         <v>16</v>
       </c>
       <c r="G702" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="H702" t="s">
         <v>80</v>
@@ -23554,13 +23548,13 @@
         <v>46098.731585648151</v>
       </c>
       <c r="E703" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F703" t="s">
         <v>16</v>
       </c>
       <c r="G703" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="H703" t="s">
         <v>34</v>
@@ -23589,7 +23583,7 @@
         <v>11</v>
       </c>
       <c r="G704" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="H704" t="s">
         <v>13</v>
@@ -23612,13 +23606,13 @@
         <v>46099.405185185184</v>
       </c>
       <c r="E705" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F705" t="s">
         <v>11</v>
       </c>
       <c r="G705" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="H705" t="s">
         <v>13</v>
@@ -23647,7 +23641,7 @@
         <v>11</v>
       </c>
       <c r="G706" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="H706" t="s">
         <v>13</v>
@@ -23676,7 +23670,7 @@
         <v>16</v>
       </c>
       <c r="G707" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H707" t="s">
         <v>34</v>
@@ -23705,7 +23699,7 @@
         <v>16</v>
       </c>
       <c r="G708" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="H708" t="s">
         <v>18</v>
@@ -23734,7 +23728,7 @@
         <v>16</v>
       </c>
       <c r="G709" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H709" t="s">
         <v>18</v>
@@ -23757,13 +23751,13 @@
         <v>46099.509108796294</v>
       </c>
       <c r="E710" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F710" t="s">
         <v>11</v>
       </c>
       <c r="G710" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="H710" t="s">
         <v>13</v>
@@ -23792,13 +23786,13 @@
         <v>11</v>
       </c>
       <c r="G711" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="H711" t="s">
         <v>18</v>
       </c>
       <c r="I711" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="712" spans="1:9" x14ac:dyDescent="0.25">
@@ -23821,7 +23815,7 @@
         <v>11</v>
       </c>
       <c r="G712" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="H712" t="s">
         <v>13</v>
@@ -23850,7 +23844,7 @@
         <v>16</v>
       </c>
       <c r="G713" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="H713" t="s">
         <v>13</v>
@@ -23873,13 +23867,13 @@
         <v>46100.433576388888</v>
       </c>
       <c r="E714" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F714" t="s">
         <v>16</v>
       </c>
       <c r="G714" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="H714" t="s">
         <v>152</v>
@@ -23908,13 +23902,13 @@
         <v>16</v>
       </c>
       <c r="G715" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="H715" t="s">
         <v>18</v>
       </c>
       <c r="I715" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="716" spans="1:9" x14ac:dyDescent="0.25">
@@ -23937,7 +23931,7 @@
         <v>16</v>
       </c>
       <c r="G716" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="H716" t="s">
         <v>18</v>
@@ -23966,7 +23960,7 @@
         <v>11</v>
       </c>
       <c r="G717" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H717" t="s">
         <v>31</v>
@@ -23995,7 +23989,7 @@
         <v>16</v>
       </c>
       <c r="G718" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H718" t="s">
         <v>31</v>
@@ -24024,7 +24018,7 @@
         <v>11</v>
       </c>
       <c r="G719" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="H719" t="s">
         <v>13</v>
@@ -24053,7 +24047,7 @@
         <v>16</v>
       </c>
       <c r="G720" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="H720" t="s">
         <v>18</v>
@@ -24082,7 +24076,7 @@
         <v>11</v>
       </c>
       <c r="G721" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="H721" t="s">
         <v>34</v>
@@ -24105,13 +24099,13 @@
         <v>46100.5077662037</v>
       </c>
       <c r="E722" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F722" t="s">
         <v>16</v>
       </c>
       <c r="G722" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="H722" t="s">
         <v>152</v>
@@ -24134,13 +24128,13 @@
         <v>46100.545555555553</v>
       </c>
       <c r="E723" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F723" t="s">
         <v>16</v>
       </c>
       <c r="G723" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="H723" t="s">
         <v>18</v>
@@ -24163,13 +24157,13 @@
         <v>46100.554837962962</v>
       </c>
       <c r="E724" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F724" t="s">
         <v>11</v>
       </c>
       <c r="G724" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="H724" t="s">
         <v>18</v>
@@ -24198,7 +24192,7 @@
         <v>11</v>
       </c>
       <c r="G725" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="H725" t="s">
         <v>18</v>
@@ -24227,7 +24221,7 @@
         <v>16</v>
       </c>
       <c r="G726" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="H726" t="s">
         <v>80</v>
@@ -24256,7 +24250,7 @@
         <v>16</v>
       </c>
       <c r="G727" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H727" t="s">
         <v>31</v>
@@ -24285,7 +24279,7 @@
         <v>16</v>
       </c>
       <c r="G728" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="H728" t="s">
         <v>31</v>
@@ -24308,13 +24302,13 @@
         <v>46101.459456018521</v>
       </c>
       <c r="E729" t="s">
+        <v>806</v>
+      </c>
+      <c r="F729" t="s">
+        <v>16</v>
+      </c>
+      <c r="G729" t="s">
         <v>807</v>
-      </c>
-      <c r="F729" t="s">
-        <v>16</v>
-      </c>
-      <c r="G729" t="s">
-        <v>808</v>
       </c>
       <c r="H729" t="s">
         <v>31</v>
@@ -24343,7 +24337,7 @@
         <v>11</v>
       </c>
       <c r="G730" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="H730" t="s">
         <v>80</v>
@@ -24366,13 +24360,13 @@
         <v>46101.497627314813</v>
       </c>
       <c r="E731" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F731" t="s">
         <v>11</v>
       </c>
       <c r="G731" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="H731" t="s">
         <v>13</v>
@@ -24401,7 +24395,7 @@
         <v>16</v>
       </c>
       <c r="G732" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H732" t="s">
         <v>18</v>
@@ -24424,13 +24418,13 @@
         <v>46101.506539351853</v>
       </c>
       <c r="E733" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="F733" t="s">
         <v>16</v>
       </c>
       <c r="G733" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="H733" t="s">
         <v>13</v>
@@ -24459,7 +24453,7 @@
         <v>16</v>
       </c>
       <c r="G734" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="H734" t="s">
         <v>152</v>
@@ -24482,13 +24476,13 @@
         <v>46101.558171296296</v>
       </c>
       <c r="E735" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F735" t="s">
         <v>16</v>
       </c>
       <c r="G735" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="H735" t="s">
         <v>31</v>
@@ -24517,7 +24511,7 @@
         <v>11</v>
       </c>
       <c r="G736" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="H736" t="s">
         <v>31</v>
@@ -24546,7 +24540,7 @@
         <v>11</v>
       </c>
       <c r="G737" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="H737" t="s">
         <v>13</v>
@@ -24569,13 +24563,13 @@
         <v>46101.652129629627</v>
       </c>
       <c r="E738" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F738" t="s">
         <v>11</v>
       </c>
       <c r="G738" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="H738" t="s">
         <v>80</v>
@@ -24604,7 +24598,7 @@
         <v>11</v>
       </c>
       <c r="G739" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="H739" t="s">
         <v>13</v>
@@ -24627,13 +24621,13 @@
         <v>46102.621527777781</v>
       </c>
       <c r="E740" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F740" t="s">
         <v>16</v>
       </c>
       <c r="G740" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="H740" t="s">
         <v>18</v>
@@ -24662,7 +24656,7 @@
         <v>16</v>
       </c>
       <c r="G741" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="H741" t="s">
         <v>13</v>
@@ -24685,13 +24679,13 @@
         <v>46103.692395833335</v>
       </c>
       <c r="E742" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F742" t="s">
         <v>16</v>
       </c>
       <c r="G742" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="H742" t="s">
         <v>18</v>
@@ -24714,13 +24708,13 @@
         <v>46104.444074074076</v>
       </c>
       <c r="E743" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F743" t="s">
         <v>16</v>
       </c>
       <c r="G743" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="H743" t="s">
         <v>34</v>
@@ -24749,7 +24743,7 @@
         <v>16</v>
       </c>
       <c r="G744" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="H744" t="s">
         <v>18</v>
@@ -24772,13 +24766,13 @@
         <v>46104.501087962963</v>
       </c>
       <c r="E745" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F745" t="s">
         <v>11</v>
       </c>
       <c r="G745" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="H745" t="s">
         <v>34</v>
@@ -24807,7 +24801,7 @@
         <v>11</v>
       </c>
       <c r="G746" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="H746" t="s">
         <v>31</v>
@@ -24836,7 +24830,7 @@
         <v>11</v>
       </c>
       <c r="G747" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="H747" t="s">
         <v>31</v>
@@ -24865,13 +24859,13 @@
         <v>16</v>
       </c>
       <c r="G748" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="H748" t="s">
         <v>18</v>
       </c>
       <c r="I748" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="749" spans="1:9" x14ac:dyDescent="0.25">
@@ -24894,7 +24888,7 @@
         <v>11</v>
       </c>
       <c r="G749" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="H749" t="s">
         <v>13</v>
@@ -24923,7 +24917,7 @@
         <v>16</v>
       </c>
       <c r="G750" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H750" t="s">
         <v>18</v>
@@ -24952,7 +24946,7 @@
         <v>16</v>
       </c>
       <c r="G751" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="H751" t="s">
         <v>13</v>
@@ -24975,13 +24969,13 @@
         <v>46104.54991898148</v>
       </c>
       <c r="E752" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F752" t="s">
         <v>16</v>
       </c>
       <c r="G752" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="H752" t="s">
         <v>18</v>
@@ -25010,7 +25004,7 @@
         <v>11</v>
       </c>
       <c r="G753" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="H753" t="s">
         <v>31</v>
@@ -25039,7 +25033,7 @@
         <v>11</v>
       </c>
       <c r="G754" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="H754" t="s">
         <v>18</v>
@@ -25068,7 +25062,7 @@
         <v>11</v>
       </c>
       <c r="G755" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H755" t="s">
         <v>13</v>
@@ -25097,13 +25091,13 @@
         <v>16</v>
       </c>
       <c r="G756" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="H756" t="s">
         <v>18</v>
       </c>
       <c r="I756" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="757" spans="1:9" x14ac:dyDescent="0.25">
@@ -25126,13 +25120,13 @@
         <v>16</v>
       </c>
       <c r="G757" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="H757" t="s">
         <v>18</v>
       </c>
       <c r="I757" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="758" spans="1:9" x14ac:dyDescent="0.25">
@@ -25155,13 +25149,13 @@
         <v>16</v>
       </c>
       <c r="G758" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="H758" t="s">
         <v>18</v>
       </c>
       <c r="I758" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="759" spans="1:9" x14ac:dyDescent="0.25">
@@ -25178,13 +25172,13 @@
         <v>46105.504745370374</v>
       </c>
       <c r="E759" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F759" t="s">
         <v>16</v>
       </c>
       <c r="G759" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H759" t="s">
         <v>18</v>
@@ -25213,7 +25207,7 @@
         <v>11</v>
       </c>
       <c r="G760" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="H760" t="s">
         <v>31</v>
@@ -25236,13 +25230,13 @@
         <v>46105.540034722224</v>
       </c>
       <c r="E761" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F761" t="s">
         <v>16</v>
       </c>
       <c r="G761" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="H761" t="s">
         <v>34</v>
@@ -25265,13 +25259,13 @@
         <v>46105.60355324074</v>
       </c>
       <c r="E762" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F762" t="s">
         <v>16</v>
       </c>
       <c r="G762" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="H762" t="s">
         <v>31</v>
@@ -25294,13 +25288,13 @@
         <v>46105.623518518521</v>
       </c>
       <c r="E763" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F763" t="s">
         <v>11</v>
       </c>
       <c r="G763" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="H763" t="s">
         <v>34</v>
@@ -25323,13 +25317,13 @@
         <v>46105.638287037036</v>
       </c>
       <c r="E764" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F764" t="s">
         <v>16</v>
       </c>
       <c r="G764" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="H764" t="s">
         <v>152</v>
@@ -25352,13 +25346,13 @@
         <v>46106.421979166669</v>
       </c>
       <c r="E765" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F765" t="s">
         <v>16</v>
       </c>
       <c r="G765" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="H765" t="s">
         <v>34</v>
@@ -25381,13 +25375,13 @@
         <v>46106.451365740744</v>
       </c>
       <c r="E766" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F766" t="s">
         <v>16</v>
       </c>
       <c r="G766" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="H766" t="s">
         <v>31</v>
@@ -25410,13 +25404,13 @@
         <v>46106.463831018518</v>
       </c>
       <c r="E767" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F767" t="s">
         <v>11</v>
       </c>
       <c r="G767" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="H767" t="s">
         <v>18</v>
@@ -25445,7 +25439,7 @@
         <v>11</v>
       </c>
       <c r="G768" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="H768" t="s">
         <v>18</v>
@@ -25474,13 +25468,13 @@
         <v>16</v>
       </c>
       <c r="G769" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="H769" t="s">
         <v>18</v>
       </c>
       <c r="I769" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="770" spans="1:9" x14ac:dyDescent="0.25">
@@ -25497,13 +25491,13 @@
         <v>46107.376805555556</v>
       </c>
       <c r="E770" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F770" t="s">
         <v>16</v>
       </c>
       <c r="G770" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="H770" t="s">
         <v>80</v>
@@ -25532,13 +25526,13 @@
         <v>11</v>
       </c>
       <c r="G771" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="H771" t="s">
         <v>18</v>
       </c>
       <c r="I771" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="772" spans="1:9" x14ac:dyDescent="0.25">
@@ -25555,13 +25549,13 @@
         <v>46107.429212962961</v>
       </c>
       <c r="E772" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F772" t="s">
         <v>16</v>
       </c>
       <c r="G772" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="H772" t="s">
         <v>13</v>
@@ -25590,7 +25584,7 @@
         <v>16</v>
       </c>
       <c r="G773" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="H773" t="s">
         <v>18</v>
@@ -25619,7 +25613,7 @@
         <v>16</v>
       </c>
       <c r="G774" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="H774" t="s">
         <v>34</v>
@@ -25642,13 +25636,13 @@
         <v>46107.477037037039</v>
       </c>
       <c r="E775" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F775" t="s">
         <v>11</v>
       </c>
       <c r="G775" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="H775" t="s">
         <v>13</v>
@@ -25677,7 +25671,7 @@
         <v>11</v>
       </c>
       <c r="G776" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="H776" t="s">
         <v>18</v>
@@ -25700,13 +25694,13 @@
         <v>46107.496307870373</v>
       </c>
       <c r="E777" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F777" t="s">
         <v>11</v>
       </c>
       <c r="G777" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="H777" t="s">
         <v>13</v>
@@ -25735,7 +25729,7 @@
         <v>16</v>
       </c>
       <c r="G778" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="H778" t="s">
         <v>18</v>
@@ -25764,7 +25758,7 @@
         <v>11</v>
       </c>
       <c r="G779" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="H779" t="s">
         <v>13</v>
@@ -25787,13 +25781,13 @@
         <v>46107.579282407409</v>
       </c>
       <c r="E780" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F780" t="s">
         <v>16</v>
       </c>
       <c r="G780" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="H780" t="s">
         <v>13</v>
@@ -25822,7 +25816,7 @@
         <v>16</v>
       </c>
       <c r="G781" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="H781" t="s">
         <v>18</v>
@@ -25851,7 +25845,7 @@
         <v>16</v>
       </c>
       <c r="G782" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="H782" t="s">
         <v>31</v>
@@ -25880,7 +25874,7 @@
         <v>16</v>
       </c>
       <c r="G783" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="H783" t="s">
         <v>31</v>
@@ -25909,13 +25903,13 @@
         <v>16</v>
       </c>
       <c r="G784" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="H784" t="s">
         <v>18</v>
       </c>
       <c r="I784" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="785" spans="1:9" x14ac:dyDescent="0.25">
@@ -25938,7 +25932,7 @@
         <v>16</v>
       </c>
       <c r="G785" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="H785" t="s">
         <v>18</v>
@@ -25967,7 +25961,7 @@
         <v>16</v>
       </c>
       <c r="G786" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="H786" t="s">
         <v>18</v>
@@ -25996,7 +25990,7 @@
         <v>16</v>
       </c>
       <c r="G787" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="H787" t="s">
         <v>31</v>
@@ -26025,13 +26019,13 @@
         <v>16</v>
       </c>
       <c r="G788" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="H788" t="s">
         <v>18</v>
       </c>
       <c r="I788" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="789" spans="1:9" x14ac:dyDescent="0.25">
@@ -26048,13 +26042,13 @@
         <v>46108.851666666669</v>
       </c>
       <c r="E789" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F789" t="s">
         <v>16</v>
       </c>
       <c r="G789" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="H789" t="s">
         <v>80</v>
@@ -26083,7 +26077,7 @@
         <v>16</v>
       </c>
       <c r="G790" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="H790" t="s">
         <v>31</v>
@@ -26106,13 +26100,13 @@
         <v>46109.517407407409</v>
       </c>
       <c r="E791" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F791" t="s">
         <v>16</v>
       </c>
       <c r="G791" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H791" t="s">
         <v>80</v>
@@ -26141,7 +26135,7 @@
         <v>16</v>
       </c>
       <c r="G792" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H792" t="s">
         <v>18</v>
@@ -26170,13 +26164,13 @@
         <v>16</v>
       </c>
       <c r="G793" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H793" t="s">
         <v>18</v>
       </c>
       <c r="I793" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="794" spans="1:9" x14ac:dyDescent="0.25">
@@ -26199,7 +26193,7 @@
         <v>11</v>
       </c>
       <c r="G794" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H794" t="s">
         <v>152</v>
@@ -26228,7 +26222,7 @@
         <v>11</v>
       </c>
       <c r="G795" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="H795" t="s">
         <v>13</v>
@@ -26257,7 +26251,7 @@
         <v>16</v>
       </c>
       <c r="G796" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="H796" t="s">
         <v>18</v>
@@ -26286,7 +26280,7 @@
         <v>16</v>
       </c>
       <c r="G797" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="H797" t="s">
         <v>152</v>
@@ -26315,7 +26309,7 @@
         <v>16</v>
       </c>
       <c r="G798" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="H798" t="s">
         <v>31</v>
@@ -26344,7 +26338,7 @@
         <v>11</v>
       </c>
       <c r="G799" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="H799" t="s">
         <v>34</v>
@@ -26373,10 +26367,10 @@
         <v>16</v>
       </c>
       <c r="G800" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="H800" t="s">
-        <v>880</v>
+        <v>34</v>
       </c>
       <c r="I800" t="s">
         <v>35</v>
@@ -26402,7 +26396,7 @@
         <v>11</v>
       </c>
       <c r="G801" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="H801" t="s">
         <v>13</v>
@@ -26431,7 +26425,7 @@
         <v>16</v>
       </c>
       <c r="G802" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="H802" t="s">
         <v>34</v>
@@ -26460,13 +26454,13 @@
         <v>16</v>
       </c>
       <c r="G803" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="H803" t="s">
         <v>18</v>
       </c>
       <c r="I803" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="804" spans="1:9" x14ac:dyDescent="0.25">
@@ -26489,13 +26483,13 @@
         <v>11</v>
       </c>
       <c r="G804" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="H804" t="s">
         <v>18</v>
       </c>
       <c r="I804" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="805" spans="1:9" x14ac:dyDescent="0.25">
@@ -26512,13 +26506,13 @@
         <v>46112.584629629629</v>
       </c>
       <c r="E805" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F805" t="s">
         <v>11</v>
       </c>
       <c r="G805" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="H805" t="s">
         <v>34</v>
@@ -26547,13 +26541,13 @@
         <v>16</v>
       </c>
       <c r="G806" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="H806" t="s">
         <v>18</v>
       </c>
       <c r="I806" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="807" spans="1:9" x14ac:dyDescent="0.25">
@@ -26576,7 +26570,7 @@
         <v>11</v>
       </c>
       <c r="G807" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="H807" t="s">
         <v>34</v>
@@ -26605,7 +26599,7 @@
         <v>11</v>
       </c>
       <c r="G808" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="H808" t="s">
         <v>13</v>
@@ -26634,7 +26628,7 @@
         <v>16</v>
       </c>
       <c r="G809" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="H809" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 20/04/2026 12:24:18,98
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74301CE5-1CDE-4843-9CDD-CDBB84287D1B}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4F77609-BB1C-4DF1-ABF5-FDA13609C281}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$836</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$905</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5019" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5433" uniqueCount="1004">
   <si>
     <t>ID</t>
   </si>
@@ -2903,6 +2903,246 @@
   <si>
     <t>Depois de alguns anos de reclamações finalmente foi instalado o filtro MIBGEO e finalmente a qualidade da agua ficou boa</t>
   </si>
+  <si>
+    <t>Tenho o purificador ha muitos anos, mas nos últimos dois anos a qualidade do filtro piorou muito, nao dura, a água fica com gosto ruim muito rápido,  os técnicos sao atenciosos e nos atendem muito bem,porem , e difícil agendar a visita pra uma data próxima, tem.sempre que esperar em.media 1 mês,  dessa forma ,estou estudando a possibilidade de mudar de purificador</t>
+  </si>
+  <si>
+    <t>FRQ SP SAO PAULO</t>
+  </si>
+  <si>
+    <t>Aguardando retorno do técnico com novo purificador.</t>
+  </si>
+  <si>
+    <t>FRQ CENTRO NORTE RJ</t>
+  </si>
+  <si>
+    <t>O técnico veio ver um problema no purificador em que a água está esfriando pouco. Ele veio, foi embora e não resolveu o problema.</t>
+  </si>
+  <si>
+    <t>Acho a assinatura cara e vejo que consumidores novos pagam menos do que eu, o que não acho correto!!</t>
+  </si>
+  <si>
+    <t>FRQ RECIFE PE</t>
+  </si>
+  <si>
+    <t>Fui informado que o purificador está quebrado, sendo necessária a troca. Até o momento não me foi informado nada, nem quando será realizada.</t>
+  </si>
+  <si>
+    <t>2 meses pra resolver uma troca por defeito</t>
+  </si>
+  <si>
+    <t>Falar com a Brastemp é um grande oroblema</t>
+  </si>
+  <si>
+    <t>Meu problema não foi resolvido.O filtro está “super” aquecendo e estou aguardando retorno p trocar o aparelho.Muito demorado!!!</t>
+  </si>
+  <si>
+    <t>Se fosse um tempo atrás eu indicaria com certeza. Mas, após ficar mais de um mês com o filtro avariado, aguardando atendimento, fica difícil de indicar para alguém.</t>
+  </si>
+  <si>
+    <t>O serviço não foi realizado.</t>
+  </si>
+  <si>
+    <t>Serviço de manutenção é muito demorada, sem contar os canais de comunicação para sanar algum problema!Fiquei mais de 1 mês em espera para manutenção de um dos filtros com alegação que seria necessário a troca, porém nunca foi aberto a solicitação de troca pelo técnico!Para o final a técnica que foi na ultima visita depois de muita insistência, disse que só era necessário a troca de uma peça!</t>
+  </si>
+  <si>
+    <t>Demorou mais de mês para virem instalar o equipamento, que depois de instalado parou de soltar agua gelada depois de 3 horas de uso.</t>
+  </si>
+  <si>
+    <t>Único porém quando precisa de visita agendam muito longe</t>
+  </si>
+  <si>
+    <t>Já vieram 3 vezes para arrumar o meu filtro e não conseguiram , continua saindo água quente</t>
+  </si>
+  <si>
+    <t>FRQ CURITIBA PR</t>
+  </si>
+  <si>
+    <t>Agilidade</t>
+  </si>
+  <si>
+    <t>Já tenha bastante tempo mas precisei de suporte semana passada tive muita dificuldade para agendar e não há nenhuma solicitação no meu e-mail para autorizar outra empresa no caso coligar a debita minhas fatura o vazamento foi resolvido mas o barulho do filtro continua e várias peças oxidadas</t>
+  </si>
+  <si>
+    <t>Muito bom equipamento. Porém, acredito que a logística de manutenção tenha mudado. Isso me incomodou muito porque não avisaram. Não confirmaram. O tecnico veio e não tinha a OS anterior, somente a nova e a qual nao tive acesso. Esta bem confuso.</t>
+  </si>
+  <si>
+    <t>FRQ BAIXADA SERRANA RJ</t>
+  </si>
+  <si>
+    <t>Falo do serviço da Brastemp em si. Não do último serviço e nem do anterior. O problema é que demorou meses até resolverem algo que deveria ser imediato! Fora as ausências do representande Brastemp nos dias combinados.</t>
+  </si>
+  <si>
+    <t>Gosto muito, mas acho o preço da mensalidade um pouco elevado. A assistência técnica não é rápida quando solicitada. Estes dois pontos poderiam melhorar.</t>
+  </si>
+  <si>
+    <t>Purificador ficou vazando, a pessoa estava perdida no atendimento, nao sabia se era reparo ou manutenção preventiva, trocou o filtro e ficou vazando,  terei quw abrir novo chamado</t>
+  </si>
+  <si>
+    <t>FRQ LAGOS RJ</t>
+  </si>
+  <si>
+    <t>Liguei solicitando um atendimento pois o purificador está vazando. O técnico viu o problema e ficou de avisar que precisa ser trocado. Até agora não recebi nenhum contato agendando a troca do aparelho. A Brastemp só entra em contato qdo tem algum problema no cartão, qto a satisfação do cliente fica muuuito a desejar.</t>
+  </si>
+  <si>
+    <t>Técnico condenou a máquina e até hoje não trouxeram outra só estou esperando cobrar para eu entrar com ação. Falta de respeito com o cliente , tô sem água até hoje tendo que comprar galões de agua por causa de vcs . Pode deixar que TDS peço nota fiscal .</t>
+  </si>
+  <si>
+    <t>FRQ BRAGANCA PAULISTA SP</t>
+  </si>
+  <si>
+    <t>Deixaram um filtro com problema e vazou agua nos armarios, que agora esta estufando toda a madeira.</t>
+  </si>
+  <si>
+    <t>Estou gostando</t>
+  </si>
+  <si>
+    <t>Estava muito boa , mas na última vez que o técnico veio, não trocou a vela e aí surgiu o problema , pois a água no local não é boa e há necessidade de trocar n para continuar Boa. Precisei solicitar que o técnico viesse trocar a vela que não tinha sido trocada e surgiu outro problema a água está fraca . Solicitei novamente o técnico .</t>
+  </si>
+  <si>
+    <t>Não trocou meu filtro com mais de 6 meses desde a última visita.</t>
+  </si>
+  <si>
+    <t>Muito bom, não tenho q reclamar do purificador Brastemp</t>
+  </si>
+  <si>
+    <t>Dei essa nota, pois para o uso residencial, eu entendo que o preço é salgado. Esse é o unico motivo.</t>
+  </si>
+  <si>
+    <t>FRQ GALEAO SUL RJ</t>
+  </si>
+  <si>
+    <t>Bom dia, na minha solicitação de troca do purificador solicitei o modelo caribe e o técnico trouxe o mesmo modelo do antigo, o técnico bem simpático e atencioso.</t>
+  </si>
+  <si>
+    <t>O purificador atual demora muito para gelar a água. Depois de dois copos leva entre 10 e 15 minutos para ter água gelada novamente.Os purificadores mais antigos não eram assim.</t>
+  </si>
+  <si>
+    <t>Não foi resolvido defeito, purificador não está gelando.</t>
+  </si>
+  <si>
+    <t>O serviço prestado cem decaindo assustadoramente. Última visita em maio/2025. A manutenção não é mais feita a cada 6 meses. Total dificuldade para falar com a brastemp sobre problema no produto e quando a empresa nos liga temos que praticamente aceitar por imposição a data indicada para visita. Totalmente insatisfeita com o Serviço que vem sendo ofertado.</t>
+  </si>
+  <si>
+    <t>FRQ SJCAMPOS SP</t>
+  </si>
+  <si>
+    <t>Era ótimo mas agora deixa a desejar</t>
+  </si>
+  <si>
+    <t>A experiência com o aparelho está muito boa, o problema é esse formato travado de agendamento que não permite flexibilidade.</t>
+  </si>
+  <si>
+    <t>Equipamento ficou vazando água em dois pontos de conexão do filtro</t>
+  </si>
+  <si>
+    <t>FOI BOA</t>
+  </si>
+  <si>
+    <t>Por muito tempo foi bom, mas de uns 3 anos pra cá, vem caindo a qualidade do atendimento. Por exemplo, agendei para o dia 09/04 e o técnico não apareceu, não deu satisfação. Liguei para a central que disse não poder fazer nada!MAs eu tive que deixar uma pessoa disponível aguardando o técnico que não apareceu...e se fosse o contrário?Outra vez, o técnico retirou os parafusos do meu aparelho, eu questionei e ele disse que não precisava dos parafusos. Mas se não precisa, porque vem da fábricacom parafusos? Estou sem os parafusos no aparelho esse último técnico que me atendeu questionou. Explicamos o que aconteceu e ele disse que precisa sim, mas que ele não tinha nenhum para repor no dia...enfim, estamos à mercê das vontades dos técnicos.spu cliente há mais de 10 anos e percebo a queda da qualidade.</t>
+  </si>
+  <si>
+    <t>Tenho tido alguns problemas pp no agendamento Marquei pela manhã não veio nem de manhã e nem a tarde , foi reagendada para dia 13/04 para tarde e apareceu de manhã  ( eu já estava saindo ) parece até que estamos a disposição para que agendar então , seria melhor só agendar o dia e deixar o horário sendo comercial Assim a pessoa já fica o tempo todo em casa</t>
+  </si>
+  <si>
+    <t>NÃO HOUVE VISITA TECNICA</t>
+  </si>
+  <si>
+    <t>Tenho este purificador a alguns anos. Tem me servido muito bem.</t>
+  </si>
+  <si>
+    <t>Atendimento péssimo via telefone pesssimo! Suporte via chat péssimo!!! Única coisa muito boa são os atendimentos dos técnicos.</t>
+  </si>
+  <si>
+    <t>Ele é realmente mto bom...Mas achei mto grande para uso doméstico... E faz um pouco de barulho.. rsrsrs</t>
+  </si>
+  <si>
+    <t>Tudo bem quanto ao purificador. Quanto ao atendimento, peço que o funcionário tenha mais panos de limpeza, pois veio só com um, sujo. Ele que só dão um por dia.Tem que dar um para cada casa visitada.Obrigado.</t>
+  </si>
+  <si>
+    <t>Segunda ou terceira vez que o técnico não troca o elemento filtrante. Será que a água da Sabesp tá tão boa, que não preciso mais de filtros?</t>
+  </si>
+  <si>
+    <t>AT FORTALEZA CE</t>
+  </si>
+  <si>
+    <t>O purificador está com períodos curtos de validade,ficando a água com odor e gosto ruim.Tenho dificuldade de marcar com brevidade nos causando transtornos. Espero que melhorem os agendamentos</t>
+  </si>
+  <si>
+    <t>Pessima! Não compareceu</t>
+  </si>
+  <si>
+    <t>Técnico apenas retirou a água do filtro e colocou uma solução para avaliação, mais nada. A visita durou 5 minutos.</t>
+  </si>
+  <si>
+    <t>O atendimento do técnico é excelente, mas a nota 7 é devido a demora na troca do equipamento, que já foi solicitada pelo técnico na última visita.O equipamento atual está com problema no compressor, vaza muito, está sempre cheio da água dentro dele, a água natural sai quente quase fervendo e a gelada é quase natural.Gostaria de saber quando irei receber um novo purificador de água, pois continuo pagando a mensalidade normalmente.Atenciosamente,Aureci</t>
+  </si>
+  <si>
+    <t>Funcionou muito bem, mas ultimamente parou de gelar a água e o técnico já esteve por três vezes em casa. Aparentemente ele vai sugerir a troca do produto e espero que isso não demore</t>
+  </si>
+  <si>
+    <t>Não realizarem a troca do filtro, já se passo mais de 6 meses.</t>
+  </si>
+  <si>
+    <t>Muito atencioso e rapido!Mas para o agendamento foi muito longo o prazo e fiquei 15 dias com o purificador sem poder usar!</t>
+  </si>
+  <si>
+    <t>Boa qualidade e serviço manutenção</t>
+  </si>
+  <si>
+    <t>Só uma reclamação. Quando falta luz ficamos sem água.</t>
+  </si>
+  <si>
+    <t>FRQ BELO HORIZONTE MG</t>
+  </si>
+  <si>
+    <t>O produto apresenta muitos defeitos. Não entrega o que promete: a água com gás é bastante limitada. Nesse último defeito a 1a visita agendada não foi realizada e a 2a demorou bastante ( fiquei muito tempo sem poder utilizar o purificador com todas as suas funcionalidades)</t>
+  </si>
+  <si>
+    <t>Mensalidade muito cara</t>
+  </si>
+  <si>
+    <t>Tinha o filtro Brastemp há muitos anos . Sempre bem atendida e nunca tive problemas. Meu filtro quebrou e tentei por 5 vezes algum técnico para ver o problema e simplesmente ninguém apareceu . Cancelei o plano e não quero mais 😡</t>
+  </si>
+  <si>
+    <t>ZERO -a empresa esta sem filtro desde o dia 17/03/2026, visita tecnica agendada e não apareceu ninguém</t>
+  </si>
+  <si>
+    <t>Depois de alguns maus atendimentos, o ultimo tecnico veio e trocou o porificador que agora esta funcionando bem.</t>
+  </si>
+  <si>
+    <t>O atendimento para agendamento de serviços de manutenção é muito burocrático. Por exemplo, tenho 05 purificadores e não consigo agendamento para manutenção de todos no mesmo dia. Estou a duas semanas recebendo técnicos dia sim, dia não para manutenção de um purificador por vez. Por exemplo, estou com um purificador parado tem 10 mês e o agendamento de troca do equipamento - registrado via laudo por outro técnico que realizou a vistoria e não realizava a troca - ficou para maio (mesmo tendo sido solicitado pela pp Brastemp no inicio de abril).</t>
+  </si>
+  <si>
+    <t>Demorou muito pra atender a solicitação</t>
+  </si>
+  <si>
+    <t>Eu estava aguardando a visita desde Out/2025 por quatro vezes agendaram e não apareceram , tentei até cancelar mas a atendente com muita educação explicou as mudanças que estão acontecendo na empresa então resolvi dar um voto de confiança, o técnico que veio foi muito gentil, cuidados  e ágil , por isso estou aqui perdendo meu tempo, mas no geral não indicaria vcs , quase 6 meses com o filtro vencido não é atendimento que se preze, pago caro pra ter qualidade e não foi isso que recebi . Espero que vcs melhorem bastante . Boa sorte !</t>
+  </si>
+  <si>
+    <t>Não estão mais fazendo manutenção preventiva . Tenho 2 purificadores e só atenderam um por chamado . Um absurdo</t>
+  </si>
+  <si>
+    <t>No dia pareceu que ficou bom, porém já está com o mesmo problema de novo. Vao precisar voltar</t>
+  </si>
+  <si>
+    <t>Em poucos meses o equipamento quebrou duas vezes, fiz a assinatura mas no próprio site da Brastemp não tinha refil do gás. O atendimento ao cliente por telefone na assistência técnica é horrível. Só não cancelei porque o técnico Eduardo foi 1000!</t>
+  </si>
+  <si>
+    <t>Os tecnicos estão teimosos, antes trocavam sempre o filtro, agora a gente tem que pedir. Aqui no centro do Rio de Janeiro a agua é podre, não podem deixar de trocar sempre o filtro, a cada seis meses. desta vez ele trocou mas disse que não está autorizado a trocar de 6/6 meses. Por favor alinhem essa postura pois antes o serviço era melhor.</t>
+  </si>
+  <si>
+    <t>Para o técnico comparecer a minha residência foi preciso eu agendar a visita duas vezes, e mesmo assim quase tive que agendar mais outra vez, porque o horário que estava marcado foi de 8:00 as 13:oo hs, e ele chegou depois deste horário, sorte que eu ainda estava em casa. O técnico solicitou a troca do purificador mas até o momento ninguem entrou em contato de quando será feito a troca. E enquanto isto estou tendo problema com o barulho que ele está fazendo enquanto estiver ligado. Estou aguardando uma solução.</t>
+  </si>
+  <si>
+    <t>A visita foi fiscalizada por minha mãe, a qual foi destratada pelo técnico, apenas por solicitar que ele retirasse o sapato para entrar na residência. Após, ele fez a manutenção básica como previsto, mas o acontecimento inicial reduziu a satisfação para nota 2</t>
+  </si>
+  <si>
+    <t>Pos venda e atendimento, já sou cliente a muito tempo e ultimamente tenho diversos contratempos em relação a manutenção, sempre o técnico que é de uma empresa terceirizada(o que temos a ver com isso?) fala que não pode trocar o filtro, sendo que passados mais de 6 meses, e a agua sempre costuma mudar o gosto quando está proximo de vencer este prazo, justificando que não são autorizados a fazer a troca se o teste feito não acusar alteração na cor, mas e o gosto? então não assinando nenhuma Ordem de Serviço, mesmo ele insistindo que iria fazer, ou seja, saiu daqui sem ordem assinada, se houver alguma assinatura, não foi a nossa, obs: continuo com os dois filtros sem manutenção.</t>
+  </si>
+  <si>
+    <t>Solicitei um serviço e veio outro, disseram que voltariam na parte da tarde para finalizar e não apareceram.</t>
+  </si>
 </sst>
 </file>
 
@@ -2920,6 +3160,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2969,7 +3210,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3273,7 +3514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I836"/>
+  <dimension ref="A1:I905"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -27532,6 +27773,2007 @@
         <v>65</v>
       </c>
     </row>
+    <row r="837" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A837" s="4">
+        <v>836</v>
+      </c>
+      <c r="B837" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C837" s="4">
+        <v>16845</v>
+      </c>
+      <c r="D837" s="2">
+        <v>46122.418773148151</v>
+      </c>
+      <c r="E837" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F837" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G837" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="H837" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I837" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="838" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A838" s="4">
+        <v>837</v>
+      </c>
+      <c r="B838" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C838" s="4">
+        <v>16460</v>
+      </c>
+      <c r="D838" s="2">
+        <v>46122.428414351853</v>
+      </c>
+      <c r="E838" s="4" t="s">
+        <v>925</v>
+      </c>
+      <c r="F838" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G838" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="H838" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I838" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="839" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A839" s="4">
+        <v>838</v>
+      </c>
+      <c r="B839" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C839" s="4">
+        <v>21937</v>
+      </c>
+      <c r="D839" s="2">
+        <v>46122.452303240738</v>
+      </c>
+      <c r="E839" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="F839" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G839" s="4" t="s">
+        <v>928</v>
+      </c>
+      <c r="H839" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I839" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="840" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A840" s="4">
+        <v>839</v>
+      </c>
+      <c r="B840" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C840" s="4">
+        <v>13639</v>
+      </c>
+      <c r="D840" s="2">
+        <v>46122.476840277777</v>
+      </c>
+      <c r="E840" s="4" t="s">
+        <v>925</v>
+      </c>
+      <c r="F840" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G840" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="H840" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I840" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="841" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A841" s="4">
+        <v>840</v>
+      </c>
+      <c r="B841" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C841" s="4">
+        <v>23150</v>
+      </c>
+      <c r="D841" s="2">
+        <v>46122.496539351851</v>
+      </c>
+      <c r="E841" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="F841" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G841" s="4" t="s">
+        <v>931</v>
+      </c>
+      <c r="H841" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I841" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="842" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A842" s="4">
+        <v>841</v>
+      </c>
+      <c r="B842" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C842" s="4">
+        <v>21967</v>
+      </c>
+      <c r="D842" s="2">
+        <v>46122.497175925928</v>
+      </c>
+      <c r="E842" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F842" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G842" s="4" t="s">
+        <v>932</v>
+      </c>
+      <c r="H842" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I842" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="843" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A843" s="4">
+        <v>842</v>
+      </c>
+      <c r="B843" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C843" s="4">
+        <v>23679</v>
+      </c>
+      <c r="D843" s="2">
+        <v>46122.504259259258</v>
+      </c>
+      <c r="E843" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F843" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G843" s="4" t="s">
+        <v>933</v>
+      </c>
+      <c r="H843" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I843" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="844" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A844" s="4">
+        <v>843</v>
+      </c>
+      <c r="B844" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C844" s="4">
+        <v>22641</v>
+      </c>
+      <c r="D844" s="2">
+        <v>46122.507511574076</v>
+      </c>
+      <c r="E844" s="4" t="s">
+        <v>910</v>
+      </c>
+      <c r="F844" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G844" s="4" t="s">
+        <v>934</v>
+      </c>
+      <c r="H844" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I844" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="845" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A845" s="4">
+        <v>844</v>
+      </c>
+      <c r="B845" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C845" s="4">
+        <v>11077</v>
+      </c>
+      <c r="D845" s="2">
+        <v>46122.744756944441</v>
+      </c>
+      <c r="E845" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F845" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G845" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="H845" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I845" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="846" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A846" s="4">
+        <v>845</v>
+      </c>
+      <c r="B846" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C846" s="4">
+        <v>15266</v>
+      </c>
+      <c r="D846" s="2">
+        <v>46123.383101851854</v>
+      </c>
+      <c r="E846" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="F846" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G846" s="4" t="s">
+        <v>936</v>
+      </c>
+      <c r="H846" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I846" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="847" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A847" s="4">
+        <v>846</v>
+      </c>
+      <c r="B847" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C847" s="4">
+        <v>22452</v>
+      </c>
+      <c r="D847" s="2">
+        <v>46125.49113425926</v>
+      </c>
+      <c r="E847" s="4" t="s">
+        <v>890</v>
+      </c>
+      <c r="F847" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G847" s="4" t="s">
+        <v>937</v>
+      </c>
+      <c r="H847" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I847" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="848" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A848" s="4">
+        <v>847</v>
+      </c>
+      <c r="B848" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C848" s="4">
+        <v>23491</v>
+      </c>
+      <c r="D848" s="2">
+        <v>46125.49858796296</v>
+      </c>
+      <c r="E848" s="4" t="s">
+        <v>890</v>
+      </c>
+      <c r="F848" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G848" s="4" t="s">
+        <v>938</v>
+      </c>
+      <c r="H848" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I848" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="849" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A849" s="4">
+        <v>848</v>
+      </c>
+      <c r="B849" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C849" s="4">
+        <v>16892</v>
+      </c>
+      <c r="D849" s="2">
+        <v>46125.509745370371</v>
+      </c>
+      <c r="E849" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F849" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G849" s="4" t="s">
+        <v>939</v>
+      </c>
+      <c r="H849" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I849" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="850" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A850" s="4">
+        <v>849</v>
+      </c>
+      <c r="B850" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C850" s="4">
+        <v>24959</v>
+      </c>
+      <c r="D850" s="2">
+        <v>46125.516909722224</v>
+      </c>
+      <c r="E850" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F850" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G850" s="4" t="s">
+        <v>940</v>
+      </c>
+      <c r="H850" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I850" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="851" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A851" s="4">
+        <v>850</v>
+      </c>
+      <c r="B851" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C851" s="4">
+        <v>25528</v>
+      </c>
+      <c r="D851" s="2">
+        <v>46125.522083333337</v>
+      </c>
+      <c r="E851" s="4" t="s">
+        <v>941</v>
+      </c>
+      <c r="F851" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G851" s="4" t="s">
+        <v>942</v>
+      </c>
+      <c r="H851" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I851" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="852" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A852" s="4">
+        <v>851</v>
+      </c>
+      <c r="B852" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C852" s="4">
+        <v>25865</v>
+      </c>
+      <c r="D852" s="2">
+        <v>46125.524826388886</v>
+      </c>
+      <c r="E852" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F852" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G852" s="4" t="s">
+        <v>943</v>
+      </c>
+      <c r="H852" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I852" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="853" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A853" s="4">
+        <v>852</v>
+      </c>
+      <c r="B853" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C853" s="4">
+        <v>17616</v>
+      </c>
+      <c r="D853" s="2">
+        <v>46125.52920138889</v>
+      </c>
+      <c r="E853" s="4" t="s">
+        <v>915</v>
+      </c>
+      <c r="F853" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G853" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="H853" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I853" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="854" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A854" s="4">
+        <v>853</v>
+      </c>
+      <c r="B854" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C854" s="4">
+        <v>20983</v>
+      </c>
+      <c r="D854" s="2">
+        <v>46125.537465277775</v>
+      </c>
+      <c r="E854" s="4" t="s">
+        <v>945</v>
+      </c>
+      <c r="F854" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G854" s="4" t="s">
+        <v>946</v>
+      </c>
+      <c r="H854" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I854" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="855" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A855" s="4">
+        <v>854</v>
+      </c>
+      <c r="B855" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C855" s="4">
+        <v>13063</v>
+      </c>
+      <c r="D855" s="2">
+        <v>46125.554016203707</v>
+      </c>
+      <c r="E855" s="4" t="s">
+        <v>915</v>
+      </c>
+      <c r="F855" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G855" s="4" t="s">
+        <v>947</v>
+      </c>
+      <c r="H855" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I855" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="856" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A856" s="4">
+        <v>855</v>
+      </c>
+      <c r="B856" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C856" s="4">
+        <v>16095</v>
+      </c>
+      <c r="D856" s="2">
+        <v>46125.556990740741</v>
+      </c>
+      <c r="E856" s="4" t="s">
+        <v>917</v>
+      </c>
+      <c r="F856" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G856" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="H856" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I856" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="857" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A857" s="4">
+        <v>856</v>
+      </c>
+      <c r="B857" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C857" s="4">
+        <v>24608</v>
+      </c>
+      <c r="D857" s="2">
+        <v>46125.57539351852</v>
+      </c>
+      <c r="E857" s="4" t="s">
+        <v>949</v>
+      </c>
+      <c r="F857" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G857" s="4" t="s">
+        <v>950</v>
+      </c>
+      <c r="H857" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I857" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="858" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A858" s="4">
+        <v>857</v>
+      </c>
+      <c r="B858" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C858" s="4">
+        <v>23276</v>
+      </c>
+      <c r="D858" s="2">
+        <v>46125.576666666668</v>
+      </c>
+      <c r="E858" s="4" t="s">
+        <v>945</v>
+      </c>
+      <c r="F858" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G858" s="4" t="s">
+        <v>951</v>
+      </c>
+      <c r="H858" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I858" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="859" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A859" s="4">
+        <v>858</v>
+      </c>
+      <c r="B859" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C859" s="4">
+        <v>24487</v>
+      </c>
+      <c r="D859" s="2">
+        <v>46125.614027777781</v>
+      </c>
+      <c r="E859" s="4" t="s">
+        <v>952</v>
+      </c>
+      <c r="F859" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G859" s="4" t="s">
+        <v>953</v>
+      </c>
+      <c r="H859" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I859" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="860" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A860" s="4">
+        <v>859</v>
+      </c>
+      <c r="B860" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C860" s="4">
+        <v>16733</v>
+      </c>
+      <c r="D860" s="2">
+        <v>46125.65729166667</v>
+      </c>
+      <c r="E860" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="F860" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G860" s="4" t="s">
+        <v>954</v>
+      </c>
+      <c r="H860" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I860" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="861" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A861" s="4">
+        <v>860</v>
+      </c>
+      <c r="B861" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C861" s="4">
+        <v>22158</v>
+      </c>
+      <c r="D861" s="2">
+        <v>46125.799456018518</v>
+      </c>
+      <c r="E861" s="4" t="s">
+        <v>915</v>
+      </c>
+      <c r="F861" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G861" s="4" t="s">
+        <v>955</v>
+      </c>
+      <c r="H861" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I861" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="862" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A862" s="4">
+        <v>861</v>
+      </c>
+      <c r="B862" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C862" s="4">
+        <v>15462</v>
+      </c>
+      <c r="D862" s="2">
+        <v>46125.859236111108</v>
+      </c>
+      <c r="E862" s="4" t="s">
+        <v>945</v>
+      </c>
+      <c r="F862" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G862" s="4" t="s">
+        <v>956</v>
+      </c>
+      <c r="H862" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I862" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="863" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A863" s="4">
+        <v>862</v>
+      </c>
+      <c r="B863" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C863" s="4">
+        <v>13866</v>
+      </c>
+      <c r="D863" s="2">
+        <v>46126.382893518516</v>
+      </c>
+      <c r="E863" s="4" t="s">
+        <v>945</v>
+      </c>
+      <c r="F863" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G863" s="4" t="s">
+        <v>957</v>
+      </c>
+      <c r="H863" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I863" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="864" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A864" s="4">
+        <v>863</v>
+      </c>
+      <c r="B864" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C864" s="4">
+        <v>25485</v>
+      </c>
+      <c r="D864" s="2">
+        <v>46126.424039351848</v>
+      </c>
+      <c r="E864" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F864" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G864" s="4" t="s">
+        <v>958</v>
+      </c>
+      <c r="H864" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I864" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="865" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A865" s="4">
+        <v>864</v>
+      </c>
+      <c r="B865" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C865" s="4">
+        <v>23489</v>
+      </c>
+      <c r="D865" s="2">
+        <v>46126.437303240738</v>
+      </c>
+      <c r="E865" s="4" t="s">
+        <v>959</v>
+      </c>
+      <c r="F865" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G865" s="4" t="s">
+        <v>960</v>
+      </c>
+      <c r="H865" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I865" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="866" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A866" s="4">
+        <v>865</v>
+      </c>
+      <c r="B866" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C866" s="4">
+        <v>26639</v>
+      </c>
+      <c r="D866" s="2">
+        <v>46126.519062500003</v>
+      </c>
+      <c r="E866" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="F866" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G866" s="4" t="s">
+        <v>961</v>
+      </c>
+      <c r="H866" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I866" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="867" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A867" s="4">
+        <v>866</v>
+      </c>
+      <c r="B867" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C867" s="4">
+        <v>26686</v>
+      </c>
+      <c r="D867" s="2">
+        <v>46126.520370370374</v>
+      </c>
+      <c r="E867" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F867" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G867" s="4" t="s">
+        <v>962</v>
+      </c>
+      <c r="H867" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I867" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="868" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A868" s="4">
+        <v>867</v>
+      </c>
+      <c r="B868" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C868" s="4">
+        <v>26076</v>
+      </c>
+      <c r="D868" s="2">
+        <v>46126.523321759261</v>
+      </c>
+      <c r="E868" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="F868" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G868" s="4" t="s">
+        <v>963</v>
+      </c>
+      <c r="H868" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I868" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="869" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A869" s="4">
+        <v>868</v>
+      </c>
+      <c r="B869" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C869" s="4">
+        <v>24683</v>
+      </c>
+      <c r="D869" s="2">
+        <v>46126.524062500001</v>
+      </c>
+      <c r="E869" s="4" t="s">
+        <v>964</v>
+      </c>
+      <c r="F869" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G869" s="4" t="s">
+        <v>965</v>
+      </c>
+      <c r="H869" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I869" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="870" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A870" s="4">
+        <v>869</v>
+      </c>
+      <c r="B870" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C870" s="4">
+        <v>13085</v>
+      </c>
+      <c r="D870" s="2">
+        <v>46126.550162037034</v>
+      </c>
+      <c r="E870" s="4" t="s">
+        <v>890</v>
+      </c>
+      <c r="F870" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G870" s="4" t="s">
+        <v>966</v>
+      </c>
+      <c r="H870" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I870" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="871" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A871" s="4">
+        <v>870</v>
+      </c>
+      <c r="B871" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C871" s="4">
+        <v>16569</v>
+      </c>
+      <c r="D871" s="2">
+        <v>46126.556284722225</v>
+      </c>
+      <c r="E871" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="F871" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G871" s="4" t="s">
+        <v>967</v>
+      </c>
+      <c r="H871" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I871" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="872" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A872" s="4">
+        <v>871</v>
+      </c>
+      <c r="B872" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C872" s="4">
+        <v>15203</v>
+      </c>
+      <c r="D872" s="2">
+        <v>46126.596377314818</v>
+      </c>
+      <c r="E872" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F872" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G872" s="4" t="s">
+        <v>968</v>
+      </c>
+      <c r="H872" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I872" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="873" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A873" s="4">
+        <v>872</v>
+      </c>
+      <c r="B873" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C873" s="4">
+        <v>25852</v>
+      </c>
+      <c r="D873" s="2">
+        <v>46126.597326388888</v>
+      </c>
+      <c r="E873" s="4" t="s">
+        <v>915</v>
+      </c>
+      <c r="F873" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G873" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="H873" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I873" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="874" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A874" s="4">
+        <v>873</v>
+      </c>
+      <c r="B874" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C874" s="4">
+        <v>14457</v>
+      </c>
+      <c r="D874" s="2">
+        <v>46126.716921296298</v>
+      </c>
+      <c r="E874" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="F874" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G874" s="4" t="s">
+        <v>970</v>
+      </c>
+      <c r="H874" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I874" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="875" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A875" s="4">
+        <v>874</v>
+      </c>
+      <c r="B875" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C875" s="4">
+        <v>15047</v>
+      </c>
+      <c r="D875" s="2">
+        <v>46127.370266203703</v>
+      </c>
+      <c r="E875" s="4" t="s">
+        <v>925</v>
+      </c>
+      <c r="F875" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G875" s="4" t="s">
+        <v>971</v>
+      </c>
+      <c r="H875" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I875" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="876" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A876" s="4">
+        <v>875</v>
+      </c>
+      <c r="B876" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C876" s="4">
+        <v>27144</v>
+      </c>
+      <c r="D876" s="2">
+        <v>46127.470659722225</v>
+      </c>
+      <c r="E876" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="F876" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G876" s="4" t="s">
+        <v>972</v>
+      </c>
+      <c r="H876" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I876" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="877" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A877" s="4">
+        <v>876</v>
+      </c>
+      <c r="B877" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C877" s="4">
+        <v>27873</v>
+      </c>
+      <c r="D877" s="2">
+        <v>46127.540439814817</v>
+      </c>
+      <c r="E877" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F877" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G877" s="4" t="s">
+        <v>973</v>
+      </c>
+      <c r="H877" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I877" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="878" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A878" s="4">
+        <v>877</v>
+      </c>
+      <c r="B878" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C878" s="4">
+        <v>22090</v>
+      </c>
+      <c r="D878" s="2">
+        <v>46127.548252314817</v>
+      </c>
+      <c r="E878" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F878" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G878" s="4" t="s">
+        <v>974</v>
+      </c>
+      <c r="H878" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I878" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="879" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A879" s="4">
+        <v>878</v>
+      </c>
+      <c r="B879" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C879" s="4">
+        <v>25146</v>
+      </c>
+      <c r="D879" s="2">
+        <v>46127.553726851853</v>
+      </c>
+      <c r="E879" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F879" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G879" s="4" t="s">
+        <v>975</v>
+      </c>
+      <c r="H879" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I879" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="880" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A880" s="4">
+        <v>879</v>
+      </c>
+      <c r="B880" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C880" s="4">
+        <v>16756</v>
+      </c>
+      <c r="D880" s="2">
+        <v>46127.639687499999</v>
+      </c>
+      <c r="E880" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F880" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G880" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="H880" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I880" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="881" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A881" s="4">
+        <v>880</v>
+      </c>
+      <c r="B881" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C881" s="4">
+        <v>24953</v>
+      </c>
+      <c r="D881" s="2">
+        <v>46127.900729166664</v>
+      </c>
+      <c r="E881" s="4" t="s">
+        <v>977</v>
+      </c>
+      <c r="F881" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G881" s="4" t="s">
+        <v>978</v>
+      </c>
+      <c r="H881" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I881" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="882" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A882" s="4">
+        <v>881</v>
+      </c>
+      <c r="B882" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C882" s="4">
+        <v>6736</v>
+      </c>
+      <c r="D882" s="2">
+        <v>46128.459178240744</v>
+      </c>
+      <c r="E882" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F882" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G882" s="4" t="s">
+        <v>979</v>
+      </c>
+      <c r="H882" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I882" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="883" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A883" s="4">
+        <v>882</v>
+      </c>
+      <c r="B883" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C883" s="4">
+        <v>26578</v>
+      </c>
+      <c r="D883" s="2">
+        <v>46128.465775462966</v>
+      </c>
+      <c r="E883" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F883" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G883" s="4" t="s">
+        <v>980</v>
+      </c>
+      <c r="H883" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I883" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="884" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A884" s="4">
+        <v>883</v>
+      </c>
+      <c r="B884" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C884" s="4">
+        <v>17340</v>
+      </c>
+      <c r="D884" s="2">
+        <v>46128.4921875</v>
+      </c>
+      <c r="E884" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="F884" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G884" s="4" t="s">
+        <v>981</v>
+      </c>
+      <c r="H884" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I884" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="885" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A885" s="4">
+        <v>884</v>
+      </c>
+      <c r="B885" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C885" s="4">
+        <v>26763</v>
+      </c>
+      <c r="D885" s="2">
+        <v>46128.501400462963</v>
+      </c>
+      <c r="E885" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F885" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G885" s="4" t="s">
+        <v>982</v>
+      </c>
+      <c r="H885" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I885" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="886" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A886" s="4">
+        <v>885</v>
+      </c>
+      <c r="B886" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C886" s="4">
+        <v>25413</v>
+      </c>
+      <c r="D886" s="2">
+        <v>46128.50340277778</v>
+      </c>
+      <c r="E886" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F886" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G886" s="4" t="s">
+        <v>983</v>
+      </c>
+      <c r="H886" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I886" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="887" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A887" s="4">
+        <v>886</v>
+      </c>
+      <c r="B887" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C887" s="4">
+        <v>22521</v>
+      </c>
+      <c r="D887" s="2">
+        <v>46128.510763888888</v>
+      </c>
+      <c r="E887" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F887" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G887" s="4" t="s">
+        <v>984</v>
+      </c>
+      <c r="H887" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I887" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="888" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A888" s="4">
+        <v>887</v>
+      </c>
+      <c r="B888" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C888" s="4">
+        <v>27290</v>
+      </c>
+      <c r="D888" s="2">
+        <v>46128.514062499999</v>
+      </c>
+      <c r="E888" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F888" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G888" s="4" t="s">
+        <v>985</v>
+      </c>
+      <c r="H888" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I888" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="889" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A889" s="4">
+        <v>888</v>
+      </c>
+      <c r="B889" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C889" s="4">
+        <v>27259</v>
+      </c>
+      <c r="D889" s="2">
+        <v>46128.520358796297</v>
+      </c>
+      <c r="E889" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="F889" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G889" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="H889" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I889" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="890" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A890" s="4">
+        <v>889</v>
+      </c>
+      <c r="B890" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C890" s="4">
+        <v>23975</v>
+      </c>
+      <c r="D890" s="2">
+        <v>46128.522592592592</v>
+      </c>
+      <c r="E890" s="4" t="s">
+        <v>987</v>
+      </c>
+      <c r="F890" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G890" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="H890" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I890" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="891" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A891" s="4">
+        <v>890</v>
+      </c>
+      <c r="B891" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C891" s="4">
+        <v>25634</v>
+      </c>
+      <c r="D891" s="2">
+        <v>46128.531331018516</v>
+      </c>
+      <c r="E891" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F891" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G891" s="4" t="s">
+        <v>989</v>
+      </c>
+      <c r="H891" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I891" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="892" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A892" s="4">
+        <v>891</v>
+      </c>
+      <c r="B892" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C892" s="4">
+        <v>26192</v>
+      </c>
+      <c r="D892" s="2">
+        <v>46129.414282407408</v>
+      </c>
+      <c r="E892" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F892" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G892" s="4" t="s">
+        <v>990</v>
+      </c>
+      <c r="H892" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I892" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="893" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A893" s="4">
+        <v>892</v>
+      </c>
+      <c r="B893" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C893" s="4">
+        <v>12342</v>
+      </c>
+      <c r="D893" s="2">
+        <v>46129.44091435185</v>
+      </c>
+      <c r="E893" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F893" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G893" s="4" t="s">
+        <v>991</v>
+      </c>
+      <c r="H893" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I893" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="894" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A894" s="4">
+        <v>893</v>
+      </c>
+      <c r="B894" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C894" s="4">
+        <v>26882</v>
+      </c>
+      <c r="D894" s="2">
+        <v>46129.46334490741</v>
+      </c>
+      <c r="E894" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F894" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G894" s="4" t="s">
+        <v>992</v>
+      </c>
+      <c r="H894" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I894" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="895" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A895" s="4">
+        <v>894</v>
+      </c>
+      <c r="B895" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C895" s="4">
+        <v>15251</v>
+      </c>
+      <c r="D895" s="2">
+        <v>46129.467581018522</v>
+      </c>
+      <c r="E895" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F895" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G895" s="4" t="s">
+        <v>993</v>
+      </c>
+      <c r="H895" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I895" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="896" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A896" s="4">
+        <v>895</v>
+      </c>
+      <c r="B896" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C896" s="4">
+        <v>11693</v>
+      </c>
+      <c r="D896" s="2">
+        <v>46129.492662037039</v>
+      </c>
+      <c r="E896" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F896" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G896" s="4" t="s">
+        <v>994</v>
+      </c>
+      <c r="H896" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I896" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="897" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A897" s="4">
+        <v>896</v>
+      </c>
+      <c r="B897" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C897" s="4">
+        <v>26646</v>
+      </c>
+      <c r="D897" s="2">
+        <v>46129.582013888888</v>
+      </c>
+      <c r="E897" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F897" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G897" s="4" t="s">
+        <v>995</v>
+      </c>
+      <c r="H897" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I897" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="898" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A898" s="4">
+        <v>897</v>
+      </c>
+      <c r="B898" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C898" s="4">
+        <v>26980</v>
+      </c>
+      <c r="D898" s="2">
+        <v>46129.588877314818</v>
+      </c>
+      <c r="E898" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F898" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G898" s="4" t="s">
+        <v>996</v>
+      </c>
+      <c r="H898" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I898" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="899" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A899" s="4">
+        <v>898</v>
+      </c>
+      <c r="B899" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C899" s="4">
+        <v>25044</v>
+      </c>
+      <c r="D899" s="2">
+        <v>46129.989432870374</v>
+      </c>
+      <c r="E899" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F899" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G899" s="4" t="s">
+        <v>997</v>
+      </c>
+      <c r="H899" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I899" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="900" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A900" s="4">
+        <v>899</v>
+      </c>
+      <c r="B900" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C900" s="4">
+        <v>24562</v>
+      </c>
+      <c r="D900" s="2">
+        <v>46130.076574074075</v>
+      </c>
+      <c r="E900" s="4" t="s">
+        <v>949</v>
+      </c>
+      <c r="F900" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G900" s="4" t="s">
+        <v>998</v>
+      </c>
+      <c r="H900" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I900" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="901" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A901" s="4">
+        <v>900</v>
+      </c>
+      <c r="B901" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C901" s="4">
+        <v>14470</v>
+      </c>
+      <c r="D901" s="2">
+        <v>46131.370949074073</v>
+      </c>
+      <c r="E901" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="F901" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G901" s="4" t="s">
+        <v>999</v>
+      </c>
+      <c r="H901" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I901" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="902" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A902" s="4">
+        <v>901</v>
+      </c>
+      <c r="B902" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C902" s="4">
+        <v>26295</v>
+      </c>
+      <c r="D902" s="2">
+        <v>46132.418773148151</v>
+      </c>
+      <c r="E902" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="F902" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G902" s="4" t="s">
+        <v>1000</v>
+      </c>
+      <c r="H902" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I902" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="903" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A903" s="4">
+        <v>902</v>
+      </c>
+      <c r="B903" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C903" s="4">
+        <v>13273</v>
+      </c>
+      <c r="D903" s="2">
+        <v>46132.439699074072</v>
+      </c>
+      <c r="E903" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="F903" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G903" s="4" t="s">
+        <v>1001</v>
+      </c>
+      <c r="H903" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I903" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="904" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A904" s="4">
+        <v>903</v>
+      </c>
+      <c r="B904" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C904" s="4">
+        <v>30803</v>
+      </c>
+      <c r="D904" s="2">
+        <v>46132.439768518518</v>
+      </c>
+      <c r="E904" s="4" t="s">
+        <v>917</v>
+      </c>
+      <c r="F904" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G904" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H904" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I904" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="905" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A905" s="4">
+        <v>904</v>
+      </c>
+      <c r="B905" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C905" s="4">
+        <v>30198</v>
+      </c>
+      <c r="D905" s="2">
+        <v>46132.441759259258</v>
+      </c>
+      <c r="E905" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F905" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G905" s="4" t="s">
+        <v>1003</v>
+      </c>
+      <c r="H905" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I905" s="4" t="s">
+        <v>765</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 27/04/2026 14:42:19,34
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4F77609-BB1C-4DF1-ABF5-FDA13609C281}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55EE847D-B86D-43B1-8D54-13711B3E0ADA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$905</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$945</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5433" uniqueCount="1004">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5673" uniqueCount="1044">
   <si>
     <t>ID</t>
   </si>
@@ -2427,9 +2427,6 @@
     <t>Estou preocupada com a troca de filtro, faz hj 20 dias q o.filtro foi trocado e já está c a.agua podre. N dá pra.entender.Será q n estão tratando c rigor os filtros pra serem reutilizados</t>
   </si>
   <si>
-    <t>Técnico não cumpriu  agenda</t>
-  </si>
-  <si>
     <t>A pessoa veio até a recepção do condomínio liberei para subir e estou esperando até hoje, porque a pessoa não subiu liguei lá na Brastemp e o Atendente informou que já estava marcando como serviço concluído. Aí expliquei o ocorrido e remarquei a visita.</t>
   </si>
   <si>
@@ -3142,6 +3139,129 @@
   </si>
   <si>
     <t>Solicitei um serviço e veio outro, disseram que voltariam na parte da tarde para finalizar e não apareceram.</t>
+  </si>
+  <si>
+    <t>É bom. Mas não ótimo.</t>
+  </si>
+  <si>
+    <t>AT JOAO PESSOA PB</t>
+  </si>
+  <si>
+    <t>Não foi nada fácil, já tenho um purificador na minha residência, pedi um pra minha mãe, mas foi uma luta, entrei em contato, fiz a solicitação na sexta-feira, a atendente ficou de me enviar o link de pagamento logo depois que desligasse o telefone, não enviou, tive que ligar na segunda uma 4 vezes até que ela entrou em contato e fez o agendamento, o profissional disse que foi até o local na terça-feira, mas meu pai e minha mãe estavam em casa e não escutaram ele chamar, só conseguiram ir na sexta-feira, fizeram a instalação mas deixaram uma mangueira “solta” falando que nãoTinha como fixar, tanto que ela está pedindo para eu ir tentar resolver, eu nunca tive problema, mas a dela foi lamentável.</t>
+  </si>
+  <si>
+    <t>Meu filtro não funciona desde que chegou e agr estão me passando 15 dias para trocarSurrealE eu nem comecei a usar</t>
+  </si>
+  <si>
+    <t>O purificador é ótimo, mas a assistência técnica é péssima.</t>
+  </si>
+  <si>
+    <t>O serviço prestado por vocês é de péssima qualidade. Um total descaso com o cliente.</t>
+  </si>
+  <si>
+    <t>Bem prático</t>
+  </si>
+  <si>
+    <t>Foi boa mas meu purificador está gotejando!</t>
+  </si>
+  <si>
+    <t>Em dois agendamentos de manutenção não houve o comparecimento do técnico e aguardo informações de quando o purificador será substituído, diante do pedido feito pela técnica que veio em visita.</t>
+  </si>
+  <si>
+    <t>Técnico não cumpriu agenda</t>
+  </si>
+  <si>
+    <t>o tempo é  longo de manutenção ( agendamentos )</t>
+  </si>
+  <si>
+    <t>Pessimo atendimento!Marcaram a manutenção após 7 meses , comprometendo a qualidade e fluxo da água.Marquei para o dia 16/04 e ninguém apareceu , tive que marcar novamente para o dia 20/04.O pagamento sempre em dia mas o pós venda sofrível.</t>
+  </si>
+  <si>
+    <t>Lamentável - estou a 2 meses tentando concertar o filtro de água - sistema de refrigeração não funciona - me deram data de 20 de Abril e ninguém apareceu Tentei ligar e fiquei 30 minutos na espera até cair a linha - vou teclar no reclame aqui e na ouvidoria</t>
+  </si>
+  <si>
+    <t>Mesmo após visita do técnico , o barulho é alto do filtro e o jato da água espirra por vezes . Tenho parente que possui o mesmo modelo e não acontece isso</t>
+  </si>
+  <si>
+    <t>Estou tendo um problema pois não está produzindo água gelada. Quando era Brastemp eu nunca tive problemas com o atendimento.O técnico foi em casa e nao solucionou. Estou em viagem nos EUA.Volto pro Brasil em Agosto. Assim que eu voltar vou providenciar o cancelamento da assinatura.</t>
+  </si>
+  <si>
+    <t>Frequência de problemas técnicos</t>
+  </si>
+  <si>
+    <t>Quando o produto dá problema, complicado para resolver. Há mais de um mês com problema no aparelho, falha no atendimento na central. Não confio mais.</t>
+  </si>
+  <si>
+    <t>Muito caro</t>
+  </si>
+  <si>
+    <t>Agendamento e atendimento foram ótimos Porém ter a água fora das condições de consumo em 3 meses é mt desagradável</t>
+  </si>
+  <si>
+    <t>Tudo é excepcional, mas o preço poderia ser melhor e ter mais algum benefício com a mensalidade.</t>
+  </si>
+  <si>
+    <t>O serviço de manutenção do equipamento,  caiu grosseiramente.Anteriormente o técnico trocava o elemento filtrante e limpava o equipamento, também "sangrava" até sair água limpa.Dessa vez, temos três chamados, fora o tempo de atendimento. Nessa 3a vez o equipamento apresentou barulho e o técnico informou que precisará ser trocado.</t>
+  </si>
+  <si>
+    <t>O purificador não se modernizou continua muito grande, toma muito espaço na cozinhal</t>
+  </si>
+  <si>
+    <t>Temos um filtro na empresa , a manutenção preventiva foi feita em 2025 , o tecnico que esteve só limpou o bico com cotonete e não foi realizado a troca do filtro nem a limpeza das tampas que foram desmontadas para a revisão .filtro continou sujo internamente .</t>
+  </si>
+  <si>
+    <t>Após 30 dias solicitando assistencia técnica, finalmente foi dia 23/4. Ficamos 30 dias comprando água. Muito ruim</t>
+  </si>
+  <si>
+    <t>usamos muito o produto e gostamos, mas sempre que temos que agendar uma visita técnica, demora MUITO para acontecer, muitas vezes 2 semanas, isso é inviável para o escritório.</t>
+  </si>
+  <si>
+    <t>Agendei a manutenção do purificador e, após o atendimento, o problema piorou significativamente. O equipamento passou a apresentar vazamento intenso, algo que não ocorria antes.Tentei contato pelo mesmo canal utilizado no agendamento, porém fui orientada a ligar e aguardar atendimento, o que torna o processo pouco eficiente diante da urgência.Além disso, já solicitei a troca ou reparo definitivo do equipamento em outras ocasiões, mas até o momento não houve solução efetiva. Apenas novos chamados são abertos, sem resolução. Inclusive, alguns técnicos informaram que também registraram a necessidade de troca, mas sem qualquer previsão concreta de atendimento. 🤡Neste momento, tenho um problema agravado após a manutenção e preciso de uma solução definitiva, com a maior brevidade possível. Por favor, somente entre em contato para trazer uma solução.</t>
+  </si>
+  <si>
+    <t>Para uma família pequena, como a minha, a relação de custo/benefício não fica tão palatável, no entanto, a praticidade e a qualidade da água fornecida compensam o atual investimento.</t>
+  </si>
+  <si>
+    <t>O técnico foi rápido e solicito.</t>
+  </si>
+  <si>
+    <t>Agendei visita para Dezembro de 2025, porém a mesma não  foi realizada,  a pessoa não  compareceu. Reagendei depois de muito sacrifício para 23/04/2026. A manutenção ocorreu  no período da manhã. No período  da tarde o problema voltou a ocorrer.  Estou insatisfeito,  preciso que seja feito a substituição do aparelho ou cancelamento do contrato.</t>
+  </si>
+  <si>
+    <t>melhorar na identificação do problema de uma simples problema técnico para um problema que impede o uso do purificador e que acaba gerando outro problema que você terá que correr para providenciar galão de água para beber pois o purificador não está funcionando.</t>
+  </si>
+  <si>
+    <t>Atraso, era no expediente da manhã e o técnico veio à tarde.</t>
+  </si>
+  <si>
+    <t>Após a última visita técnica, passou a aquecer demais e a água não está mais gelando. Já solicitei nova visita, mas vou ter que esperar mais de uma semana. Lamentável !!!</t>
+  </si>
+  <si>
+    <t>Após pouco mais de 6 meses de uso, o técnico não trocou o elemento filtrante</t>
+  </si>
+  <si>
+    <t>Água gelada está saindo morna (literalmente). Técnico não orientou sobre a necessidade da compra do gás.Demora para agendamento de visita técnica para corrigir problema relatado no dia da instalação.</t>
+  </si>
+  <si>
+    <t>Marquei tres visitas técnicas, consecutivas,  e ninguem apareceu .Não consigo utilizar os filtros , por que um deles não esta gelando e tivemos casos no predio de hepatite .</t>
+  </si>
+  <si>
+    <t>Vcs dão o cano sem avisar, atrasam e falam que não sabem o apartamento - sendo que já foram várias vezes…Atendimento péssimo e suporte ao cliente horrível.</t>
+  </si>
+  <si>
+    <t>A pessoa veio verificar o problema aqui na minha casa, informe quais eram. Ela me disse que estava "normal". Na verdade a agua não está gelando como sempre gelou e as vezes faz um barulho estranho. Outro ponto, muitas vezes na hora do almoço ou a tarde a agua nem gela - para mim isso é um problema.Sugeri que o filtro fosse trocado, mas ela disse que não poderia fazer pois estava ok.Já tenho contrato com vocês a muito tempo, se não tivesse problema e se não estivesse me incomodando não estaria perdendo meu tempo reclamando a vocês. Esperava uma atitude mais pro ativa da empresa, neste caso me surpreendeu para o mau.</t>
+  </si>
+  <si>
+    <t>Olá, sou cliente desde 2014, estou satisfeita com a qualidade da água, mas há 1 ano meu purificador está superaquecendo e já pedi diversas vezes a substituição, nada foi resolvido. No ano passado o Bruno, técnico, fez um vídeo, enviou para o gerente e não teve solução, vejo que impacta significativamente na conta de energia. Desligo o aparelho sempre que saio e à noite, mas preciso que seja substituído por um mais eficiente.</t>
+  </si>
+  <si>
+    <t>Fiquei mais de 1 mês sem poder usar o purificador porque ele deu defeito e não consegui agendar data. Quando agendei o técnico não veio e da segunda vez que agendei o técnico veio sem a peça necessária para o conserto.</t>
+  </si>
+  <si>
+    <t>Produto de qualidade,  contudo o filtro tem que ser trocado a cada 6 meses, e não por definição da empresa. A solicitação do cliente precisa ser respeitada.</t>
+  </si>
+  <si>
+    <t>O atendimento da Brastemp costumava ser impecável,mas tem piorado. Principalmente nessa mudança de sistema , pq tudo que dá  errado, colocam a culpa na mudança.</t>
   </si>
 </sst>
 </file>
@@ -3514,7 +3634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I905"/>
+  <dimension ref="A1:I945"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -3729,7 +3849,7 @@
         <v>18</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3874,7 +3994,7 @@
         <v>18</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4193,7 +4313,7 @@
         <v>18</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4512,7 +4632,7 @@
         <v>18</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4773,7 +4893,7 @@
         <v>18</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5150,7 +5270,7 @@
         <v>18</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5237,7 +5357,7 @@
         <v>18</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5353,7 +5473,7 @@
         <v>18</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5498,7 +5618,7 @@
         <v>18</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5585,7 +5705,7 @@
         <v>18</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5991,7 +6111,7 @@
         <v>18</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6049,7 +6169,7 @@
         <v>18</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6078,7 +6198,7 @@
         <v>18</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6107,7 +6227,7 @@
         <v>18</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6368,7 +6488,7 @@
         <v>18</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
@@ -6484,7 +6604,7 @@
         <v>18</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6658,7 +6778,7 @@
         <v>18</v>
       </c>
       <c r="I108" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6977,7 +7097,7 @@
         <v>18</v>
       </c>
       <c r="I119" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
@@ -7151,7 +7271,7 @@
         <v>18</v>
       </c>
       <c r="I125" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7441,7 +7561,7 @@
         <v>18</v>
       </c>
       <c r="I135" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7470,7 +7590,7 @@
         <v>18</v>
       </c>
       <c r="I136" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7557,7 +7677,7 @@
         <v>18</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7818,7 +7938,7 @@
         <v>18</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8688,7 +8808,7 @@
         <v>18</v>
       </c>
       <c r="I178" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8775,7 +8895,7 @@
         <v>18</v>
       </c>
       <c r="I181" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8804,7 +8924,7 @@
         <v>18</v>
       </c>
       <c r="I182" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8833,7 +8953,7 @@
         <v>18</v>
       </c>
       <c r="I183" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -8862,7 +8982,7 @@
         <v>18</v>
       </c>
       <c r="I184" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -8920,7 +9040,7 @@
         <v>18</v>
       </c>
       <c r="I186" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9007,7 +9127,7 @@
         <v>18</v>
       </c>
       <c r="I189" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9065,7 +9185,7 @@
         <v>18</v>
       </c>
       <c r="I191" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9152,7 +9272,7 @@
         <v>18</v>
       </c>
       <c r="I194" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9181,7 +9301,7 @@
         <v>18</v>
       </c>
       <c r="I195" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9268,7 +9388,7 @@
         <v>18</v>
       </c>
       <c r="I198" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9384,7 +9504,7 @@
         <v>18</v>
       </c>
       <c r="I202" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9732,7 +9852,7 @@
         <v>18</v>
       </c>
       <c r="I214" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.25">
@@ -9964,7 +10084,7 @@
         <v>18</v>
       </c>
       <c r="I222" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -9993,7 +10113,7 @@
         <v>18</v>
       </c>
       <c r="I223" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10138,7 +10258,7 @@
         <v>18</v>
       </c>
       <c r="I228" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10225,7 +10345,7 @@
         <v>18</v>
       </c>
       <c r="I231" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10341,7 +10461,7 @@
         <v>276</v>
       </c>
       <c r="I235" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10805,7 +10925,7 @@
         <v>18</v>
       </c>
       <c r="I251" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.25">
@@ -10863,7 +10983,7 @@
         <v>18</v>
       </c>
       <c r="I253" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.25">
@@ -11008,7 +11128,7 @@
         <v>18</v>
       </c>
       <c r="I258" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.25">
@@ -11124,7 +11244,7 @@
         <v>18</v>
       </c>
       <c r="I262" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="263" spans="1:9" x14ac:dyDescent="0.25">
@@ -11211,7 +11331,7 @@
         <v>18</v>
       </c>
       <c r="I265" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.25">
@@ -11269,7 +11389,7 @@
         <v>18</v>
       </c>
       <c r="I267" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="268" spans="1:9" x14ac:dyDescent="0.25">
@@ -11588,7 +11708,7 @@
         <v>18</v>
       </c>
       <c r="I278" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="279" spans="1:9" x14ac:dyDescent="0.25">
@@ -11820,7 +11940,7 @@
         <v>18</v>
       </c>
       <c r="I286" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="287" spans="1:9" x14ac:dyDescent="0.25">
@@ -11878,7 +11998,7 @@
         <v>18</v>
       </c>
       <c r="I288" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="289" spans="1:9" x14ac:dyDescent="0.25">
@@ -12052,7 +12172,7 @@
         <v>18</v>
       </c>
       <c r="I294" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.25">
@@ -12139,7 +12259,7 @@
         <v>18</v>
       </c>
       <c r="I297" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
@@ -12197,7 +12317,7 @@
         <v>18</v>
       </c>
       <c r="I299" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="300" spans="1:9" x14ac:dyDescent="0.25">
@@ -12255,7 +12375,7 @@
         <v>18</v>
       </c>
       <c r="I301" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.25">
@@ -12313,7 +12433,7 @@
         <v>18</v>
       </c>
       <c r="I303" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="304" spans="1:9" x14ac:dyDescent="0.25">
@@ -12429,7 +12549,7 @@
         <v>18</v>
       </c>
       <c r="I307" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="308" spans="1:9" x14ac:dyDescent="0.25">
@@ -13183,7 +13303,7 @@
         <v>18</v>
       </c>
       <c r="I333" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="334" spans="1:9" x14ac:dyDescent="0.25">
@@ -13763,7 +13883,7 @@
         <v>18</v>
       </c>
       <c r="I353" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="354" spans="1:9" x14ac:dyDescent="0.25">
@@ -13995,7 +14115,7 @@
         <v>18</v>
       </c>
       <c r="I361" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="362" spans="1:9" x14ac:dyDescent="0.25">
@@ -14285,7 +14405,7 @@
         <v>18</v>
       </c>
       <c r="I371" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="372" spans="1:9" x14ac:dyDescent="0.25">
@@ -14430,7 +14550,7 @@
         <v>18</v>
       </c>
       <c r="I376" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="377" spans="1:9" x14ac:dyDescent="0.25">
@@ -15068,7 +15188,7 @@
         <v>18</v>
       </c>
       <c r="I398" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="399" spans="1:9" x14ac:dyDescent="0.25">
@@ -15329,7 +15449,7 @@
         <v>18</v>
       </c>
       <c r="I407" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="408" spans="1:9" x14ac:dyDescent="0.25">
@@ -15358,7 +15478,7 @@
         <v>18</v>
       </c>
       <c r="I408" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="409" spans="1:9" x14ac:dyDescent="0.25">
@@ -15677,7 +15797,7 @@
         <v>18</v>
       </c>
       <c r="I419" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="420" spans="1:9" x14ac:dyDescent="0.25">
@@ -15706,7 +15826,7 @@
         <v>18</v>
       </c>
       <c r="I420" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="421" spans="1:9" x14ac:dyDescent="0.25">
@@ -15967,7 +16087,7 @@
         <v>18</v>
       </c>
       <c r="I429" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="430" spans="1:9" x14ac:dyDescent="0.25">
@@ -16344,7 +16464,7 @@
         <v>18</v>
       </c>
       <c r="I442" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="443" spans="1:9" x14ac:dyDescent="0.25">
@@ -16460,7 +16580,7 @@
         <v>18</v>
       </c>
       <c r="I446" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="447" spans="1:9" x14ac:dyDescent="0.25">
@@ -17446,7 +17566,7 @@
         <v>18</v>
       </c>
       <c r="I480" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="481" spans="1:9" x14ac:dyDescent="0.25">
@@ -17475,7 +17595,7 @@
         <v>18</v>
       </c>
       <c r="I481" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="482" spans="1:9" x14ac:dyDescent="0.25">
@@ -17707,7 +17827,7 @@
         <v>18</v>
       </c>
       <c r="I489" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="490" spans="1:9" x14ac:dyDescent="0.25">
@@ -17765,7 +17885,7 @@
         <v>18</v>
       </c>
       <c r="I491" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="492" spans="1:9" x14ac:dyDescent="0.25">
@@ -17823,7 +17943,7 @@
         <v>18</v>
       </c>
       <c r="I493" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="494" spans="1:9" x14ac:dyDescent="0.25">
@@ -17939,7 +18059,7 @@
         <v>18</v>
       </c>
       <c r="I497" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="498" spans="1:9" x14ac:dyDescent="0.25">
@@ -18084,7 +18204,7 @@
         <v>18</v>
       </c>
       <c r="I502" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="503" spans="1:9" x14ac:dyDescent="0.25">
@@ -18345,7 +18465,7 @@
         <v>18</v>
       </c>
       <c r="I511" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="512" spans="1:9" x14ac:dyDescent="0.25">
@@ -18519,7 +18639,7 @@
         <v>18</v>
       </c>
       <c r="I517" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="518" spans="1:9" x14ac:dyDescent="0.25">
@@ -18577,7 +18697,7 @@
         <v>18</v>
       </c>
       <c r="I519" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="520" spans="1:9" x14ac:dyDescent="0.25">
@@ -18780,7 +18900,7 @@
         <v>18</v>
       </c>
       <c r="I526" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="527" spans="1:9" x14ac:dyDescent="0.25">
@@ -19650,7 +19770,7 @@
         <v>18</v>
       </c>
       <c r="I556" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.25">
@@ -19708,7 +19828,7 @@
         <v>18</v>
       </c>
       <c r="I558" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="559" spans="1:9" x14ac:dyDescent="0.25">
@@ -19853,7 +19973,7 @@
         <v>18</v>
       </c>
       <c r="I563" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="564" spans="1:9" x14ac:dyDescent="0.25">
@@ -20201,7 +20321,7 @@
         <v>18</v>
       </c>
       <c r="I575" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="576" spans="1:9" x14ac:dyDescent="0.25">
@@ -20723,7 +20843,7 @@
         <v>18</v>
       </c>
       <c r="I593" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="594" spans="1:9" x14ac:dyDescent="0.25">
@@ -21100,7 +21220,7 @@
         <v>18</v>
       </c>
       <c r="I606" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="607" spans="1:9" x14ac:dyDescent="0.25">
@@ -21129,7 +21249,7 @@
         <v>18</v>
       </c>
       <c r="I607" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="608" spans="1:9" x14ac:dyDescent="0.25">
@@ -21883,7 +22003,7 @@
         <v>18</v>
       </c>
       <c r="I633" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="634" spans="1:9" x14ac:dyDescent="0.25">
@@ -21941,7 +22061,7 @@
         <v>18</v>
       </c>
       <c r="I635" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="636" spans="1:9" x14ac:dyDescent="0.25">
@@ -22202,7 +22322,7 @@
         <v>18</v>
       </c>
       <c r="I644" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="645" spans="1:9" x14ac:dyDescent="0.25">
@@ -23501,13 +23621,13 @@
         <v>16</v>
       </c>
       <c r="G689" s="4" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="H689" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I689" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="690" spans="1:9" x14ac:dyDescent="0.25">
@@ -23530,7 +23650,7 @@
         <v>11</v>
       </c>
       <c r="G690" s="4" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="H690" s="4" t="s">
         <v>34</v>
@@ -23559,7 +23679,7 @@
         <v>16</v>
       </c>
       <c r="G691" s="4" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="H691" s="4" t="s">
         <v>18</v>
@@ -23588,7 +23708,7 @@
         <v>16</v>
       </c>
       <c r="G692" s="4" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="H692" s="4" t="s">
         <v>34</v>
@@ -23617,7 +23737,7 @@
         <v>11</v>
       </c>
       <c r="G693" s="4" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="H693" s="4" t="s">
         <v>13</v>
@@ -23646,7 +23766,7 @@
         <v>16</v>
       </c>
       <c r="G694" s="4" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="H694" s="4" t="s">
         <v>18</v>
@@ -23675,13 +23795,13 @@
         <v>16</v>
       </c>
       <c r="G695" s="4" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H695" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I695" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="696" spans="1:9" x14ac:dyDescent="0.25">
@@ -23704,7 +23824,7 @@
         <v>16</v>
       </c>
       <c r="G696" s="4" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="H696" s="4" t="s">
         <v>34</v>
@@ -23733,7 +23853,7 @@
         <v>16</v>
       </c>
       <c r="G697" s="4" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="H697" s="4" t="s">
         <v>18</v>
@@ -23762,7 +23882,7 @@
         <v>11</v>
       </c>
       <c r="G698" s="4" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="H698" s="4" t="s">
         <v>13</v>
@@ -23791,7 +23911,7 @@
         <v>11</v>
       </c>
       <c r="G699" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="H699" s="4" t="s">
         <v>18</v>
@@ -23820,7 +23940,7 @@
         <v>16</v>
       </c>
       <c r="G700" s="4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="H700" s="4" t="s">
         <v>18</v>
@@ -23849,7 +23969,7 @@
         <v>11</v>
       </c>
       <c r="G701" s="4" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="H701" s="4" t="s">
         <v>13</v>
@@ -23878,7 +23998,7 @@
         <v>16</v>
       </c>
       <c r="G702" s="4" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="H702" s="4" t="s">
         <v>80</v>
@@ -23907,7 +24027,7 @@
         <v>16</v>
       </c>
       <c r="G703" s="4" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="H703" s="4" t="s">
         <v>34</v>
@@ -23936,7 +24056,7 @@
         <v>11</v>
       </c>
       <c r="G704" s="4" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="H704" s="4" t="s">
         <v>13</v>
@@ -23965,7 +24085,7 @@
         <v>11</v>
       </c>
       <c r="G705" s="4" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="H705" s="4" t="s">
         <v>13</v>
@@ -23994,7 +24114,7 @@
         <v>11</v>
       </c>
       <c r="G706" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="H706" s="4" t="s">
         <v>13</v>
@@ -24023,7 +24143,7 @@
         <v>16</v>
       </c>
       <c r="G707" s="4" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="H707" s="4" t="s">
         <v>34</v>
@@ -24052,7 +24172,7 @@
         <v>16</v>
       </c>
       <c r="G708" s="4" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H708" s="4" t="s">
         <v>18</v>
@@ -24081,7 +24201,7 @@
         <v>16</v>
       </c>
       <c r="G709" s="4" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="H709" s="4" t="s">
         <v>18</v>
@@ -24110,7 +24230,7 @@
         <v>11</v>
       </c>
       <c r="G710" s="4" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H710" s="4" t="s">
         <v>13</v>
@@ -24139,13 +24259,13 @@
         <v>11</v>
       </c>
       <c r="G711" s="4" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="H711" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I711" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="712" spans="1:9" x14ac:dyDescent="0.25">
@@ -24168,7 +24288,7 @@
         <v>11</v>
       </c>
       <c r="G712" s="4" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="H712" s="4" t="s">
         <v>13</v>
@@ -24197,7 +24317,7 @@
         <v>16</v>
       </c>
       <c r="G713" s="4" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="H713" s="4" t="s">
         <v>13</v>
@@ -24226,7 +24346,7 @@
         <v>16</v>
       </c>
       <c r="G714" s="4" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="H714" s="4" t="s">
         <v>152</v>
@@ -24255,13 +24375,13 @@
         <v>16</v>
       </c>
       <c r="G715" s="4" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="H715" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I715" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="716" spans="1:9" x14ac:dyDescent="0.25">
@@ -24284,7 +24404,7 @@
         <v>16</v>
       </c>
       <c r="G716" s="4" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="H716" s="4" t="s">
         <v>18</v>
@@ -24313,7 +24433,7 @@
         <v>11</v>
       </c>
       <c r="G717" s="4" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="H717" s="4" t="s">
         <v>31</v>
@@ -24342,7 +24462,7 @@
         <v>16</v>
       </c>
       <c r="G718" s="4" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H718" s="4" t="s">
         <v>31</v>
@@ -24371,7 +24491,7 @@
         <v>11</v>
       </c>
       <c r="G719" s="4" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H719" s="4" t="s">
         <v>13</v>
@@ -24400,7 +24520,7 @@
         <v>16</v>
       </c>
       <c r="G720" s="4" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="H720" s="4" t="s">
         <v>18</v>
@@ -24429,7 +24549,7 @@
         <v>11</v>
       </c>
       <c r="G721" s="4" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="H721" s="4" t="s">
         <v>34</v>
@@ -24458,7 +24578,7 @@
         <v>16</v>
       </c>
       <c r="G722" s="4" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="H722" s="4" t="s">
         <v>152</v>
@@ -24487,7 +24607,7 @@
         <v>16</v>
       </c>
       <c r="G723" s="4" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="H723" s="4" t="s">
         <v>18</v>
@@ -24516,7 +24636,7 @@
         <v>11</v>
       </c>
       <c r="G724" s="4" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="H724" s="4" t="s">
         <v>18</v>
@@ -24545,7 +24665,7 @@
         <v>11</v>
       </c>
       <c r="G725" s="4" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="H725" s="4" t="s">
         <v>18</v>
@@ -24574,7 +24694,7 @@
         <v>16</v>
       </c>
       <c r="G726" s="4" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="H726" s="4" t="s">
         <v>80</v>
@@ -24603,7 +24723,7 @@
         <v>16</v>
       </c>
       <c r="G727" s="4" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="H727" s="4" t="s">
         <v>31</v>
@@ -24632,7 +24752,7 @@
         <v>16</v>
       </c>
       <c r="G728" s="4" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H728" s="4" t="s">
         <v>31</v>
@@ -24655,13 +24775,13 @@
         <v>46101.459456018521</v>
       </c>
       <c r="E729" s="4" t="s">
+        <v>805</v>
+      </c>
+      <c r="F729" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G729" s="4" t="s">
         <v>806</v>
-      </c>
-      <c r="F729" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G729" s="4" t="s">
-        <v>807</v>
       </c>
       <c r="H729" s="4" t="s">
         <v>31</v>
@@ -24690,7 +24810,7 @@
         <v>11</v>
       </c>
       <c r="G730" s="4" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="H730" s="4" t="s">
         <v>80</v>
@@ -24719,7 +24839,7 @@
         <v>11</v>
       </c>
       <c r="G731" s="4" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="H731" s="4" t="s">
         <v>13</v>
@@ -24748,7 +24868,7 @@
         <v>16</v>
       </c>
       <c r="G732" s="4" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="H732" s="4" t="s">
         <v>18</v>
@@ -24771,13 +24891,13 @@
         <v>46101.506539351853</v>
       </c>
       <c r="E733" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F733" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G733" s="4" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H733" s="4" t="s">
         <v>13</v>
@@ -24806,7 +24926,7 @@
         <v>16</v>
       </c>
       <c r="G734" s="4" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="H734" s="4" t="s">
         <v>152</v>
@@ -24835,7 +24955,7 @@
         <v>16</v>
       </c>
       <c r="G735" s="4" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="H735" s="4" t="s">
         <v>31</v>
@@ -24864,7 +24984,7 @@
         <v>11</v>
       </c>
       <c r="G736" s="4" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="H736" s="4" t="s">
         <v>31</v>
@@ -24893,7 +25013,7 @@
         <v>11</v>
       </c>
       <c r="G737" s="4" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="H737" s="4" t="s">
         <v>13</v>
@@ -24922,7 +25042,7 @@
         <v>11</v>
       </c>
       <c r="G738" s="4" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="H738" s="4" t="s">
         <v>80</v>
@@ -24951,7 +25071,7 @@
         <v>11</v>
       </c>
       <c r="G739" s="4" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="H739" s="4" t="s">
         <v>13</v>
@@ -24980,7 +25100,7 @@
         <v>16</v>
       </c>
       <c r="G740" s="4" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="H740" s="4" t="s">
         <v>18</v>
@@ -25009,7 +25129,7 @@
         <v>16</v>
       </c>
       <c r="G741" s="4" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="H741" s="4" t="s">
         <v>13</v>
@@ -25038,7 +25158,7 @@
         <v>16</v>
       </c>
       <c r="G742" s="4" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="H742" s="4" t="s">
         <v>18</v>
@@ -25067,7 +25187,7 @@
         <v>16</v>
       </c>
       <c r="G743" s="4" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="H743" s="4" t="s">
         <v>34</v>
@@ -25096,7 +25216,7 @@
         <v>16</v>
       </c>
       <c r="G744" s="4" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="H744" s="4" t="s">
         <v>18</v>
@@ -25125,7 +25245,7 @@
         <v>11</v>
       </c>
       <c r="G745" s="4" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="H745" s="4" t="s">
         <v>34</v>
@@ -25154,7 +25274,7 @@
         <v>11</v>
       </c>
       <c r="G746" s="4" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="H746" s="4" t="s">
         <v>31</v>
@@ -25183,7 +25303,7 @@
         <v>11</v>
       </c>
       <c r="G747" s="4" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="H747" s="4" t="s">
         <v>31</v>
@@ -25212,13 +25332,13 @@
         <v>16</v>
       </c>
       <c r="G748" s="4" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="H748" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I748" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="749" spans="1:9" x14ac:dyDescent="0.25">
@@ -25241,7 +25361,7 @@
         <v>11</v>
       </c>
       <c r="G749" s="4" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="H749" s="4" t="s">
         <v>13</v>
@@ -25270,7 +25390,7 @@
         <v>16</v>
       </c>
       <c r="G750" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="H750" s="4" t="s">
         <v>18</v>
@@ -25299,7 +25419,7 @@
         <v>16</v>
       </c>
       <c r="G751" s="4" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H751" s="4" t="s">
         <v>13</v>
@@ -25328,7 +25448,7 @@
         <v>16</v>
       </c>
       <c r="G752" s="4" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="H752" s="4" t="s">
         <v>18</v>
@@ -25357,7 +25477,7 @@
         <v>11</v>
       </c>
       <c r="G753" s="4" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="H753" s="4" t="s">
         <v>31</v>
@@ -25386,7 +25506,7 @@
         <v>11</v>
       </c>
       <c r="G754" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="H754" s="4" t="s">
         <v>18</v>
@@ -25415,7 +25535,7 @@
         <v>11</v>
       </c>
       <c r="G755" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="H755" s="4" t="s">
         <v>13</v>
@@ -25444,13 +25564,13 @@
         <v>16</v>
       </c>
       <c r="G756" s="4" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H756" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I756" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="757" spans="1:9" x14ac:dyDescent="0.25">
@@ -25473,13 +25593,13 @@
         <v>16</v>
       </c>
       <c r="G757" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="H757" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I757" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="758" spans="1:9" x14ac:dyDescent="0.25">
@@ -25502,13 +25622,13 @@
         <v>16</v>
       </c>
       <c r="G758" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="H758" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I758" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="759" spans="1:9" x14ac:dyDescent="0.25">
@@ -25531,7 +25651,7 @@
         <v>16</v>
       </c>
       <c r="G759" s="4" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="H759" s="4" t="s">
         <v>18</v>
@@ -25560,7 +25680,7 @@
         <v>11</v>
       </c>
       <c r="G760" s="4" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H760" s="4" t="s">
         <v>31</v>
@@ -25589,7 +25709,7 @@
         <v>16</v>
       </c>
       <c r="G761" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="H761" s="4" t="s">
         <v>34</v>
@@ -25618,7 +25738,7 @@
         <v>16</v>
       </c>
       <c r="G762" s="4" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="H762" s="4" t="s">
         <v>31</v>
@@ -25647,7 +25767,7 @@
         <v>11</v>
       </c>
       <c r="G763" s="4" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="H763" s="4" t="s">
         <v>34</v>
@@ -25676,7 +25796,7 @@
         <v>16</v>
       </c>
       <c r="G764" s="4" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="H764" s="4" t="s">
         <v>152</v>
@@ -25705,7 +25825,7 @@
         <v>16</v>
       </c>
       <c r="G765" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="H765" s="4" t="s">
         <v>34</v>
@@ -25734,7 +25854,7 @@
         <v>16</v>
       </c>
       <c r="G766" s="4" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="H766" s="4" t="s">
         <v>31</v>
@@ -25763,7 +25883,7 @@
         <v>11</v>
       </c>
       <c r="G767" s="4" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="H767" s="4" t="s">
         <v>18</v>
@@ -25792,7 +25912,7 @@
         <v>11</v>
       </c>
       <c r="G768" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="H768" s="4" t="s">
         <v>18</v>
@@ -25821,13 +25941,13 @@
         <v>16</v>
       </c>
       <c r="G769" s="4" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="H769" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I769" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="770" spans="1:9" x14ac:dyDescent="0.25">
@@ -25850,7 +25970,7 @@
         <v>16</v>
       </c>
       <c r="G770" s="4" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="H770" s="4" t="s">
         <v>80</v>
@@ -25879,13 +25999,13 @@
         <v>11</v>
       </c>
       <c r="G771" s="4" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="H771" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I771" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="772" spans="1:9" x14ac:dyDescent="0.25">
@@ -25908,7 +26028,7 @@
         <v>16</v>
       </c>
       <c r="G772" s="4" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="H772" s="4" t="s">
         <v>13</v>
@@ -25937,7 +26057,7 @@
         <v>16</v>
       </c>
       <c r="G773" s="4" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="H773" s="4" t="s">
         <v>18</v>
@@ -25966,7 +26086,7 @@
         <v>16</v>
       </c>
       <c r="G774" s="4" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="H774" s="4" t="s">
         <v>34</v>
@@ -25995,7 +26115,7 @@
         <v>11</v>
       </c>
       <c r="G775" s="4" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="H775" s="4" t="s">
         <v>13</v>
@@ -26024,7 +26144,7 @@
         <v>11</v>
       </c>
       <c r="G776" s="4" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="H776" s="4" t="s">
         <v>18</v>
@@ -26053,7 +26173,7 @@
         <v>11</v>
       </c>
       <c r="G777" s="4" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="H777" s="4" t="s">
         <v>13</v>
@@ -26082,7 +26202,7 @@
         <v>16</v>
       </c>
       <c r="G778" s="4" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="H778" s="4" t="s">
         <v>18</v>
@@ -26111,7 +26231,7 @@
         <v>11</v>
       </c>
       <c r="G779" s="4" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="H779" s="4" t="s">
         <v>13</v>
@@ -26140,7 +26260,7 @@
         <v>16</v>
       </c>
       <c r="G780" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="H780" s="4" t="s">
         <v>13</v>
@@ -26169,7 +26289,7 @@
         <v>16</v>
       </c>
       <c r="G781" s="4" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="H781" s="4" t="s">
         <v>18</v>
@@ -26198,7 +26318,7 @@
         <v>16</v>
       </c>
       <c r="G782" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="H782" s="4" t="s">
         <v>31</v>
@@ -26227,7 +26347,7 @@
         <v>16</v>
       </c>
       <c r="G783" s="4" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="H783" s="4" t="s">
         <v>31</v>
@@ -26256,13 +26376,13 @@
         <v>16</v>
       </c>
       <c r="G784" s="4" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="H784" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I784" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="785" spans="1:9" x14ac:dyDescent="0.25">
@@ -26285,7 +26405,7 @@
         <v>16</v>
       </c>
       <c r="G785" s="4" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="H785" s="4" t="s">
         <v>18</v>
@@ -26314,7 +26434,7 @@
         <v>16</v>
       </c>
       <c r="G786" s="4" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="H786" s="4" t="s">
         <v>18</v>
@@ -26343,7 +26463,7 @@
         <v>16</v>
       </c>
       <c r="G787" s="4" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="H787" s="4" t="s">
         <v>31</v>
@@ -26372,13 +26492,13 @@
         <v>16</v>
       </c>
       <c r="G788" s="4" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="H788" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I788" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="789" spans="1:9" x14ac:dyDescent="0.25">
@@ -26401,7 +26521,7 @@
         <v>16</v>
       </c>
       <c r="G789" s="4" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="H789" s="4" t="s">
         <v>80</v>
@@ -26430,7 +26550,7 @@
         <v>16</v>
       </c>
       <c r="G790" s="4" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="H790" s="4" t="s">
         <v>31</v>
@@ -26459,7 +26579,7 @@
         <v>16</v>
       </c>
       <c r="G791" s="4" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="H791" s="4" t="s">
         <v>80</v>
@@ -26488,7 +26608,7 @@
         <v>16</v>
       </c>
       <c r="G792" s="4" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H792" s="4" t="s">
         <v>18</v>
@@ -26517,13 +26637,13 @@
         <v>16</v>
       </c>
       <c r="G793" s="4" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H793" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I793" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="794" spans="1:9" x14ac:dyDescent="0.25">
@@ -26546,7 +26666,7 @@
         <v>11</v>
       </c>
       <c r="G794" s="4" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H794" s="4" t="s">
         <v>152</v>
@@ -26575,7 +26695,7 @@
         <v>11</v>
       </c>
       <c r="G795" s="4" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H795" s="4" t="s">
         <v>13</v>
@@ -26604,7 +26724,7 @@
         <v>16</v>
       </c>
       <c r="G796" s="4" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="H796" s="4" t="s">
         <v>18</v>
@@ -26633,7 +26753,7 @@
         <v>16</v>
       </c>
       <c r="G797" s="4" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="H797" s="4" t="s">
         <v>152</v>
@@ -26662,7 +26782,7 @@
         <v>16</v>
       </c>
       <c r="G798" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="H798" s="4" t="s">
         <v>31</v>
@@ -26691,7 +26811,7 @@
         <v>11</v>
       </c>
       <c r="G799" s="4" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="H799" s="4" t="s">
         <v>34</v>
@@ -26720,7 +26840,7 @@
         <v>16</v>
       </c>
       <c r="G800" s="4" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="H800" s="4" t="s">
         <v>34</v>
@@ -26749,7 +26869,7 @@
         <v>11</v>
       </c>
       <c r="G801" s="4" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="H801" s="4" t="s">
         <v>13</v>
@@ -26778,7 +26898,7 @@
         <v>16</v>
       </c>
       <c r="G802" s="4" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="H802" s="4" t="s">
         <v>34</v>
@@ -26807,13 +26927,13 @@
         <v>16</v>
       </c>
       <c r="G803" s="4" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="H803" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I803" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="804" spans="1:9" x14ac:dyDescent="0.25">
@@ -26836,13 +26956,13 @@
         <v>11</v>
       </c>
       <c r="G804" s="4" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="H804" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I804" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="805" spans="1:9" x14ac:dyDescent="0.25">
@@ -26865,7 +26985,7 @@
         <v>11</v>
       </c>
       <c r="G805" s="4" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="H805" s="4" t="s">
         <v>34</v>
@@ -26894,13 +27014,13 @@
         <v>16</v>
       </c>
       <c r="G806" s="4" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="H806" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I806" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="807" spans="1:9" x14ac:dyDescent="0.25">
@@ -26923,7 +27043,7 @@
         <v>11</v>
       </c>
       <c r="G807" s="4" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="H807" s="4" t="s">
         <v>34</v>
@@ -26952,7 +27072,7 @@
         <v>11</v>
       </c>
       <c r="G808" s="4" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="H808" s="4" t="s">
         <v>13</v>
@@ -26981,7 +27101,7 @@
         <v>16</v>
       </c>
       <c r="G809" s="4" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="H809" s="4" t="s">
         <v>31</v>
@@ -27010,7 +27130,7 @@
         <v>11</v>
       </c>
       <c r="G810" s="4" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="H810" s="4" t="s">
         <v>13</v>
@@ -27039,7 +27159,7 @@
         <v>11</v>
       </c>
       <c r="G811" s="4" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="H811" s="4" t="s">
         <v>18</v>
@@ -27062,13 +27182,13 @@
         <v>46119.454583333332</v>
       </c>
       <c r="E812" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F812" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G812" s="4" t="s">
         <v>890</v>
-      </c>
-      <c r="F812" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G812" s="4" t="s">
-        <v>891</v>
       </c>
       <c r="H812" s="4" t="s">
         <v>13</v>
@@ -27097,7 +27217,7 @@
         <v>16</v>
       </c>
       <c r="G813" s="4" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H813" s="4" t="s">
         <v>18</v>
@@ -27126,7 +27246,7 @@
         <v>16</v>
       </c>
       <c r="G814" s="4" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="H814" s="4" t="s">
         <v>13</v>
@@ -27149,7 +27269,7 @@
         <v>46119.501319444447</v>
       </c>
       <c r="E815" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F815" s="4" t="s">
         <v>11</v>
@@ -27184,13 +27304,13 @@
         <v>16</v>
       </c>
       <c r="G816" s="4" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="H816" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I816" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="817" spans="1:9" x14ac:dyDescent="0.25">
@@ -27207,13 +27327,13 @@
         <v>46119.519618055558</v>
       </c>
       <c r="E817" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="F817" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G817" s="4" t="s">
         <v>896</v>
-      </c>
-      <c r="F817" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G817" s="4" t="s">
-        <v>897</v>
       </c>
       <c r="H817" s="4" t="s">
         <v>18</v>
@@ -27236,13 +27356,13 @@
         <v>46119.525277777779</v>
       </c>
       <c r="E818" s="4" t="s">
+        <v>897</v>
+      </c>
+      <c r="F818" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G818" s="4" t="s">
         <v>898</v>
-      </c>
-      <c r="F818" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G818" s="4" t="s">
-        <v>899</v>
       </c>
       <c r="H818" s="4" t="s">
         <v>80</v>
@@ -27271,7 +27391,7 @@
         <v>16</v>
       </c>
       <c r="G819" s="4" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="H819" s="4" t="s">
         <v>31</v>
@@ -27300,7 +27420,7 @@
         <v>16</v>
       </c>
       <c r="G820" s="4" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="H820" s="4" t="s">
         <v>31</v>
@@ -27329,7 +27449,7 @@
         <v>16</v>
       </c>
       <c r="G821" s="4" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="H821" s="4" t="s">
         <v>80</v>
@@ -27352,13 +27472,13 @@
         <v>46119.668356481481</v>
       </c>
       <c r="E822" s="4" t="s">
+        <v>902</v>
+      </c>
+      <c r="F822" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G822" s="4" t="s">
         <v>903</v>
-      </c>
-      <c r="F822" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G822" s="4" t="s">
-        <v>904</v>
       </c>
       <c r="H822" s="4" t="s">
         <v>31</v>
@@ -27387,7 +27507,7 @@
         <v>16</v>
       </c>
       <c r="G823" s="4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="H823" s="4" t="s">
         <v>18</v>
@@ -27410,19 +27530,19 @@
         <v>46119.913877314815</v>
       </c>
       <c r="E824" s="4" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F824" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G824" s="4" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="H824" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I824" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="825" spans="1:9" x14ac:dyDescent="0.25">
@@ -27445,7 +27565,7 @@
         <v>16</v>
       </c>
       <c r="G825" s="4" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H825" s="4" t="s">
         <v>13</v>
@@ -27474,7 +27594,7 @@
         <v>16</v>
       </c>
       <c r="G826" s="4" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="H826" s="4" t="s">
         <v>18</v>
@@ -27503,7 +27623,7 @@
         <v>16</v>
       </c>
       <c r="G827" s="4" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H827" s="4" t="s">
         <v>62</v>
@@ -27526,13 +27646,13 @@
         <v>46121.387361111112</v>
       </c>
       <c r="E828" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F828" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G828" s="4" t="s">
         <v>910</v>
-      </c>
-      <c r="F828" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G828" s="4" t="s">
-        <v>911</v>
       </c>
       <c r="H828" s="4" t="s">
         <v>18</v>
@@ -27555,13 +27675,13 @@
         <v>46121.431064814817</v>
       </c>
       <c r="E829" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F829" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G829" s="4" t="s">
         <v>912</v>
-      </c>
-      <c r="F829" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G829" s="4" t="s">
-        <v>913</v>
       </c>
       <c r="H829" s="4" t="s">
         <v>18</v>
@@ -27590,7 +27710,7 @@
         <v>16</v>
       </c>
       <c r="G830" s="4" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="H830" s="4" t="s">
         <v>18</v>
@@ -27613,13 +27733,13 @@
         <v>46121.518912037034</v>
       </c>
       <c r="E831" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F831" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G831" s="4" t="s">
         <v>915</v>
-      </c>
-      <c r="F831" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G831" s="4" t="s">
-        <v>916</v>
       </c>
       <c r="H831" s="4" t="s">
         <v>18</v>
@@ -27642,13 +27762,13 @@
         <v>46121.521967592591</v>
       </c>
       <c r="E832" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F832" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G832" s="4" t="s">
         <v>917</v>
-      </c>
-      <c r="F832" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G832" s="4" t="s">
-        <v>918</v>
       </c>
       <c r="H832" s="4" t="s">
         <v>18</v>
@@ -27671,19 +27791,19 @@
         <v>46121.554814814815</v>
       </c>
       <c r="E833" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F833" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G833" s="4" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="H833" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I833" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="834" spans="1:9" x14ac:dyDescent="0.25">
@@ -27700,13 +27820,13 @@
         <v>46121.571666666663</v>
       </c>
       <c r="E834" s="4" t="s">
+        <v>919</v>
+      </c>
+      <c r="F834" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G834" s="4" t="s">
         <v>920</v>
-      </c>
-      <c r="F834" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G834" s="4" t="s">
-        <v>921</v>
       </c>
       <c r="H834" s="4" t="s">
         <v>34</v>
@@ -27729,19 +27849,19 @@
         <v>46121.777638888889</v>
       </c>
       <c r="E835" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F835" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G835" s="4" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="H835" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I835" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="836" spans="1:9" x14ac:dyDescent="0.25">
@@ -27758,13 +27878,13 @@
         <v>46122.372777777775</v>
       </c>
       <c r="E836" s="4" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="F836" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G836" s="4" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="H836" s="4" t="s">
         <v>34</v>
@@ -27787,13 +27907,13 @@
         <v>46122.418773148151</v>
       </c>
       <c r="E837" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F837" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G837" s="4" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="H837" s="4" t="s">
         <v>34</v>
@@ -27816,13 +27936,13 @@
         <v>46122.428414351853</v>
       </c>
       <c r="E838" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F838" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G838" s="4" t="s">
         <v>925</v>
-      </c>
-      <c r="F838" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G838" s="4" t="s">
-        <v>926</v>
       </c>
       <c r="H838" s="4" t="s">
         <v>34</v>
@@ -27845,13 +27965,13 @@
         <v>46122.452303240738</v>
       </c>
       <c r="E839" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F839" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G839" s="4" t="s">
         <v>927</v>
-      </c>
-      <c r="F839" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G839" s="4" t="s">
-        <v>928</v>
       </c>
       <c r="H839" s="4" t="s">
         <v>18</v>
@@ -27874,13 +27994,13 @@
         <v>46122.476840277777</v>
       </c>
       <c r="E840" s="4" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="F840" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G840" s="4" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="H840" s="4" t="s">
         <v>13</v>
@@ -27903,13 +28023,13 @@
         <v>46122.496539351851</v>
       </c>
       <c r="E841" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F841" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G841" s="4" t="s">
         <v>930</v>
-      </c>
-      <c r="F841" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G841" s="4" t="s">
-        <v>931</v>
       </c>
       <c r="H841" s="4" t="s">
         <v>34</v>
@@ -27938,7 +28058,7 @@
         <v>16</v>
       </c>
       <c r="G842" s="4" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="H842" s="4" t="s">
         <v>31</v>
@@ -27967,7 +28087,7 @@
         <v>16</v>
       </c>
       <c r="G843" s="4" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H843" s="4" t="s">
         <v>80</v>
@@ -27990,13 +28110,13 @@
         <v>46122.507511574076</v>
       </c>
       <c r="E844" s="4" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="F844" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G844" s="4" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="H844" s="4" t="s">
         <v>31</v>
@@ -28025,7 +28145,7 @@
         <v>16</v>
       </c>
       <c r="G845" s="4" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="H845" s="4" t="s">
         <v>31</v>
@@ -28048,19 +28168,19 @@
         <v>46123.383101851854</v>
       </c>
       <c r="E846" s="4" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F846" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G846" s="4" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="H846" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I846" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="847" spans="1:9" x14ac:dyDescent="0.25">
@@ -28077,13 +28197,13 @@
         <v>46125.49113425926</v>
       </c>
       <c r="E847" s="4" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F847" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G847" s="4" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="H847" s="4" t="s">
         <v>18</v>
@@ -28106,13 +28226,13 @@
         <v>46125.49858796296</v>
       </c>
       <c r="E848" s="4" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F848" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G848" s="4" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="H848" s="4" t="s">
         <v>31</v>
@@ -28135,13 +28255,13 @@
         <v>46125.509745370371</v>
       </c>
       <c r="E849" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F849" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G849" s="4" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="H849" s="4" t="s">
         <v>31</v>
@@ -28164,13 +28284,13 @@
         <v>46125.516909722224</v>
       </c>
       <c r="E850" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F850" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G850" s="4" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H850" s="4" t="s">
         <v>18</v>
@@ -28193,13 +28313,13 @@
         <v>46125.522083333337</v>
       </c>
       <c r="E851" s="4" t="s">
+        <v>940</v>
+      </c>
+      <c r="F851" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G851" s="4" t="s">
         <v>941</v>
-      </c>
-      <c r="F851" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G851" s="4" t="s">
-        <v>942</v>
       </c>
       <c r="H851" s="4" t="s">
         <v>13</v>
@@ -28228,7 +28348,7 @@
         <v>11</v>
       </c>
       <c r="G852" s="4" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H852" s="4" t="s">
         <v>31</v>
@@ -28251,13 +28371,13 @@
         <v>46125.52920138889</v>
       </c>
       <c r="E853" s="4" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="F853" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G853" s="4" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H853" s="4" t="s">
         <v>18</v>
@@ -28280,19 +28400,19 @@
         <v>46125.537465277775</v>
       </c>
       <c r="E854" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="F854" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G854" s="4" t="s">
         <v>945</v>
       </c>
-      <c r="F854" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G854" s="4" t="s">
-        <v>946</v>
-      </c>
       <c r="H854" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I854" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="855" spans="1:9" x14ac:dyDescent="0.25">
@@ -28309,13 +28429,13 @@
         <v>46125.554016203707</v>
       </c>
       <c r="E855" s="4" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="F855" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G855" s="4" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H855" s="4" t="s">
         <v>13</v>
@@ -28338,13 +28458,13 @@
         <v>46125.556990740741</v>
       </c>
       <c r="E856" s="4" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="F856" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G856" s="4" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="H856" s="4" t="s">
         <v>18</v>
@@ -28367,13 +28487,13 @@
         <v>46125.57539351852</v>
       </c>
       <c r="E857" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="F857" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G857" s="4" t="s">
         <v>949</v>
-      </c>
-      <c r="F857" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G857" s="4" t="s">
-        <v>950</v>
       </c>
       <c r="H857" s="4" t="s">
         <v>34</v>
@@ -28396,13 +28516,13 @@
         <v>46125.576666666668</v>
       </c>
       <c r="E858" s="4" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="F858" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G858" s="4" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H858" s="4" t="s">
         <v>34</v>
@@ -28425,13 +28545,13 @@
         <v>46125.614027777781</v>
       </c>
       <c r="E859" s="4" t="s">
+        <v>951</v>
+      </c>
+      <c r="F859" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G859" s="4" t="s">
         <v>952</v>
-      </c>
-      <c r="F859" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G859" s="4" t="s">
-        <v>953</v>
       </c>
       <c r="H859" s="4" t="s">
         <v>18</v>
@@ -28454,13 +28574,13 @@
         <v>46125.65729166667</v>
       </c>
       <c r="E860" s="4" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="F860" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G860" s="4" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="H860" s="4" t="s">
         <v>13</v>
@@ -28483,13 +28603,13 @@
         <v>46125.799456018518</v>
       </c>
       <c r="E861" s="4" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="F861" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G861" s="4" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="H861" s="4" t="s">
         <v>18</v>
@@ -28512,13 +28632,13 @@
         <v>46125.859236111108</v>
       </c>
       <c r="E862" s="4" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="F862" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G862" s="4" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H862" s="4" t="s">
         <v>18</v>
@@ -28541,13 +28661,13 @@
         <v>46126.382893518516</v>
       </c>
       <c r="E863" s="4" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="F863" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G863" s="4" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="H863" s="4" t="s">
         <v>13</v>
@@ -28576,7 +28696,7 @@
         <v>11</v>
       </c>
       <c r="G864" s="4" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="H864" s="4" t="s">
         <v>13</v>
@@ -28599,13 +28719,13 @@
         <v>46126.437303240738</v>
       </c>
       <c r="E865" s="4" t="s">
+        <v>958</v>
+      </c>
+      <c r="F865" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G865" s="4" t="s">
         <v>959</v>
-      </c>
-      <c r="F865" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G865" s="4" t="s">
-        <v>960</v>
       </c>
       <c r="H865" s="4" t="s">
         <v>34</v>
@@ -28628,13 +28748,13 @@
         <v>46126.519062500003</v>
       </c>
       <c r="E866" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F866" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G866" s="4" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="H866" s="4" t="s">
         <v>34</v>
@@ -28663,7 +28783,7 @@
         <v>11</v>
       </c>
       <c r="G867" s="4" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="H867" s="4" t="s">
         <v>18</v>
@@ -28686,13 +28806,13 @@
         <v>46126.523321759261</v>
       </c>
       <c r="E868" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F868" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G868" s="4" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="H868" s="4" t="s">
         <v>31</v>
@@ -28715,13 +28835,13 @@
         <v>46126.524062500001</v>
       </c>
       <c r="E869" s="4" t="s">
+        <v>963</v>
+      </c>
+      <c r="F869" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G869" s="4" t="s">
         <v>964</v>
-      </c>
-      <c r="F869" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G869" s="4" t="s">
-        <v>965</v>
       </c>
       <c r="H869" s="4" t="s">
         <v>13</v>
@@ -28744,13 +28864,13 @@
         <v>46126.550162037034</v>
       </c>
       <c r="E870" s="4" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F870" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G870" s="4" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="H870" s="4" t="s">
         <v>31</v>
@@ -28773,13 +28893,13 @@
         <v>46126.556284722225</v>
       </c>
       <c r="E871" s="4" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F871" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G871" s="4" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="H871" s="4" t="s">
         <v>34</v>
@@ -28802,13 +28922,13 @@
         <v>46126.596377314818</v>
       </c>
       <c r="E872" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F872" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G872" s="4" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="H872" s="4" t="s">
         <v>13</v>
@@ -28831,19 +28951,19 @@
         <v>46126.597326388888</v>
       </c>
       <c r="E873" s="4" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="F873" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G873" s="4" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="H873" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I873" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="874" spans="1:9" x14ac:dyDescent="0.25">
@@ -28860,13 +28980,13 @@
         <v>46126.716921296298</v>
       </c>
       <c r="E874" s="4" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="F874" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G874" s="4" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="H874" s="4" t="s">
         <v>18</v>
@@ -28889,19 +29009,19 @@
         <v>46127.370266203703</v>
       </c>
       <c r="E875" s="4" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="F875" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G875" s="4" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="H875" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I875" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="876" spans="1:9" x14ac:dyDescent="0.25">
@@ -28918,13 +29038,13 @@
         <v>46127.470659722225</v>
       </c>
       <c r="E876" s="4" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="F876" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G876" s="4" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="H876" s="4" t="s">
         <v>13</v>
@@ -28953,7 +29073,7 @@
         <v>16</v>
       </c>
       <c r="G877" s="4" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="H877" s="4" t="s">
         <v>80</v>
@@ -28982,7 +29102,7 @@
         <v>11</v>
       </c>
       <c r="G878" s="4" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="H878" s="4" t="s">
         <v>34</v>
@@ -29011,7 +29131,7 @@
         <v>11</v>
       </c>
       <c r="G879" s="4" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="H879" s="4" t="s">
         <v>18</v>
@@ -29034,13 +29154,13 @@
         <v>46127.639687499999</v>
       </c>
       <c r="E880" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F880" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G880" s="4" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="H880" s="4" t="s">
         <v>18</v>
@@ -29063,13 +29183,13 @@
         <v>46127.900729166664</v>
       </c>
       <c r="E881" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F881" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G881" s="4" t="s">
         <v>977</v>
-      </c>
-      <c r="F881" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G881" s="4" t="s">
-        <v>978</v>
       </c>
       <c r="H881" s="4" t="s">
         <v>34</v>
@@ -29098,13 +29218,13 @@
         <v>16</v>
       </c>
       <c r="G882" s="4" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="H882" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I882" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="883" spans="1:9" x14ac:dyDescent="0.25">
@@ -29127,7 +29247,7 @@
         <v>11</v>
       </c>
       <c r="G883" s="4" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="H883" s="4" t="s">
         <v>18</v>
@@ -29150,13 +29270,13 @@
         <v>46128.4921875</v>
       </c>
       <c r="E884" s="4" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F884" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G884" s="4" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="H884" s="4" t="s">
         <v>31</v>
@@ -29179,13 +29299,13 @@
         <v>46128.501400462963</v>
       </c>
       <c r="E885" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F885" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G885" s="4" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="H885" s="4" t="s">
         <v>18</v>
@@ -29214,7 +29334,7 @@
         <v>16</v>
       </c>
       <c r="G886" s="4" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="H886" s="4" t="s">
         <v>18</v>
@@ -29243,7 +29363,7 @@
         <v>16</v>
       </c>
       <c r="G887" s="4" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="H887" s="4" t="s">
         <v>31</v>
@@ -29272,7 +29392,7 @@
         <v>11</v>
       </c>
       <c r="G888" s="4" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="H888" s="4" t="s">
         <v>13</v>
@@ -29295,13 +29415,13 @@
         <v>46128.520358796297</v>
       </c>
       <c r="E889" s="4" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="F889" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G889" s="4" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="H889" s="4" t="s">
         <v>34</v>
@@ -29324,13 +29444,13 @@
         <v>46128.522592592592</v>
       </c>
       <c r="E890" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F890" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G890" s="4" t="s">
         <v>987</v>
-      </c>
-      <c r="F890" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G890" s="4" t="s">
-        <v>988</v>
       </c>
       <c r="H890" s="4" t="s">
         <v>34</v>
@@ -29359,7 +29479,7 @@
         <v>16</v>
       </c>
       <c r="G891" s="4" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="H891" s="4" t="s">
         <v>13</v>
@@ -29388,13 +29508,13 @@
         <v>16</v>
       </c>
       <c r="G892" s="4" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="H892" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I892" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="893" spans="1:9" x14ac:dyDescent="0.25">
@@ -29417,7 +29537,7 @@
         <v>16</v>
       </c>
       <c r="G893" s="4" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="H893" s="4" t="s">
         <v>152</v>
@@ -29446,7 +29566,7 @@
         <v>11</v>
       </c>
       <c r="G894" s="4" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="H894" s="4" t="s">
         <v>13</v>
@@ -29469,13 +29589,13 @@
         <v>46129.467581018522</v>
       </c>
       <c r="E895" s="4" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F895" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G895" s="4" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="H895" s="4" t="s">
         <v>31</v>
@@ -29504,7 +29624,7 @@
         <v>11</v>
       </c>
       <c r="G896" s="4" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="H896" s="4" t="s">
         <v>31</v>
@@ -29533,13 +29653,13 @@
         <v>16</v>
       </c>
       <c r="G897" s="4" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="H897" s="4" t="s">
         <v>18</v>
       </c>
       <c r="I897" s="4" t="s">
-        <v>765</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="898" spans="1:9" x14ac:dyDescent="0.25">
@@ -29562,7 +29682,7 @@
         <v>16</v>
       </c>
       <c r="G898" s="4" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="H898" s="4" t="s">
         <v>18</v>
@@ -29591,7 +29711,7 @@
         <v>11</v>
       </c>
       <c r="G899" s="4" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="H899" s="4" t="s">
         <v>18</v>
@@ -29614,13 +29734,13 @@
         <v>46130.076574074075</v>
       </c>
       <c r="E900" s="4" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="F900" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G900" s="4" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="H900" s="4" t="s">
         <v>80</v>
@@ -29643,13 +29763,13 @@
         <v>46131.370949074073</v>
       </c>
       <c r="E901" s="4" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="F901" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G901" s="4" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="H901" s="4" t="s">
         <v>18</v>
@@ -29672,13 +29792,13 @@
         <v>46132.418773148151</v>
       </c>
       <c r="E902" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F902" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G902" s="4" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="H902" s="4" t="s">
         <v>18</v>
@@ -29701,13 +29821,13 @@
         <v>46132.439699074072</v>
       </c>
       <c r="E903" s="4" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F903" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G903" s="4" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="H903" s="4" t="s">
         <v>18</v>
@@ -29730,13 +29850,13 @@
         <v>46132.439768518518</v>
       </c>
       <c r="E904" s="4" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="F904" s="4" t="s">
         <v>16</v>
       </c>
       <c r="G904" s="4" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="H904" s="4" t="s">
         <v>18</v>
@@ -29765,13 +29885,1173 @@
         <v>16</v>
       </c>
       <c r="G905" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H905" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I905" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="906" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A906" s="4">
+        <v>905</v>
+      </c>
+      <c r="B906" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C906" s="4">
+        <v>14480</v>
+      </c>
+      <c r="D906" s="2">
+        <v>46132.513807870368</v>
+      </c>
+      <c r="E906" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F906" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G906" s="4" t="s">
         <v>1003</v>
       </c>
-      <c r="H905" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I905" s="4" t="s">
-        <v>765</v>
+      <c r="H906" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I906" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="907" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A907" s="4">
+        <v>906</v>
+      </c>
+      <c r="B907" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C907" s="4">
+        <v>28800</v>
+      </c>
+      <c r="D907" s="2">
+        <v>46132.515462962961</v>
+      </c>
+      <c r="E907" s="4" t="s">
+        <v>1004</v>
+      </c>
+      <c r="F907" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G907" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="H907" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I907" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="908" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A908" s="4">
+        <v>907</v>
+      </c>
+      <c r="B908" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C908" s="4">
+        <v>30289</v>
+      </c>
+      <c r="D908" s="2">
+        <v>46132.515787037039</v>
+      </c>
+      <c r="E908" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F908" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G908" s="4" t="s">
+        <v>1006</v>
+      </c>
+      <c r="H908" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I908" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="909" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A909" s="4">
+        <v>908</v>
+      </c>
+      <c r="B909" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C909" s="4">
+        <v>28832</v>
+      </c>
+      <c r="D909" s="2">
+        <v>46132.523530092592</v>
+      </c>
+      <c r="E909" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F909" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G909" s="4" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H909" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I909" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="910" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A910" s="4">
+        <v>909</v>
+      </c>
+      <c r="B910" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C910" s="4">
+        <v>24194</v>
+      </c>
+      <c r="D910" s="2">
+        <v>46132.535717592589</v>
+      </c>
+      <c r="E910" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F910" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G910" s="4" t="s">
+        <v>1008</v>
+      </c>
+      <c r="H910" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I910" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="911" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A911" s="4">
+        <v>910</v>
+      </c>
+      <c r="B911" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C911" s="4">
+        <v>16562</v>
+      </c>
+      <c r="D911" s="2">
+        <v>46132.54247685185</v>
+      </c>
+      <c r="E911" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F911" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G911" s="4" t="s">
+        <v>1009</v>
+      </c>
+      <c r="H911" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I911" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="912" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A912" s="4">
+        <v>911</v>
+      </c>
+      <c r="B912" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C912" s="4">
+        <v>28290</v>
+      </c>
+      <c r="D912" s="2">
+        <v>46132.655300925922</v>
+      </c>
+      <c r="E912" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F912" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G912" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H912" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I912" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="913" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A913" s="4">
+        <v>912</v>
+      </c>
+      <c r="B913" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C913" s="4">
+        <v>28358</v>
+      </c>
+      <c r="D913" s="2">
+        <v>46132.671620370369</v>
+      </c>
+      <c r="E913" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F913" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G913" s="4" t="s">
+        <v>1011</v>
+      </c>
+      <c r="H913" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I913" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="914" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A914" s="4">
+        <v>913</v>
+      </c>
+      <c r="B914" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C914" s="4">
+        <v>15835</v>
+      </c>
+      <c r="D914" s="2">
+        <v>46134.421516203707</v>
+      </c>
+      <c r="E914" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F914" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G914" s="4" t="s">
+        <v>1013</v>
+      </c>
+      <c r="H914" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I914" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="915" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A915" s="4">
+        <v>914</v>
+      </c>
+      <c r="B915" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C915" s="4">
+        <v>14147</v>
+      </c>
+      <c r="D915" s="2">
+        <v>46134.509826388887</v>
+      </c>
+      <c r="E915" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F915" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G915" s="4" t="s">
+        <v>1014</v>
+      </c>
+      <c r="H915" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I915" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="916" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A916" s="4">
+        <v>915</v>
+      </c>
+      <c r="B916" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C916" s="4">
+        <v>8852</v>
+      </c>
+      <c r="D916" s="2">
+        <v>46134.517928240741</v>
+      </c>
+      <c r="E916" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F916" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G916" s="4" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H916" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I916" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="917" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A917" s="4">
+        <v>916</v>
+      </c>
+      <c r="B917" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C917" s="4">
+        <v>26673</v>
+      </c>
+      <c r="D917" s="2">
+        <v>46134.540775462963</v>
+      </c>
+      <c r="E917" s="4" t="s">
+        <v>963</v>
+      </c>
+      <c r="F917" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G917" s="4" t="s">
+        <v>1016</v>
+      </c>
+      <c r="H917" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I917" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="918" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A918" s="4">
+        <v>917</v>
+      </c>
+      <c r="B918" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C918" s="4">
+        <v>10890</v>
+      </c>
+      <c r="D918" s="2">
+        <v>46134.614398148151</v>
+      </c>
+      <c r="E918" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F918" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G918" s="4" t="s">
+        <v>1017</v>
+      </c>
+      <c r="H918" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I918" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="919" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A919" s="4">
+        <v>918</v>
+      </c>
+      <c r="B919" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C919" s="4">
+        <v>27790</v>
+      </c>
+      <c r="D919" s="2">
+        <v>46134.769641203704</v>
+      </c>
+      <c r="E919" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F919" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G919" s="4" t="s">
+        <v>1018</v>
+      </c>
+      <c r="H919" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I919" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="920" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A920" s="4">
+        <v>919</v>
+      </c>
+      <c r="B920" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C920" s="4">
+        <v>30428</v>
+      </c>
+      <c r="D920" s="2">
+        <v>46135.401435185187</v>
+      </c>
+      <c r="E920" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F920" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G920" s="4" t="s">
+        <v>1019</v>
+      </c>
+      <c r="H920" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I920" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="921" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A921" s="4">
+        <v>920</v>
+      </c>
+      <c r="B921" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C921" s="4">
+        <v>16685</v>
+      </c>
+      <c r="D921" s="2">
+        <v>46135.413784722223</v>
+      </c>
+      <c r="E921" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F921" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G921" s="4" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H921" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I921" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="922" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A922" s="4">
+        <v>921</v>
+      </c>
+      <c r="B922" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C922" s="4">
+        <v>33179</v>
+      </c>
+      <c r="D922" s="2">
+        <v>46135.508981481478</v>
+      </c>
+      <c r="E922" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F922" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G922" s="4" t="s">
+        <v>1021</v>
+      </c>
+      <c r="H922" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I922" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="923" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A923" s="4">
+        <v>922</v>
+      </c>
+      <c r="B923" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C923" s="4">
+        <v>22790</v>
+      </c>
+      <c r="D923" s="2">
+        <v>46135.558796296296</v>
+      </c>
+      <c r="E923" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F923" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G923" s="4" t="s">
+        <v>1022</v>
+      </c>
+      <c r="H923" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I923" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="924" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A924" s="4">
+        <v>923</v>
+      </c>
+      <c r="B924" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C924" s="4">
+        <v>32181</v>
+      </c>
+      <c r="D924" s="2">
+        <v>46135.654236111113</v>
+      </c>
+      <c r="E924" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F924" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G924" s="4" t="s">
+        <v>1023</v>
+      </c>
+      <c r="H924" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I924" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="925" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A925" s="4">
+        <v>924</v>
+      </c>
+      <c r="B925" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C925" s="4">
+        <v>31439</v>
+      </c>
+      <c r="D925" s="2">
+        <v>46135.690983796296</v>
+      </c>
+      <c r="E925" s="4" t="s">
+        <v>902</v>
+      </c>
+      <c r="F925" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G925" s="4" t="s">
+        <v>1024</v>
+      </c>
+      <c r="H925" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I925" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="926" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A926" s="4">
+        <v>925</v>
+      </c>
+      <c r="B926" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C926" s="4">
+        <v>32429</v>
+      </c>
+      <c r="D926" s="2">
+        <v>46136.377106481479</v>
+      </c>
+      <c r="E926" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F926" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G926" s="4" t="s">
+        <v>1025</v>
+      </c>
+      <c r="H926" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I926" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="927" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A927" s="4">
+        <v>926</v>
+      </c>
+      <c r="B927" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C927" s="4">
+        <v>31703</v>
+      </c>
+      <c r="D927" s="2">
+        <v>46136.409166666665</v>
+      </c>
+      <c r="E927" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="F927" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G927" s="4" t="s">
+        <v>1026</v>
+      </c>
+      <c r="H927" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I927" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="928" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A928" s="4">
+        <v>927</v>
+      </c>
+      <c r="B928" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C928" s="4">
+        <v>27899</v>
+      </c>
+      <c r="D928" s="2">
+        <v>46136.493888888886</v>
+      </c>
+      <c r="E928" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F928" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G928" s="4" t="s">
+        <v>1027</v>
+      </c>
+      <c r="H928" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I928" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="929" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A929" s="4">
+        <v>928</v>
+      </c>
+      <c r="B929" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C929" s="4">
+        <v>32578</v>
+      </c>
+      <c r="D929" s="2">
+        <v>46136.527511574073</v>
+      </c>
+      <c r="E929" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F929" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G929" s="4" t="s">
+        <v>1028</v>
+      </c>
+      <c r="H929" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I929" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="930" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A930" s="4">
+        <v>929</v>
+      </c>
+      <c r="B930" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C930" s="4">
+        <v>28627</v>
+      </c>
+      <c r="D930" s="2">
+        <v>46136.587106481478</v>
+      </c>
+      <c r="E930" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F930" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G930" s="4" t="s">
+        <v>1029</v>
+      </c>
+      <c r="H930" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I930" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="931" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A931" s="4">
+        <v>930</v>
+      </c>
+      <c r="B931" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C931" s="4">
+        <v>33568</v>
+      </c>
+      <c r="D931" s="2">
+        <v>46136.609791666669</v>
+      </c>
+      <c r="E931" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F931" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G931" s="4" t="s">
+        <v>1030</v>
+      </c>
+      <c r="H931" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I931" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="932" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A932" s="4">
+        <v>931</v>
+      </c>
+      <c r="B932" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C932" s="4">
+        <v>26609</v>
+      </c>
+      <c r="D932" s="2">
+        <v>46136.61078703704</v>
+      </c>
+      <c r="E932" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F932" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G932" s="4" t="s">
+        <v>1031</v>
+      </c>
+      <c r="H932" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I932" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="933" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A933" s="4">
+        <v>932</v>
+      </c>
+      <c r="B933" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C933" s="4">
+        <v>25833</v>
+      </c>
+      <c r="D933" s="2">
+        <v>46137.382187499999</v>
+      </c>
+      <c r="E933" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F933" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G933" s="4" t="s">
+        <v>1032</v>
+      </c>
+      <c r="H933" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I933" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="934" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A934" s="4">
+        <v>933</v>
+      </c>
+      <c r="B934" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C934" s="4">
+        <v>27804</v>
+      </c>
+      <c r="D934" s="2">
+        <v>46137.4219212963</v>
+      </c>
+      <c r="E934" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F934" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G934" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="H934" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I934" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="935" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A935" s="4">
+        <v>934</v>
+      </c>
+      <c r="B935" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C935" s="4">
+        <v>31974</v>
+      </c>
+      <c r="D935" s="2">
+        <v>46139.397303240738</v>
+      </c>
+      <c r="E935" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F935" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G935" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="H935" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I935" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="936" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A936" s="4">
+        <v>935</v>
+      </c>
+      <c r="B936" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C936" s="4">
+        <v>10899</v>
+      </c>
+      <c r="D936" s="2">
+        <v>46139.397997685184</v>
+      </c>
+      <c r="E936" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F936" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G936" s="4" t="s">
+        <v>1035</v>
+      </c>
+      <c r="H936" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I936" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="937" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A937" s="4">
+        <v>936</v>
+      </c>
+      <c r="B937" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C937" s="4">
+        <v>34943</v>
+      </c>
+      <c r="D937" s="2">
+        <v>46139.403055555558</v>
+      </c>
+      <c r="E937" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F937" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G937" s="4" t="s">
+        <v>1036</v>
+      </c>
+      <c r="H937" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I937" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="938" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A938" s="4">
+        <v>937</v>
+      </c>
+      <c r="B938" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C938" s="4">
+        <v>14194</v>
+      </c>
+      <c r="D938" s="2">
+        <v>46139.411620370367</v>
+      </c>
+      <c r="E938" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F938" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G938" s="4" t="s">
+        <v>1037</v>
+      </c>
+      <c r="H938" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I938" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="939" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A939" s="4">
+        <v>938</v>
+      </c>
+      <c r="B939" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C939" s="4">
+        <v>28006</v>
+      </c>
+      <c r="D939" s="2">
+        <v>46139.455428240741</v>
+      </c>
+      <c r="E939" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F939" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G939" s="4" t="s">
+        <v>1038</v>
+      </c>
+      <c r="H939" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I939" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="940" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A940" s="4">
+        <v>939</v>
+      </c>
+      <c r="B940" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C940" s="4">
+        <v>33160</v>
+      </c>
+      <c r="D940" s="2">
+        <v>46139.495034722226</v>
+      </c>
+      <c r="E940" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F940" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G940" s="4" t="s">
+        <v>1039</v>
+      </c>
+      <c r="H940" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I940" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="941" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A941" s="4">
+        <v>940</v>
+      </c>
+      <c r="B941" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C941" s="4">
+        <v>32127</v>
+      </c>
+      <c r="D941" s="2">
+        <v>46139.507094907407</v>
+      </c>
+      <c r="E941" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F941" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G941" s="4" t="s">
+        <v>1040</v>
+      </c>
+      <c r="H941" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I941" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="942" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A942" s="4">
+        <v>941</v>
+      </c>
+      <c r="B942" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C942" s="4">
+        <v>30901</v>
+      </c>
+      <c r="D942" s="2">
+        <v>46139.522291666668</v>
+      </c>
+      <c r="E942" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F942" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G942" s="4" t="s">
+        <v>1041</v>
+      </c>
+      <c r="H942" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I942" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="943" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A943" s="4">
+        <v>942</v>
+      </c>
+      <c r="B943" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C943" s="4">
+        <v>16481</v>
+      </c>
+      <c r="D943" s="2">
+        <v>46139.530162037037</v>
+      </c>
+      <c r="E943" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F943" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G943" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H943" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I943" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="944" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A944" s="4">
+        <v>943</v>
+      </c>
+      <c r="B944" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C944" s="4">
+        <v>32785</v>
+      </c>
+      <c r="D944" s="2">
+        <v>46139.558923611112</v>
+      </c>
+      <c r="E944" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F944" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G944" s="4" t="s">
+        <v>1042</v>
+      </c>
+      <c r="H944" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I944" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="945" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A945" s="4">
+        <v>944</v>
+      </c>
+      <c r="B945" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C945" s="4">
+        <v>31243</v>
+      </c>
+      <c r="D945" s="2">
+        <v>46139.568159722221</v>
+      </c>
+      <c r="E945" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F945" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G945" s="4" t="s">
+        <v>1043</v>
+      </c>
+      <c r="H945" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I945" s="4" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 04/05/2026 11:12:17,15
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55EE847D-B86D-43B1-8D54-13711B3E0ADA}"/>
+  <xr:revisionPtr revIDLastSave="237" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E91F81A3-AD50-4F44-A1A1-3790C2269483}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$945</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$977</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5673" uniqueCount="1044">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5865" uniqueCount="1077">
   <si>
     <t>ID</t>
   </si>
@@ -3262,6 +3262,105 @@
   </si>
   <si>
     <t>O atendimento da Brastemp costumava ser impecável,mas tem piorado. Principalmente nessa mudança de sistema , pq tudo que dá  errado, colocam a culpa na mudança.</t>
+  </si>
+  <si>
+    <t>o problema nao foi resolvido.</t>
+  </si>
+  <si>
+    <t>O processo de instalação foi rápido, porém o equipamento apresentou defeito por não ter vindo de fábrica convertido para 220v</t>
+  </si>
+  <si>
+    <t>O horário da visita de vocês é lamentável13:00 hs hora de almoço17:00 hs hora que a responsável pelo atendimento vai emboraVisita apenas periódca faz o teste da agua e vai embora, duração de 5 minutos</t>
+  </si>
+  <si>
+    <t>Purificador é  bom, mas de vez em quando a assistência técnica falha</t>
+  </si>
+  <si>
+    <t>Foi a 3a visita realizada e mais 2 onde não houve comparecimento. O purificador foi trocado e no mesmo dia a água gelada já não funcionava mais. E cada vez que agendo uma visita são 2 semanas pra frente para que ela aconteça.</t>
+  </si>
+  <si>
+    <t>Péssima, pensando em cancelar,pois já faz mas de 1ano que não resolve meu problema cada um que vem fala uma coisa, meu filtro não sai água.</t>
+  </si>
+  <si>
+    <t>FRQ GOIANIA GO</t>
+  </si>
+  <si>
+    <t>Boa tarde segunda vou ligar foi difícil a instalação o cara despreparado.. se não fosse um amigo com uma chave de pressão não teria tirado se quer a torneira do lugar sem matérial.. O purificador não está gelando a água... Eu não indico a Brastemp nem. Para o pior inimigo do mundo....vou ligar segunda e quero providencia..ficar paga só por mês esse valor não dá por um produto....jamais</t>
+  </si>
+  <si>
+    <t>O técnico, chegou após 13hsvisita muito rápido. Trocou somente o filtro e foi embora.Antes qdo era Brastemp limpava o aparelho, testava a água e mostrava.</t>
+  </si>
+  <si>
+    <t>A visita foi agendada com mais de 30 dias de antecedência e simplesmente o técnico não apareceu, não avisou. Estou a oito meses sem manutenção preventiva. Atendimento péssimo, datas para agendamento péssimas. Vou cancelar meu contrato.</t>
+  </si>
+  <si>
+    <t>Toda vez que eu entro em contato para troca do filtro, a agenda leva mais de um mês.Acho inviável.</t>
+  </si>
+  <si>
+    <t>Boa tarde, vai ter que ser trocado devido a quem. E preciso que seja no prazo que o técnico deu 48 horas.Sueli</t>
+  </si>
+  <si>
+    <t>Tudo ok.</t>
+  </si>
+  <si>
+    <t>Gosto bastante do filtro, mas para trocá-lo só temos opção muito cara</t>
+  </si>
+  <si>
+    <t>O aparelho é muito bom, porém, quando é necessário um atendimento técnico, é complicado: datas prevista para visita distante, problemática dos técnicos atenderem no período da tarde, por questão logístico, só atendem minha área no período da manhã, se o cliente trabalhar ou precisar sair neste período, fica sem atendimento, sugiro então, que coloquem técnico que atendam, uns no período da manhã e outros no período da tarde. Fica a dica.</t>
+  </si>
+  <si>
+    <t>Valores superiores ao mercado.</t>
+  </si>
+  <si>
+    <t>Manutenção contratual péssima</t>
+  </si>
+  <si>
+    <t>UM ÓTIMO EQUIPAMENTO, MAS MENSALIDADE CARA PARA ASSALARIADO, ESTOU QUASE DESISTINDO PARA COMPRAR UM SEMILAR, SUM PARCELAS MENSAIS, QUE AJUDA A CORROER AINDA MAIS NOSSO SALÁRIO DE APOSENTADO.</t>
+  </si>
+  <si>
+    <t>1 mês sem água gelada, novamente o técnico veio em minha casa, mexeu e permaneço com água quente. Vocês são bons em produtos, já em serviços prestados é uma desgraça. Estou indignado novamente marcar assistência com agenda lá pra casa do caralho, pois nunca tem data próxima.</t>
+  </si>
+  <si>
+    <t>Acho a assinatura cara demais, mas gosto da qualidade da agua</t>
+  </si>
+  <si>
+    <t>O aparelho funciona bem, mas a reposição do próprio é um processo difícil. O técnico diz que temos que solicitar a troca, pois a anotação na ordem de serviço nao é lida,ao fazer isso a atendente diz que ele que tem que pedir . Enfim estou com fluxo de agua fraco e sem solução</t>
+  </si>
+  <si>
+    <t>Foi tranquilo</t>
+  </si>
+  <si>
+    <t>Normal.</t>
+  </si>
+  <si>
+    <t>O aparelho atende bem, mas poderia ser mais moderno e tecnológico</t>
+  </si>
+  <si>
+    <t>Faz muito tempo que tenho...gosto muito</t>
+  </si>
+  <si>
+    <t>NÃO RECEBEMOS A VISITA TECNICA. POR FAVOR, QUANDO MARCAREM, VENHAM...</t>
+  </si>
+  <si>
+    <t>PROBLEMA NAO RESOLVIDO , FIZ UMA RECLAMAÇÃO DA VISITA ANTERIOR QUE FOI SOLICITADO UMA PEÇA , E VCS ANOTARAM UMA NOVA VISITA TECNICA</t>
+  </si>
+  <si>
+    <t>A instalação foi rápida e tranquila</t>
+  </si>
+  <si>
+    <t>O purificador foi instalado mas a água não está gelando e o técnico não observou isso ou  testou a temperatura para perceber que a água não está gelada , inclusive a água corrente da torneira está numa temperatura mais fresca do que a do purificador</t>
+  </si>
+  <si>
+    <t>Estou com o purificador a 4 meses pingando gerando risco de escorregamento de pessoas.Já foram realizadas mais de 5 visitas sem sucesso em sanar o vazamento</t>
+  </si>
+  <si>
+    <t>Tive péssimas experiências desde a instalação que foi trocada a data várias vzs. Depois, padaria a manutenção, agendei um horário e o técnico foi em outro. Agendei mais 3x e na segunda e terceira não compareceu e na 4a me ligaram dizendo q estava no portão e que não estava funcionando o interfone. Desci pra ver e não tinha ninguém e o interfone estava funcionando sim.Enfim, na 4a vez ele apareceu e fez a troca. Ainda pro cima tentei falar com os telefones que indicam pelo WhatsApp e nada, retornei a ligação para a atendente e não atendia. Enfim, horrível!</t>
+  </si>
+  <si>
+    <t>O purificador 30 minutos após a instalação parou de sair água. Liguei para assistência e me deram até o dia 08 para enviar alguém. Resultado: estou sem água na minha residência e sem perspectiva de retorno</t>
+  </si>
+  <si>
+    <t>Muito boa</t>
   </si>
 </sst>
 </file>
@@ -3634,7 +3733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I945"/>
+  <dimension ref="A1:I977"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -31054,6 +31153,934 @@
         <v>26</v>
       </c>
     </row>
+    <row r="946" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A946" s="4">
+        <v>945</v>
+      </c>
+      <c r="B946" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C946" s="4">
+        <v>33492</v>
+      </c>
+      <c r="D946" s="2">
+        <v>46139.594583333332</v>
+      </c>
+      <c r="E946" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F946" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G946" s="4" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H946" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I946" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="947" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A947" s="4">
+        <v>946</v>
+      </c>
+      <c r="B947" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C947" s="4">
+        <v>33823</v>
+      </c>
+      <c r="D947" s="2">
+        <v>46139.703796296293</v>
+      </c>
+      <c r="E947" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F947" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G947" s="4" t="s">
+        <v>1045</v>
+      </c>
+      <c r="H947" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I947" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="948" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A948" s="4">
+        <v>947</v>
+      </c>
+      <c r="B948" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C948" s="4">
+        <v>31018</v>
+      </c>
+      <c r="D948" s="2">
+        <v>46139.758287037039</v>
+      </c>
+      <c r="E948" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F948" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G948" s="4" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H948" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I948" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="949" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A949" s="4">
+        <v>948</v>
+      </c>
+      <c r="B949" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C949" s="4">
+        <v>35105</v>
+      </c>
+      <c r="D949" s="2">
+        <v>46139.767152777778</v>
+      </c>
+      <c r="E949" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F949" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G949" s="4" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H949" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I949" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="950" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A950" s="4">
+        <v>949</v>
+      </c>
+      <c r="B950" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C950" s="4">
+        <v>21580</v>
+      </c>
+      <c r="D950" s="2">
+        <v>46139.783680555556</v>
+      </c>
+      <c r="E950" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="F950" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G950" s="4" t="s">
+        <v>1048</v>
+      </c>
+      <c r="H950" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I950" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="951" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A951" s="4">
+        <v>950</v>
+      </c>
+      <c r="B951" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C951" s="4">
+        <v>32632</v>
+      </c>
+      <c r="D951" s="2">
+        <v>46139.851458333331</v>
+      </c>
+      <c r="E951" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F951" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G951" s="4" t="s">
+        <v>1049</v>
+      </c>
+      <c r="H951" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I951" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="952" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A952" s="4">
+        <v>951</v>
+      </c>
+      <c r="B952" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C952" s="4">
+        <v>30374</v>
+      </c>
+      <c r="D952" s="2">
+        <v>46140.237013888887</v>
+      </c>
+      <c r="E952" s="4" t="s">
+        <v>1050</v>
+      </c>
+      <c r="F952" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G952" s="4" t="s">
+        <v>1051</v>
+      </c>
+      <c r="H952" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I952" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="953" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A953" s="4">
+        <v>952</v>
+      </c>
+      <c r="B953" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C953" s="4">
+        <v>33664</v>
+      </c>
+      <c r="D953" s="2">
+        <v>46140.390613425923</v>
+      </c>
+      <c r="E953" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F953" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G953" s="4" t="s">
+        <v>1052</v>
+      </c>
+      <c r="H953" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I953" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="954" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A954" s="4">
+        <v>953</v>
+      </c>
+      <c r="B954" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C954" s="4">
+        <v>13602</v>
+      </c>
+      <c r="D954" s="2">
+        <v>46140.406377314815</v>
+      </c>
+      <c r="E954" s="4" t="s">
+        <v>897</v>
+      </c>
+      <c r="F954" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G954" s="4" t="s">
+        <v>1053</v>
+      </c>
+      <c r="H954" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I954" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="955" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A955" s="4">
+        <v>954</v>
+      </c>
+      <c r="B955" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C955" s="4">
+        <v>31161</v>
+      </c>
+      <c r="D955" s="2">
+        <v>46140.408310185187</v>
+      </c>
+      <c r="E955" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F955" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G955" s="4" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H955" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I955" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="956" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A956" s="4">
+        <v>955</v>
+      </c>
+      <c r="B956" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C956" s="4">
+        <v>32150</v>
+      </c>
+      <c r="D956" s="2">
+        <v>46140.572395833333</v>
+      </c>
+      <c r="E956" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F956" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G956" s="4" t="s">
+        <v>1055</v>
+      </c>
+      <c r="H956" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I956" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="957" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A957" s="4">
+        <v>956</v>
+      </c>
+      <c r="B957" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C957" s="4">
+        <v>15584</v>
+      </c>
+      <c r="D957" s="2">
+        <v>46140.580081018517</v>
+      </c>
+      <c r="E957" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F957" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G957" s="4" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H957" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I957" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="958" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A958" s="4">
+        <v>957</v>
+      </c>
+      <c r="B958" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C958" s="4">
+        <v>35589</v>
+      </c>
+      <c r="D958" s="2">
+        <v>46140.581412037034</v>
+      </c>
+      <c r="E958" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F958" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G958" s="4" t="s">
+        <v>1057</v>
+      </c>
+      <c r="H958" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I958" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="959" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A959" s="4">
+        <v>958</v>
+      </c>
+      <c r="B959" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C959" s="4">
+        <v>35974</v>
+      </c>
+      <c r="D959" s="2">
+        <v>46140.58697916667</v>
+      </c>
+      <c r="E959" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F959" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G959" s="4" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H959" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I959" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="960" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A960" s="4">
+        <v>959</v>
+      </c>
+      <c r="B960" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C960" s="4">
+        <v>33020</v>
+      </c>
+      <c r="D960" s="2">
+        <v>46140.638449074075</v>
+      </c>
+      <c r="E960" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F960" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G960" s="4" t="s">
+        <v>1059</v>
+      </c>
+      <c r="H960" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I960" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="961" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A961" s="4">
+        <v>960</v>
+      </c>
+      <c r="B961" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C961" s="4">
+        <v>25498</v>
+      </c>
+      <c r="D961" s="2">
+        <v>46140.710856481484</v>
+      </c>
+      <c r="E961" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F961" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G961" s="4" t="s">
+        <v>1060</v>
+      </c>
+      <c r="H961" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I961" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="962" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A962" s="4">
+        <v>961</v>
+      </c>
+      <c r="B962" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C962" s="4">
+        <v>27088</v>
+      </c>
+      <c r="D962" s="2">
+        <v>46140.788784722223</v>
+      </c>
+      <c r="E962" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F962" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G962" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="H962" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I962" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="963" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A963" s="4">
+        <v>962</v>
+      </c>
+      <c r="B963" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C963" s="4">
+        <v>32542</v>
+      </c>
+      <c r="D963" s="2">
+        <v>46140.878530092596</v>
+      </c>
+      <c r="E963" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F963" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G963" s="4" t="s">
+        <v>1062</v>
+      </c>
+      <c r="H963" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I963" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="964" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A964" s="4">
+        <v>963</v>
+      </c>
+      <c r="B964" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C964" s="4">
+        <v>30409</v>
+      </c>
+      <c r="D964" s="2">
+        <v>46140.97284722222</v>
+      </c>
+      <c r="E964" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F964" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G964" s="4" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H964" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I964" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="965" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A965" s="4">
+        <v>964</v>
+      </c>
+      <c r="B965" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C965" s="4">
+        <v>28441</v>
+      </c>
+      <c r="D965" s="2">
+        <v>46141.409768518519</v>
+      </c>
+      <c r="E965" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F965" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G965" s="4" t="s">
+        <v>1064</v>
+      </c>
+      <c r="H965" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I965" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="966" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A966" s="4">
+        <v>965</v>
+      </c>
+      <c r="B966" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C966" s="4">
+        <v>37198</v>
+      </c>
+      <c r="D966" s="2">
+        <v>46141.503009259257</v>
+      </c>
+      <c r="E966" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F966" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G966" s="4" t="s">
+        <v>1065</v>
+      </c>
+      <c r="H966" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I966" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="967" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A967" s="4">
+        <v>966</v>
+      </c>
+      <c r="B967" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C967" s="4">
+        <v>34368</v>
+      </c>
+      <c r="D967" s="2">
+        <v>46141.518946759257</v>
+      </c>
+      <c r="E967" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F967" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G967" s="4" t="s">
+        <v>1066</v>
+      </c>
+      <c r="H967" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I967" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="968" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A968" s="4">
+        <v>967</v>
+      </c>
+      <c r="B968" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C968" s="4">
+        <v>37144</v>
+      </c>
+      <c r="D968" s="2">
+        <v>46141.54828703704</v>
+      </c>
+      <c r="E968" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F968" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G968" s="4" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H968" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I968" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="969" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A969" s="4">
+        <v>968</v>
+      </c>
+      <c r="B969" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C969" s="4">
+        <v>28428</v>
+      </c>
+      <c r="D969" s="2">
+        <v>46141.6247337963</v>
+      </c>
+      <c r="E969" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F969" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G969" s="4" t="s">
+        <v>1068</v>
+      </c>
+      <c r="H969" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I969" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="970" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A970" s="4">
+        <v>969</v>
+      </c>
+      <c r="B970" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C970" s="4">
+        <v>36435</v>
+      </c>
+      <c r="D970" s="2">
+        <v>46142.381412037037</v>
+      </c>
+      <c r="E970" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F970" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G970" s="4" t="s">
+        <v>1069</v>
+      </c>
+      <c r="H970" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I970" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="971" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A971" s="4">
+        <v>970</v>
+      </c>
+      <c r="B971" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C971" s="4">
+        <v>38103</v>
+      </c>
+      <c r="D971" s="2">
+        <v>46142.501736111109</v>
+      </c>
+      <c r="E971" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F971" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G971" s="4" t="s">
+        <v>1070</v>
+      </c>
+      <c r="H971" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I971" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="972" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A972" s="4">
+        <v>971</v>
+      </c>
+      <c r="B972" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C972" s="4">
+        <v>36141</v>
+      </c>
+      <c r="D972" s="2">
+        <v>46142.504259259258</v>
+      </c>
+      <c r="E972" s="4" t="s">
+        <v>940</v>
+      </c>
+      <c r="F972" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G972" s="4" t="s">
+        <v>1071</v>
+      </c>
+      <c r="H972" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I972" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="973" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A973" s="4">
+        <v>972</v>
+      </c>
+      <c r="B973" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C973" s="4">
+        <v>36982</v>
+      </c>
+      <c r="D973" s="2">
+        <v>46142.514953703707</v>
+      </c>
+      <c r="E973" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F973" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G973" s="4" t="s">
+        <v>1072</v>
+      </c>
+      <c r="H973" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I973" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="974" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A974" s="4">
+        <v>973</v>
+      </c>
+      <c r="B974" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C974" s="4">
+        <v>36539</v>
+      </c>
+      <c r="D974" s="2">
+        <v>46142.516956018517</v>
+      </c>
+      <c r="E974" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F974" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G974" s="4" t="s">
+        <v>1073</v>
+      </c>
+      <c r="H974" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I974" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="975" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A975" s="4">
+        <v>974</v>
+      </c>
+      <c r="B975" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C975" s="4">
+        <v>32833</v>
+      </c>
+      <c r="D975" s="2">
+        <v>46142.519791666666</v>
+      </c>
+      <c r="E975" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F975" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G975" s="4" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H975" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I975" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="976" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A976" s="4">
+        <v>975</v>
+      </c>
+      <c r="B976" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C976" s="4">
+        <v>38299</v>
+      </c>
+      <c r="D976" s="2">
+        <v>46142.523831018516</v>
+      </c>
+      <c r="E976" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F976" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G976" s="4" t="s">
+        <v>1075</v>
+      </c>
+      <c r="H976" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I976" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="977" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A977" s="4">
+        <v>976</v>
+      </c>
+      <c r="B977" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C977" s="4">
+        <v>27403</v>
+      </c>
+      <c r="D977" s="2">
+        <v>46142.543009259258</v>
+      </c>
+      <c r="E977" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F977" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G977" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="H977" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I977" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 11/05/2026 11:48:04,67
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="237" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E91F81A3-AD50-4F44-A1A1-3790C2269483}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E8A968B-EB8E-490A-AE20-57410259325B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5865" uniqueCount="1077">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6237" uniqueCount="1140">
   <si>
     <t>ID</t>
   </si>
@@ -3361,6 +3361,195 @@
   </si>
   <si>
     <t>Muito boa</t>
+  </si>
+  <si>
+    <t>Os técnicos ao trocarem o filtro deveria amostrar ao consumidor lacrado, já que levam o anterior a troca, nada garante que não será usado pra outra pessoa.</t>
+  </si>
+  <si>
+    <t>O atendimento online é péssimoo técnico nunca vem na hora certa</t>
+  </si>
+  <si>
+    <t>Bom dia, depois de muito tempo com vazamento... TRÊS técnicos... troca seria necessária</t>
+  </si>
+  <si>
+    <t>Já quebrou 2 vezes em 3 meses. Não tem o cilindro de gas no site...</t>
+  </si>
+  <si>
+    <t>O defeito permanece e será necessária a substituição de uma peça, que está demorando para ocorrer !</t>
+  </si>
+  <si>
+    <t>Péssima, mesmo com todas as informações enviadas o chamado foi aberto para o técnico com um defeito totalmente diferente</t>
+  </si>
+  <si>
+    <t>A instalação em si não foi problemática... Problemática foi confirmar a instalação. Ora passaram-me números telefônicos...</t>
+  </si>
+  <si>
+    <t>A visita estava agendada para sábado... a técnica veio na quinta sem avisar... não conseguiu reparar</t>
+  </si>
+  <si>
+    <t>Foi realizada a troca do filtro no entanto ele não está gelando como deveria.</t>
+  </si>
+  <si>
+    <t>Não arrumou meu problema</t>
+  </si>
+  <si>
+    <t>Muito bom</t>
+  </si>
+  <si>
+    <t>Desde que entraram em contato... péssimo atendimento... técnico arrogante</t>
+  </si>
+  <si>
+    <t>Serviço mensal caro</t>
+  </si>
+  <si>
+    <t>Após precisar de reparo no purificador, a prestação de serviços tem sido péssima</t>
+  </si>
+  <si>
+    <t>Funciona bem, mas agendar e precisar de assitencia tecnica é uma experiencia bem mediana</t>
+  </si>
+  <si>
+    <t>Pessima experiencia. Marcaram visita, não compareceu... técnico não veio</t>
+  </si>
+  <si>
+    <t>O técnico trocou o filtro, e a pressão da água está muito reduzida</t>
+  </si>
+  <si>
+    <t>LIMPEZA MUITO RÁPIDA E INSATISFATÓRIA</t>
+  </si>
+  <si>
+    <t>unica reclamação que é muito demorado prazo para virem fazer a visita</t>
+  </si>
+  <si>
+    <t>Está vazando desde a instalação. E não consigo agendar reparo urgente</t>
+  </si>
+  <si>
+    <t>Ô purificador de água é satisfatório, contudo tenho observado que ele tem ficado quente</t>
+  </si>
+  <si>
+    <t>Demorou quase 2 meses desde o 1º pedido</t>
+  </si>
+  <si>
+    <t>O rapaz da instalação... muito atencioso... porém após a instalação... água iria gelar após 40 minutos, estou aguardando 4 dias</t>
+  </si>
+  <si>
+    <t>Não tivemos um bom retorno, precisamos de uma nova visita</t>
+  </si>
+  <si>
+    <t>Problema foi resolvido, mas tivemos que esperar mais de uma semana</t>
+  </si>
+  <si>
+    <t>Gosto muito do Purificador Brastemp, porém acho a mensalidade cara.</t>
+  </si>
+  <si>
+    <t>Estava marcado no sábado, técnico não apareceu. Foi aparecer na segunda, sem avisar.</t>
+  </si>
+  <si>
+    <t>marquei o horario tarde , veio 2x pela manhã</t>
+  </si>
+  <si>
+    <t>Não apareceu nenhum técnico para a manutenção</t>
+  </si>
+  <si>
+    <t>toda a vez que é feito a visita o tecnico diz que nunca precisa trocar o filtro</t>
+  </si>
+  <si>
+    <t>a pessoa que veio instalar era extremamente preguiçosa... grosseiro... deixou instalado de qualquer jeito</t>
+  </si>
+  <si>
+    <t>P minha família atende muito bem estamos gostando</t>
+  </si>
+  <si>
+    <t>O purificador é bom! O único porém é o serviço de manutenção que agenda e não comparece.</t>
+  </si>
+  <si>
+    <t>O técnico estava agendado hj na parte da manhã. Ele veio a tarde</t>
+  </si>
+  <si>
+    <t>na anterior, o elemento filtrante não foi trocado... tive que esperar quase 15 dias</t>
+  </si>
+  <si>
+    <t>FRQ PORTO ALEGRE RS</t>
+  </si>
+  <si>
+    <t>Um parente recebeu o técnico.</t>
+  </si>
+  <si>
+    <t>a visita em si foi rápida... Porém o jato de água ficou muito forte</t>
+  </si>
+  <si>
+    <t>a assistência técnica está um pouco demorada</t>
+  </si>
+  <si>
+    <t>o filtro não foi trocado, o técnico disse que estava bom</t>
+  </si>
+  <si>
+    <t>Os serviços não foram efetuados... peças necessárias terão de ser substituídas em nova visita</t>
+  </si>
+  <si>
+    <t>FRQ LIMEIRA SP</t>
+  </si>
+  <si>
+    <t>A manutenção não foi pedida pelo cliente. Foi de rotina.</t>
+  </si>
+  <si>
+    <t>nada</t>
+  </si>
+  <si>
+    <t>Vcs marcam a visita e não aparece ninguém isso já aconteceu 2 x</t>
+  </si>
+  <si>
+    <t>Tive um Problema... agendado uma semana depois. Tive que comprar água</t>
+  </si>
+  <si>
+    <t>quando o mesmo apresenta problemas a comunicação... espera de reparo muito demorada</t>
+  </si>
+  <si>
+    <t>Estou com problema e não foi resolvido.</t>
+  </si>
+  <si>
+    <t>recentemente tenho problemas da máquina e não resolvem na visita técnica</t>
+  </si>
+  <si>
+    <t>Em menos de 1 ano a agua ficou com cheiro de enxofre duas vezes.</t>
+  </si>
+  <si>
+    <t>Nc</t>
+  </si>
+  <si>
+    <t>Qdo precisamos de um tecnico, sempre deixa a desejar, muitas vezes marcam e nao vao</t>
+  </si>
+  <si>
+    <t>Atendimento péssimo Não levaram a borracha para trocar</t>
+  </si>
+  <si>
+    <t>A água é de excelente qualidade, o atendimento técnico é maravilhoso</t>
+  </si>
+  <si>
+    <t>O aparelho é bom e atende as minhas necessidades.</t>
+  </si>
+  <si>
+    <t>pedi troca da vela... não trouxe... pessima experiencia</t>
+  </si>
+  <si>
+    <t>Não trocaram o produto e continua não gelando</t>
+  </si>
+  <si>
+    <t>Praticidade da água gelada</t>
+  </si>
+  <si>
+    <t>Demoraram 2 meses pra vir instalar... cobrança de mensalidade continuou</t>
+  </si>
+  <si>
+    <t>Após a instalação, foi identificado vazamento de água na conexão</t>
+  </si>
+  <si>
+    <t>Veio no horário errado.Bom atendimento.</t>
+  </si>
+  <si>
+    <t>Devido vazamento foi trocado o botão, mas no dia seguinte voltou a dar problema</t>
+  </si>
+  <si>
+    <t>Gosto do purificador, atende a nossa demanda</t>
   </si>
 </sst>
 </file>
@@ -3733,7 +3922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I977"/>
+  <dimension ref="A1:I1039"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -32081,6 +32270,1804 @@
         <v>14</v>
       </c>
     </row>
+    <row r="978" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A978" s="4">
+        <v>977</v>
+      </c>
+      <c r="B978" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C978" s="4">
+        <v>32012</v>
+      </c>
+      <c r="D978" s="2">
+        <v>46143.617372685185</v>
+      </c>
+      <c r="E978" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F978" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G978" s="4" t="s">
+        <v>1077</v>
+      </c>
+      <c r="H978" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I978" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="979" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A979" s="4">
+        <v>978</v>
+      </c>
+      <c r="B979" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C979" s="4">
+        <v>29191</v>
+      </c>
+      <c r="D979" s="2">
+        <v>46144.336875000001</v>
+      </c>
+      <c r="E979" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F979" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G979" s="4" t="s">
+        <v>1078</v>
+      </c>
+      <c r="H979" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I979" s="4" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="980" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A980" s="4">
+        <v>979</v>
+      </c>
+      <c r="B980" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C980" s="4">
+        <v>29089</v>
+      </c>
+      <c r="D980" s="2">
+        <v>46144.402187500003</v>
+      </c>
+      <c r="E980" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F980" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G980" s="4" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H980" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I980" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="981" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A981" s="4">
+        <v>980</v>
+      </c>
+      <c r="B981" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C981" s="4">
+        <v>31383</v>
+      </c>
+      <c r="D981" s="2">
+        <v>46144.652187500003</v>
+      </c>
+      <c r="E981" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="F981" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G981" s="4" t="s">
+        <v>1080</v>
+      </c>
+      <c r="H981" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I981" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="982" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A982" s="4">
+        <v>981</v>
+      </c>
+      <c r="B982" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C982" s="4">
+        <v>36478</v>
+      </c>
+      <c r="D982" s="2">
+        <v>46145.457928240743</v>
+      </c>
+      <c r="E982" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F982" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G982" s="4" t="s">
+        <v>1081</v>
+      </c>
+      <c r="H982" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I982" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="983" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A983" s="4">
+        <v>982</v>
+      </c>
+      <c r="B983" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C983" s="4">
+        <v>28294</v>
+      </c>
+      <c r="D983" s="2">
+        <v>46146.280173611114</v>
+      </c>
+      <c r="E983" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F983" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G983" s="4" t="s">
+        <v>1082</v>
+      </c>
+      <c r="H983" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I983" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="984" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A984" s="4">
+        <v>983</v>
+      </c>
+      <c r="B984" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C984" s="4">
+        <v>34220</v>
+      </c>
+      <c r="D984" s="2">
+        <v>46146.402083333334</v>
+      </c>
+      <c r="E984" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F984" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G984" s="4" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H984" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I984" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="985" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A985" s="4">
+        <v>984</v>
+      </c>
+      <c r="B985" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C985" s="4">
+        <v>36392</v>
+      </c>
+      <c r="D985" s="2">
+        <v>46146.505706018521</v>
+      </c>
+      <c r="E985" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F985" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G985" s="4" t="s">
+        <v>1084</v>
+      </c>
+      <c r="H985" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I985" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="986" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A986" s="4">
+        <v>985</v>
+      </c>
+      <c r="B986" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C986" s="4">
+        <v>36035</v>
+      </c>
+      <c r="D986" s="2">
+        <v>46146.511874999997</v>
+      </c>
+      <c r="E986" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F986" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G986" s="4" t="s">
+        <v>1085</v>
+      </c>
+      <c r="H986" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I986" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="987" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A987" s="4">
+        <v>986</v>
+      </c>
+      <c r="B987" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C987" s="4">
+        <v>38236</v>
+      </c>
+      <c r="D987" s="2">
+        <v>46146.539814814816</v>
+      </c>
+      <c r="E987" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F987" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G987" s="4" t="s">
+        <v>1086</v>
+      </c>
+      <c r="H987" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I987" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="988" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A988" s="4">
+        <v>987</v>
+      </c>
+      <c r="B988" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C988" s="4">
+        <v>40701</v>
+      </c>
+      <c r="D988" s="2">
+        <v>46146.541875000003</v>
+      </c>
+      <c r="E988" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F988" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G988" s="4" t="s">
+        <v>1087</v>
+      </c>
+      <c r="H988" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I988" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="989" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A989" s="4">
+        <v>988</v>
+      </c>
+      <c r="B989" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C989" s="4">
+        <v>38440</v>
+      </c>
+      <c r="D989" s="2">
+        <v>46146.559120370373</v>
+      </c>
+      <c r="E989" s="4" t="s">
+        <v>1050</v>
+      </c>
+      <c r="F989" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G989" s="4" t="s">
+        <v>1088</v>
+      </c>
+      <c r="H989" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I989" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="990" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A990" s="4">
+        <v>989</v>
+      </c>
+      <c r="B990" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C990" s="4">
+        <v>38904</v>
+      </c>
+      <c r="D990" s="2">
+        <v>46146.560567129629</v>
+      </c>
+      <c r="E990" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F990" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G990" s="4" t="s">
+        <v>1089</v>
+      </c>
+      <c r="H990" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I990" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="991" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A991" s="4">
+        <v>990</v>
+      </c>
+      <c r="B991" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C991" s="4">
+        <v>36979</v>
+      </c>
+      <c r="D991" s="2">
+        <v>46146.604699074072</v>
+      </c>
+      <c r="E991" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F991" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G991" s="4" t="s">
+        <v>1090</v>
+      </c>
+      <c r="H991" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I991" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="992" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A992" s="4">
+        <v>991</v>
+      </c>
+      <c r="B992" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C992" s="4">
+        <v>34903</v>
+      </c>
+      <c r="D992" s="2">
+        <v>46146.648182870369</v>
+      </c>
+      <c r="E992" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F992" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G992" s="4" t="s">
+        <v>1091</v>
+      </c>
+      <c r="H992" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I992" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="993" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A993" s="4">
+        <v>992</v>
+      </c>
+      <c r="B993" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C993" s="4">
+        <v>36355</v>
+      </c>
+      <c r="D993" s="2">
+        <v>46146.72215277778</v>
+      </c>
+      <c r="E993" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F993" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G993" s="4" t="s">
+        <v>1092</v>
+      </c>
+      <c r="H993" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I993" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="994" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A994" s="4">
+        <v>993</v>
+      </c>
+      <c r="B994" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C994" s="4">
+        <v>27217</v>
+      </c>
+      <c r="D994" s="2">
+        <v>46146.837314814817</v>
+      </c>
+      <c r="E994" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F994" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G994" s="4" t="s">
+        <v>1093</v>
+      </c>
+      <c r="H994" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I994" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="995" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A995" s="4">
+        <v>994</v>
+      </c>
+      <c r="B995" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C995" s="4">
+        <v>39032</v>
+      </c>
+      <c r="D995" s="2">
+        <v>46147.374340277776</v>
+      </c>
+      <c r="E995" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F995" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G995" s="4" t="s">
+        <v>1094</v>
+      </c>
+      <c r="H995" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I995" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="996" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A996" s="4">
+        <v>995</v>
+      </c>
+      <c r="B996" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C996" s="4">
+        <v>34594</v>
+      </c>
+      <c r="D996" s="2">
+        <v>46147.392372685186</v>
+      </c>
+      <c r="E996" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F996" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G996" s="4" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H996" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I996" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="997" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A997" s="4">
+        <v>996</v>
+      </c>
+      <c r="B997" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C997" s="4">
+        <v>40542</v>
+      </c>
+      <c r="D997" s="2">
+        <v>46147.478333333333</v>
+      </c>
+      <c r="E997" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F997" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G997" s="4" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H997" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I997" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="998" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A998" s="4">
+        <v>997</v>
+      </c>
+      <c r="B998" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C998" s="4">
+        <v>36228</v>
+      </c>
+      <c r="D998" s="2">
+        <v>46147.603125000001</v>
+      </c>
+      <c r="E998" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F998" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G998" s="4" t="s">
+        <v>1097</v>
+      </c>
+      <c r="H998" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I998" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="999" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A999" s="4">
+        <v>998</v>
+      </c>
+      <c r="B999" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C999" s="4">
+        <v>39951</v>
+      </c>
+      <c r="D999" s="2">
+        <v>46147.995289351849</v>
+      </c>
+      <c r="E999" s="4" t="s">
+        <v>958</v>
+      </c>
+      <c r="F999" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G999" s="4" t="s">
+        <v>1098</v>
+      </c>
+      <c r="H999" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I999" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1000" s="4">
+        <v>999</v>
+      </c>
+      <c r="B1000" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1000" s="4">
+        <v>35209</v>
+      </c>
+      <c r="D1000" s="2">
+        <v>46148.181770833333</v>
+      </c>
+      <c r="E1000" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1000" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1000" s="4" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H1000" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1000" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1001" s="4">
+        <v>1000</v>
+      </c>
+      <c r="B1001" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1001" s="4">
+        <v>37352</v>
+      </c>
+      <c r="D1001" s="2">
+        <v>46148.311192129629</v>
+      </c>
+      <c r="E1001" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1001" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1001" s="4" t="s">
+        <v>1100</v>
+      </c>
+      <c r="H1001" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1001" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1002" s="4">
+        <v>1001</v>
+      </c>
+      <c r="B1002" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1002" s="4">
+        <v>33514</v>
+      </c>
+      <c r="D1002" s="2">
+        <v>46148.409745370373</v>
+      </c>
+      <c r="E1002" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1002" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1002" s="4" t="s">
+        <v>1101</v>
+      </c>
+      <c r="H1002" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1002" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1003" s="4">
+        <v>1002</v>
+      </c>
+      <c r="B1003" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1003" s="4">
+        <v>41642</v>
+      </c>
+      <c r="D1003" s="2">
+        <v>46148.474745370368</v>
+      </c>
+      <c r="E1003" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1003" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1003" s="4" t="s">
+        <v>1102</v>
+      </c>
+      <c r="H1003" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1003" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1004" s="4">
+        <v>1003</v>
+      </c>
+      <c r="B1004" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1004" s="4">
+        <v>35222</v>
+      </c>
+      <c r="D1004" s="2">
+        <v>46148.487847222219</v>
+      </c>
+      <c r="E1004" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F1004" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1004" s="4" t="s">
+        <v>1103</v>
+      </c>
+      <c r="H1004" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1004" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1005" s="4">
+        <v>1004</v>
+      </c>
+      <c r="B1005" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1005" s="4">
+        <v>39342</v>
+      </c>
+      <c r="D1005" s="2">
+        <v>46148.492592592593</v>
+      </c>
+      <c r="E1005" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1005" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1005" s="4" t="s">
+        <v>1104</v>
+      </c>
+      <c r="H1005" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1005" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1006" s="4">
+        <v>1005</v>
+      </c>
+      <c r="B1006" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1006" s="4">
+        <v>38814</v>
+      </c>
+      <c r="D1006" s="2">
+        <v>46148.50105324074</v>
+      </c>
+      <c r="E1006" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1006" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1006" s="4" t="s">
+        <v>1105</v>
+      </c>
+      <c r="H1006" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1006" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1007" s="4">
+        <v>1006</v>
+      </c>
+      <c r="B1007" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1007" s="4">
+        <v>39952</v>
+      </c>
+      <c r="D1007" s="2">
+        <v>46148.502650462964</v>
+      </c>
+      <c r="E1007" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1007" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1007" s="4" t="s">
+        <v>1106</v>
+      </c>
+      <c r="H1007" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1007" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1008" s="4">
+        <v>1007</v>
+      </c>
+      <c r="B1008" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1008" s="4">
+        <v>40862</v>
+      </c>
+      <c r="D1008" s="2">
+        <v>46148.503125000003</v>
+      </c>
+      <c r="E1008" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1008" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1008" s="4" t="s">
+        <v>1107</v>
+      </c>
+      <c r="H1008" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1008" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1009" s="4">
+        <v>1008</v>
+      </c>
+      <c r="B1009" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1009" s="4">
+        <v>40136</v>
+      </c>
+      <c r="D1009" s="2">
+        <v>46148.508194444446</v>
+      </c>
+      <c r="E1009" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1009" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1009" s="4" t="s">
+        <v>1108</v>
+      </c>
+      <c r="H1009" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1009" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1010" s="4">
+        <v>1009</v>
+      </c>
+      <c r="B1010" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1010" s="4">
+        <v>39950</v>
+      </c>
+      <c r="D1010" s="2">
+        <v>46148.594085648147</v>
+      </c>
+      <c r="E1010" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1010" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1010" s="4" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H1010" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1010" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1011" s="4">
+        <v>1010</v>
+      </c>
+      <c r="B1011" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1011" s="4">
+        <v>39586</v>
+      </c>
+      <c r="D1011" s="2">
+        <v>46148.696574074071</v>
+      </c>
+      <c r="E1011" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1011" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1011" s="4" t="s">
+        <v>1110</v>
+      </c>
+      <c r="H1011" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1011" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1012" s="4">
+        <v>1011</v>
+      </c>
+      <c r="B1012" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1012" s="4">
+        <v>35612</v>
+      </c>
+      <c r="D1012" s="2">
+        <v>46148.733148148145</v>
+      </c>
+      <c r="E1012" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1012" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1012" s="4" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H1012" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1012" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1013" s="4">
+        <v>1012</v>
+      </c>
+      <c r="B1013" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1013" s="4">
+        <v>32692</v>
+      </c>
+      <c r="D1013" s="2">
+        <v>46149.045590277776</v>
+      </c>
+      <c r="E1013" s="4" t="s">
+        <v>1112</v>
+      </c>
+      <c r="F1013" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1013" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H1013" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1013" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1014" s="4">
+        <v>1013</v>
+      </c>
+      <c r="B1014" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1014" s="4">
+        <v>32982</v>
+      </c>
+      <c r="D1014" s="2">
+        <v>46149.330312500002</v>
+      </c>
+      <c r="E1014" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1014" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1014" s="4" t="s">
+        <v>1114</v>
+      </c>
+      <c r="H1014" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1014" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1015" s="4">
+        <v>1014</v>
+      </c>
+      <c r="B1015" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1015" s="4">
+        <v>30933</v>
+      </c>
+      <c r="D1015" s="2">
+        <v>46149.352280092593</v>
+      </c>
+      <c r="E1015" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1015" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1015" s="4" t="s">
+        <v>1115</v>
+      </c>
+      <c r="H1015" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1015" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1016" s="4">
+        <v>1015</v>
+      </c>
+      <c r="B1016" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1016" s="4">
+        <v>34702</v>
+      </c>
+      <c r="D1016" s="2">
+        <v>46149.504351851851</v>
+      </c>
+      <c r="E1016" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F1016" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1016" s="4" t="s">
+        <v>1116</v>
+      </c>
+      <c r="H1016" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1016" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1017" s="4">
+        <v>1016</v>
+      </c>
+      <c r="B1017" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1017" s="4">
+        <v>34674</v>
+      </c>
+      <c r="D1017" s="2">
+        <v>46149.507951388892</v>
+      </c>
+      <c r="E1017" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1017" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1017" s="4" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H1017" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1017" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1018" s="4">
+        <v>1017</v>
+      </c>
+      <c r="B1018" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1018" s="4">
+        <v>39061</v>
+      </c>
+      <c r="D1018" s="2">
+        <v>46149.508159722223</v>
+      </c>
+      <c r="E1018" s="4" t="s">
+        <v>1118</v>
+      </c>
+      <c r="F1018" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1018" s="4" t="s">
+        <v>1119</v>
+      </c>
+      <c r="H1018" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1018" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1019" s="4">
+        <v>1018</v>
+      </c>
+      <c r="B1019" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1019" s="4">
+        <v>40393</v>
+      </c>
+      <c r="D1019" s="2">
+        <v>46149.509317129632</v>
+      </c>
+      <c r="E1019" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1019" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1019" s="4" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H1019" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1019" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1020" s="4">
+        <v>1019</v>
+      </c>
+      <c r="B1020" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1020" s="4">
+        <v>26780</v>
+      </c>
+      <c r="D1020" s="2">
+        <v>46149.520231481481</v>
+      </c>
+      <c r="E1020" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1020" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1020" s="4" t="s">
+        <v>1121</v>
+      </c>
+      <c r="H1020" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1020" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1021" s="4">
+        <v>1020</v>
+      </c>
+      <c r="B1021" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1021" s="4">
+        <v>36395</v>
+      </c>
+      <c r="D1021" s="2">
+        <v>46149.528819444444</v>
+      </c>
+      <c r="E1021" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1021" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1021" s="4" t="s">
+        <v>1122</v>
+      </c>
+      <c r="H1021" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1021" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1022" s="4">
+        <v>1021</v>
+      </c>
+      <c r="B1022" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1022" s="4">
+        <v>40105</v>
+      </c>
+      <c r="D1022" s="2">
+        <v>46149.56695601852</v>
+      </c>
+      <c r="E1022" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1022" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1022" s="4" t="s">
+        <v>1123</v>
+      </c>
+      <c r="H1022" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1022" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1023" s="4">
+        <v>1022</v>
+      </c>
+      <c r="B1023" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1023" s="4">
+        <v>41029</v>
+      </c>
+      <c r="D1023" s="2">
+        <v>46149.619560185187</v>
+      </c>
+      <c r="E1023" s="4" t="s">
+        <v>902</v>
+      </c>
+      <c r="F1023" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1023" s="4" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H1023" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1023" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1024" s="4">
+        <v>1023</v>
+      </c>
+      <c r="B1024" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1024" s="4">
+        <v>41832</v>
+      </c>
+      <c r="D1024" s="2">
+        <v>46149.645185185182</v>
+      </c>
+      <c r="E1024" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1024" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1024" s="4" t="s">
+        <v>1125</v>
+      </c>
+      <c r="H1024" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1024" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1025" s="4">
+        <v>1024</v>
+      </c>
+      <c r="B1025" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1025" s="4">
+        <v>37597</v>
+      </c>
+      <c r="D1025" s="2">
+        <v>46149.817847222221</v>
+      </c>
+      <c r="E1025" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1025" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1025" s="4" t="s">
+        <v>1126</v>
+      </c>
+      <c r="H1025" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1025" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1026" s="4">
+        <v>1025</v>
+      </c>
+      <c r="B1026" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1026" s="4">
+        <v>40346</v>
+      </c>
+      <c r="D1026" s="2">
+        <v>46150.501261574071</v>
+      </c>
+      <c r="E1026" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1026" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1026" s="4" t="s">
+        <v>1127</v>
+      </c>
+      <c r="H1026" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1026" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1027" s="4">
+        <v>1026</v>
+      </c>
+      <c r="B1027" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1027" s="4">
+        <v>43126</v>
+      </c>
+      <c r="D1027" s="2">
+        <v>46150.502835648149</v>
+      </c>
+      <c r="E1027" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1027" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1027" s="4" t="s">
+        <v>1087</v>
+      </c>
+      <c r="H1027" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1027" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1028" s="4">
+        <v>1027</v>
+      </c>
+      <c r="B1028" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1028" s="4">
+        <v>43155</v>
+      </c>
+      <c r="D1028" s="2">
+        <v>46150.512187499997</v>
+      </c>
+      <c r="E1028" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="F1028" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1028" s="4" t="s">
+        <v>1128</v>
+      </c>
+      <c r="H1028" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1028" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1029" s="4">
+        <v>1028</v>
+      </c>
+      <c r="B1029" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1029" s="4">
+        <v>41244</v>
+      </c>
+      <c r="D1029" s="2">
+        <v>46150.518171296295</v>
+      </c>
+      <c r="E1029" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="F1029" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1029" s="4" t="s">
+        <v>1129</v>
+      </c>
+      <c r="H1029" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1029" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1030" s="4">
+        <v>1029</v>
+      </c>
+      <c r="B1030" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1030" s="4">
+        <v>37569</v>
+      </c>
+      <c r="D1030" s="2">
+        <v>46150.552083333336</v>
+      </c>
+      <c r="E1030" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1030" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1030" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H1030" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1030" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1031" s="4">
+        <v>1030</v>
+      </c>
+      <c r="B1031" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1031" s="4">
+        <v>38732</v>
+      </c>
+      <c r="D1031" s="2">
+        <v>46150.561122685183</v>
+      </c>
+      <c r="E1031" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1031" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1031" s="4" t="s">
+        <v>1131</v>
+      </c>
+      <c r="H1031" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1031" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1032" s="4">
+        <v>1031</v>
+      </c>
+      <c r="B1032" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1032" s="4">
+        <v>39752</v>
+      </c>
+      <c r="D1032" s="2">
+        <v>46150.57267361111</v>
+      </c>
+      <c r="E1032" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1032" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1032" s="4" t="s">
+        <v>1132</v>
+      </c>
+      <c r="H1032" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1032" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1033" s="4">
+        <v>1032</v>
+      </c>
+      <c r="B1033" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1033" s="4">
+        <v>43055</v>
+      </c>
+      <c r="D1033" s="2">
+        <v>46150.750613425924</v>
+      </c>
+      <c r="E1033" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1033" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1033" s="4" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H1033" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1033" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1034" s="4">
+        <v>1033</v>
+      </c>
+      <c r="B1034" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1034" s="4">
+        <v>40032</v>
+      </c>
+      <c r="D1034" s="2">
+        <v>46151.575972222221</v>
+      </c>
+      <c r="E1034" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1034" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1034" s="4" t="s">
+        <v>1134</v>
+      </c>
+      <c r="H1034" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1034" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1035" s="4">
+        <v>1034</v>
+      </c>
+      <c r="B1035" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1035" s="4">
+        <v>42705</v>
+      </c>
+      <c r="D1035" s="2">
+        <v>46152.373668981483</v>
+      </c>
+      <c r="E1035" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1035" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1035" s="4" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H1035" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1035" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1036" s="4">
+        <v>1035</v>
+      </c>
+      <c r="B1036" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1036" s="4">
+        <v>36238</v>
+      </c>
+      <c r="D1036" s="2">
+        <v>46152.657222222224</v>
+      </c>
+      <c r="E1036" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1036" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1036" s="4" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1036" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1036" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1037" s="4">
+        <v>1036</v>
+      </c>
+      <c r="B1037" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1037" s="4">
+        <v>41417</v>
+      </c>
+      <c r="D1037" s="2">
+        <v>46152.740879629629</v>
+      </c>
+      <c r="E1037" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F1037" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1037" s="4" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H1037" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1037" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1038" s="4">
+        <v>1037</v>
+      </c>
+      <c r="B1038" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1038" s="4">
+        <v>39071</v>
+      </c>
+      <c r="D1038" s="2">
+        <v>46153.376805555556</v>
+      </c>
+      <c r="E1038" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1038" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1038" s="4" t="s">
+        <v>1138</v>
+      </c>
+      <c r="H1038" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1038" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1039" s="4">
+        <v>1038</v>
+      </c>
+      <c r="B1039" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1039" s="4">
+        <v>30630</v>
+      </c>
+      <c r="D1039" s="2">
+        <v>46153.412476851852</v>
+      </c>
+      <c r="E1039" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1039" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1039" s="4" t="s">
+        <v>1139</v>
+      </c>
+      <c r="H1039" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1039" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 21/05/2026 11:14:06,91
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="238" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E8A968B-EB8E-490A-AE20-57410259325B}"/>
+  <xr:revisionPtr revIDLastSave="247" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{828ADCCC-FB78-402F-8DB9-B575A1F24DB8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$977</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6237" uniqueCount="1140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6699" uniqueCount="1220">
   <si>
     <t>ID</t>
   </si>
@@ -3550,6 +3550,246 @@
   </si>
   <si>
     <t>Gosto do purificador, atende a nossa demanda</t>
+  </si>
+  <si>
+    <t>Fiquei muito decepcionada com o atendimento, na hora da visita quem atendeu foi meu filho. A técnica que foi abriu o filtro e falou para meu filho que não precisava trocar o filtro, mas eu já estou sentindo gosto de água de torneira. Desde que voltei a ter o filtro Brastemp é a segunda visita técnica de manutenção que recebo, na primeira o técnico falou que estava tudo certo, fez o teste na minha frente e orientou que precisava ser trocado na próxima. Dessa vez meu filho não viu fazendo o teste ou talvez não tenha se atentado, mas minha chateação é a falta de troca de filtro, eu optei em alugar ao invés de comprar um filtro justamente para não me preocupar com a manutenção, mas infelizmente o atendimento caiu muito. Estou pensando seriamente em cancelar a locação. Já tive o filtro Brastemp anteriormente, há uns 6 anos atrás, e nessa época a manutenção era maravilhosa, mas infelizmente agora que voltei a ter só vem me decepcionando.</t>
+  </si>
+  <si>
+    <t>FRQ BRASILIA DF</t>
+  </si>
+  <si>
+    <t>O técnico que vem normalmente fazendo as manutenções periódicas nos atende com muita cordialidade e competência. Entretanto o técnico que realizou a troca do aparelho na semana passada foi muito grosseiro e mal educado.</t>
+  </si>
+  <si>
+    <t>Meu purificador com 10 dias de instalação apresentou problema. Solicitei manutenção. O técnico veio, trocou todas as peças e não resolveu o problema. Solicitou a troca. Entrei em contato com a central e me informaram que o pedido de troca não está no sistema. Tenho que aguardar . Pedi a suspensão do meu faturamento até que chegue o novo purificador , me informaram que não é possível, que posso solicitar o decréscimo da fatura depois. Ou seja, estou pagando por algo que não estou usando e sem previsão para resolver o problema. A atendente por telefone, completamente perdida, não sabia me informar nada.</t>
+  </si>
+  <si>
+    <t>Atendimento um lixo</t>
+  </si>
+  <si>
+    <t>O serviço não foi executado conforme solicitação estou no aguardo com agendamento hoje</t>
+  </si>
+  <si>
+    <t>O canal de atendimento mecanizado é pessimo, não permite compreender o que foi falado.</t>
+  </si>
+  <si>
+    <t>Foi diferente!</t>
+  </si>
+  <si>
+    <t>excelente, apesar de o valor ser muito alto</t>
+  </si>
+  <si>
+    <t>Preço Elevado</t>
+  </si>
+  <si>
+    <t>Meu purificador e maravilhoso.</t>
+  </si>
+  <si>
+    <t>Quando assinei o contrato disponibilizava troca do elemento filtrante a cada 6 meses.Desde 2025 os técnicos relutam para fazer a troca e alegam ser ordem da Brastemp.Isso me faz pensar se devo contar o contrato.A venda para Culligan foi mau comunicada e gerou contatos estranhos para troca do meio de pagamento e deu medo pq eu não sabia quem era Culligan e recebi várias ligações de números que não conheço e links de pagamento. Horrível.</t>
+  </si>
+  <si>
+    <t>o Purificador é ótimo. Só o valor que precisaria ser um pouco mais acessível principalmente para clientes antigos como eu.</t>
+  </si>
+  <si>
+    <t>Atendimento educado, sem problema nenhum com respeito ao profissional,  mas não foi resolvido o problema, e na minha opinião, deveria ter esperado para saber se o problema foi sanado.</t>
+  </si>
+  <si>
+    <t>Nao teve nenhuma visita tecnica nenhuma; Ate faturamento voces tem dificuldade para elitir corretamente e nunca respondem nosso emails e pedidos</t>
+  </si>
+  <si>
+    <t>Tenho marcado várias visitas e nada aconteceu, agora veio e infelizmente eu não estava e fizeram a troca do aparelho e esta danificado porém foi anterior  a essa visita e pelo visto o próprio também não viu</t>
+  </si>
+  <si>
+    <t>Qualidade do produto</t>
+  </si>
+  <si>
+    <t>O técnico não fez nada, não explicou direito e ainda pediu para que eu assinasse um papel, sem ter resolvido nada.</t>
+  </si>
+  <si>
+    <t>Demora excessiva na manutenção...tive que solicitar por 3 vezes...</t>
+  </si>
+  <si>
+    <t>Não houve a manutenção preventiva.  O técnico não apareceu.</t>
+  </si>
+  <si>
+    <t>compareceu 2 horas antes do horario agendado e não me aguardou para informar todos os problemas observados em purificador muito antigo .Fez a manutenção e vou observar seu  funcionamento</t>
+  </si>
+  <si>
+    <t>FRQ MOGI GUACU SP</t>
+  </si>
+  <si>
+    <t>O aparelho está com problema de pouco fluxo de água . Por ser um aparelho modelo mais antigo ( vcs já deveriam ter trocado automaticamente e não o fizeram ) não há peças de reposição . Continuo com o aparelho com problemas , sem previsão de troca e pagando a mensalidade normalmente .</t>
+  </si>
+  <si>
+    <t>Atende nossa necessidade</t>
+  </si>
+  <si>
+    <t>A visita foi boa, técnico educado.O que de fato me incomoda é a dificuldade para a empresa trocar o filtro.Esse serviço era realizado com frequência antes (já chegaram a substituir com  6 meses), agora recebo a informação do técnico que somente daqui a 3 anos. É serio isso? Não deveria ter higienização? Temos altíssimo consumo, uma vez que temos mais de 40 pessoas no escritório. Peço que uma revisão no nosso caso e retorno referente a informação.</t>
+  </si>
+  <si>
+    <t>Péssimo retorno no atendimento ao cliente, aqui é um consultório e fiquei mais de 15 dias sem água, pois estava com cheiro horrível, muita demora na manutenção.</t>
+  </si>
+  <si>
+    <t>Acho cara a mensalidade, na hr do gás nem sempre entra, e o técnico atrasou pra chegar na visita.</t>
+  </si>
+  <si>
+    <t>Lamentável no último ano</t>
+  </si>
+  <si>
+    <t>Equipamento apresenta falhas constantes e péssimo conhecimento e serviço no atendimento técnico!</t>
+  </si>
+  <si>
+    <t>Preço Custo benefício- não estou vendo mais vantagens como no início</t>
+  </si>
+  <si>
+    <t>O aparelho sempre apresenta algum tipo de problema.</t>
+  </si>
+  <si>
+    <t>O técnico diminuiu muito a pressão da água e agora cai um ínfimo fio de água.  Preciso que outro técnico venha corrigir isso.</t>
+  </si>
+  <si>
+    <t>Precisa trocar o equipamento jatem mais de 15 anos</t>
+  </si>
+  <si>
+    <t>Nao trocaram filtro. Fiquei decrpcionada uma vez que a limpeza  ultoma foi em outubro. A tecnica nao tinha foltro pata repor</t>
+  </si>
+  <si>
+    <t>É uma boa opção para quem consome água com gás e quer evitar a garrafa de plástico. O serviço de manutenção foi prático, informativo e eficiente. O preço do cilindro de gás é alto, e a oferta limitada. É preciso melhorar a informação inicial quanto às trocas de cilindro (tipos de cilindros que são compatíveis, onde adquirí-los e como descartá-los)</t>
+  </si>
+  <si>
+    <t>O aparelho é bom mas...</t>
+  </si>
+  <si>
+    <t>Foi ok a visita, mas o técnico na portaria não sabia a senha. Deixamos entrar, mas isso nos deixou muito inseguras. Na verdade, não deveríamos tê-lo recebido.</t>
+  </si>
+  <si>
+    <t>Chamei a assistência técnica porque o purificador estava vazando água. O técnico foi muito gentil ao explicar que será necessária a substituição do aparelho, para o que eu teria de aguardar o contato de outra assessoria técnica. Pena não poder a mesma equipe fazer a substituição. Estou no aguardo.</t>
+  </si>
+  <si>
+    <t>O atendimento é muito ruum, demorou mais de 1 mes pra chegar a uma solução.</t>
+  </si>
+  <si>
+    <t>Agora que troquei o aparelho estou satisfeita</t>
+  </si>
+  <si>
+    <t>Tenho o purificador a algum tempo com vcs, solicitei o técnico para resolver um pequeno vazamento na mangueira, por já ter o equipamento a algum tempo e estou repaginado toda minha casa com móveis novos e planejados sugeri ao técnico a troca por um equipamento mais novo e moderno, e que não tivesse nenhum problema ou vazamento pois poderia danificar os moveis e o prejuízo poderia ser grande, simplesmente o técnico informou que não era possível a troca e que não havia mais vazamento e não era necessário a troca, fiquei chateado com sua resposta pois nem sequer entrou em contato com vcs verificando se havia possibilidade, acho que merecia um outro tratamento por ser cliente a muito tempo.</t>
+  </si>
+  <si>
+    <t>O técnico veio ontem mas deixou o purificador com um vazamento, que só percebemos hoje pela manhã.</t>
+  </si>
+  <si>
+    <t>O purificador precisaria ser trocado por um modelo mais novo, o comprensor está fazendo ruído. É difícil, no entanto, conseguir um atendimento com um representante, que não seja robô, para fazer a solicitação.</t>
+  </si>
+  <si>
+    <t>Gosto muito do purificador. Já uso há muitos anos porém, desde a última visita que ocorreu em novembro/25, foi constatado pelo técnico um defeito no botão da água gelada. O técnico nos informou que informaria a central sobre o problema. Quando fiz este último agendamento, reforcei o defeito não resolvido e novamente o técnico não consertou por nao ter recebido a demanda da central. Portanto continuamos com o botao com defeito. Outro problema é que faço os agendamentos a tarde e o técnico sempre aparece de manhã.</t>
+  </si>
+  <si>
+    <t>Técnico não compareceu na data agendada e não deu nenhum retorno</t>
+  </si>
+  <si>
+    <t>O serviço é bom, mas a manutenção demora a acontecer e o custo é alto.</t>
+  </si>
+  <si>
+    <t>O atendimento é sempre muito solicito, mas por uma problema de logística (falta do equipamento no CD) eu não consegui fazer o upgrade. Soube pelo técnico que meu aparelho está fora de comercialização e não tive uma busca ativa da empresa em me oferecer um novo aparelho</t>
+  </si>
+  <si>
+    <t>Estou sinceramente cansada de prestadores de serviço que não fazem o menor esforço para prestar um atendimento ok, estão sempre agindo e pensando dentro da caixa e jamais podem ir além do mínimo. No agendamento eu solicitei que realizassem a organização da fiação que ficou bagunçada no dia da instalação e solicitei também a instalação do suporte. O prestador disse que só faria a manutenção preventiva porque era o que estava escrito na ordem de serviço.Acontece que eu já havia solicitado as outras coisas no agendamento, mas mesmo assim, só colocaram a manutenção preventiva para ele fazer, e ele só fez o que foi pedido. Zero boa vontade dele e de toda a equipe, que por sinal, nunca tem disponibilidade de data próxima.</t>
+  </si>
+  <si>
+    <t>O purificador foi instalado no dia 22/04 e somente no dia 12/05 foi resolvido o problema do mesmo não estar gelando. Além disso, o problema da instalação do suporte ainda ficou pendente.  Muitos transtornos para um cliente novo.</t>
+  </si>
+  <si>
+    <t>Não veio técnico algum na minha residência....</t>
+  </si>
+  <si>
+    <t>Preço caro</t>
+  </si>
+  <si>
+    <t>Preço alto</t>
+  </si>
+  <si>
+    <t>Carissimo</t>
+  </si>
+  <si>
+    <t>Gosto do produto, mas percebo que não há cuidado com a jornada do cliente, as falhas não são reconhecidas e prontamente solucionadas, para que aconteça qualquer movimento por parte da empresa em direção a solução, seja de falhas financeiras, ou de manutenção, nós os consumidores, somos obrigados a passar por muitos dissabores, esperas longuíssimas, o que tem me feito repensar muito se vale a pena mesmo.</t>
+  </si>
+  <si>
+    <t>Purificador é bom, mas as visitas nao acontecem dentro do planejado</t>
+  </si>
+  <si>
+    <t>Demorou muito - mais de 30 dias - a troca do purificador.</t>
+  </si>
+  <si>
+    <t>Hoje darei nota 07, pois não vieram fazer a manutenção no período correto. No atendimento via fone, a atendente me informou que se ele não ligam agendando, nos clientes que devemos entrar em contato. Achei um absurdo.Tecnico de manuteção não tenho o que reclamar.</t>
+  </si>
+  <si>
+    <t>Não foi pois o técnico simplesmente não apareceu….</t>
+  </si>
+  <si>
+    <t>O atendimento técnico e o agendamento são bem ruins...Eu não agendei nenhuma visita técnica e o técnico simplesmente apareceu na minha casa.</t>
+  </si>
+  <si>
+    <t>to a mais de mês sem água com gás e pagando por isso</t>
+  </si>
+  <si>
+    <t>Ainda não visitaram para resolver o problema</t>
+  </si>
+  <si>
+    <t>Filtro está fazendo muito barulho e agua com gas nao está funcionando.</t>
+  </si>
+  <si>
+    <t>A qualidade do filtro é boa, embora o aparelho seja bastante antigo. A relação custo-benefício poderia ser melhor, ou seja, o custo está elevado para o que é oferecido.</t>
+  </si>
+  <si>
+    <t>Tenho o purificador já faz umbom tempo</t>
+  </si>
+  <si>
+    <t>Ultimamente, minha experiência com o purificador tem sido extremamente frustrante. Enfrentamos problemas com o produto, atraso na troca e, infelizmente, falta de transparência e veracidade nas informações sobre a reposição.Sou cliente há bastante tempo, com uma assinatura de longa data, e é bastante decepcionante perceber que essa fidelidade aparentemente não tem a devida importância para a marca.Esperava um atendimento muito mais respeitoso, transparente e compatível com a confiança que depositei na empresa ao longo de todos esses anos.</t>
+  </si>
+  <si>
+    <t>MUITO DIFICIL. INFORMACOES CONTRADITORIAS SOBRE O MESMO ASSUNTO, NAO HA RETORNO NEM RESPOSTAS, ATENDIMENTO DEMORADO. PRECISEI LIGAR  MAIS VEZES PARA 0BTER RESPOSTAS . SO TROQUEI O PURIFICADOR PARA  ATENDER O DEPARTAMENTO DE CANCELAMENTO . E PRECISO MAIS ATENCAO E EMPENHO DE VOCES COM OS CLIENTES</t>
+  </si>
+  <si>
+    <t>O filtro é muito bom, mas a visita do tecnico nem sempre é adequada.</t>
+  </si>
+  <si>
+    <t>TEMOS DOIS APARELHOS NO MESMO CONTRATO, POREM EM LOJAS DIFERENTESMAS NO MESMO ENDEREÇO! O TECNICO MUNCA SABE DESTA INFORMAÇÃO´, E VÁRIAS VEZES ELE TROCA SOMENTE DE UM FILTRO DE UMA MÁQUINA SÓ</t>
+  </si>
+  <si>
+    <t>Gerenciamento muito ruim, falta de comprometimento, cobranças indevidas sem o cliente ter o produto funcionando. Se possivel gostaria de falar com o responsável pela administração da empresa.</t>
+  </si>
+  <si>
+    <t>Muitas vezes não sai água gaseificada mesmo o reservatório estando com água gelada. Mas nos testes com o técnico no dia da visita , funcionou.</t>
+  </si>
+  <si>
+    <t>O equipamento em si é muito bom. Contudo o nível de serviço ja foi melhor. Principalmente por inicialmente ser um produto diferenciado.</t>
+  </si>
+  <si>
+    <t>Foi péssima, os colaboradores ao invés de resolver o problema acabaram deixando outros, e vazamentos e aborrecimentos... Não indico para ninguém.Outra coisa, NÃO foi da parte do último colaborador que veio aqui em 18/05/26, esse coitado nem sabia de nada só veio como técnico de visita técnica,  e colher minha assinatura referente aos serviços anteriores, e inclusive não havia nem agendamento para o atendimento dele podem consultar desde minha solicitação de datas anteriores foi um sacrifício para tentarem vir até o local da instalação pois o problema originou- se desde 28/03/26</t>
+  </si>
+  <si>
+    <t>Aparelho bom, mas demoram demais para efetuar a troca do filtro.  Para nossa segurança e confiança na empresa, é indispensável conferir  se o filtro está em perfeitas condições de realizar excelente purificação da água. Agendamento da visita técnica é meio demorado  e, dessa vez, atrasou 3 meses.</t>
+  </si>
+  <si>
+    <t>A dificuldade de fazer o pagamento é imensa, vc tenta todos os canais e eles falam liguas diferentes.</t>
+  </si>
+  <si>
+    <t>Sem problema  nenhum. Tudo muito tranquilo cumprindo o que foi determinado no contrato.</t>
+  </si>
+  <si>
+    <t>Não gostei , pois agendei no período da tarde das 13hs as 18hs, e o técnico chegou 11:50 da manhã na minha residência, minha mãe uma senhora idosa de 90 anos teve que atende lo , sendo que eu estaria as 13 HS na minha residência para acompanhar o processo. Detalhe o técnico nem fez a limpeza do purificador</t>
+  </si>
+  <si>
+    <t>Tenho alguns problemas, com a comunicação .</t>
+  </si>
+  <si>
+    <t>Ha mais de 6 meses tentando resolver mas agora acho que vai</t>
+  </si>
+  <si>
+    <t>Bom dia.Solicitei uma visita para verificar resíduos cinzas que estavam saindo na água. Durante a visita, a técnica informou que a pressão da água estava muito forte e que, por isso, os resíduos estavam saindo. Ela reduziu a pressão da água do purificador, porém, mesmo assim, após alguns minutos, a água continua saindo muito forte.Para completar, o local onde fica o cano que liga o purificador à água está vazando.</t>
+  </si>
+  <si>
+    <t>O técnico veio fez o serviço, porem falou que tínhamos que entrar em contato com a central para troca do equipamento, porem a central disse que o técnico deveria solicitar.</t>
   </si>
 </sst>
 </file>
@@ -3922,7 +4162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1039"/>
+  <dimension ref="A1:I1116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -34068,6 +34308,2239 @@
         <v>14</v>
       </c>
     </row>
+    <row r="1040" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1040" s="4">
+        <v>1039</v>
+      </c>
+      <c r="B1040" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1040" s="4">
+        <v>39502</v>
+      </c>
+      <c r="D1040" s="2">
+        <v>46153.430578703701</v>
+      </c>
+      <c r="E1040" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1040" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1040" s="4" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H1040" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1040" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1041" s="4">
+        <v>1040</v>
+      </c>
+      <c r="B1041" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1041" s="4">
+        <v>42656</v>
+      </c>
+      <c r="D1041" s="2">
+        <v>46153.437962962962</v>
+      </c>
+      <c r="E1041" s="4" t="s">
+        <v>1141</v>
+      </c>
+      <c r="F1041" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1041" s="4" t="s">
+        <v>1142</v>
+      </c>
+      <c r="H1041" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1041" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1042" s="4">
+        <v>1041</v>
+      </c>
+      <c r="B1042" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1042" s="4">
+        <v>45349</v>
+      </c>
+      <c r="D1042" s="2">
+        <v>46153.472569444442</v>
+      </c>
+      <c r="E1042" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1042" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1042" s="4" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H1042" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1042" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1043" s="4">
+        <v>1042</v>
+      </c>
+      <c r="B1043" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1043" s="4">
+        <v>42605</v>
+      </c>
+      <c r="D1043" s="2">
+        <v>46153.513923611114</v>
+      </c>
+      <c r="E1043" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1043" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1043" s="4" t="s">
+        <v>1144</v>
+      </c>
+      <c r="H1043" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1043" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1044" s="4">
+        <v>1043</v>
+      </c>
+      <c r="B1044" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1044" s="4">
+        <v>45245</v>
+      </c>
+      <c r="D1044" s="2">
+        <v>46153.514409722222</v>
+      </c>
+      <c r="E1044" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F1044" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1044" s="4" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H1044" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1044" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1045" s="4">
+        <v>1044</v>
+      </c>
+      <c r="B1045" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1045" s="4">
+        <v>42047</v>
+      </c>
+      <c r="D1045" s="2">
+        <v>46153.514560185184</v>
+      </c>
+      <c r="E1045" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1045" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1045" s="4" t="s">
+        <v>1146</v>
+      </c>
+      <c r="H1045" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1045" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1046" s="4">
+        <v>1045</v>
+      </c>
+      <c r="B1046" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1046" s="4">
+        <v>28017</v>
+      </c>
+      <c r="D1046" s="2">
+        <v>46153.521180555559</v>
+      </c>
+      <c r="E1046" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1046" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1046" s="4" t="s">
+        <v>1147</v>
+      </c>
+      <c r="H1046" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1046" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1047" s="4">
+        <v>1046</v>
+      </c>
+      <c r="B1047" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1047" s="4">
+        <v>43475</v>
+      </c>
+      <c r="D1047" s="2">
+        <v>46153.532430555555</v>
+      </c>
+      <c r="E1047" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1047" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1047" s="4" t="s">
+        <v>1148</v>
+      </c>
+      <c r="H1047" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1047" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1048" s="4">
+        <v>1047</v>
+      </c>
+      <c r="B1048" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1048" s="4">
+        <v>39783</v>
+      </c>
+      <c r="D1048" s="2">
+        <v>46153.53869212963</v>
+      </c>
+      <c r="E1048" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1048" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1048" s="4" t="s">
+        <v>1150</v>
+      </c>
+      <c r="H1048" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1048" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1049" s="4">
+        <v>1048</v>
+      </c>
+      <c r="B1049" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1049" s="4">
+        <v>23289</v>
+      </c>
+      <c r="D1049" s="2">
+        <v>46153.674826388888</v>
+      </c>
+      <c r="E1049" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1049" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1049" s="4" t="s">
+        <v>1151</v>
+      </c>
+      <c r="H1049" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1049" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1050" s="4">
+        <v>1049</v>
+      </c>
+      <c r="B1050" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1050" s="4">
+        <v>44371</v>
+      </c>
+      <c r="D1050" s="2">
+        <v>46153.694097222222</v>
+      </c>
+      <c r="E1050" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1050" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1050" s="4" t="s">
+        <v>1152</v>
+      </c>
+      <c r="H1050" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1050" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1051" s="4">
+        <v>1050</v>
+      </c>
+      <c r="B1051" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1051" s="4">
+        <v>42303</v>
+      </c>
+      <c r="D1051" s="2">
+        <v>46154.485324074078</v>
+      </c>
+      <c r="E1051" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F1051" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1051" s="4" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H1051" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1051" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1052" s="4">
+        <v>1051</v>
+      </c>
+      <c r="B1052" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1052" s="4">
+        <v>29831</v>
+      </c>
+      <c r="D1052" s="2">
+        <v>46154.488692129627</v>
+      </c>
+      <c r="E1052" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1052" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1052" s="4" t="s">
+        <v>1154</v>
+      </c>
+      <c r="H1052" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1052" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1053" s="4">
+        <v>1052</v>
+      </c>
+      <c r="B1053" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1053" s="4">
+        <v>43404</v>
+      </c>
+      <c r="D1053" s="2">
+        <v>46154.509212962963</v>
+      </c>
+      <c r="E1053" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1053" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1053" s="4" t="s">
+        <v>1155</v>
+      </c>
+      <c r="H1053" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1053" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1054" s="4">
+        <v>1053</v>
+      </c>
+      <c r="B1054" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1054" s="4">
+        <v>45660</v>
+      </c>
+      <c r="D1054" s="2">
+        <v>46154.513773148145</v>
+      </c>
+      <c r="E1054" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1054" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1054" s="4" t="s">
+        <v>1157</v>
+      </c>
+      <c r="H1054" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1054" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1055" s="4">
+        <v>1054</v>
+      </c>
+      <c r="B1055" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1055" s="4">
+        <v>44104</v>
+      </c>
+      <c r="D1055" s="2">
+        <v>46154.525497685187</v>
+      </c>
+      <c r="E1055" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1055" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1055" s="4" t="s">
+        <v>1158</v>
+      </c>
+      <c r="H1055" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1055" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1056" s="4">
+        <v>1055</v>
+      </c>
+      <c r="B1056" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1056" s="4">
+        <v>31205</v>
+      </c>
+      <c r="D1056" s="2">
+        <v>46154.526666666665</v>
+      </c>
+      <c r="E1056" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1056" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1056" s="4" t="s">
+        <v>1159</v>
+      </c>
+      <c r="H1056" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1056" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1057" s="4">
+        <v>1056</v>
+      </c>
+      <c r="B1057" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1057" s="4">
+        <v>44385</v>
+      </c>
+      <c r="D1057" s="2">
+        <v>46155.386076388888</v>
+      </c>
+      <c r="E1057" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1057" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1057" s="4" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H1057" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1057" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1058" s="4">
+        <v>1057</v>
+      </c>
+      <c r="B1058" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1058" s="4">
+        <v>45595</v>
+      </c>
+      <c r="D1058" s="2">
+        <v>46155.447615740741</v>
+      </c>
+      <c r="E1058" s="4" t="s">
+        <v>1161</v>
+      </c>
+      <c r="F1058" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1058" s="4" t="s">
+        <v>1162</v>
+      </c>
+      <c r="H1058" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1058" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1059" s="4">
+        <v>1058</v>
+      </c>
+      <c r="B1059" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1059" s="4">
+        <v>44238</v>
+      </c>
+      <c r="D1059" s="2">
+        <v>46155.463819444441</v>
+      </c>
+      <c r="E1059" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1059" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1059" s="4" t="s">
+        <v>1163</v>
+      </c>
+      <c r="H1059" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1059" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1060" s="4">
+        <v>1059</v>
+      </c>
+      <c r="B1060" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1060" s="4">
+        <v>47157</v>
+      </c>
+      <c r="D1060" s="2">
+        <v>46155.474224537036</v>
+      </c>
+      <c r="E1060" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1060" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1060" s="4" t="s">
+        <v>1164</v>
+      </c>
+      <c r="H1060" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1060" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1061" s="4">
+        <v>1060</v>
+      </c>
+      <c r="B1061" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1061" s="4">
+        <v>36914</v>
+      </c>
+      <c r="D1061" s="2">
+        <v>46155.515300925923</v>
+      </c>
+      <c r="E1061" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1061" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1061" s="4" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H1061" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1061" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1062" s="4">
+        <v>1061</v>
+      </c>
+      <c r="B1062" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1062" s="4">
+        <v>44645</v>
+      </c>
+      <c r="D1062" s="2">
+        <v>46155.517071759263</v>
+      </c>
+      <c r="E1062" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1062" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1062" s="4" t="s">
+        <v>1166</v>
+      </c>
+      <c r="H1062" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1062" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1063" s="4">
+        <v>1062</v>
+      </c>
+      <c r="B1063" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1063" s="4">
+        <v>35651</v>
+      </c>
+      <c r="D1063" s="2">
+        <v>46155.560937499999</v>
+      </c>
+      <c r="E1063" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1063" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1063" s="4" t="s">
+        <v>1167</v>
+      </c>
+      <c r="H1063" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1063" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1064" s="4">
+        <v>1063</v>
+      </c>
+      <c r="B1064" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1064" s="4">
+        <v>42991</v>
+      </c>
+      <c r="D1064" s="2">
+        <v>46155.596203703702</v>
+      </c>
+      <c r="E1064" s="4" t="s">
+        <v>963</v>
+      </c>
+      <c r="F1064" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1064" s="4" t="s">
+        <v>1168</v>
+      </c>
+      <c r="H1064" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1064" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1065" s="4">
+        <v>1064</v>
+      </c>
+      <c r="B1065" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1065" s="4">
+        <v>44352</v>
+      </c>
+      <c r="D1065" s="2">
+        <v>46155.657442129632</v>
+      </c>
+      <c r="E1065" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1065" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1065" s="4" t="s">
+        <v>1169</v>
+      </c>
+      <c r="H1065" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1065" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1066" s="4">
+        <v>1065</v>
+      </c>
+      <c r="B1066" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1066" s="4">
+        <v>40115</v>
+      </c>
+      <c r="D1066" s="2">
+        <v>46155.996481481481</v>
+      </c>
+      <c r="E1066" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="F1066" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1066" s="4" t="s">
+        <v>1170</v>
+      </c>
+      <c r="H1066" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1066" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1067" s="4">
+        <v>1066</v>
+      </c>
+      <c r="B1067" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1067" s="4">
+        <v>46604</v>
+      </c>
+      <c r="D1067" s="2">
+        <v>46156.451504629629</v>
+      </c>
+      <c r="E1067" s="4" t="s">
+        <v>1118</v>
+      </c>
+      <c r="F1067" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1067" s="4" t="s">
+        <v>1171</v>
+      </c>
+      <c r="H1067" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1067" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1068" s="4">
+        <v>1067</v>
+      </c>
+      <c r="B1068" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1068" s="4">
+        <v>47929</v>
+      </c>
+      <c r="D1068" s="2">
+        <v>46156.479143518518</v>
+      </c>
+      <c r="E1068" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1068" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1068" s="4" t="s">
+        <v>1172</v>
+      </c>
+      <c r="H1068" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1068" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1069" s="4">
+        <v>1068</v>
+      </c>
+      <c r="B1069" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1069" s="4">
+        <v>47050</v>
+      </c>
+      <c r="D1069" s="2">
+        <v>46156.510625000003</v>
+      </c>
+      <c r="E1069" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1069" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1069" s="4" t="s">
+        <v>1173</v>
+      </c>
+      <c r="H1069" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1069" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1070" s="4">
+        <v>1069</v>
+      </c>
+      <c r="B1070" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1070" s="4">
+        <v>40709</v>
+      </c>
+      <c r="D1070" s="2">
+        <v>46156.518900462965</v>
+      </c>
+      <c r="E1070" s="4" t="s">
+        <v>1141</v>
+      </c>
+      <c r="F1070" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1070" s="4" t="s">
+        <v>1174</v>
+      </c>
+      <c r="H1070" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1070" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1071" s="4">
+        <v>1070</v>
+      </c>
+      <c r="B1071" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1071" s="4">
+        <v>39207</v>
+      </c>
+      <c r="D1071" s="2">
+        <v>46156.547395833331</v>
+      </c>
+      <c r="E1071" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1071" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1071" s="4" t="s">
+        <v>1175</v>
+      </c>
+      <c r="H1071" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1071" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1072" s="4">
+        <v>1071</v>
+      </c>
+      <c r="B1072" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1072" s="4">
+        <v>47550</v>
+      </c>
+      <c r="D1072" s="2">
+        <v>46156.597349537034</v>
+      </c>
+      <c r="E1072" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1072" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1072" s="4" t="s">
+        <v>1176</v>
+      </c>
+      <c r="H1072" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1072" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1073" s="4">
+        <v>1072</v>
+      </c>
+      <c r="B1073" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1073" s="4">
+        <v>48146</v>
+      </c>
+      <c r="D1073" s="2">
+        <v>46156.615277777775</v>
+      </c>
+      <c r="E1073" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F1073" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1073" s="4" t="s">
+        <v>1177</v>
+      </c>
+      <c r="H1073" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1073" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1074" s="4">
+        <v>1073</v>
+      </c>
+      <c r="B1074" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1074" s="4">
+        <v>41416</v>
+      </c>
+      <c r="D1074" s="2">
+        <v>46156.729560185187</v>
+      </c>
+      <c r="E1074" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1074" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1074" s="4" t="s">
+        <v>1178</v>
+      </c>
+      <c r="H1074" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1074" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1075" s="4">
+        <v>1074</v>
+      </c>
+      <c r="B1075" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1075" s="4">
+        <v>31728</v>
+      </c>
+      <c r="D1075" s="2">
+        <v>46156.776805555557</v>
+      </c>
+      <c r="E1075" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1075" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1075" s="4" t="s">
+        <v>1179</v>
+      </c>
+      <c r="H1075" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1075" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1076" s="4">
+        <v>1075</v>
+      </c>
+      <c r="B1076" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1076" s="4">
+        <v>44194</v>
+      </c>
+      <c r="D1076" s="2">
+        <v>46156.779745370368</v>
+      </c>
+      <c r="E1076" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1076" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1076" s="4" t="s">
+        <v>1180</v>
+      </c>
+      <c r="H1076" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1076" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1077" s="4">
+        <v>1076</v>
+      </c>
+      <c r="B1077" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1077" s="4">
+        <v>44260</v>
+      </c>
+      <c r="D1077" s="2">
+        <v>46157.433715277781</v>
+      </c>
+      <c r="E1077" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1077" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1077" s="4" t="s">
+        <v>1181</v>
+      </c>
+      <c r="H1077" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1077" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1078" s="4">
+        <v>1077</v>
+      </c>
+      <c r="B1078" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1078" s="4">
+        <v>44772</v>
+      </c>
+      <c r="D1078" s="2">
+        <v>46157.438136574077</v>
+      </c>
+      <c r="E1078" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1078" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1078" s="4" t="s">
+        <v>1182</v>
+      </c>
+      <c r="H1078" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1078" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1079" s="4">
+        <v>1078</v>
+      </c>
+      <c r="B1079" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1079" s="4">
+        <v>39094</v>
+      </c>
+      <c r="D1079" s="2">
+        <v>46157.481296296297</v>
+      </c>
+      <c r="E1079" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1079" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1079" s="4" t="s">
+        <v>1183</v>
+      </c>
+      <c r="H1079" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1079" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1080" s="4">
+        <v>1079</v>
+      </c>
+      <c r="B1080" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1080" s="4">
+        <v>49594</v>
+      </c>
+      <c r="D1080" s="2">
+        <v>46157.630057870374</v>
+      </c>
+      <c r="E1080" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F1080" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1080" s="4" t="s">
+        <v>1184</v>
+      </c>
+      <c r="H1080" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1080" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1081" s="4">
+        <v>1080</v>
+      </c>
+      <c r="B1081" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1081" s="4">
+        <v>36611</v>
+      </c>
+      <c r="D1081" s="2">
+        <v>46157.643587962964</v>
+      </c>
+      <c r="E1081" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1081" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1081" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="H1081" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1081" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1082" s="4">
+        <v>1081</v>
+      </c>
+      <c r="B1082" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1082" s="4">
+        <v>43245</v>
+      </c>
+      <c r="D1082" s="2">
+        <v>46157.646423611113</v>
+      </c>
+      <c r="E1082" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F1082" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1082" s="4" t="s">
+        <v>1186</v>
+      </c>
+      <c r="H1082" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1082" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1083" s="4">
+        <v>1082</v>
+      </c>
+      <c r="B1083" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1083" s="4">
+        <v>44753</v>
+      </c>
+      <c r="D1083" s="2">
+        <v>46157.646770833337</v>
+      </c>
+      <c r="E1083" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1083" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1083" s="4" t="s">
+        <v>1187</v>
+      </c>
+      <c r="H1083" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1083" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1084" s="4">
+        <v>1083</v>
+      </c>
+      <c r="B1084" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1084" s="4">
+        <v>46548</v>
+      </c>
+      <c r="D1084" s="2">
+        <v>46157.670590277776</v>
+      </c>
+      <c r="E1084" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1084" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1084" s="4" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H1084" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1084" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1085" s="4">
+        <v>1084</v>
+      </c>
+      <c r="B1085" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1085" s="4">
+        <v>25069</v>
+      </c>
+      <c r="D1085" s="2">
+        <v>46157.854212962964</v>
+      </c>
+      <c r="E1085" s="4" t="s">
+        <v>951</v>
+      </c>
+      <c r="F1085" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1085" s="4" t="s">
+        <v>1189</v>
+      </c>
+      <c r="H1085" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1085" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1086" s="4">
+        <v>1085</v>
+      </c>
+      <c r="B1086" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1086" s="4">
+        <v>46551</v>
+      </c>
+      <c r="D1086" s="2">
+        <v>46158.297534722224</v>
+      </c>
+      <c r="E1086" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1086" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1086" s="4" t="s">
+        <v>1190</v>
+      </c>
+      <c r="H1086" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1086" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1087" s="4">
+        <v>1086</v>
+      </c>
+      <c r="B1087" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1087" s="4">
+        <v>43110</v>
+      </c>
+      <c r="D1087" s="2">
+        <v>46158.425138888888</v>
+      </c>
+      <c r="E1087" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1087" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1087" s="4" t="s">
+        <v>1191</v>
+      </c>
+      <c r="H1087" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1087" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1088" s="4">
+        <v>1087</v>
+      </c>
+      <c r="B1088" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1088" s="4">
+        <v>44510</v>
+      </c>
+      <c r="D1088" s="2">
+        <v>46158.582256944443</v>
+      </c>
+      <c r="E1088" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1088" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1088" s="4" t="s">
+        <v>1192</v>
+      </c>
+      <c r="H1088" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1088" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1089" s="4">
+        <v>1088</v>
+      </c>
+      <c r="B1089" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1089" s="4">
+        <v>41180</v>
+      </c>
+      <c r="D1089" s="2">
+        <v>46159.47587962963</v>
+      </c>
+      <c r="E1089" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1089" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1089" s="4" t="s">
+        <v>1193</v>
+      </c>
+      <c r="H1089" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1089" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1090" s="4">
+        <v>1089</v>
+      </c>
+      <c r="B1090" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1090" s="4">
+        <v>39418</v>
+      </c>
+      <c r="D1090" s="2">
+        <v>46160.369618055556</v>
+      </c>
+      <c r="E1090" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1090" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1090" s="4" t="s">
+        <v>1194</v>
+      </c>
+      <c r="H1090" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1090" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1091" s="4">
+        <v>1090</v>
+      </c>
+      <c r="B1091" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1091" s="4">
+        <v>40383</v>
+      </c>
+      <c r="D1091" s="2">
+        <v>46160.369756944441</v>
+      </c>
+      <c r="E1091" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1091" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1091" s="4" t="s">
+        <v>1195</v>
+      </c>
+      <c r="H1091" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1091" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1092" s="4">
+        <v>1091</v>
+      </c>
+      <c r="B1092" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1092" s="4">
+        <v>48305</v>
+      </c>
+      <c r="D1092" s="2">
+        <v>46160.376307870371</v>
+      </c>
+      <c r="E1092" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1092" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1092" s="4" t="s">
+        <v>1196</v>
+      </c>
+      <c r="H1092" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1092" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1093" s="4">
+        <v>1092</v>
+      </c>
+      <c r="B1093" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1093" s="4">
+        <v>40775</v>
+      </c>
+      <c r="D1093" s="2">
+        <v>46160.387662037036</v>
+      </c>
+      <c r="E1093" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1093" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1093" s="4" t="s">
+        <v>1197</v>
+      </c>
+      <c r="H1093" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1093" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1094" s="4">
+        <v>1093</v>
+      </c>
+      <c r="B1094" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1094" s="4">
+        <v>41135</v>
+      </c>
+      <c r="D1094" s="2">
+        <v>46160.469340277778</v>
+      </c>
+      <c r="E1094" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1094" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1094" s="4" t="s">
+        <v>1198</v>
+      </c>
+      <c r="H1094" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1094" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1095" s="4">
+        <v>1094</v>
+      </c>
+      <c r="B1095" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1095" s="4">
+        <v>50933</v>
+      </c>
+      <c r="D1095" s="2">
+        <v>46160.501030092593</v>
+      </c>
+      <c r="E1095" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1095" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1095" s="4" t="s">
+        <v>1199</v>
+      </c>
+      <c r="H1095" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1095" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1096" s="4">
+        <v>1095</v>
+      </c>
+      <c r="B1096" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1096" s="4">
+        <v>43694</v>
+      </c>
+      <c r="D1096" s="2">
+        <v>46160.501064814816</v>
+      </c>
+      <c r="E1096" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1096" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1096" s="4" t="s">
+        <v>1200</v>
+      </c>
+      <c r="H1096" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1096" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1097" s="4">
+        <v>1096</v>
+      </c>
+      <c r="B1097" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1097" s="4">
+        <v>47545</v>
+      </c>
+      <c r="D1097" s="2">
+        <v>46160.501168981478</v>
+      </c>
+      <c r="E1097" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1097" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1097" s="4" t="s">
+        <v>1201</v>
+      </c>
+      <c r="H1097" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1097" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1098" s="4">
+        <v>1097</v>
+      </c>
+      <c r="B1098" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1098" s="4">
+        <v>48869</v>
+      </c>
+      <c r="D1098" s="2">
+        <v>46160.503298611111</v>
+      </c>
+      <c r="E1098" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1098" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1098" s="4" t="s">
+        <v>1202</v>
+      </c>
+      <c r="H1098" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1098" s="4" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1099" s="4">
+        <v>1098</v>
+      </c>
+      <c r="B1099" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1099" s="4">
+        <v>43249</v>
+      </c>
+      <c r="D1099" s="2">
+        <v>46160.545601851853</v>
+      </c>
+      <c r="E1099" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1099" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1099" s="4" t="s">
+        <v>1203</v>
+      </c>
+      <c r="H1099" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1099" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1100" s="4">
+        <v>1099</v>
+      </c>
+      <c r="B1100" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1100" s="4">
+        <v>44218</v>
+      </c>
+      <c r="D1100" s="2">
+        <v>46160.545706018522</v>
+      </c>
+      <c r="E1100" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1100" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1100" s="4" t="s">
+        <v>1204</v>
+      </c>
+      <c r="H1100" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1100" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1101" s="4">
+        <v>1100</v>
+      </c>
+      <c r="B1101" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1101" s="4">
+        <v>49085</v>
+      </c>
+      <c r="D1101" s="2">
+        <v>46160.602083333331</v>
+      </c>
+      <c r="E1101" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F1101" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1101" s="4" t="s">
+        <v>1205</v>
+      </c>
+      <c r="H1101" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1101" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1102" s="4">
+        <v>1101</v>
+      </c>
+      <c r="B1102" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1102" s="4">
+        <v>45545</v>
+      </c>
+      <c r="D1102" s="2">
+        <v>46160.977708333332</v>
+      </c>
+      <c r="E1102" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1102" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1102" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H1102" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1102" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1103" s="4">
+        <v>1102</v>
+      </c>
+      <c r="B1103" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1103" s="4">
+        <v>47248</v>
+      </c>
+      <c r="D1103" s="2">
+        <v>46161.253391203703</v>
+      </c>
+      <c r="E1103" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1103" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1103" s="4" t="s">
+        <v>1206</v>
+      </c>
+      <c r="H1103" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1103" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1104" s="4">
+        <v>1103</v>
+      </c>
+      <c r="B1104" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1104" s="4">
+        <v>26472</v>
+      </c>
+      <c r="D1104" s="2">
+        <v>46161.466921296298</v>
+      </c>
+      <c r="E1104" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1104" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1104" s="4" t="s">
+        <v>1207</v>
+      </c>
+      <c r="H1104" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1104" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1105" s="4">
+        <v>1104</v>
+      </c>
+      <c r="B1105" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1105" s="4">
+        <v>53697</v>
+      </c>
+      <c r="D1105" s="2">
+        <v>46161.516655092593</v>
+      </c>
+      <c r="E1105" s="4" t="s">
+        <v>1112</v>
+      </c>
+      <c r="F1105" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1105" s="4" t="s">
+        <v>1208</v>
+      </c>
+      <c r="H1105" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1105" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1106" s="4">
+        <v>1105</v>
+      </c>
+      <c r="B1106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1106" s="4">
+        <v>44071</v>
+      </c>
+      <c r="D1106" s="2">
+        <v>46161.533692129633</v>
+      </c>
+      <c r="E1106" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1106" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1106" s="4" t="s">
+        <v>1209</v>
+      </c>
+      <c r="H1106" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I1106" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1107" s="4">
+        <v>1106</v>
+      </c>
+      <c r="B1107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1107" s="4">
+        <v>40354</v>
+      </c>
+      <c r="D1107" s="2">
+        <v>46161.542881944442</v>
+      </c>
+      <c r="E1107" s="4" t="s">
+        <v>963</v>
+      </c>
+      <c r="F1107" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1107" s="4" t="s">
+        <v>1210</v>
+      </c>
+      <c r="H1107" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1107" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1108" s="4">
+        <v>1107</v>
+      </c>
+      <c r="B1108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1108" s="4">
+        <v>40427</v>
+      </c>
+      <c r="D1108" s="2">
+        <v>46162.383738425924</v>
+      </c>
+      <c r="E1108" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1108" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1108" s="4" t="s">
+        <v>1211</v>
+      </c>
+      <c r="H1108" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1108" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1109" s="4">
+        <v>1108</v>
+      </c>
+      <c r="B1109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1109" s="4">
+        <v>37056</v>
+      </c>
+      <c r="D1109" s="2">
+        <v>46162.385300925926</v>
+      </c>
+      <c r="E1109" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1109" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1109" s="4" t="s">
+        <v>1212</v>
+      </c>
+      <c r="H1109" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1109" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1110" s="4">
+        <v>1109</v>
+      </c>
+      <c r="B1110" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1110" s="4">
+        <v>53827</v>
+      </c>
+      <c r="D1110" s="2">
+        <v>46162.499398148146</v>
+      </c>
+      <c r="E1110" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1110" s="4" t="s">
+        <v>1213</v>
+      </c>
+      <c r="H1110" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1110" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1111" s="4">
+        <v>1110</v>
+      </c>
+      <c r="B1111" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1111" s="4">
+        <v>48224</v>
+      </c>
+      <c r="D1111" s="2">
+        <v>46162.501944444448</v>
+      </c>
+      <c r="E1111" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1111" s="4" t="s">
+        <v>1214</v>
+      </c>
+      <c r="H1111" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1111" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1112" s="4">
+        <v>1111</v>
+      </c>
+      <c r="B1112" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1112" s="4">
+        <v>53243</v>
+      </c>
+      <c r="D1112" s="2">
+        <v>46162.51972222222</v>
+      </c>
+      <c r="E1112" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F1112" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1112" s="4" t="s">
+        <v>1215</v>
+      </c>
+      <c r="H1112" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1112" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1113" s="4">
+        <v>1112</v>
+      </c>
+      <c r="B1113" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1113" s="4">
+        <v>49807</v>
+      </c>
+      <c r="D1113" s="2">
+        <v>46162.57440972222</v>
+      </c>
+      <c r="E1113" s="4" t="s">
+        <v>1161</v>
+      </c>
+      <c r="F1113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1113" s="4" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H1113" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1113" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1114" s="4">
+        <v>1113</v>
+      </c>
+      <c r="B1114" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1114" s="4">
+        <v>50445</v>
+      </c>
+      <c r="D1114" s="2">
+        <v>46162.591481481482</v>
+      </c>
+      <c r="E1114" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1114" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1114" s="4" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H1114" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1114" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1115" s="4">
+        <v>1114</v>
+      </c>
+      <c r="B1115" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1115" s="4">
+        <v>52298</v>
+      </c>
+      <c r="D1115" s="2">
+        <v>46163.401967592596</v>
+      </c>
+      <c r="E1115" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1115" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1115" s="4" t="s">
+        <v>1218</v>
+      </c>
+      <c r="H1115" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1115" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1116" s="4">
+        <v>1115</v>
+      </c>
+      <c r="B1116" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1116" s="4">
+        <v>40922</v>
+      </c>
+      <c r="D1116" s="2">
+        <v>46163.406689814816</v>
+      </c>
+      <c r="E1116" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1116" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1116" s="4" t="s">
+        <v>1219</v>
+      </c>
+      <c r="H1116" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1116" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 29/05/2026 17:54:58,60
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="247" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{828ADCCC-FB78-402F-8DB9-B575A1F24DB8}"/>
+  <xr:revisionPtr revIDLastSave="250" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13E6E693-60A2-49A6-B963-AD5BB472AB69}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$1196</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6699" uniqueCount="1220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7179" uniqueCount="1310">
   <si>
     <t>ID</t>
   </si>
@@ -3790,6 +3790,276 @@
   </si>
   <si>
     <t>O técnico veio fez o serviço, porem falou que tínhamos que entrar em contato com a central para troca do equipamento, porem a central disse que o técnico deveria solicitar.</t>
+  </si>
+  <si>
+    <t>O técnico não veio na data agendada</t>
+  </si>
+  <si>
+    <t>Foi bom</t>
+  </si>
+  <si>
+    <t>Os sistemas de atendimento e chamados da Brastemp são péssimos. Abri um chamado de assistência técnica relatando um problema e na visita o técnico trouxe outras peças diferentes, pois no chamado constava um defeito totalmente diferente do que descrevi, tive que aguardar semanas pela peça correta mesmo descrito o problema com o parecer técnico da visita na nova visita não trouxeram um novo cilindro de gás. Conforme identificado pelo técnico havia instalado um novo cilindro e no dia seguinte estava vazio por defeito do equipamento.</t>
+  </si>
+  <si>
+    <t>NÃO HOUVE VISITA TECNICA.</t>
+  </si>
+  <si>
+    <t>Atendimento excelente,  o técnico.detectou.um.problema.que eu já tinha reclamado,. precisa trocar o aparelho pois está com.um.barulhao e não gela muito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Não gela</t>
+  </si>
+  <si>
+    <t>O técnico veio deixou a cuba descongelando disse que tem que trocar o sensor de temperatura gritou com minha tia idosa e foi embora</t>
+  </si>
+  <si>
+    <t>O técnico fez a “troca” do filtro utilizando um usado, ou seja, imagino ter pego de outro cliente e colocado no meu como se fosse novo. Isso foi observado pela minha funcionária que já presenciou outras manutenções. Não fiquei satisfeita com essa atitude além da dificuldade de marcação de manutenção. A falta de confiança na qualidade da água consumida pelo filtro de vcs me fez repensar a continuidade do serviço. Aguardo retorno de vcs.</t>
+  </si>
+  <si>
+    <t>Aluguei a dois meses e já até foi trocado ontem, porque vazava e continua vazando! Absurdo</t>
+  </si>
+  <si>
+    <t>não trocou ofiltro</t>
+  </si>
+  <si>
+    <t>O aparelho é bom, mas o custo é extremamente alto</t>
+  </si>
+  <si>
+    <t>Mais uma vez não houve atendimento, estou pensando até de entregar o bebedouro.</t>
+  </si>
+  <si>
+    <t>Dessa vez o problema foi resolvido</t>
+  </si>
+  <si>
+    <t>O purificador continua com problemas. Agora está vazando. Peço que retornem</t>
+  </si>
+  <si>
+    <t>Muito ruim. O técnico não apareceu na data agendada. Liguei para reclamar, disseram que viria à tarde.  Também não veio. Perdi meu dia de trabalho. Finalmente veio na nova data agendada.   Veio, trocou o filtro e foi embora.  Antigamente desinfetava a máquina, fazia o teste de filtro de cloro.  Nada, só a troca do filtro. O filtro “novo” veio fora de qualquer embalagem. Será que era realmente novo?  Muito estranho. Estou perdendo o prazer e a confiança em ter o produto em casa.</t>
+  </si>
+  <si>
+    <t>Meu aparelho é novo, mas já deu problema em uma peça que não foi possível reparar no mesmo dia. Estou aguardando a OS para que peçam a peça para trocar. Estou um pouco triste, pois meu aparelho é muito recente e novo.</t>
+  </si>
+  <si>
+    <t>Meu agendamento estava para o perido manha - 8h as 13h.Tive de reagendar e alocar outra pessoa para atender o técnico que chegou as 17h30.Fez a vistoria e vai voltar com troca de uma nova peça do equipamento.Foi atencioso e profissional.</t>
+  </si>
+  <si>
+    <t>O purificador "não é lá uma Brastemp!"Instalaram o purificador, mas até hoje não funciona bem. A água sai fraca e não está gelando. Além do técnico que fez a instalação, mais 2 técnicos já foram fazer visita técnica, mas chegaram perdidos porque não foram informados das peças que deveriam trocar.Eu só tenho certeza de uma coisa: a parcela vai bater em dia no meu cartão, mesmo o produto não estar funcionando da maneira correta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Vazão/pressão da água</t>
+  </si>
+  <si>
+    <t>Trocou o filtro mas na deixou comprovante nem laudo da manutenção</t>
+  </si>
+  <si>
+    <t>O purificador vem nos atendendo de modo satisfatório, apenas com respeito a esta visita técnica,o técnico chegou ao local após o horário estabelecido e agendado por vocês, ocorrendo que a supervisora da unidade não se encontrava mais presente no local, outra pessoa teve de acompanhá-lo.</t>
+  </si>
+  <si>
+    <t>Precisava mudar para 220v e ele nao mudou</t>
+  </si>
+  <si>
+    <t>Funcionou muito bem, até parar de gelar e me deixar na mão</t>
+  </si>
+  <si>
+    <t>Demora é burocracia para substituir o equipamento quebrado.</t>
+  </si>
+  <si>
+    <t>FRQ OESTE RJ R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Não teve visita técnica</t>
+  </si>
+  <si>
+    <t>FRQ SBC SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>A visita foi somente a periódica e boa parte da avaliação abaixo refere-se a ela. Porém, há meses tento resolver o problema do filtro aquecer excessivamente e de tentar ligar a refrigeração, por vezes, mais de 10 tentativas. Como os técnicos dizem que só podem efetuar a trica do filtro se este apresentar o problema descrito quando estão presentes, estou aguardando o filtro “pegar fogo” ou a refrigeração parar de funcionar. Até lá, ele vai gastando muita energia.</t>
+  </si>
+  <si>
+    <t>FRQ OSASCO SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>visita técnica ocorreu na semana anterior - sábado dia 23/05/2026 veio outro técnico que não foi recebido porque não havia solicitação</t>
+  </si>
+  <si>
+    <t>FRQ ZONA SUL SP 01 R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>A técnica muito simpática e eficiente. Porém a nota é 8 devido a falta de compromisso ai marcarem em 1 data e não vir, e o cliente precisar ficar correndo atrás para ser atendido.</t>
+  </si>
+  <si>
+    <t>atendeu dentro das expectativas, apenas manutenção do filtro.</t>
+  </si>
+  <si>
+    <t>Não houve solução do problema que chamei o técnico. Ele informou que a Brastemp ia entrar em contato para novo agendamento e isso não aconteceu.</t>
+  </si>
+  <si>
+    <t>FRQ ZONA SUL SP 02 R01</t>
+  </si>
+  <si>
+    <t>A visita não aconteceu.</t>
+  </si>
+  <si>
+    <t>Serviço ruim, última visita técnica não levou material correto, não trocou filtro e não fez higienização, disse que voltaria depois e não deu mais notícias</t>
+  </si>
+  <si>
+    <t>Está sendo estável</t>
+  </si>
+  <si>
+    <t>FRQ CENTRO NORTE RJ R02</t>
+  </si>
+  <si>
+    <t>Estou a mais de 10 dias sem filtro, veio um técnico na minha casa,demorou 2 horas tentando arrumar, e no final condenou o filtro pedindo a troca, sendo que hj tive a surpresa qd liguei e falaram que não havia laudo do técnico, sendo que teria que fazer uma nova visita pra reavaliar meu filtro,que absurdo de falta de consideração com o cliente. Espero retorno urgente de vcs</t>
+  </si>
+  <si>
+    <t>Agendamos a troca do filtro para esse sábado, mas ao chegar em casa o técnico disse que o purificador saiu de linha e saiu sem trocar o filtro.</t>
+  </si>
+  <si>
+    <t>FRQ SALVADOR BA R02</t>
+  </si>
+  <si>
+    <t>O aparelho foi instalado e funcionando sem problemas, mas o técnico, como o mesmo declarou que é o único da BRASTEMP na Bahia, levou o meu cilindro de gás, que estava cheio, deixando o que era de uso dele ligado no aparelho.A BRASTEMP é uma ótima marca que a 50 anos, somente uso seus produtos, mas a assistência técnica aqui na Bahia é amadora e sem escrúpulos e cuidado com o cliente .Lamentável, fiquei no prejuízo e tenho agora que comprar um cilindro de gás para o aparelho.NÃO QUERO MAIS ESSE TÉCNICO NA MINHA RESIDÊNCIA E VOU RELATAR O FATO NO RECLAMANTE AQUI.</t>
+  </si>
+  <si>
+    <t>AT SJRPRETO SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Muito boa, mas fica caro por um ano</t>
+  </si>
+  <si>
+    <t>Equipamento muito bom, porém começam a aparecer ruídos de trepidação e de funcionamento do sistema elétrico, que incomodam muito a noite.</t>
+  </si>
+  <si>
+    <t>Depois da manutenção realizada o filtro está vazando agua</t>
+  </si>
+  <si>
+    <t>Poedeira ter sido nota 10 porem , o prestador é uma pessoa muito boa e prestativa mas teve um problema ele sem querer afetou a mangueira e esta vazado água</t>
+  </si>
+  <si>
+    <t>O técnico veio e mediu a qualidade da água falando que ela, a água estava boa, o atendimento durou segundos, não sei se esse é o procedimento certo, porque nas outras vezes os técnicos que vinham abriam a máquina e verificavam se estava tudo ok, de qualquer forma ele falou que estava tudo certo!</t>
+  </si>
+  <si>
+    <t>O purificador é muito bom, mas o atendimento e interface com o cliente contratante é péssima, extremamente demorada e trabalhosa.</t>
+  </si>
+  <si>
+    <t>Está com preço altos, fiz uma nova pesquisa para o mesmo serviço e o custo nao está mais compensando.</t>
+  </si>
+  <si>
+    <t>Já utilizo a anos. Me atende e eu gosto muito</t>
+  </si>
+  <si>
+    <t>A favor: atendimento realizado na data agendada com qualidade da água garantida.Contra: agendamento não imediato (- 01 ponto), materiais descartáveis fornecidos a técnico(a) por cliente (-01 ponto) e Ordem de Serviço não recebida por e-mail ou SMS (- 01 ponto) = 07 pontos.</t>
+  </si>
+  <si>
+    <t>Péssimo. Vcs pensam q fazem favor.  Eu pago a vcs.</t>
+  </si>
+  <si>
+    <t>Esta tudo bem. O preço ainda é um tanto alto!</t>
+  </si>
+  <si>
+    <t>1) as visitas deveriam ser semestrais e marcadas pela Bratemp. Mas eu tive de ir atrás e marcar, porque a Brastemp não marcou. 2) a técnica que foi primeiro não abriu o filtro, alegou falta de pressão do prédio e foi embora. 3) após falar novamente com a Brastemp fui informado de que poderia haver a troca do filtro. concordei. 4) Quase 20 dias depois, novo técnico abriu o filtro atual, fez manutenção e foi embora. Não houve a troca do aparelho.</t>
+  </si>
+  <si>
+    <t>Muito chateada com a troca do purificador no dia 22/5/26. Não tiveram consideração em relação ao horário, já que agendaram pela manhã e só vieram perto de 18h. Se eu não reclamasse várias vezes durante o dia não teria acontecido.O aparelho que veio na troca é inferior ao que tinha na minha casa. Não trouxe o suporte correspondente ao aparelho novo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora do período agendado </t>
+  </si>
+  <si>
+    <t>Preço desestimula</t>
+  </si>
+  <si>
+    <t>O purificador é espetacular, a central de atendimento pelo sistema BA(burrice artificial) é vergonhoso, é um lixo. Portanto 5 é a nota merecida.Contrate uma pessoa de TI que faça um agente que identifique o cliente pelo telefone, especialmente os que tem mais de uma assinatura.</t>
+  </si>
+  <si>
+    <t>Atendimento excelente, profissional super prestativo, mas não entendi porque não foi substituído o filtro.</t>
+  </si>
+  <si>
+    <t>Péssimo atendimento para um cliente de 15 anos com o mesmo aparelho e assinatura.</t>
+  </si>
+  <si>
+    <t>Péssimo, o técnico foi para uma visita periódica e deixou a água do meu purificador com gosto horrível,  com o jato forte, estou bastante chateada. O purificador estava 100% ,agora não podemos nem tomar água com medo de passar mal.</t>
+  </si>
+  <si>
+    <t>Cordial, explicou de forma clara, resolveu o problema</t>
+  </si>
+  <si>
+    <t>Serviço rápido e limpo, mas sem muitas explicações.</t>
+  </si>
+  <si>
+    <t>Uma situação que não me agradou foi que mudaram de empresa pra fazer a Manutenção e não fui avisada antes... simplesmente mudaram e passou a cobrança pra empresa atual. Claro que não autorizei! Não sabia de onde vinha aquela cobrança... aí acabou que eu fui procurar saber de onde vinha a cobrança por tanta insistência</t>
+  </si>
+  <si>
+    <t>Serviço realizado ok, mas não tem responsabilidade com horário marcado</t>
+  </si>
+  <si>
+    <t>Fornece água pura, natural ou gelada, por um custo mensal, incluindo a manutenção do purificador.</t>
+  </si>
+  <si>
+    <t>Bom dia, a peça que solicitei para trocar o tecnico não trocou, por isso a minha insatisfação.</t>
+  </si>
+  <si>
+    <t>indicação de problema a ser corrigido pelo tecnico foi mal feito e técnico veio para resolver somente parte do problema deixando problemas (piores) para trás. Deixo claro que o problema não foi o técnico enviado, mas, a comunicação interna para posicionamento do problema</t>
+  </si>
+  <si>
+    <t>0 ninguém apareceu</t>
+  </si>
+  <si>
+    <t>SOU CLIENTE (PURIFICADOR) DESDE O INICIO O QUERO UM APARELHO MENOR, SE NÃO EXISTEDEVEM PRODUZIR OUTROESTA NA HORA DE PODERMOS ESCOLHER O QUE MELHOR SE ADAPTA</t>
+  </si>
+  <si>
+    <t>Nada negativo quanto ao produto, porém, quanto ao atendimento sempre tenho problemas. Ficam ligando e mandando mensagens sendo redundantes e o técnico ainda não cumpre o período agendado.</t>
+  </si>
+  <si>
+    <t>Fui ignorado por semanas. Só depois que me queixei no Reclame Aqui eu tive minja demanda atendida. O serviço já foi muito melhor...</t>
+  </si>
+  <si>
+    <t>Nos últimos anos está sendo péssima a realização de manutenção e comunicação com a empresa</t>
+  </si>
+  <si>
+    <t>Bem complicado o atendimento técnico. Tive que agendar 3 datas porque apesar de confirmadas as visitas o técnico não compareceu e nem recebi qualquer justificativa/ comunicação da empresa.Ontem o técnico compareceu sem qualquer agendamento/comunicação prévia… uma bagunça</t>
+  </si>
+  <si>
+    <t>Quando marquei a visita era pq tinha gosto na água, a pessoa me disse que não estava programado para troca, fez um teste e a água estava amarelada. Ele pegou um elemento filtrante sem embalagem ou lacrado e trocou. No dia seguinte minha bancada estava totalmente encharcado de água. Não sei o que ele fez só sei que estragou o que está certo além de colocar um elemento filtrante sem lembalagem e lacrado, que estava aberto em sua mochila. Nem fez higiene da própria e tb não fez a limpeza que sempre quem vem trocar ao abrir o purificador para troca o faz.Higiene  fundamental pois pode contaminar o resto do ambiente já que nem fez a higiene das mãos .Segurança é muito importante, precisamos ter segurança de que tudo garanta nossa saúde.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vazamento </t>
+  </si>
+  <si>
+    <t>A visita técnica somente fez a limpeza e não trocou o que foi solicitado pelo telefone</t>
+  </si>
+  <si>
+    <t>Estou com problema a meses e ninguémResolve</t>
+  </si>
+  <si>
+    <t>Não vieram fazer a manutenção !</t>
+  </si>
+  <si>
+    <t>Já tenho, uma experiência de longos anos! No momento estou satisfeita, tanto com o produto e com a manutenção..</t>
+  </si>
+  <si>
+    <t>Não recebemos visita técnica na data e horário marcado.</t>
+  </si>
+  <si>
+    <t>Tive até agora 3 visitas de técnico. O meu bebedouro continua c problema isto é, não está refrigerando. Esta situação já está pelo menos a 30 dias. Preciso de um atendimento urgente e eficaz.</t>
+  </si>
+  <si>
+    <t>Muito bom! Feito como se esperava.Observação: pedido para trocar o bico da saída água, técnico não o possuía e pediu entrar em contato com a empresa</t>
+  </si>
+  <si>
+    <t>Os equipamentos apresentam problemas com frequência e, quando é necessário realizar a troca, mesmo com parecer técnico, há uma demora demasiada em fazer. Muito ruim!</t>
+  </si>
+  <si>
+    <t>O purificar é otimo mas a assistencia tecnica e muito complicada. o APP deles e pessimo, voce fica um tempão para finalizar um atendimento. Coisa que não temos mais hoje em dia. Sem contar que agendaram parte da manha, e so apareceram as 1530 h. Foi muito desgastante.</t>
+  </si>
+  <si>
+    <t>Tenho 13 anos de purificador e o descaso da Brastemp com o atendimento de manutenção está horrível, liguei cinco vezes para poder ser atendido por uma coisa básica, manutenção semestral quando deveria ser um serviço automático, só recebi a visita do técnico quando informei que só realizaria os pagamentos das próximas faturas depois da visita técnica, espero que não ocorra nas próximas manutenções, devido ao tempo da demora água do purificador estava com gosto ruim</t>
+  </si>
+  <si>
+    <t>O purificador é eficiente e cumpre seu papel, contudo os purificadores deveriam sofrer substituição após o período de depreciação de forma que os assinantes possam usufruir de produtos mais eficientes e atualizados. A simples comodidade da manutenção não justifica o valor cobrado mensalmente. Eu sou cliente de vocês, há 17 anos e só tive meu purificador trocado há 5 anos atrás e pagando mensalidade muito proxima dos contratos referentes aos novos modelos.</t>
+  </si>
+  <si>
+    <t>Ultimamente,  sempre está dando problemas nos aparelhos</t>
   </si>
 </sst>
 </file>
@@ -4162,7 +4432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1116"/>
+  <dimension ref="A1:I1196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -36541,6 +36811,2326 @@
         <v>50</v>
       </c>
     </row>
+    <row r="1117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1117" s="4">
+        <v>116</v>
+      </c>
+      <c r="B1117" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1117" s="4">
+        <v>52484</v>
+      </c>
+      <c r="D1117" s="2">
+        <v>46163.412106481483</v>
+      </c>
+      <c r="E1117" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F1117" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1117" s="4" t="s">
+        <v>1220</v>
+      </c>
+      <c r="H1117" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1117" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1118" s="4">
+        <v>117</v>
+      </c>
+      <c r="B1118" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1118" s="4">
+        <v>52840</v>
+      </c>
+      <c r="D1118" s="2">
+        <v>46163.423263888886</v>
+      </c>
+      <c r="E1118" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1118" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1118" s="4" t="s">
+        <v>1221</v>
+      </c>
+      <c r="H1118" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1118" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1119" s="4">
+        <v>118</v>
+      </c>
+      <c r="B1119" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1119" s="4">
+        <v>39386</v>
+      </c>
+      <c r="D1119" s="2">
+        <v>46163.425162037034</v>
+      </c>
+      <c r="E1119" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1119" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1119" s="4" t="s">
+        <v>1222</v>
+      </c>
+      <c r="H1119" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1119" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1120" s="4">
+        <v>119</v>
+      </c>
+      <c r="B1120" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1120" s="4">
+        <v>39716</v>
+      </c>
+      <c r="D1120" s="2">
+        <v>46163.431979166664</v>
+      </c>
+      <c r="E1120" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1120" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1120" s="4" t="s">
+        <v>1223</v>
+      </c>
+      <c r="H1120" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1120" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1121" s="4">
+        <v>120</v>
+      </c>
+      <c r="B1121" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1121" s="4">
+        <v>47382</v>
+      </c>
+      <c r="D1121" s="2">
+        <v>46163.44604166667</v>
+      </c>
+      <c r="E1121" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1121" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1121" s="4" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H1121" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1121" s="4" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1122" s="4">
+        <v>121</v>
+      </c>
+      <c r="B1122" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1122" s="4">
+        <v>53662</v>
+      </c>
+      <c r="D1122" s="2">
+        <v>46163.446157407408</v>
+      </c>
+      <c r="E1122" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1122" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1122" s="4" t="s">
+        <v>1226</v>
+      </c>
+      <c r="H1122" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1122" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1123" s="4">
+        <v>122</v>
+      </c>
+      <c r="B1123" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1123" s="4">
+        <v>47902</v>
+      </c>
+      <c r="D1123" s="2">
+        <v>46163.448125000003</v>
+      </c>
+      <c r="E1123" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1123" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1123" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="H1123" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1123" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1124" s="4">
+        <v>123</v>
+      </c>
+      <c r="B1124" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1124" s="4">
+        <v>50119</v>
+      </c>
+      <c r="D1124" s="2">
+        <v>46163.526875000003</v>
+      </c>
+      <c r="E1124" s="4" t="s">
+        <v>916</v>
+      </c>
+      <c r="F1124" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1124" s="4" t="s">
+        <v>1228</v>
+      </c>
+      <c r="H1124" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1124" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1125" s="4">
+        <v>124</v>
+      </c>
+      <c r="B1125" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1125" s="4">
+        <v>40867</v>
+      </c>
+      <c r="D1125" s="2">
+        <v>46163.529988425929</v>
+      </c>
+      <c r="E1125" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F1125" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1125" s="4" t="s">
+        <v>1229</v>
+      </c>
+      <c r="H1125" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1125" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1126" s="4">
+        <v>125</v>
+      </c>
+      <c r="B1126" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1126" s="4">
+        <v>48393</v>
+      </c>
+      <c r="D1126" s="2">
+        <v>46163.535578703704</v>
+      </c>
+      <c r="E1126" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1126" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1126" s="4" t="s">
+        <v>1230</v>
+      </c>
+      <c r="H1126" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1126" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1127" s="4">
+        <v>126</v>
+      </c>
+      <c r="B1127" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1127" s="4">
+        <v>49366</v>
+      </c>
+      <c r="D1127" s="2">
+        <v>46163.546944444446</v>
+      </c>
+      <c r="E1127" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1127" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1127" s="4" t="s">
+        <v>1231</v>
+      </c>
+      <c r="H1127" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1127" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1128" s="4">
+        <v>127</v>
+      </c>
+      <c r="B1128" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1128" s="4">
+        <v>50519</v>
+      </c>
+      <c r="D1128" s="2">
+        <v>46163.592511574076</v>
+      </c>
+      <c r="E1128" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="F1128" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1128" s="4" t="s">
+        <v>1232</v>
+      </c>
+      <c r="H1128" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1128" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1129" s="4">
+        <v>128</v>
+      </c>
+      <c r="B1129" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1129" s="4">
+        <v>48070</v>
+      </c>
+      <c r="D1129" s="2">
+        <v>46163.600636574076</v>
+      </c>
+      <c r="E1129" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1129" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1129" s="4" t="s">
+        <v>1233</v>
+      </c>
+      <c r="H1129" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1129" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1130" s="4">
+        <v>129</v>
+      </c>
+      <c r="B1130" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1130" s="4">
+        <v>40382</v>
+      </c>
+      <c r="D1130" s="2">
+        <v>46163.620625000003</v>
+      </c>
+      <c r="E1130" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="F1130" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1130" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="H1130" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1130" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1131" s="4">
+        <v>130</v>
+      </c>
+      <c r="B1131" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1131" s="4">
+        <v>55562</v>
+      </c>
+      <c r="D1131" s="2">
+        <v>46164.391006944446</v>
+      </c>
+      <c r="E1131" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1131" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1131" s="4" t="s">
+        <v>1234</v>
+      </c>
+      <c r="H1131" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1131" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1132" s="4">
+        <v>131</v>
+      </c>
+      <c r="B1132" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1132" s="4">
+        <v>55801</v>
+      </c>
+      <c r="D1132" s="2">
+        <v>46164.515416666669</v>
+      </c>
+      <c r="E1132" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="F1132" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1132" s="4" t="s">
+        <v>1235</v>
+      </c>
+      <c r="H1132" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1132" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1133" s="4">
+        <v>132</v>
+      </c>
+      <c r="B1133" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1133" s="4">
+        <v>52047</v>
+      </c>
+      <c r="D1133" s="2">
+        <v>46164.517291666663</v>
+      </c>
+      <c r="E1133" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1133" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1133" s="4" t="s">
+        <v>1236</v>
+      </c>
+      <c r="H1133" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1133" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1134" s="4">
+        <v>133</v>
+      </c>
+      <c r="B1134" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1134" s="4">
+        <v>44961</v>
+      </c>
+      <c r="D1134" s="2">
+        <v>46164.523020833331</v>
+      </c>
+      <c r="E1134" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1134" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1134" s="4" t="s">
+        <v>1237</v>
+      </c>
+      <c r="H1134" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1134" s="4" t="s">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1135" s="4">
+        <v>134</v>
+      </c>
+      <c r="B1135" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1135" s="4">
+        <v>50117</v>
+      </c>
+      <c r="D1135" s="2">
+        <v>46164.534467592595</v>
+      </c>
+      <c r="E1135" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1135" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1135" s="4" t="s">
+        <v>1239</v>
+      </c>
+      <c r="H1135" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1135" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1136" s="4">
+        <v>135</v>
+      </c>
+      <c r="B1136" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1136" s="4">
+        <v>51319</v>
+      </c>
+      <c r="D1136" s="2">
+        <v>46164.558356481481</v>
+      </c>
+      <c r="E1136" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1136" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1136" s="4" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H1136" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1136" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1137" s="4">
+        <v>136</v>
+      </c>
+      <c r="B1137" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1137" s="4">
+        <v>49347</v>
+      </c>
+      <c r="D1137" s="2">
+        <v>46164.633148148147</v>
+      </c>
+      <c r="E1137" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1137" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1137" s="4" t="s">
+        <v>1241</v>
+      </c>
+      <c r="H1137" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1137" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1138" s="4">
+        <v>137</v>
+      </c>
+      <c r="B1138" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1138" s="4">
+        <v>54945</v>
+      </c>
+      <c r="D1138" s="2">
+        <v>46164.73101851852</v>
+      </c>
+      <c r="E1138" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1138" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1138" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="H1138" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1138" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1139" s="4">
+        <v>138</v>
+      </c>
+      <c r="B1139" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1139" s="4">
+        <v>46552</v>
+      </c>
+      <c r="D1139" s="2">
+        <v>46167.276979166665</v>
+      </c>
+      <c r="E1139" s="4" t="s">
+        <v>902</v>
+      </c>
+      <c r="F1139" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1139" s="4" t="s">
+        <v>1243</v>
+      </c>
+      <c r="H1139" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1139" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1140" s="4">
+        <v>139</v>
+      </c>
+      <c r="B1140" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1140" s="4">
+        <v>53969</v>
+      </c>
+      <c r="D1140" s="2">
+        <v>46167.379629629628</v>
+      </c>
+      <c r="E1140" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1140" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1140" s="4" t="s">
+        <v>1245</v>
+      </c>
+      <c r="H1140" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1140" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1141" s="4">
+        <v>140</v>
+      </c>
+      <c r="B1141" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1141" s="4">
+        <v>49597</v>
+      </c>
+      <c r="D1141" s="2">
+        <v>46167.385462962964</v>
+      </c>
+      <c r="E1141" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1141" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1141" s="4" t="s">
+        <v>1247</v>
+      </c>
+      <c r="H1141" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1141" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1142" s="4">
+        <v>141</v>
+      </c>
+      <c r="B1142" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1142" s="4">
+        <v>52963</v>
+      </c>
+      <c r="D1142" s="2">
+        <v>46167.401770833334</v>
+      </c>
+      <c r="E1142" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1142" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1142" s="4" t="s">
+        <v>1249</v>
+      </c>
+      <c r="H1142" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1142" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1143" s="4">
+        <v>142</v>
+      </c>
+      <c r="B1143" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1143" s="4">
+        <v>39637</v>
+      </c>
+      <c r="D1143" s="2">
+        <v>46167.406064814815</v>
+      </c>
+      <c r="E1143" s="4" t="s">
+        <v>1250</v>
+      </c>
+      <c r="F1143" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1143" s="4" t="s">
+        <v>1251</v>
+      </c>
+      <c r="H1143" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1143" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1144" s="4">
+        <v>143</v>
+      </c>
+      <c r="B1144" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1144" s="4">
+        <v>49739</v>
+      </c>
+      <c r="D1144" s="2">
+        <v>46167.435416666667</v>
+      </c>
+      <c r="E1144" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1144" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1144" s="4" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H1144" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1144" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1145" s="4">
+        <v>144</v>
+      </c>
+      <c r="B1145" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1145" s="4">
+        <v>49566</v>
+      </c>
+      <c r="D1145" s="2">
+        <v>46167.437094907407</v>
+      </c>
+      <c r="E1145" s="4" t="s">
+        <v>1250</v>
+      </c>
+      <c r="F1145" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1145" s="4" t="s">
+        <v>1253</v>
+      </c>
+      <c r="H1145" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1145" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1146" s="4">
+        <v>145</v>
+      </c>
+      <c r="B1146" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1146" s="4">
+        <v>53459</v>
+      </c>
+      <c r="D1146" s="2">
+        <v>46167.482997685183</v>
+      </c>
+      <c r="E1146" s="4" t="s">
+        <v>1254</v>
+      </c>
+      <c r="F1146" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1146" s="4" t="s">
+        <v>1255</v>
+      </c>
+      <c r="H1146" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1146" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1147" s="4">
+        <v>146</v>
+      </c>
+      <c r="B1147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1147" s="4">
+        <v>53223</v>
+      </c>
+      <c r="D1147" s="2">
+        <v>46167.524618055555</v>
+      </c>
+      <c r="E1147" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1147" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1147" s="4" t="s">
+        <v>1256</v>
+      </c>
+      <c r="H1147" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1147" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1148" s="4">
+        <v>147</v>
+      </c>
+      <c r="B1148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1148" s="4">
+        <v>52330</v>
+      </c>
+      <c r="D1148" s="2">
+        <v>46167.527696759258</v>
+      </c>
+      <c r="E1148" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1148" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1148" s="4" t="s">
+        <v>1257</v>
+      </c>
+      <c r="H1148" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1148" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1149" s="4">
+        <v>148</v>
+      </c>
+      <c r="B1149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1149" s="4">
+        <v>56241</v>
+      </c>
+      <c r="D1149" s="2">
+        <v>46167.533009259256</v>
+      </c>
+      <c r="E1149" s="4" t="s">
+        <v>1258</v>
+      </c>
+      <c r="F1149" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1149" s="4" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H1149" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1149" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1150" s="4">
+        <v>149</v>
+      </c>
+      <c r="B1150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1150" s="4">
+        <v>59000</v>
+      </c>
+      <c r="D1150" s="2">
+        <v>46167.548067129632</v>
+      </c>
+      <c r="E1150" s="4" t="s">
+        <v>1254</v>
+      </c>
+      <c r="F1150" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1150" s="4" t="s">
+        <v>1260</v>
+      </c>
+      <c r="H1150" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1150" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1151" s="4">
+        <v>150</v>
+      </c>
+      <c r="B1151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1151" s="4">
+        <v>56606</v>
+      </c>
+      <c r="D1151" s="2">
+        <v>46167.570023148146</v>
+      </c>
+      <c r="E1151" s="4" t="s">
+        <v>1261</v>
+      </c>
+      <c r="F1151" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1151" s="4" t="s">
+        <v>1262</v>
+      </c>
+      <c r="H1151" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1151" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1152" s="4">
+        <v>151</v>
+      </c>
+      <c r="B1152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1152" s="4">
+        <v>56418</v>
+      </c>
+      <c r="D1152" s="2">
+        <v>46167.576493055552</v>
+      </c>
+      <c r="E1152" s="4" t="s">
+        <v>1263</v>
+      </c>
+      <c r="F1152" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1152" s="4" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H1152" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1152" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1153" s="4">
+        <v>152</v>
+      </c>
+      <c r="B1153" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1153" s="4">
+        <v>55770</v>
+      </c>
+      <c r="D1153" s="2">
+        <v>46167.612407407411</v>
+      </c>
+      <c r="E1153" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="F1153" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1153" s="4" t="s">
+        <v>1265</v>
+      </c>
+      <c r="H1153" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1153" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1154" s="4">
+        <v>153</v>
+      </c>
+      <c r="B1154" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1154" s="4">
+        <v>55431</v>
+      </c>
+      <c r="D1154" s="2">
+        <v>46167.623333333337</v>
+      </c>
+      <c r="E1154" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="F1154" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1154" s="4" t="s">
+        <v>1266</v>
+      </c>
+      <c r="H1154" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1154" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1155" s="4">
+        <v>154</v>
+      </c>
+      <c r="B1155" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1155" s="4">
+        <v>58774</v>
+      </c>
+      <c r="D1155" s="2">
+        <v>46167.65865740741</v>
+      </c>
+      <c r="E1155" s="4" t="s">
+        <v>1254</v>
+      </c>
+      <c r="F1155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1155" s="4" t="s">
+        <v>1267</v>
+      </c>
+      <c r="H1155" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1155" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1156" s="4">
+        <v>155</v>
+      </c>
+      <c r="B1156" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1156" s="4">
+        <v>54294</v>
+      </c>
+      <c r="D1156" s="2">
+        <v>46167.667696759258</v>
+      </c>
+      <c r="E1156" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1156" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1156" s="4" t="s">
+        <v>1268</v>
+      </c>
+      <c r="H1156" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1156" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1157" s="4">
+        <v>156</v>
+      </c>
+      <c r="B1157" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1157" s="4">
+        <v>47621</v>
+      </c>
+      <c r="D1157" s="2">
+        <v>46167.734166666669</v>
+      </c>
+      <c r="E1157" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1157" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1157" s="4" t="s">
+        <v>1269</v>
+      </c>
+      <c r="H1157" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1157" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1158" s="4">
+        <v>157</v>
+      </c>
+      <c r="B1158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1158" s="4">
+        <v>54899</v>
+      </c>
+      <c r="D1158" s="2">
+        <v>46167.739224537036</v>
+      </c>
+      <c r="E1158" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="F1158" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1158" s="4" t="s">
+        <v>1270</v>
+      </c>
+      <c r="H1158" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1158" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1159" s="4">
+        <v>158</v>
+      </c>
+      <c r="B1159" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1159" s="4">
+        <v>33391</v>
+      </c>
+      <c r="D1159" s="2">
+        <v>46168.483761574076</v>
+      </c>
+      <c r="E1159" s="4" t="s">
+        <v>926</v>
+      </c>
+      <c r="F1159" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1159" s="4" t="s">
+        <v>1271</v>
+      </c>
+      <c r="H1159" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1159" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1160" s="4">
+        <v>159</v>
+      </c>
+      <c r="B1160" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1160" s="4">
+        <v>41275</v>
+      </c>
+      <c r="D1160" s="2">
+        <v>46168.552893518521</v>
+      </c>
+      <c r="E1160" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1160" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1160" s="4" t="s">
+        <v>1272</v>
+      </c>
+      <c r="H1160" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1160" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1161" s="4">
+        <v>160</v>
+      </c>
+      <c r="B1161" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1161" s="4">
+        <v>54782</v>
+      </c>
+      <c r="D1161" s="2">
+        <v>46168.597361111111</v>
+      </c>
+      <c r="E1161" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1161" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1161" s="4" t="s">
+        <v>1273</v>
+      </c>
+      <c r="H1161" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1161" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1162" s="4">
+        <v>161</v>
+      </c>
+      <c r="B1162" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1162" s="4">
+        <v>50375</v>
+      </c>
+      <c r="D1162" s="2">
+        <v>46168.59784722222</v>
+      </c>
+      <c r="E1162" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1162" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1162" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="H1162" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1162" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1163" s="4">
+        <v>162</v>
+      </c>
+      <c r="B1163" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1163" s="4">
+        <v>41157</v>
+      </c>
+      <c r="D1163" s="2">
+        <v>46168.598379629628</v>
+      </c>
+      <c r="E1163" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1163" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1163" s="4" t="s">
+        <v>1275</v>
+      </c>
+      <c r="H1163" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1163" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1164" s="4">
+        <v>163</v>
+      </c>
+      <c r="B1164" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1164" s="4">
+        <v>54115</v>
+      </c>
+      <c r="D1164" s="2">
+        <v>46168.59988425926</v>
+      </c>
+      <c r="E1164" s="4" t="s">
+        <v>1258</v>
+      </c>
+      <c r="F1164" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1164" s="4" t="s">
+        <v>1276</v>
+      </c>
+      <c r="H1164" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1164" s="4" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1165" s="4">
+        <v>164</v>
+      </c>
+      <c r="B1165" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1165" s="4">
+        <v>51135</v>
+      </c>
+      <c r="D1165" s="2">
+        <v>46168.599930555552</v>
+      </c>
+      <c r="E1165" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1165" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1165" s="4" t="s">
+        <v>1278</v>
+      </c>
+      <c r="H1165" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1165" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1166" s="4">
+        <v>165</v>
+      </c>
+      <c r="B1166" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1166" s="4">
+        <v>52826</v>
+      </c>
+      <c r="D1166" s="2">
+        <v>46168.600243055553</v>
+      </c>
+      <c r="E1166" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1166" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1166" s="4" t="s">
+        <v>1279</v>
+      </c>
+      <c r="H1166" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1166" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1167" s="4">
+        <v>166</v>
+      </c>
+      <c r="B1167" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1167" s="4">
+        <v>49372</v>
+      </c>
+      <c r="D1167" s="2">
+        <v>46168.601759259262</v>
+      </c>
+      <c r="E1167" s="4" t="s">
+        <v>924</v>
+      </c>
+      <c r="F1167" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1167" s="4" t="s">
+        <v>1280</v>
+      </c>
+      <c r="H1167" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1167" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1168" s="4">
+        <v>167</v>
+      </c>
+      <c r="B1168" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1168" s="4">
+        <v>58597</v>
+      </c>
+      <c r="D1168" s="2">
+        <v>46168.621851851851</v>
+      </c>
+      <c r="E1168" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1168" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1168" s="4" t="s">
+        <v>1281</v>
+      </c>
+      <c r="H1168" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1168" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1169" s="4">
+        <v>168</v>
+      </c>
+      <c r="B1169" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1169" s="4">
+        <v>52479</v>
+      </c>
+      <c r="D1169" s="2">
+        <v>46168.626793981479</v>
+      </c>
+      <c r="E1169" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1169" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1169" s="4" t="s">
+        <v>1282</v>
+      </c>
+      <c r="H1169" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1169" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1170" s="4">
+        <v>169</v>
+      </c>
+      <c r="B1170" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1170" s="4">
+        <v>54071</v>
+      </c>
+      <c r="D1170" s="2">
+        <v>46168.648032407407</v>
+      </c>
+      <c r="E1170" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1170" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1170" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H1170" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1170" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1171" s="4">
+        <v>170</v>
+      </c>
+      <c r="B1171" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1171" s="4">
+        <v>54665</v>
+      </c>
+      <c r="D1171" s="2">
+        <v>46168.724305555559</v>
+      </c>
+      <c r="E1171" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1171" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1171" s="4" t="s">
+        <v>1284</v>
+      </c>
+      <c r="H1171" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1171" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1172" s="4">
+        <v>171</v>
+      </c>
+      <c r="B1172" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1172" s="4">
+        <v>46703</v>
+      </c>
+      <c r="D1172" s="2">
+        <v>46169.333564814813</v>
+      </c>
+      <c r="E1172" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1172" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1172" s="4" t="s">
+        <v>1285</v>
+      </c>
+      <c r="H1172" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1172" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1173" s="4">
+        <v>172</v>
+      </c>
+      <c r="B1173" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1173" s="4">
+        <v>25971</v>
+      </c>
+      <c r="D1173" s="2">
+        <v>46169.361956018518</v>
+      </c>
+      <c r="E1173" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1173" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1173" s="4" t="s">
+        <v>1286</v>
+      </c>
+      <c r="H1173" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1173" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1174" s="4">
+        <v>173</v>
+      </c>
+      <c r="B1174" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1174" s="4">
+        <v>48383</v>
+      </c>
+      <c r="D1174" s="2">
+        <v>46169.367002314815</v>
+      </c>
+      <c r="E1174" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1174" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1174" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="H1174" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1174" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1175" s="4">
+        <v>174</v>
+      </c>
+      <c r="B1175" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1175" s="4">
+        <v>49998</v>
+      </c>
+      <c r="D1175" s="2">
+        <v>46169.370486111111</v>
+      </c>
+      <c r="E1175" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="F1175" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1175" s="4" t="s">
+        <v>1288</v>
+      </c>
+      <c r="H1175" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1175" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1176" s="4">
+        <v>175</v>
+      </c>
+      <c r="B1176" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1176" s="4">
+        <v>54329</v>
+      </c>
+      <c r="D1176" s="2">
+        <v>46169.418136574073</v>
+      </c>
+      <c r="E1176" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1176" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1176" s="4" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H1176" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1176" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1177" s="4">
+        <v>176</v>
+      </c>
+      <c r="B1177" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1177" s="4">
+        <v>21252</v>
+      </c>
+      <c r="D1177" s="2">
+        <v>46169.527372685188</v>
+      </c>
+      <c r="E1177" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1177" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1177" s="4" t="s">
+        <v>1290</v>
+      </c>
+      <c r="H1177" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1177" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1178" s="4">
+        <v>177</v>
+      </c>
+      <c r="B1178" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1178" s="4">
+        <v>55832</v>
+      </c>
+      <c r="D1178" s="2">
+        <v>46169.527430555558</v>
+      </c>
+      <c r="E1178" s="4" t="s">
+        <v>679</v>
+      </c>
+      <c r="F1178" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1178" s="4" t="s">
+        <v>1291</v>
+      </c>
+      <c r="H1178" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1178" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1179" s="4">
+        <v>178</v>
+      </c>
+      <c r="B1179" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1179" s="4">
+        <v>58695</v>
+      </c>
+      <c r="D1179" s="2">
+        <v>46169.528958333336</v>
+      </c>
+      <c r="E1179" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1179" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1179" s="4" t="s">
+        <v>1292</v>
+      </c>
+      <c r="H1179" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1179" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1180" s="4">
+        <v>179</v>
+      </c>
+      <c r="B1180" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1180" s="4">
+        <v>55975</v>
+      </c>
+      <c r="D1180" s="2">
+        <v>46169.529664351852</v>
+      </c>
+      <c r="E1180" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="F1180" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1180" s="4" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H1180" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1180" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1181" s="4">
+        <v>180</v>
+      </c>
+      <c r="B1181" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1181" s="4">
+        <v>57004</v>
+      </c>
+      <c r="D1181" s="2">
+        <v>46169.547534722224</v>
+      </c>
+      <c r="E1181" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1181" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1181" s="4" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H1181" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1181" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1182" s="4">
+        <v>181</v>
+      </c>
+      <c r="B1182" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1182" s="4">
+        <v>56049</v>
+      </c>
+      <c r="D1182" s="2">
+        <v>46169.552916666667</v>
+      </c>
+      <c r="E1182" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="F1182" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1182" s="4" t="s">
+        <v>1295</v>
+      </c>
+      <c r="H1182" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1182" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1183" s="4">
+        <v>182</v>
+      </c>
+      <c r="B1183" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1183" s="4">
+        <v>51830</v>
+      </c>
+      <c r="D1183" s="2">
+        <v>46169.555775462963</v>
+      </c>
+      <c r="E1183" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F1183" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1183" s="4" t="s">
+        <v>1296</v>
+      </c>
+      <c r="H1183" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1183" s="4" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1184" s="4">
+        <v>183</v>
+      </c>
+      <c r="B1184" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1184" s="4">
+        <v>58776</v>
+      </c>
+      <c r="D1184" s="2">
+        <v>46169.560034722221</v>
+      </c>
+      <c r="E1184" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1184" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1184" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H1184" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1184" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1185" s="4">
+        <v>184</v>
+      </c>
+      <c r="B1185" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1185" s="4">
+        <v>48611</v>
+      </c>
+      <c r="D1185" s="2">
+        <v>46169.596851851849</v>
+      </c>
+      <c r="E1185" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1185" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1185" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H1185" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1185" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1186" s="4">
+        <v>185</v>
+      </c>
+      <c r="B1186" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1186" s="4">
+        <v>59306</v>
+      </c>
+      <c r="D1186" s="2">
+        <v>46169.681180555555</v>
+      </c>
+      <c r="E1186" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1186" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1186" s="4" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H1186" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1186" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1187" s="4">
+        <v>186</v>
+      </c>
+      <c r="B1187" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1187" s="4">
+        <v>51669</v>
+      </c>
+      <c r="D1187" s="2">
+        <v>46169.842928240738</v>
+      </c>
+      <c r="E1187" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="F1187" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1187" s="4" t="s">
+        <v>1300</v>
+      </c>
+      <c r="H1187" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1187" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1188" s="4">
+        <v>187</v>
+      </c>
+      <c r="B1188" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1188" s="4">
+        <v>50802</v>
+      </c>
+      <c r="D1188" s="2">
+        <v>46169.883275462962</v>
+      </c>
+      <c r="E1188" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1188" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1188" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="H1188" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1188" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1189" s="4">
+        <v>188</v>
+      </c>
+      <c r="B1189" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1189" s="4">
+        <v>33365</v>
+      </c>
+      <c r="D1189" s="2">
+        <v>46170.453831018516</v>
+      </c>
+      <c r="E1189" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="F1189" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1189" s="4" t="s">
+        <v>1302</v>
+      </c>
+      <c r="H1189" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1189" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1190" s="4">
+        <v>189</v>
+      </c>
+      <c r="B1190" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1190" s="4">
+        <v>60221</v>
+      </c>
+      <c r="D1190" s="2">
+        <v>46170.503692129627</v>
+      </c>
+      <c r="E1190" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="F1190" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1190" s="4" t="s">
+        <v>1303</v>
+      </c>
+      <c r="H1190" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1190" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1191" s="4">
+        <v>190</v>
+      </c>
+      <c r="B1191" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1191" s="4">
+        <v>50885</v>
+      </c>
+      <c r="D1191" s="2">
+        <v>46170.89435185185</v>
+      </c>
+      <c r="E1191" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="F1191" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1191" s="4" t="s">
+        <v>1304</v>
+      </c>
+      <c r="H1191" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1191" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1192" s="4">
+        <v>191</v>
+      </c>
+      <c r="B1192" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1192" s="4">
+        <v>61323</v>
+      </c>
+      <c r="D1192" s="2">
+        <v>46171.374918981484</v>
+      </c>
+      <c r="E1192" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="F1192" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1192" s="4" t="s">
+        <v>1305</v>
+      </c>
+      <c r="H1192" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1192" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1193" s="4">
+        <v>192</v>
+      </c>
+      <c r="B1193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1193" s="4">
+        <v>50131</v>
+      </c>
+      <c r="D1193" s="2">
+        <v>46171.427499999998</v>
+      </c>
+      <c r="E1193" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1193" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1193" s="4" t="s">
+        <v>1306</v>
+      </c>
+      <c r="H1193" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1193" s="4" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1194" s="4">
+        <v>193</v>
+      </c>
+      <c r="B1194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1194" s="4">
+        <v>60108</v>
+      </c>
+      <c r="D1194" s="2">
+        <v>46171.619050925925</v>
+      </c>
+      <c r="E1194" s="4" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1194" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1194" s="4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="H1194" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1194" s="4" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1195" s="4">
+        <v>194</v>
+      </c>
+      <c r="B1195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1195" s="4">
+        <v>51390</v>
+      </c>
+      <c r="D1195" s="2">
+        <v>46171.638101851851</v>
+      </c>
+      <c r="E1195" s="4" t="s">
+        <v>889</v>
+      </c>
+      <c r="F1195" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1195" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="H1195" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1195" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1196" s="4">
+        <v>195</v>
+      </c>
+      <c r="B1196" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1196" s="4">
+        <v>55963</v>
+      </c>
+      <c r="D1196" s="2">
+        <v>46171.658993055556</v>
+      </c>
+      <c r="E1196" s="4" t="s">
+        <v>1254</v>
+      </c>
+      <c r="F1196" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1196" s="4" t="s">
+        <v>1309</v>
+      </c>
+      <c r="H1196" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1196" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/07/2026 14:15:15,68
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="322" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{557AC962-AC73-40DD-BA07-ACBA862F8EFE}"/>
+  <xr:revisionPtr revIDLastSave="342" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3BF358E-CF34-4945-B1B9-F26F1BA47FB6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10403" uniqueCount="1444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10547" uniqueCount="1465">
   <si>
     <t>ID</t>
   </si>
@@ -4477,6 +4477,69 @@
   </si>
   <si>
     <t>Medium Corporate</t>
+  </si>
+  <si>
+    <t>Descontinuar os Robôs nos atendimento, ou atualizar. Aumentar numero de tecnicos disponiveis para tentar melhorar a disponibilidade dos serviços. Cumprir com as datas dos agendamentos (sempre adiam o dia agendado).</t>
+  </si>
+  <si>
+    <t>Repair</t>
+  </si>
+  <si>
+    <t>Preciso de uma data e que resolvam o problema do cliente.</t>
+  </si>
+  <si>
+    <t>Comunicação para evitar desencontros.</t>
+  </si>
+  <si>
+    <t>FRQ PORTO ALEGRE RS R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>A comunicação é muito ruim, precisa melhorar ,uito.</t>
+  </si>
+  <si>
+    <t>manutenção preventiva mais regular</t>
+  </si>
+  <si>
+    <t>Precisam oferecer uma aparelho para alta demanda e menos reparos.</t>
+  </si>
+  <si>
+    <t>Cumprir com prazos e mais qualidade no serviço prestado.</t>
+  </si>
+  <si>
+    <t>O agendamento do atendimento</t>
+  </si>
+  <si>
+    <t>o tempo de troca</t>
+  </si>
+  <si>
+    <t>atendimento completo no mesmo dia</t>
+  </si>
+  <si>
+    <t>Comunicacao, retorno efetivo ou pessoa dedicada para cada cliente.</t>
+  </si>
+  <si>
+    <t>Se temos 10 purificadores de água, porque não agendar um dia para a manutenção preventiva de todos, com o diagnóstico dos problemas de todos, e o profissional para resolver todos de uma vez, ao invés de 15 visitas (e retorno de visitas)...</t>
+  </si>
+  <si>
+    <t>Melhor atendimento e clareza nas informações o que abrange uma manutenção.</t>
+  </si>
+  <si>
+    <t>Atender com profissionalismo, cumprir prazos e entender que o cliente é sempre prioridade.</t>
+  </si>
+  <si>
+    <t>Respeitar os horários indicados - períodos da manhã ou tarde, ex.: das 09 as 12h, não adianta o técnico chegar as 08h, não vai ter ninguém na empresa. Em caso de dificuldade no atendimento, informar a Central de Atendimento imediatamente, agilidade nos agendamento, uma semana é muito tempo para uma instalação em empresa com diversos colaboradores. É preciso filtrar e agilizar alguns serviços. Atendentes com capacidade de identificar o que é urgente e ter autonomia para priorizar o atendimento. Central deve ter alguém que consiga contato com a equipe em campo (técnico).</t>
+  </si>
+  <si>
+    <t>Agilidade, eficiência, tempo de resposta.</t>
+  </si>
+  <si>
+    <t>Preciso que ao confirmar o reparo de 03 filtros, a pessoa venha para realizar o serviço solicitado.</t>
+  </si>
+  <si>
+    <t>retorno das solicitações, serviços executados, informações repassadas para execução do prestador.</t>
+  </si>
+  <si>
+    <t>Large Corporate</t>
   </si>
 </sst>
 </file>
@@ -4849,7 +4912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1300"/>
+  <dimension ref="A1:K1318"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -50366,6 +50429,636 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1301" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1301" s="4">
+        <v>300</v>
+      </c>
+      <c r="B1301" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1301" s="4">
+        <v>38058</v>
+      </c>
+      <c r="D1301" s="2">
+        <v>46160.451111111113</v>
+      </c>
+      <c r="E1301" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1301" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1301" s="4" t="s">
+        <v>1444</v>
+      </c>
+      <c r="H1301" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1301" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1301" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1301" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1302" s="4">
+        <v>301</v>
+      </c>
+      <c r="B1302" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1302" s="4">
+        <v>47729</v>
+      </c>
+      <c r="D1302" s="2">
+        <v>46155.373749999999</v>
+      </c>
+      <c r="E1302" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1302" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1302" s="4" t="s">
+        <v>1446</v>
+      </c>
+      <c r="H1302" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1302" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1302" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1302" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1303" s="4">
+        <v>302</v>
+      </c>
+      <c r="B1303" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1303" s="4">
+        <v>32850</v>
+      </c>
+      <c r="D1303" s="2">
+        <v>46142.267291666663</v>
+      </c>
+      <c r="E1303" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1303" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1303" s="4" t="s">
+        <v>1447</v>
+      </c>
+      <c r="H1303" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1303" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1303" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1303" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1304" s="4">
+        <v>303</v>
+      </c>
+      <c r="B1304" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1304" s="4">
+        <v>13035</v>
+      </c>
+      <c r="D1304" s="2">
+        <v>46141.312245370369</v>
+      </c>
+      <c r="E1304" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1304" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1304" s="4" t="s">
+        <v>1449</v>
+      </c>
+      <c r="H1304" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1304" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1304" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1304" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1305" s="4">
+        <v>304</v>
+      </c>
+      <c r="B1305" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1305" s="4">
+        <v>32906</v>
+      </c>
+      <c r="D1305" s="2">
+        <v>46139.258009259262</v>
+      </c>
+      <c r="E1305" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1305" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1305" s="4" t="s">
+        <v>1450</v>
+      </c>
+      <c r="H1305" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1305" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1305" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1305" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1306" s="4">
+        <v>305</v>
+      </c>
+      <c r="B1306" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1306" s="4">
+        <v>23781</v>
+      </c>
+      <c r="D1306" s="2">
+        <v>46128.346689814818</v>
+      </c>
+      <c r="E1306" s="4" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F1306" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1306" s="4" t="s">
+        <v>1451</v>
+      </c>
+      <c r="H1306" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1306" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1306" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1306" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1307" s="4">
+        <v>306</v>
+      </c>
+      <c r="B1307" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1307" s="4">
+        <v>8005323270</v>
+      </c>
+      <c r="D1307" s="2">
+        <v>46111.304849537039</v>
+      </c>
+      <c r="E1307" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1307" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1307" s="4" t="s">
+        <v>1452</v>
+      </c>
+      <c r="H1307" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1307" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1307" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1307" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1308" s="4">
+        <v>307</v>
+      </c>
+      <c r="B1308" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1308" s="4">
+        <v>8005331414</v>
+      </c>
+      <c r="D1308" s="2">
+        <v>46106.844189814823</v>
+      </c>
+      <c r="E1308" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1308" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1308" s="4" t="s">
+        <v>1453</v>
+      </c>
+      <c r="H1308" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1308" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1308" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1308" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1309" s="4">
+        <v>308</v>
+      </c>
+      <c r="B1309" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1309" s="4">
+        <v>8005322828</v>
+      </c>
+      <c r="D1309" s="2">
+        <v>46106.419687499998</v>
+      </c>
+      <c r="E1309" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1309" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1309" s="4" t="s">
+        <v>1454</v>
+      </c>
+      <c r="H1309" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1309" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1309" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1309" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1310" s="4">
+        <v>309</v>
+      </c>
+      <c r="B1310" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1310" s="4">
+        <v>8005297777</v>
+      </c>
+      <c r="D1310" s="2">
+        <v>46094.543796296297</v>
+      </c>
+      <c r="E1310" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1310" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1310" s="4" t="s">
+        <v>1455</v>
+      </c>
+      <c r="H1310" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1310" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1310" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1310" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1311" s="4">
+        <v>310</v>
+      </c>
+      <c r="B1311" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1311" s="4">
+        <v>1637</v>
+      </c>
+      <c r="D1311" s="2">
+        <v>46087.469074074077</v>
+      </c>
+      <c r="E1311" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="F1311" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1311" s="4" t="s">
+        <v>1456</v>
+      </c>
+      <c r="H1311" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1311" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1311" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1311" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1312" s="4">
+        <v>311</v>
+      </c>
+      <c r="B1312" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1312" s="4">
+        <v>8005267857</v>
+      </c>
+      <c r="D1312" s="2">
+        <v>46076.368449074071</v>
+      </c>
+      <c r="E1312" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1312" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1312" s="4" t="s">
+        <v>1457</v>
+      </c>
+      <c r="H1312" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1312" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1312" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1312" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1313" s="4">
+        <v>312</v>
+      </c>
+      <c r="B1313" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1313" s="4">
+        <v>8005273824</v>
+      </c>
+      <c r="D1313" s="2">
+        <v>46059.434490740743</v>
+      </c>
+      <c r="E1313" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1313" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1313" s="4" t="s">
+        <v>1458</v>
+      </c>
+      <c r="H1313" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1313" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1313" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1313" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1314" s="4">
+        <v>313</v>
+      </c>
+      <c r="B1314" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1314" s="4">
+        <v>8005268010</v>
+      </c>
+      <c r="D1314" s="2">
+        <v>46050.186805555553</v>
+      </c>
+      <c r="E1314" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1314" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1314" s="4" t="s">
+        <v>1459</v>
+      </c>
+      <c r="H1314" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1314" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1314" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1314" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1315" s="4">
+        <v>314</v>
+      </c>
+      <c r="B1315" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1315" s="4">
+        <v>8005262964</v>
+      </c>
+      <c r="D1315" s="2">
+        <v>46041.472581018519</v>
+      </c>
+      <c r="E1315" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1315" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1315" s="4" t="s">
+        <v>1460</v>
+      </c>
+      <c r="H1315" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1315" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1315" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1315" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1316" s="4">
+        <v>315</v>
+      </c>
+      <c r="B1316" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1316" s="4">
+        <v>8005261580</v>
+      </c>
+      <c r="D1316" s="2">
+        <v>46041.344097222223</v>
+      </c>
+      <c r="E1316" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1316" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1316" s="4" t="s">
+        <v>1461</v>
+      </c>
+      <c r="H1316" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1316" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1316" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1316" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1317" s="4">
+        <v>316</v>
+      </c>
+      <c r="B1317" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1317" s="4">
+        <v>8005267856</v>
+      </c>
+      <c r="D1317" s="2">
+        <v>46038.343310185177</v>
+      </c>
+      <c r="E1317" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1317" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1317" s="4" t="s">
+        <v>1462</v>
+      </c>
+      <c r="H1317" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1317" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1317" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1317" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1318" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1318" s="4">
+        <v>317</v>
+      </c>
+      <c r="B1318" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1318" s="4">
+        <v>8005237058</v>
+      </c>
+      <c r="D1318" s="2">
+        <v>46036.277233796303</v>
+      </c>
+      <c r="E1318" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1318" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1318" s="4" t="s">
+        <v>1463</v>
+      </c>
+      <c r="H1318" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1318" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1318" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1318" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/07/2026 14:25:56,57
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="342" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3BF358E-CF34-4945-B1B9-F26F1BA47FB6}"/>
+  <xr:revisionPtr revIDLastSave="346" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D73799EE-65B4-4451-B537-577971CD0735}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1318</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 13/07/2026 18:30:11,10
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/eduardacjr_algartech_com/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="346" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D73799EE-65B4-4451-B537-577971CD0735}"/>
+  <xr:revisionPtr revIDLastSave="353" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3BA484-D7CA-4030-9C81-A2893A9ACDE6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10547" uniqueCount="1465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10835" uniqueCount="1509">
   <si>
     <t>ID</t>
   </si>
@@ -4540,6 +4540,154 @@
   </si>
   <si>
     <t>Large Corporate</t>
+  </si>
+  <si>
+    <t>Detrator</t>
+  </si>
+  <si>
+    <t>Porque antecipou a visita e não fui informada e também não concluiu o reparo, tive que solicitar outro serviço.</t>
+  </si>
+  <si>
+    <t>Foram necessários 4 agendamentos para finalmente um técnico aparecer e resolver o problema, além disso, durante os INÚMEROS protocolos abertos solicitando a correção de vazamento e o fornecimento de água com gás, nenhum dos atendentes tinha autonomia para resolver um problema criado pela própria Culligan.</t>
+  </si>
+  <si>
+    <t>AT FORTALEZA CE R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Solicitei durante todo o mês de junho para manutenção do purificador. Só vieram em primeiro de julho, assim mesmo porque falei para encerrar minha assinatura.</t>
+  </si>
+  <si>
+    <t>Foi o terceiro agendamento cancela e informei ao atendente que a água está com gosto ruim!!!! Desprezo total com o cliente!!!</t>
+  </si>
+  <si>
+    <t>1) Por que nessa página deveria ser separado SEM acento.
+2) Porque o filtro era novinho e já precisou de reparo
+3) Porque VOCÊS mudaram de razão social e simplesmente não transferiram meu débito automático e quando eu precisei de conserto ainda fui tratada como mal pagante porque vocês não haviam feito o débito de 3 meses. 
+Cada vez que eu tenho que falar com vocês, o atendimento é difícil porque sempre tem aquele bot que não quer me mandar para um ser humano e muitas vezes não entende o que precisamos.
+Sou cliente há muitos anos e só agora considero seriamente cancelar. Recomendar, não recomendo mais para ninguém...</t>
+  </si>
+  <si>
+    <t>Pq até agora não foi resolvido o meu problema, empresa totalmente sem compromisso com cliente, inclusive já estou certa de pedir cancelamento do contrato.</t>
+  </si>
+  <si>
+    <t>Por que nn houve a manutenção. O técnico nn compareceu e nn fui avisada pelo setor responsável.</t>
+  </si>
+  <si>
+    <t>FRQ GUARULHOS SP R05</t>
+  </si>
+  <si>
+    <t>nao consigo contato para abertura de chamados a mais de uma semana tentando</t>
+  </si>
+  <si>
+    <t>dificuldade de resolver um problema no meu purificador, a 90 dias estou com o mesmo com defeito, mesmo tendo feito  várias ligações.
+Recentemente trocaram o aparelho e o mesmo está fazendo um barulho anormal e marcaram para daqui a 15 dias para retornarem</t>
+  </si>
+  <si>
+    <t>Serviço caiu muito depois que mudou controle</t>
+  </si>
+  <si>
+    <t>Não foram fiquei esperando e o filtro continua com problema. Pago por filtro com gaz e não estou conseguindo usar</t>
+  </si>
+  <si>
+    <t>AT BAURU SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>o funcionário não compareceu</t>
+  </si>
+  <si>
+    <t>Porque o problema apresentado pelo filtro ainda não foi solucionado. Desde o início do mês de junho tenho aberto chamados para conserto porém o problema ainda persiste.  A água na temperatura ambiente não sai. Está saindo água somente ao selecionar a opção água fria.</t>
+  </si>
+  <si>
+    <t>Visita marcada para um horário, não cumprida, apareceu sem avisar após 2 horas, ficou menos de 5 minutos no atendimento, além do mais, se eu não comunico que não havia comparecido, não iria aparecer, após muito tempo perdido e reclamação no chat, não sabiam o que estava acontecendo e até agora não me disseram o porque de tanto incompetência para realizar uma visita veloz, para esse serviço ficar ruim, precisa melhor muito, pois hoje é péssimo, vocês tem a capacidade de fazer o consumidor esperar por 8 horas e não honrar a visita, e a opção é ou remarque e espere mais 8 horas ou cancele, parabens Brastemp, pelo respeito ao consumidor</t>
+  </si>
+  <si>
+    <t>O técnico não fez a troca da vela do purificador, a água da caixa d'água do prédio que resido, é muito suja. Prefiro que faça a troca, já que feita de seis em seis meses.</t>
+  </si>
+  <si>
+    <t>Infelizmente com vários problemas de recebimento de cobranças , boletos pagos e também confusão com nomes de outra pessoa em meu E Mail. Muito desagradavel</t>
+  </si>
+  <si>
+    <t>FRQ SANTOS SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Fugiu dos padroes anteriores, nao recebi um codigo de autorizacao, nem o nome do tecnico, o tecnico nao tinha o numero do apto. Nao entendi também porque foi realizado esse agendamento, visto que nao tinha nem 6 meses da ultima visita.</t>
+  </si>
+  <si>
+    <t>Essa nota foi por causa de todo o processo e não pela a última visita e interação. Tentei a meses trocar o aparelho... Foi bem na éboca da mudança da razão social e também de sistema.... Chegaram até a trazer um purificar errado aqui em casa..... Mas nessa ultima chamada e interação fui muito bem atendido!!! Porém, não quero deixar de registrar todo o problema que eu tive.</t>
+  </si>
+  <si>
+    <t>FRQ BRAGANCA PAULISTA SP R02</t>
+  </si>
+  <si>
+    <t>Porque simplesmente não apareceu ninguém! Não se deram ao trabalho nem de avisar que não viriam atender. Tive que cancelar compromissos na parte da tarde só para ficar em casa esperando o técnico, para ele simplesmente, não aparecer nem dar satisfação!
+Estou pensando seriamente em cancelar este contrato, pois as últimas 3 vezes foi deste jeito! Só que nas 2 anteriores, o técnico apareceu em casa um ou dois dias depois...</t>
+  </si>
+  <si>
+    <t>estou impressionada com baixa qualidade do serviço de vcs!!!! trocaram meu purificador depois de meses pedindo, e agora que instalaram, VAZA SEM parar, liguei pedindo urgência e só podem
+ ir em 10 dias. ABSURDO!!! NÃO DÁ PRA CONTINUAR!!! PAGO PRLO SERVICO</t>
+  </si>
+  <si>
+    <t>FRQ ATLANTICA RJ R03</t>
+  </si>
+  <si>
+    <t>Sou cliente da Brastemp há anos e tenho tido uma dificuldade no atendimento com vocês. Marcam visitas e não comparecem, sequer avisam que não virão. Por fim trocaram meu aparelho e no dia seguinte deu defeito. Não sai agua gelada.  Absurdo</t>
+  </si>
+  <si>
+    <t>Já há uma semana meu purificador apresentou problema e o técnico, que veio verificar o problema, constatou a necessidade da trocado aparelho.  Entrando em contato com a empresa, me disseram que não há aparelho disponível em estoque, que será necessário aguardar.  Até quando vou ficar sem o purificador de água?</t>
+  </si>
+  <si>
+    <t>Não estou avaliando o serviço, mas sim chamando a atenção de vocês patra a troca da mangueira d'água, já havia pedido, a pressão no cano é muito forte, e a mangueira que vocês colocaram não me parece forte o bastante.</t>
+  </si>
+  <si>
+    <t>A VISITA NAO FOI REALIZADA, MEU APARELHO CONTINUA COM DEFEITO. SERVIÇO PÉSSIMO. UM AMIGO QUE INDIQUEI COM O MESMO PROBLEMA. PROVAVELMENTE IREI CANCELAR O SERVIÇO.</t>
+  </si>
+  <si>
+    <t>O problema não foi resolvido. Estou aguardando peça para reposição. Continuo com filtro desligado.</t>
+  </si>
+  <si>
+    <t>Passei uma semana com vazamento no filtro e sem agua filtrada. Entrei em contato muitas vezes por telefone com a Brastemp. As visitas técnicas eram desmarcadas sem aviso previo. Um tecnico acabou indo sem avisar há semanas e solucionou o problema. Passadas essas semanas, comecei a receber mensagens no WhatsApp sobre a realização da visita tecnica que já havia sido efetuada. Tecnico chegou a ir em casa recentemente e não sabia do ocorrido anteriormente. Resumo: a experiência foi péssima e a desorganização é evidente. Se ocorrer novamente, terei que cancelar a assinatura.</t>
+  </si>
+  <si>
+    <t>FRQ JOINVILLE SC R03</t>
+  </si>
+  <si>
+    <t>A manutenção foi antecipada em mais de 1 mês, não foi avisada, o técnico simplesmente apareceu aqui sem nenhum aviso prévio. Verificou a máquina, não trocou o filtro. Sendo que qualquer filtro deve ser trocado com 6 meses de uso. Ele fez testes com a água e disse que estava ok. Eu desconheço esse procedimento, mesmo porque na assinatura está muito claro de que o filtro se troca a cada 6 meses. Então ficou tudo muito estranho. Ele foi extremamente simpático, educado. Mas esses 2 fatos: aparecer sem avisar e não trocar o filtro, me deixo incomodado.</t>
+  </si>
+  <si>
+    <t>Solicitamos visita técnica desde dezembro/25 e somente em 08/07/2025 que fomos atendido.
+O técnico (infelizmente não lembro o nome) foi super atencioso, educado, mostrou o filtro que trocou etc. e fez anotações para facilitar as próximas visitas, pois os técnicos anteriores alegaram que não encontraram o endereço.</t>
+  </si>
+  <si>
+    <t>Não veio no horário combinado 
+Atrasou 1:30, fez eu faltar no meu serviço.
+Trouxe um purificador com peças que não encaixam, faltando uma perna do suporte
+Teve que arrancar as outras para nivelar 
+E a pressão da água está forte e molhando a cozinha.</t>
+  </si>
+  <si>
+    <t>o produto é ruim, a assistencia técnica é ruim e os meios de contato com a Brastemp não funcionam. Em relação a proxima pergunta sobre o que motivou minha nota zero, todos os argumentos elencados se aplicam. Selecionei apenas um porque o sistema não permite mais de 1 opção</t>
+  </si>
+  <si>
+    <t>No dia 07/07/26, o técnico veio fazer a limpeza da purificador e deixou um vazamento que infiltrou nas gavetas do armário. Ao ligar para a Brastemp informaram que só teria atendimento no dia 17/07 então a atendente disse que iria avaliar se seria possível antecipar para o dia 10/07 mas avisaria antes.  Além do móvel estragado tivemos que comprar garrafas de água.</t>
+  </si>
+  <si>
+    <t>Bom dia.
+RIDÌCULO eu não poder indicar alguém para programar a manutenção.
+Exemplo: Eu fechei com vcs porque minha esposa que é dona de casa exigiu. Mas não é comigo que tem que programar a data e o horário da manutenção e mto menos o técnico me mandar mensagem que vai mudar o horário que eu perdi umas 3hs de trabalho para conseguir marcar.
+Peço incluir minha esposa como contato da Brastemp, ou CANCELAR minha assinatura URGENTE!!!</t>
+  </si>
+  <si>
+    <t>Não foi resolvido o problema. E agora so vem em 4 dias. Estamos sem agua</t>
+  </si>
+  <si>
+    <t>Fiz agendamento para retirada do aparelho após o cancelamento em 9/06 . Ou seja demoraram 1 mês não cancelaram e marcaram com visita técnica… espero q também não estejam me cobrando já  que não cancelaram 
+Aguardo retorno</t>
+  </si>
+  <si>
+    <t>fizeram a manutenção e treocaram o filtro   porem quase não sai agua,  dizeram que vao retornar e ate agora nada</t>
+  </si>
+  <si>
+    <t>O atendimento do técnico foi bom. De fato não sei qual o diferencial do purificador Brastemp para água Sabesp.Técnico usou um reagente que muda a cor da água sinalizando a presença de cloro. Pedi para ele testar outras fontes de água:  1) Purificador: água se manteve transparente e cristalina 2) Água da torneira fria: agua da Sabesp entra,passa por uma cisterna de 8 mil litros, duas bombas distribuem água para 3 caixas dágua. Ao testar, um copo com essa água, ela se manteve transparente e cristalina. Pergunta: se essa água, fica em caixa dágua, que no máximo é feito uma limpeza a cada 2 anos, como não sinalizou nenhum problema? 3) Agua da torneira quente: além do descrito no item 2, a água vai para um boiler de 250 l. Também ao testar se manteve transparente e cristalina. 4) Água da piscina: foi a única que reagiu e ficou amarelada (por causa do cloro). Pergunta: ou o teste feito está errado, usando somente reação cloro, ou não tem diferença entre usar água da torneira e brastemp.</t>
   </si>
 </sst>
 </file>
@@ -4912,7 +5060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1318"/>
+  <dimension ref="A1:K1354"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -51059,6 +51207,1266 @@
         <v>1464</v>
       </c>
     </row>
+    <row r="1319" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1319" s="4">
+        <v>318</v>
+      </c>
+      <c r="B1319" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1319" s="4">
+        <v>77613</v>
+      </c>
+      <c r="D1319" s="2">
+        <v>46204.228113425903</v>
+      </c>
+      <c r="E1319" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1319" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1319" s="4" t="s">
+        <v>1466</v>
+      </c>
+      <c r="H1319" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1319" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1319" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1319" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1320" s="4">
+        <v>319</v>
+      </c>
+      <c r="B1320" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1320" s="4">
+        <v>86493</v>
+      </c>
+      <c r="D1320" s="2">
+        <v>46205.341307870403</v>
+      </c>
+      <c r="E1320" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1320" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1320" s="4" t="s">
+        <v>1467</v>
+      </c>
+      <c r="H1320" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1320" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1320" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1320" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1321" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1321" s="4">
+        <v>320</v>
+      </c>
+      <c r="B1321" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1321" s="4">
+        <v>85511</v>
+      </c>
+      <c r="D1321" s="2">
+        <v>46205.687384259298</v>
+      </c>
+      <c r="E1321" s="4" t="s">
+        <v>1468</v>
+      </c>
+      <c r="F1321" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1321" s="4" t="s">
+        <v>1469</v>
+      </c>
+      <c r="H1321" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1321" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1321" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1321" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1322" s="4">
+        <v>321</v>
+      </c>
+      <c r="B1322" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1322" s="4">
+        <v>87456</v>
+      </c>
+      <c r="D1322" s="2">
+        <v>46206.402025463001</v>
+      </c>
+      <c r="E1322" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1322" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1322" s="4" t="s">
+        <v>1470</v>
+      </c>
+      <c r="H1322" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1322" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1322" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1322" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1323" s="4">
+        <v>322</v>
+      </c>
+      <c r="B1323" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1323" s="4">
+        <v>84877</v>
+      </c>
+      <c r="D1323" s="2">
+        <v>46206.404606481497</v>
+      </c>
+      <c r="E1323" s="4" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1323" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1323" s="4" t="s">
+        <v>1471</v>
+      </c>
+      <c r="H1323" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1323" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1323" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1323" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1324" s="4">
+        <v>323</v>
+      </c>
+      <c r="B1324" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1324" s="4">
+        <v>88457</v>
+      </c>
+      <c r="D1324" s="2">
+        <v>46206.513159722199</v>
+      </c>
+      <c r="E1324" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1324" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1324" s="4" t="s">
+        <v>1472</v>
+      </c>
+      <c r="H1324" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1324" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1324" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1324" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1325" s="4">
+        <v>324</v>
+      </c>
+      <c r="B1325" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1325" s="4">
+        <v>71235</v>
+      </c>
+      <c r="D1325" s="2">
+        <v>46208.382118055597</v>
+      </c>
+      <c r="E1325" s="4" t="s">
+        <v>1427</v>
+      </c>
+      <c r="F1325" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1325" s="4" t="s">
+        <v>1473</v>
+      </c>
+      <c r="H1325" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1325" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1325" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1325" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1326" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1326" s="4">
+        <v>325</v>
+      </c>
+      <c r="B1326" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1326" s="4">
+        <v>77925</v>
+      </c>
+      <c r="D1326" s="2">
+        <v>46209.3108333333</v>
+      </c>
+      <c r="E1326" s="4" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F1326" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1326" s="4" t="s">
+        <v>1475</v>
+      </c>
+      <c r="H1326" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1326" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1326" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1326" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1327" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1327" s="4">
+        <v>326</v>
+      </c>
+      <c r="B1327" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1327" s="4">
+        <v>91153</v>
+      </c>
+      <c r="D1327" s="2">
+        <v>46209.324907407397</v>
+      </c>
+      <c r="E1327" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1327" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1327" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="H1327" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1327" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1327" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1327" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1328" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1328" s="4">
+        <v>327</v>
+      </c>
+      <c r="B1328" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1328" s="4">
+        <v>68303</v>
+      </c>
+      <c r="D1328" s="2">
+        <v>46209.332476851901</v>
+      </c>
+      <c r="E1328" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1328" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1328" s="4" t="s">
+        <v>1477</v>
+      </c>
+      <c r="H1328" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1328" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1328" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1328" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1329" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1329" s="4">
+        <v>328</v>
+      </c>
+      <c r="B1329" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1329" s="4">
+        <v>91068</v>
+      </c>
+      <c r="D1329" s="2">
+        <v>46209.395358796297</v>
+      </c>
+      <c r="E1329" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1329" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1329" s="4" t="s">
+        <v>1478</v>
+      </c>
+      <c r="H1329" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1329" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1329" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1329" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1330" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1330" s="4">
+        <v>329</v>
+      </c>
+      <c r="B1330" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1330" s="4">
+        <v>81209</v>
+      </c>
+      <c r="D1330" s="2">
+        <v>46209.405763888899</v>
+      </c>
+      <c r="E1330" s="4" t="s">
+        <v>1479</v>
+      </c>
+      <c r="F1330" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1330" s="4" t="s">
+        <v>1480</v>
+      </c>
+      <c r="H1330" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1330" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1330" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1330" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1331" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1331" s="4">
+        <v>330</v>
+      </c>
+      <c r="B1331" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1331" s="4">
+        <v>88667</v>
+      </c>
+      <c r="D1331" s="2">
+        <v>46209.555567129602</v>
+      </c>
+      <c r="E1331" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1331" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1331" s="4" t="s">
+        <v>1481</v>
+      </c>
+      <c r="H1331" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1331" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1331" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1331" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1332" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1332" s="4">
+        <v>331</v>
+      </c>
+      <c r="B1332" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1332" s="4">
+        <v>78632</v>
+      </c>
+      <c r="D1332" s="2">
+        <v>46209.562962962998</v>
+      </c>
+      <c r="E1332" s="4" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1332" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1332" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="H1332" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1332" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1332" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1332" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1333" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1333" s="4">
+        <v>332</v>
+      </c>
+      <c r="B1333" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1333" s="4">
+        <v>82227</v>
+      </c>
+      <c r="D1333" s="2">
+        <v>46209.716145833299</v>
+      </c>
+      <c r="E1333" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1333" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1333" s="4" t="s">
+        <v>1483</v>
+      </c>
+      <c r="H1333" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1333" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1333" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1333" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1334" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1334" s="4">
+        <v>333</v>
+      </c>
+      <c r="B1334" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1334" s="4">
+        <v>81488</v>
+      </c>
+      <c r="D1334" s="2">
+        <v>46210.286759259303</v>
+      </c>
+      <c r="E1334" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1334" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1334" s="4" t="s">
+        <v>1484</v>
+      </c>
+      <c r="H1334" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1334" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1334" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1334" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1335" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1335" s="4">
+        <v>334</v>
+      </c>
+      <c r="B1335" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1335" s="4">
+        <v>71658</v>
+      </c>
+      <c r="D1335" s="2">
+        <v>46210.397152777798</v>
+      </c>
+      <c r="E1335" s="4" t="s">
+        <v>1485</v>
+      </c>
+      <c r="F1335" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1335" s="4" t="s">
+        <v>1486</v>
+      </c>
+      <c r="H1335" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1335" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1335" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1335" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1336" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1336" s="4">
+        <v>335</v>
+      </c>
+      <c r="B1336" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1336" s="4">
+        <v>88352</v>
+      </c>
+      <c r="D1336" s="2">
+        <v>46210.605185185203</v>
+      </c>
+      <c r="E1336" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1336" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1336" s="4" t="s">
+        <v>1487</v>
+      </c>
+      <c r="H1336" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1336" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1336" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1336" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1337" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1337" s="4">
+        <v>336</v>
+      </c>
+      <c r="B1337" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1337" s="4">
+        <v>79776</v>
+      </c>
+      <c r="D1337" s="2">
+        <v>46211.625416666699</v>
+      </c>
+      <c r="E1337" s="4" t="s">
+        <v>1488</v>
+      </c>
+      <c r="F1337" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1337" s="4" t="s">
+        <v>1489</v>
+      </c>
+      <c r="H1337" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1337" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1337" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1337" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1338" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1338" s="4">
+        <v>337</v>
+      </c>
+      <c r="B1338" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1338" s="4">
+        <v>86122</v>
+      </c>
+      <c r="D1338" s="2">
+        <v>46211.6703935185</v>
+      </c>
+      <c r="E1338" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1338" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1338" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="H1338" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1338" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1338" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1338" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1339" s="4">
+        <v>338</v>
+      </c>
+      <c r="B1339" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1339" s="4">
+        <v>88500</v>
+      </c>
+      <c r="D1339" s="2">
+        <v>46211.718460648197</v>
+      </c>
+      <c r="E1339" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1339" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1339" s="4" t="s">
+        <v>1492</v>
+      </c>
+      <c r="H1339" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1339" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1339" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1339" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1340" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1340" s="4">
+        <v>339</v>
+      </c>
+      <c r="B1340" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1340" s="4">
+        <v>91901</v>
+      </c>
+      <c r="D1340" s="2">
+        <v>46212.403495370403</v>
+      </c>
+      <c r="E1340" s="4" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F1340" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1340" s="4" t="s">
+        <v>1493</v>
+      </c>
+      <c r="H1340" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1340" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1340" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1340" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1341" s="4">
+        <v>340</v>
+      </c>
+      <c r="B1341" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1341" s="4">
+        <v>90803</v>
+      </c>
+      <c r="D1341" s="2">
+        <v>46212.483738425901</v>
+      </c>
+      <c r="E1341" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1341" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1341" s="4" t="s">
+        <v>1494</v>
+      </c>
+      <c r="H1341" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1341" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="J1341" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1341" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1342" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1342" s="4">
+        <v>341</v>
+      </c>
+      <c r="B1342" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1342" s="4">
+        <v>81777</v>
+      </c>
+      <c r="D1342" s="2">
+        <v>46213.401446759301</v>
+      </c>
+      <c r="E1342" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1342" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1342" s="4" t="s">
+        <v>1495</v>
+      </c>
+      <c r="H1342" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1342" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1342" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1342" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1343" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1343" s="4">
+        <v>342</v>
+      </c>
+      <c r="B1343" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1343" s="4">
+        <v>95091</v>
+      </c>
+      <c r="D1343" s="2">
+        <v>46213.407546296301</v>
+      </c>
+      <c r="E1343" s="4" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1343" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1343" s="4" t="s">
+        <v>1496</v>
+      </c>
+      <c r="H1343" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1343" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1343" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1343" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1344" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1344" s="4">
+        <v>343</v>
+      </c>
+      <c r="B1344" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1344" s="4">
+        <v>94455</v>
+      </c>
+      <c r="D1344" s="2">
+        <v>46213.464884259301</v>
+      </c>
+      <c r="E1344" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1344" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1344" s="4" t="s">
+        <v>1497</v>
+      </c>
+      <c r="H1344" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1344" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1344" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1344" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1345" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1345" s="4">
+        <v>344</v>
+      </c>
+      <c r="B1345" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1345" s="4">
+        <v>82944</v>
+      </c>
+      <c r="D1345" s="2">
+        <v>46213.467465277798</v>
+      </c>
+      <c r="E1345" s="4" t="s">
+        <v>1498</v>
+      </c>
+      <c r="F1345" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1345" s="4" t="s">
+        <v>1499</v>
+      </c>
+      <c r="H1345" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1345" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1345" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1345" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1346" s="4">
+        <v>345</v>
+      </c>
+      <c r="B1346" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1346" s="4">
+        <v>92666</v>
+      </c>
+      <c r="D1346" s="2">
+        <v>46213.521215277797</v>
+      </c>
+      <c r="E1346" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1346" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1346" s="4" t="s">
+        <v>1500</v>
+      </c>
+      <c r="H1346" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1346" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1346" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1346" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1347" s="4">
+        <v>346</v>
+      </c>
+      <c r="B1347" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1347" s="4">
+        <v>92151</v>
+      </c>
+      <c r="D1347" s="2">
+        <v>46213.6069444444</v>
+      </c>
+      <c r="E1347" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1347" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1347" s="4" t="s">
+        <v>1501</v>
+      </c>
+      <c r="H1347" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1347" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1347" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1347" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1348" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1348" s="4">
+        <v>347</v>
+      </c>
+      <c r="B1348" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1348" s="4">
+        <v>80778</v>
+      </c>
+      <c r="D1348" s="2">
+        <v>46214.486516203702</v>
+      </c>
+      <c r="E1348" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1348" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1348" s="4" t="s">
+        <v>1502</v>
+      </c>
+      <c r="H1348" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1348" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1348" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1348" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1349" s="4">
+        <v>348</v>
+      </c>
+      <c r="B1349" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1349" s="4">
+        <v>87540</v>
+      </c>
+      <c r="D1349" s="2">
+        <v>46215.174537036997</v>
+      </c>
+      <c r="E1349" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1349" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1349" s="4" t="s">
+        <v>1503</v>
+      </c>
+      <c r="H1349" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1349" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1349" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1349" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1350" s="4">
+        <v>349</v>
+      </c>
+      <c r="B1350" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1350" s="4">
+        <v>93008</v>
+      </c>
+      <c r="D1350" s="2">
+        <v>46216.286307870403</v>
+      </c>
+      <c r="E1350" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1350" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1350" s="4" t="s">
+        <v>1504</v>
+      </c>
+      <c r="H1350" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1350" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1350" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1350" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1351" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1351" s="4">
+        <v>350</v>
+      </c>
+      <c r="B1351" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1351" s="4">
+        <v>87232</v>
+      </c>
+      <c r="D1351" s="2">
+        <v>46216.384155092601</v>
+      </c>
+      <c r="E1351" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1351" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1351" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="H1351" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1351" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1351" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1351" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1352" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1352" s="4">
+        <v>351</v>
+      </c>
+      <c r="B1352" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1352" s="4">
+        <v>83845</v>
+      </c>
+      <c r="D1352" s="2">
+        <v>46216.3851967593</v>
+      </c>
+      <c r="E1352" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1352" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1352" s="4" t="s">
+        <v>1506</v>
+      </c>
+      <c r="H1352" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1352" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1352" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1352" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1353" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1353" s="4">
+        <v>352</v>
+      </c>
+      <c r="B1353" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1353" s="4">
+        <v>91804</v>
+      </c>
+      <c r="D1353" s="2">
+        <v>46216.456053240698</v>
+      </c>
+      <c r="E1353" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1353" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1353" s="4" t="s">
+        <v>1507</v>
+      </c>
+      <c r="H1353" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1353" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="J1353" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1353" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1354" s="4">
+        <v>353</v>
+      </c>
+      <c r="B1354" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1354" s="4">
+        <v>94399</v>
+      </c>
+      <c r="D1354" s="2">
+        <v>46216.483900462998</v>
+      </c>
+      <c r="E1354" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="F1354" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1354" s="4" t="s">
+        <v>1508</v>
+      </c>
+      <c r="H1354" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1354" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1354" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1354" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/07/2026 12:35:03,14
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="353" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3BA484-D7CA-4030-9C81-A2893A9ACDE6}"/>
+  <xr:revisionPtr revIDLastSave="356" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAFE9962-B52D-428B-98FF-1EFE5AED9248}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10835" uniqueCount="1509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10955" uniqueCount="1527">
   <si>
     <t>ID</t>
   </si>
@@ -4688,6 +4688,68 @@
   </si>
   <si>
     <t>O atendimento do técnico foi bom. De fato não sei qual o diferencial do purificador Brastemp para água Sabesp.Técnico usou um reagente que muda a cor da água sinalizando a presença de cloro. Pedi para ele testar outras fontes de água:  1) Purificador: água se manteve transparente e cristalina 2) Água da torneira fria: agua da Sabesp entra,passa por uma cisterna de 8 mil litros, duas bombas distribuem água para 3 caixas dágua. Ao testar, um copo com essa água, ela se manteve transparente e cristalina. Pergunta: se essa água, fica em caixa dágua, que no máximo é feito uma limpeza a cada 2 anos, como não sinalizou nenhum problema? 3) Agua da torneira quente: além do descrito no item 2, a água vai para um boiler de 250 l. Também ao testar se manteve transparente e cristalina. 4) Água da piscina: foi a única que reagiu e ficou amarelada (por causa do cloro). Pergunta: ou o teste feito está errado, usando somente reação cloro, ou não tem diferença entre usar água da torneira e brastemp.</t>
+  </si>
+  <si>
+    <t>FRQ BELO HORIZONTE MG R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Não foi trocado o filtro, pq o rapaz falou que como foi pedido cancelamento. 
+Porém não marcaram uma data para retirada do aparelho.</t>
+  </si>
+  <si>
+    <t>A Visita não ocorreu...Não houve visita técnica.</t>
+  </si>
+  <si>
+    <t>Prestador pouco proativo.</t>
+  </si>
+  <si>
+    <t>Serviço não executado. Desorganização, não trocaram o elemento filtrante, a água ficou com gosto ruim e fluxo pior ainda. 
+Arrependido de ter contratado esse serviço. Os órgãos competentes já foram acionados.</t>
+  </si>
+  <si>
+    <t>Por não conseguir falar com ninguém, o técnico era muito bom mas estou sem respostas para o problema do meu filtro. Próximo passo cancelar a assinatura</t>
+  </si>
+  <si>
+    <t>Agendado 2 vezes e ninguém apareceu.</t>
+  </si>
+  <si>
+    <t>O profissional que veio não tenho do que reclamar, pelo contrário recomendo 100%.
+Mas como estava com problema no purificador poderiam colocar uma data mais próxima, atender mais rápido.</t>
+  </si>
+  <si>
+    <t>Primeiramente, quando solicitamos uma visita técnica, os prazos de atendimento costumam ser muito longos. Em diversas ocasiões, precisamos manter o purificador desligado até que a equipe consiga comparecer para realizar o reparo.
+Outro ponto é que a manutenção preventiva, que deveria ocorrer a cada seis meses, frequentemente ultrapassa esse prazo.
+Além disso, a comunicação com vocês é muito difícil. As devolutivas são insatisfatórias e, na maioria das vezes, conseguimos contato apenas com robôs, o que dificulta a resolução dos problemas.
+Ontem recebemos uma visita técnica para a troca do botão de um dos purificadores, que estava quebrado. Durante o atendimento, percebi que o técnico teve dificuldade para fechar o equipamento. Após a conclusão do serviço e a saída dele, o botão passou a ficar extremamente sensível, acionando sozinho diversas vezes.
+Entrei em contato imediatamente para informar o problema, porém, até o momento, não obtive retorno. Como consequência, estamos novamente</t>
+  </si>
+  <si>
+    <t>O serviçode de reparo  realizado ontem 14/07/26 não resolveu o problema. Funcionou por apenas 10 horas e o problema anterior voltou a se repetir. Só que desta vez o botão da água gelada não só não funciona corretamente como também  não gela a água. Ou seja, o problema não foi solucionado mas sim agravado, piorando consideravelmente o funcionamento do aparelho. Hoje, 15/07/26 voltei a entrar em contato para reportar o que aconteceu e solicitar nova visita para resolver o problema. Para minha surpresa e indignação,  fui informado que a nova visita só poderia ser agendada dua 28/07/26. Isso é inadmissível, pois o aparelho não funciona e eu continuo pagando por um serviço que efetivamente não está sendo prestado. Espero que a Brastemp reveja essa forma de tratar os seus clientes e reagende, com a maior brevidade possível, uma visita em que o técnico solucione definitivamente o problema. Além disso,  desconte da fatura do cliente os dias em que  o aparelho ficou inoperante.</t>
+  </si>
+  <si>
+    <t>FRQ BRASILIA DF R02</t>
+  </si>
+  <si>
+    <t>Eu marquei para a visita o turno vespertino. O técnico chegou pela manhã e causou um grande transtorno. Pra que agendar o turno se não é respeitado???</t>
+  </si>
+  <si>
+    <t>FRQ SANTOS SP R05</t>
+  </si>
+  <si>
+    <t>Foi trocado o sistema de filtragem da a impressão de ser usado pois veio mal embalado e o tecnico usou escova de dente usada na limpesa lateral e cotonete no bico e manuseio inadequado em contato com mão suja e usando o lado sujo dentro da válvula de saída de água. Decepção</t>
+  </si>
+  <si>
+    <t>estava agendadao para uma data e o tecniico veio 3 dias antes.
+por sorte estava em casa .... qual o sentido de se agendar a visita e aparecer antes?</t>
+  </si>
+  <si>
+    <t>A assistência foi rápida e aparentemente muito eficiente.. Ele até testou e estava tudo ok. Mas bastou sair e começou a apresentar defeito: barulho inédito ao acionar o aparelho e uma água completamente turva, Aos poucos conforme ia pegando água foi voltando a ficar transparente, mas o gosto não indica o uso e o barulho não cessou.Espero orientação e solução.</t>
+  </si>
+  <si>
+    <t>Porque não dei causa ao acumulo de parcelas vencidas, As respostas já vem prontas é so escolher a que quiseremj.</t>
+  </si>
+  <si>
+    <t>Ninguém veio!!!! Não houve serviço. Fiquei em casa esperando e nada!</t>
   </si>
 </sst>
 </file>
@@ -5060,7 +5122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1354"/>
+  <dimension ref="A1:K1369"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -52467,6 +52529,531 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1355" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1355" s="4">
+        <v>354</v>
+      </c>
+      <c r="B1355" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1355" s="4">
+        <v>83095</v>
+      </c>
+      <c r="D1355" s="2">
+        <v>46216.589780092603</v>
+      </c>
+      <c r="E1355" s="4" t="s">
+        <v>1509</v>
+      </c>
+      <c r="F1355" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1355" s="4" t="s">
+        <v>1510</v>
+      </c>
+      <c r="H1355" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1355" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1355" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1355" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1356" s="4">
+        <v>355</v>
+      </c>
+      <c r="B1356" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1356" s="4">
+        <v>83347</v>
+      </c>
+      <c r="D1356" s="2">
+        <v>46216.828043981477</v>
+      </c>
+      <c r="E1356" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1356" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1356" s="4" t="s">
+        <v>1511</v>
+      </c>
+      <c r="H1356" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1356" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1356" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1356" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1357" s="4">
+        <v>356</v>
+      </c>
+      <c r="B1357" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1357" s="4">
+        <v>85506</v>
+      </c>
+      <c r="D1357" s="2">
+        <v>46217.460590277777</v>
+      </c>
+      <c r="E1357" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1357" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1357" s="4" t="s">
+        <v>1512</v>
+      </c>
+      <c r="H1357" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1357" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1357" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1357" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1358" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1358" s="4">
+        <v>357</v>
+      </c>
+      <c r="B1358" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1358" s="4">
+        <v>91503</v>
+      </c>
+      <c r="D1358" s="2">
+        <v>46217.525439814817</v>
+      </c>
+      <c r="E1358" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1358" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1358" s="4" t="s">
+        <v>1513</v>
+      </c>
+      <c r="H1358" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1358" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1358" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1358" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1359" s="4">
+        <v>358</v>
+      </c>
+      <c r="B1359" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1359" s="4">
+        <v>89265</v>
+      </c>
+      <c r="D1359" s="2">
+        <v>46217.738692129627</v>
+      </c>
+      <c r="E1359" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1359" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1359" s="4" t="s">
+        <v>1514</v>
+      </c>
+      <c r="H1359" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1359" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1359" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1359" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1360" s="4">
+        <v>359</v>
+      </c>
+      <c r="B1360" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1360" s="4">
+        <v>96993</v>
+      </c>
+      <c r="D1360" s="2">
+        <v>46218.312557870369</v>
+      </c>
+      <c r="E1360" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1360" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1360" s="4" t="s">
+        <v>1515</v>
+      </c>
+      <c r="H1360" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1360" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1360" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1360" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1361" s="4">
+        <v>360</v>
+      </c>
+      <c r="B1361" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1361" s="4">
+        <v>94534</v>
+      </c>
+      <c r="D1361" s="2">
+        <v>46218.314849537041</v>
+      </c>
+      <c r="E1361" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1361" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1361" s="4" t="s">
+        <v>1516</v>
+      </c>
+      <c r="H1361" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1361" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1361" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1361" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1362" s="4">
+        <v>361</v>
+      </c>
+      <c r="B1362" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1362" s="4">
+        <v>94778</v>
+      </c>
+      <c r="D1362" s="2">
+        <v>46218.31653935185</v>
+      </c>
+      <c r="E1362" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1362" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1362" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H1362" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1362" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1362" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1362" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1363" s="4">
+        <v>362</v>
+      </c>
+      <c r="B1363" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1363" s="4">
+        <v>97056</v>
+      </c>
+      <c r="D1363" s="2">
+        <v>46218.317361111112</v>
+      </c>
+      <c r="E1363" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1363" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1363" s="4" t="s">
+        <v>1518</v>
+      </c>
+      <c r="H1363" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1363" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1363" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1363" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1364" s="4">
+        <v>363</v>
+      </c>
+      <c r="B1364" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1364" s="4">
+        <v>86551</v>
+      </c>
+      <c r="D1364" s="2">
+        <v>46218.373020833344</v>
+      </c>
+      <c r="E1364" s="4" t="s">
+        <v>1519</v>
+      </c>
+      <c r="F1364" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1364" s="4" t="s">
+        <v>1520</v>
+      </c>
+      <c r="H1364" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1364" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1364" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1364" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1365" s="4">
+        <v>364</v>
+      </c>
+      <c r="B1365" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1365" s="4">
+        <v>88899</v>
+      </c>
+      <c r="D1365" s="2">
+        <v>46218.758553240739</v>
+      </c>
+      <c r="E1365" s="4" t="s">
+        <v>1521</v>
+      </c>
+      <c r="F1365" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1365" s="4" t="s">
+        <v>1522</v>
+      </c>
+      <c r="H1365" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1365" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1365" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1365" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1366" s="4">
+        <v>365</v>
+      </c>
+      <c r="B1366" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1366" s="4">
+        <v>88814</v>
+      </c>
+      <c r="D1366" s="2">
+        <v>46220.256249999999</v>
+      </c>
+      <c r="E1366" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1366" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1366" s="4" t="s">
+        <v>1523</v>
+      </c>
+      <c r="H1366" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1366" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1366" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1366" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1367" s="4">
+        <v>366</v>
+      </c>
+      <c r="B1367" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1367" s="4">
+        <v>80608</v>
+      </c>
+      <c r="D1367" s="2">
+        <v>46220.267152777778</v>
+      </c>
+      <c r="E1367" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1367" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1367" s="4" t="s">
+        <v>1524</v>
+      </c>
+      <c r="H1367" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1367" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1367" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1367" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1368" s="4">
+        <v>367</v>
+      </c>
+      <c r="B1368" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1368" s="4">
+        <v>78193</v>
+      </c>
+      <c r="D1368" s="2">
+        <v>46220.358032407406</v>
+      </c>
+      <c r="E1368" s="4" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F1368" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1368" s="4" t="s">
+        <v>1525</v>
+      </c>
+      <c r="H1368" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1368" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1368" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1368" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1369" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1369" s="4">
+        <v>368</v>
+      </c>
+      <c r="B1369" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1369" s="4">
+        <v>85145</v>
+      </c>
+      <c r="D1369" s="2">
+        <v>46220.35869212963</v>
+      </c>
+      <c r="E1369" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1369" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1369" s="4" t="s">
+        <v>1526</v>
+      </c>
+      <c r="H1369" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1369" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1369" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1369" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 24/07/2026 12:22:48,74
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="356" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAFE9962-B52D-428B-98FF-1EFE5AED9248}"/>
+  <xr:revisionPtr revIDLastSave="375" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{214C79D5-981C-4934-94FA-774887436A38}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1318</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1369</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10955" uniqueCount="1527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11075" uniqueCount="1548">
   <si>
     <t>ID</t>
   </si>
@@ -4750,6 +4750,70 @@
   </si>
   <si>
     <t>Ninguém veio!!!! Não houve serviço. Fiquei em casa esperando e nada!</t>
+  </si>
+  <si>
+    <t>FRQ SP LIT NORTE R03</t>
+  </si>
+  <si>
+    <t>FRQ GUARULHOS SP R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>Remarcaram a visita 2 semanas para a frente, visitaram e não resolveu o problema - sigo há 1 mês sem água gelada pagando assinatura cara há 5 anos</t>
+  </si>
+  <si>
+    <t>Marquei a manutenção para o dia 08/07 e não apareceu ninguém. Precisei ligar mais 3x para ouvir que primeiro tinham que cancelar a ordem anterior e só depois avaliar se teria uma nova data. Apareceram aqui ontem sem avisar que viriam e nem retornar sobre os 3 contatos que fiz.</t>
+  </si>
+  <si>
+    <t>Não consegui falar com uma pessoa. Inteligência artificial não atende às necessidades.</t>
+  </si>
+  <si>
+    <t>O atendimento do técnico foi maravilhoso,mas as circunstâncias do atendimento não.Liguei várias vezes solicitando reparo e troca dos purificadores e nunca marcaram por problemas no sistema.Entao,do nada,sem aviso prévio ,o técnico veio para a manutenção periódica com a troca do filtro.Foi por uma questão de saúde que tinha alguém em casa.Quando a Brastemp era responsável pelos purificadores,o SAC era outra qualidade,aliás,muito superior.Agendamento por telefone prévio conforme a disponibilidade do cliente,confirmação da visita.Palavra-chave de segurança.Quando ligava para o SAc as solicitações eram atendidas.Agora,horas na linha para não resolver nada.No momento não recomendo a Culligan e pretendo rever a assinatura dos purificadores e talvez cancelar.Os aparelhos estão feios por serem velhos.Nao combinam com a estética da casa.Ja pedi a substituição e nada.</t>
+  </si>
+  <si>
+    <t>Tenho 2 contratos um deles agendado a manutenção não apareceu ninguém e muito menos tive um retorno após meu contato retornansoð</t>
+  </si>
+  <si>
+    <t>Eu recebi as notificações sobre as mudanças com um certa confusão não ficando muito claro recebi um boleto de pagamento que eu não sabia do que se tratava só depois é que eu fui entender que era do novo sistema eu tentei pagar e não consegui e eu não tenho a quem ligar não tenho eu não tenho um acesso a um sistema de reclamação então por enquanto a minha experiência tem sido bem negativa eu sou um cliente fiel há muitos anos que sempre paga em dia e eu acho que esse tipo de tratamento é desrespeitoso para conosco que somos disciplinados e pontuais nas nossas contas</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
+  </si>
+  <si>
+    <t>Boleto</t>
+  </si>
+  <si>
+    <t>Porque o reparo foi feito, mas o filtro apresentou outro defeito. Agora está pingando. Tive que marcar outra visita</t>
+  </si>
+  <si>
+    <t>Agendaram visita técnica para manutenção preventiva no sábado dia 18.07.2026 oela manhã, foi confirmado, ficamos em casa esperando e não vieram!</t>
+  </si>
+  <si>
+    <t>Porque das vezes anteriores a manutenção era mais completa do que é feita hoje.</t>
+  </si>
+  <si>
+    <t>FRQ PORTO ALEGRE RS R03</t>
+  </si>
+  <si>
+    <t>O técnico, em menos de 5 minutos deixou o local sinalizando estar pronto, pois apenas trocou o filtro, deixou tudo sujo e saiu.
+Apareceu no local para realizar a visita, sem meu conhecimento de agendamento, pois recebi um contato em 17mar, e ficou agendado para dia 17/abr, de manha. Ninguém apareceu em Abril e não recebi nenhum aviso que não seria alterado a data, ou cancelado, nada. O Serviço e atendimento, desculpe mas está MUITO RUIM. Consideração ZERO com o cliente.</t>
+  </si>
+  <si>
+    <t>Qulatics</t>
+  </si>
+  <si>
+    <t>O técnico não estava com prope ..entrou com a bota na minha casa. Eu trabalho com prestação de serviços item básico para atendimento na casa do cliente e colocar o proteção na bota.</t>
+  </si>
+  <si>
+    <t>Péssimo atendimento.</t>
+  </si>
+  <si>
+    <t>Insatisfeito</t>
+  </si>
+  <si>
+    <t>Dois agendamentos feitos, mas o técnico não compareceu ao local e não deu informação sobre o motivo do não comparecimento. A empresa não soube resolver o problema quando entrei em contato. O técnico compareceu no dia seguinte, sem avisar que ia.</t>
+  </si>
+  <si>
+    <t>Nos últimos meses, a qualidade do serviço prestado tem deixado muito a desejar. Em diversas ocasiões, as visitas técnicas foram agendadas e não ocorreram. Quando acontecem ,muitas vezes são marcadas para dias em que o escritório está fechado,( mesmo o agendamento tendo sido feito para o dia em que está aberto, não respeitando a data )sem flexibilidade ou boa vontade por parte do técnico para buscar uma alternativa. A mudança na qualidade do atendimento foi bastante significativa, infelizmente para pior. Esperamos uma melhora nesse cenário ,pois caso essa situação persista , provavelmente teremos que buscar outro fornecedor. Sem contar que solicitei alteração tanto para e-mail como para número de telefone e não ocorreu.</t>
   </si>
 </sst>
 </file>
@@ -5122,7 +5186,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1369"/>
+  <dimension ref="A1:K1384"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -53054,6 +53118,531 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1370" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1370" s="4">
+        <v>369</v>
+      </c>
+      <c r="B1370" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1370" s="4">
+        <v>72992</v>
+      </c>
+      <c r="D1370" s="2">
+        <v>46221.760682870372</v>
+      </c>
+      <c r="E1370" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F1370" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1370" s="4" t="s">
+        <v>1541</v>
+      </c>
+      <c r="H1370" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1370" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1370" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1370" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1371" s="4">
+        <v>370</v>
+      </c>
+      <c r="B1371" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1371" s="4">
+        <v>97032</v>
+      </c>
+      <c r="D1371" s="2">
+        <v>46223.288668981477</v>
+      </c>
+      <c r="E1371" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1371" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1371" s="4" t="s">
+        <v>1543</v>
+      </c>
+      <c r="H1371" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1371" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1371" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1371" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1372" s="4">
+        <v>371</v>
+      </c>
+      <c r="B1372" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1372" s="4">
+        <v>98261</v>
+      </c>
+      <c r="D1372" s="2">
+        <v>46223.300069444442</v>
+      </c>
+      <c r="E1372" s="4" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1372" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1372" s="4" t="s">
+        <v>1544</v>
+      </c>
+      <c r="H1372" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1372" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1372" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1372" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1373" s="4">
+        <v>372</v>
+      </c>
+      <c r="B1373" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1373" s="4">
+        <v>100121</v>
+      </c>
+      <c r="D1373" s="2">
+        <v>46223.557881944442</v>
+      </c>
+      <c r="E1373" s="4" t="s">
+        <v>803</v>
+      </c>
+      <c r="F1373" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1373" s="4" t="s">
+        <v>1545</v>
+      </c>
+      <c r="H1373" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1373" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1373" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1373" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1374" s="4">
+        <v>373</v>
+      </c>
+      <c r="B1374" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1374" s="4">
+        <v>75329</v>
+      </c>
+      <c r="D1374" s="2">
+        <v>46223.592349537037</v>
+      </c>
+      <c r="E1374" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1374" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1374" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="H1374" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1374" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1374" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1374" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1375" s="4">
+        <v>374</v>
+      </c>
+      <c r="B1375" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1375" s="4">
+        <v>99336</v>
+      </c>
+      <c r="D1375" s="2">
+        <v>46223.631967592592</v>
+      </c>
+      <c r="E1375" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1375" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1375" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="H1375" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1375" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1375" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1375" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1376" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1376" s="4">
+        <v>375</v>
+      </c>
+      <c r="B1376" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1376" s="4">
+        <v>94295</v>
+      </c>
+      <c r="D1376" s="2">
+        <v>46223.717152777783</v>
+      </c>
+      <c r="E1376" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1376" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1376" s="4" t="s">
+        <v>1529</v>
+      </c>
+      <c r="H1376" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1376" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1376" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1376" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1377" s="4">
+        <v>376</v>
+      </c>
+      <c r="B1377" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1377" s="4">
+        <v>88705</v>
+      </c>
+      <c r="D1377" s="2">
+        <v>46224.304930555547</v>
+      </c>
+      <c r="E1377" s="4" t="s">
+        <v>1527</v>
+      </c>
+      <c r="F1377" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1377" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="H1377" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1377" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1377" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1377" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1378" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1378" s="4">
+        <v>377</v>
+      </c>
+      <c r="B1378" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1378" s="4">
+        <v>92473</v>
+      </c>
+      <c r="D1378" s="2">
+        <v>46224.331608796303</v>
+      </c>
+      <c r="E1378" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1378" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1378" s="4" t="s">
+        <v>1531</v>
+      </c>
+      <c r="H1378" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1378" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1378" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1378" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1379" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1379" s="4">
+        <v>378</v>
+      </c>
+      <c r="B1379" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1379" s="4">
+        <v>86207</v>
+      </c>
+      <c r="D1379" s="2">
+        <v>46224.442812499998</v>
+      </c>
+      <c r="E1379" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1379" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1379" s="4" t="s">
+        <v>1532</v>
+      </c>
+      <c r="H1379" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1379" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1379" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1379" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1380" s="4">
+        <v>379</v>
+      </c>
+      <c r="B1380" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1380" s="4">
+        <v>89411</v>
+      </c>
+      <c r="D1380" s="2">
+        <v>46224.490995370368</v>
+      </c>
+      <c r="E1380" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1380" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1380" s="4" t="s">
+        <v>1533</v>
+      </c>
+      <c r="H1380" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1380" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1380" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1380" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1381" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1381" s="4">
+        <v>380</v>
+      </c>
+      <c r="B1381" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1381" s="4">
+        <v>99055</v>
+      </c>
+      <c r="D1381" s="2">
+        <v>46224.663495370369</v>
+      </c>
+      <c r="E1381" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1381" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1381" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="H1381" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="I1381" s="4" t="s">
+        <v>1536</v>
+      </c>
+      <c r="J1381" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1381" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1382" s="4">
+        <v>381</v>
+      </c>
+      <c r="B1382" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1382" s="4">
+        <v>93985</v>
+      </c>
+      <c r="D1382" s="2">
+        <v>46224.674560185187</v>
+      </c>
+      <c r="E1382" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1382" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1382" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="H1382" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1382" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1382" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1382" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1383" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1383" s="4">
+        <v>382</v>
+      </c>
+      <c r="B1383" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1383" s="4">
+        <v>87665</v>
+      </c>
+      <c r="D1383" s="2">
+        <v>46224.779664351852</v>
+      </c>
+      <c r="E1383" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1383" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1383" s="4" t="s">
+        <v>1538</v>
+      </c>
+      <c r="H1383" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1383" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1383" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1383" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1384" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1384" s="4">
+        <v>383</v>
+      </c>
+      <c r="B1384" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1384" s="4">
+        <v>87180</v>
+      </c>
+      <c r="D1384" s="2">
+        <v>46224.894201388888</v>
+      </c>
+      <c r="E1384" s="4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="F1384" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1384" s="4" t="s">
+        <v>1539</v>
+      </c>
+      <c r="H1384" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1384" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1384" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="K1384" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 31/07/2026 11:12:25,28
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="375" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{214C79D5-981C-4934-94FA-774887436A38}"/>
+  <xr:revisionPtr revIDLastSave="378" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DEBF4C1-E61D-4DF1-A915-DB6E0E3EC113}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11075" uniqueCount="1548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11259" uniqueCount="1578">
   <si>
     <t>ID</t>
   </si>
@@ -4814,6 +4814,116 @@
   </si>
   <si>
     <t>Nos últimos meses, a qualidade do serviço prestado tem deixado muito a desejar. Em diversas ocasiões, as visitas técnicas foram agendadas e não ocorreram. Quando acontecem ,muitas vezes são marcadas para dias em que o escritório está fechado,( mesmo o agendamento tendo sido feito para o dia em que está aberto, não respeitando a data )sem flexibilidade ou boa vontade por parte do técnico para buscar uma alternativa. A mudança na qualidade do atendimento foi bastante significativa, infelizmente para pior. Esperamos uma melhora nesse cenário ,pois caso essa situação persista , provavelmente teremos que buscar outro fornecedor. Sem contar que solicitei alteração tanto para e-mail como para número de telefone e não ocorreu.</t>
+  </si>
+  <si>
+    <t>Na primeira visita nao foi feito o serviço, os atendentes foram muito educados porém nao souberam e nao tinham as peças necessárias para resolver. No dia seguinte veio outra pessoa, ela trouxe a peça mas o problema não resolveu. Como não fui eu pessoalmente quem acompanhou não detectei no momento e tive que abrir outro chamado. Apesar de eu relatar que gostaria de um encaixe rápido pois havia passado por duas visitas que nao resolveram tive que esperar 1 semana para próxima, que ainda vai ocorrer.</t>
+  </si>
+  <si>
+    <t>O filtro foi trocado e ficou um barulho enorme no purificador, tentei pedir o reparo e só tem vaga para 01/08. Um absurdo!</t>
+  </si>
+  <si>
+    <t>PORQUE NAO TEM RESPOSABILIDADE EM FAZER AS MANUTEÇOES NA DATA CERTAS, PRECISA ESTA LIGANDO PRA LEMBRA QUE ESTA VENCIDA .</t>
+  </si>
+  <si>
+    <t>Vocês já marcaram a manutenção 3 vezes e nao apareceram. Pessimo serviço. Quero saber o procedimento para cancelamento do contrato.</t>
+  </si>
+  <si>
+    <t>Olá,
+Sugiro uma melhoria nos aspectos de organização, planejamento e comunicação, principalmente no envio de avisos com antecedência ao cliente sobre as visitas técnicas.
+Também é importante aprimorar o processo relacionado às Ordens de Serviço, informando de forma clara qual equipamento será atendido durante a manutenção.
+Esses pontos ainda não estão sendo atendidos de maneira satisfatória, o que impacta a qualidade do atendimento. Por esse motivo, no momento, seria pouco provável que eu recomendasse esse serviço a um amigo ou colega.
+Atenciosamente,
+Ieda Castelo -(Triospuma Ind. e Com. Ltda)</t>
+  </si>
+  <si>
+    <t>Carteira comunicação</t>
+  </si>
+  <si>
+    <t>Mais uma vez o técnico não foi no dia agendado</t>
+  </si>
+  <si>
+    <t>Compareceu sem agendamento e ouve uma instalação que o purificador esta solto e desnivelado</t>
+  </si>
+  <si>
+    <t>serviços não foi finalizado, segundo técnico retomaria no dia seguinte, até o momento não tivemos retorno, canal digital de comunicação e ruim.</t>
+  </si>
+  <si>
+    <t>Install</t>
+  </si>
+  <si>
+    <t>FRQ BAIXADA SERRANA RJ R01</t>
+  </si>
+  <si>
+    <t>Pedi instalação na parede e não veio , além de desmarcar a instalação e nem avisar</t>
+  </si>
+  <si>
+    <t>Não recebi o serviço de manutenção</t>
+  </si>
+  <si>
+    <t>Há cerca de 3 meses, estou com dificuldades para conseguir pagar, tanto débito automático quanto boleto, e também para agendamento de visitas e correção de defeito no equipamento. Há quase 2 meses sem funcionar
+Assistência está deixando muito a desejar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financeiro </t>
+  </si>
+  <si>
+    <t>Problemas no faturamento</t>
+  </si>
+  <si>
+    <t>O bebedouro passou a apresentar vazamento no mês de ABRIL/26,solicitei prontamente o reparo, fui orientado a paralisar o uso. Só que a visita do técnico para reparo só ocorreu em JULHO.
+Ressalto que os débitos em conta pelo uso do bebedouro ocorreram de abril a junho.</t>
+  </si>
+  <si>
+    <t>Meu filtro continuou estragado na água gelada, o filtro trocado ficou</t>
+  </si>
+  <si>
+    <t>FRQ GUARULHOS SP R03</t>
+  </si>
+  <si>
+    <t>Atendimento péssimo, e o problema não foi solucionado.
+O mesmo informou que o equipamento não é para uso empresarial então não comporta a saída de água com gás</t>
+  </si>
+  <si>
+    <t>Tenho 8 protocolos, debito duplicado, 20 dias esperando estorno, péssimo atendimento jo whatsap, pedido de demonstrativo financeiro negado  apesar de 2 protocolos, pedido dd verificação de débito duplicado em julho sem resposta. estou acionando o Procon, não vou pagar mensalidade de julho enquanto nao estorarem o valor. e se ninguem resolver vou proceder com o cancelamento e assinar com o concorrente</t>
+  </si>
+  <si>
+    <t>A pressão da água no meu apartamento é altíssima. O técnico da Brastemp que instalou o equipamento há pouco mais de 6 meses instalou um redutor de pressão, que funcionava muito bem. O técnico que esteve agora, ao que parece, retirou o redutor. Está muito difícil usar o filtro porque a água sai com muita força, molhando tudo em volta!!</t>
+  </si>
+  <si>
+    <t>Demora nos retornos dos emails</t>
+  </si>
+  <si>
+    <t>FRQ RIBEIRAO PRETO R04</t>
+  </si>
+  <si>
+    <t>A central de atendimento ao cliente é horrível, abem chamados errados ocasionando custos desnecessários para vocês mesmos e não resolvem o problema do cliente, os pobres dos técnicos são maravilhosos, mas as informações que chegam até eles são completamente erradas, ligo na central por um motivo o técnico chega em minha residência por motivo completamente errados e sem ter como resolver o verdadeiro problema, já estou a um mês sem conseguir utilizar meu equipamento e pagando normalmente o aluguel, e já estou no aguardo do quarto chamado pra tentar resolver, 
+completamente insatisfeito</t>
+  </si>
+  <si>
+    <t>Só tende um robo
+O técnico não comparece e nem avisa
+o robô não consegue enviar a senha para identificar o prestador
+Mandar e-mails com ofertas não solicitadas é crime</t>
+  </si>
+  <si>
+    <t>Demorou 4 meses para trocarem um equipamento antigo, que estava superaquecendo, inclusive com laudo de técnico da Brastemp pedindo a substituição.
+Desde abril.26 com problema, só deram atenção depois que paguei as mensalidades de abril a julho.26, e solicitei o cancelamento.
+Ao ligar para cancelar, logo atenderam a necessidade, trocando o equipamento.
+Sou cliente a mais de uma década, e sempre busquei o valor do serviço, não o preço, mas hoje, o valor só serviço da Brastemp é muito baixo, para o preço que cobram.
+Como proporam trocar o equipamento e não cobrar os próximos meses, para compensar o que tive que pagar, aceitar para avaliar os seus serviços, que está deixando a desejar.
+Muito insatisfeito com o tratamento da Brastemp.</t>
+  </si>
+  <si>
+    <t>É sério? Pedi a troca do purificador que estava com defeito e trocaram por outro que não funciona. A água não gela. Estou há três dias tentando falar com vcs e nada / uma vergonha. Vou cancelar</t>
+  </si>
+  <si>
+    <t>Porque fiz contato oara marcar a manutenção, que ocorreu somente 15 dias depois, o tecnico nao resolveu o probelma no dia, voltou depois de 7 dias, nao resolveu o problema, e agora disse que voltara 10 dias depois para trocar o Filtro. Serviço no qual eu ja havia sinalizado e falaram que deveria ter a avaliação do tecnico.
+Ou seja, estou pagando por um serviço de locação mensal e faz 1 mes que estou sem filtro!</t>
+  </si>
+  <si>
+    <t>Desorganização e desrespeito com o consuidor - 1) Sempre paguei a Brastemp corretamente e em debito automático. E me gerou impactos ao trocar de cnpj x meu débito automático e eu, que nunca devi na vida, fiquei com pendência e até hj não consigo mais colocar em débito automático novamente.
+2) Marcaram de vir no Sábado, das 8 às 13h. Desmarquei todos os meus compromissos para recebê-los e além de não virem, nem sequer informaram para que eu pudesse então, resolver outras responsabilidades. 
+3) Reagendei para uma 5af à tarde e me apareceu um técnico aqui antes do dia marcado. Eu estava operada. E depois apareceu um outro técnico no dia marcado, foi quando descobrimos que a ordem de serviço anterior não tinha sido fechada. Ou seja, gerou ineficiência até para o técnico do dia marcado, pois poderia atender outros clientes. .</t>
   </si>
 </sst>
 </file>
@@ -5186,7 +5296,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1384"/>
+  <dimension ref="A1:K1407"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -53643,6 +53753,811 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1385" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1385" s="4">
+        <v>387</v>
+      </c>
+      <c r="B1385" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1385" s="4">
+        <v>85699</v>
+      </c>
+      <c r="D1385" s="2">
+        <v>46226.303622685176</v>
+      </c>
+      <c r="E1385" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1385" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1385" s="4" t="s">
+        <v>1548</v>
+      </c>
+      <c r="H1385" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1385" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1385" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1385" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1386" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1386" s="4">
+        <v>389</v>
+      </c>
+      <c r="B1386" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1386" s="4">
+        <v>79599</v>
+      </c>
+      <c r="D1386" s="2">
+        <v>46226.464259259257</v>
+      </c>
+      <c r="E1386" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1386" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1386" s="4" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H1386" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1386" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1386" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1386" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1387" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1387" s="4">
+        <v>390</v>
+      </c>
+      <c r="B1387" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1387" s="4">
+        <v>101958</v>
+      </c>
+      <c r="D1387" s="2">
+        <v>46227.313773148147</v>
+      </c>
+      <c r="E1387" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1387" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1387" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="H1387" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1387" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1387" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1387" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1388" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1388" s="4">
+        <v>391</v>
+      </c>
+      <c r="B1388" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1388" s="4">
+        <v>91490</v>
+      </c>
+      <c r="D1388" s="2">
+        <v>46227.535555555558</v>
+      </c>
+      <c r="E1388" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1388" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1388" s="4" t="s">
+        <v>1551</v>
+      </c>
+      <c r="H1388" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1388" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1388" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1388" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1389" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1389" s="4">
+        <v>392</v>
+      </c>
+      <c r="B1389" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1389" s="4">
+        <v>103497</v>
+      </c>
+      <c r="D1389" s="2">
+        <v>46230.163402777784</v>
+      </c>
+      <c r="E1389" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1389" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1389" s="4" t="s">
+        <v>1552</v>
+      </c>
+      <c r="H1389" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1389" s="4" t="s">
+        <v>1553</v>
+      </c>
+      <c r="J1389" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1389" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1390" s="4">
+        <v>393</v>
+      </c>
+      <c r="B1390" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1390" s="4">
+        <v>90234</v>
+      </c>
+      <c r="D1390" s="2">
+        <v>46230.252002314817</v>
+      </c>
+      <c r="E1390" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1390" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1390" s="4" t="s">
+        <v>1554</v>
+      </c>
+      <c r="H1390" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1390" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1390" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1390" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1391" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1391" s="4">
+        <v>394</v>
+      </c>
+      <c r="B1391" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1391" s="4">
+        <v>103674</v>
+      </c>
+      <c r="D1391" s="2">
+        <v>46230.269479166673</v>
+      </c>
+      <c r="E1391" s="4" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1391" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1391" s="4" t="s">
+        <v>1555</v>
+      </c>
+      <c r="H1391" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1391" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1391" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1391" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1392" s="4">
+        <v>395</v>
+      </c>
+      <c r="B1392" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1392" s="4">
+        <v>103554</v>
+      </c>
+      <c r="D1392" s="2">
+        <v>46230.353437500002</v>
+      </c>
+      <c r="E1392" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1392" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1392" s="4" t="s">
+        <v>1556</v>
+      </c>
+      <c r="H1392" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1392" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1392" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1392" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1393" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1393" s="4">
+        <v>396</v>
+      </c>
+      <c r="B1393" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C1393" s="4">
+        <v>106661</v>
+      </c>
+      <c r="D1393" s="2">
+        <v>46230.440486111111</v>
+      </c>
+      <c r="E1393" s="4" t="s">
+        <v>1558</v>
+      </c>
+      <c r="F1393" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1393" s="4" t="s">
+        <v>1559</v>
+      </c>
+      <c r="H1393" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1393" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1393" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1393" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1394" s="4">
+        <v>397</v>
+      </c>
+      <c r="B1394" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1394" s="4">
+        <v>100515</v>
+      </c>
+      <c r="D1394" s="2">
+        <v>46230.499502314808</v>
+      </c>
+      <c r="E1394" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1394" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1394" s="4" t="s">
+        <v>1560</v>
+      </c>
+      <c r="H1394" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1394" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1394" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1394" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1395" s="4">
+        <v>398</v>
+      </c>
+      <c r="B1395" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1395" s="4">
+        <v>106143</v>
+      </c>
+      <c r="D1395" s="2">
+        <v>46230.517500000002</v>
+      </c>
+      <c r="E1395" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1395" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1395" s="4" t="s">
+        <v>1561</v>
+      </c>
+      <c r="H1395" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="I1395" s="4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="J1395" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1395" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1396" s="4">
+        <v>400</v>
+      </c>
+      <c r="B1396" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1396" s="4">
+        <v>106365</v>
+      </c>
+      <c r="D1396" s="2">
+        <v>46231.378865740742</v>
+      </c>
+      <c r="E1396" s="4" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1396" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1396" s="4" t="s">
+        <v>1564</v>
+      </c>
+      <c r="H1396" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1396" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1396" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1396" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1397" s="4">
+        <v>401</v>
+      </c>
+      <c r="B1397" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1397" s="4">
+        <v>91356</v>
+      </c>
+      <c r="D1397" s="2">
+        <v>46231.618923611109</v>
+      </c>
+      <c r="E1397" s="4" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F1397" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1397" s="4" t="s">
+        <v>1565</v>
+      </c>
+      <c r="H1397" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1397" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1397" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1397" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1398" s="4">
+        <v>402</v>
+      </c>
+      <c r="B1398" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1398" s="4">
+        <v>106419</v>
+      </c>
+      <c r="D1398" s="2">
+        <v>46232.304594907408</v>
+      </c>
+      <c r="E1398" s="4" t="s">
+        <v>1566</v>
+      </c>
+      <c r="F1398" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1398" s="4" t="s">
+        <v>1567</v>
+      </c>
+      <c r="H1398" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1398" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1398" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1398" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1399" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1399" s="4">
+        <v>403</v>
+      </c>
+      <c r="B1399" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1399" s="4">
+        <v>96662</v>
+      </c>
+      <c r="D1399" s="2">
+        <v>46232.311030092591</v>
+      </c>
+      <c r="E1399" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1399" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1399" s="4" t="s">
+        <v>1568</v>
+      </c>
+      <c r="H1399" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="I1399" s="4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="J1399" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1399" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1400" s="4">
+        <v>404</v>
+      </c>
+      <c r="B1400" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1400" s="4">
+        <v>98899</v>
+      </c>
+      <c r="D1400" s="2">
+        <v>46232.558495370373</v>
+      </c>
+      <c r="E1400" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F1400" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1400" s="4" t="s">
+        <v>1569</v>
+      </c>
+      <c r="H1400" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1400" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="J1400" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1400" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1401" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1401" s="4">
+        <v>405</v>
+      </c>
+      <c r="B1401" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1401" s="4">
+        <v>104621</v>
+      </c>
+      <c r="D1401" s="2">
+        <v>46233.339548611111</v>
+      </c>
+      <c r="E1401" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1401" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1401" s="4" t="s">
+        <v>1570</v>
+      </c>
+      <c r="H1401" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1401" s="4" t="s">
+        <v>1553</v>
+      </c>
+      <c r="J1401" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1401" s="4" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1402" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1402" s="4">
+        <v>406</v>
+      </c>
+      <c r="B1402" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1402" s="4">
+        <v>77825</v>
+      </c>
+      <c r="D1402" s="2">
+        <v>46233.38753472222</v>
+      </c>
+      <c r="E1402" s="4" t="s">
+        <v>1571</v>
+      </c>
+      <c r="F1402" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1402" s="4" t="s">
+        <v>1572</v>
+      </c>
+      <c r="H1402" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1402" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1402" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1402" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1403" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1403" s="4">
+        <v>407</v>
+      </c>
+      <c r="B1403" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1403" s="4">
+        <v>103194</v>
+      </c>
+      <c r="D1403" s="2">
+        <v>46233.558287037027</v>
+      </c>
+      <c r="E1403" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1403" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1403" s="4" t="s">
+        <v>1573</v>
+      </c>
+      <c r="H1403" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1403" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1403" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1403" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1404" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1404" s="4">
+        <v>408</v>
+      </c>
+      <c r="B1404" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1404" s="4">
+        <v>106622</v>
+      </c>
+      <c r="D1404" s="2">
+        <v>46233.631863425922</v>
+      </c>
+      <c r="E1404" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1404" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1404" s="4" t="s">
+        <v>1574</v>
+      </c>
+      <c r="H1404" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1404" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1404" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1404" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1405" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1405" s="4">
+        <v>409</v>
+      </c>
+      <c r="B1405" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1405" s="4">
+        <v>95559</v>
+      </c>
+      <c r="D1405" s="2">
+        <v>46233.677673611113</v>
+      </c>
+      <c r="E1405" s="4" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1405" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1405" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="H1405" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1405" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1405" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1405" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1406" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1406" s="4">
+        <v>410</v>
+      </c>
+      <c r="B1406" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1406" s="4">
+        <v>98178</v>
+      </c>
+      <c r="D1406" s="2">
+        <v>46233.796076388891</v>
+      </c>
+      <c r="E1406" s="4" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1406" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1406" s="4" t="s">
+        <v>1576</v>
+      </c>
+      <c r="H1406" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1406" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1406" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1406" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1407" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1407" s="4">
+        <v>411</v>
+      </c>
+      <c r="B1407" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1407" s="4">
+        <v>106837</v>
+      </c>
+      <c r="D1407" s="2">
+        <v>46234.202592592592</v>
+      </c>
+      <c r="E1407" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1407" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1407" s="4" t="s">
+        <v>1577</v>
+      </c>
+      <c r="H1407" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="I1407" s="4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="J1407" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1407" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 31/07/2026 11:23:55,44
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="378" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DEBF4C1-E61D-4DF1-A915-DB6E0E3EC113}"/>
+  <xr:revisionPtr revIDLastSave="385" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0FAECE6-0F71-4C0C-9851-7CE90029DE8E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1369</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1407</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11259" uniqueCount="1578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11259" uniqueCount="1576">
   <si>
     <t>ID</t>
   </si>
@@ -4779,9 +4779,6 @@
     <t>Financeiro</t>
   </si>
   <si>
-    <t>Boleto</t>
-  </si>
-  <si>
     <t>Porque o reparo foi feito, mas o filtro apresentou outro defeito. Agora está pingando. Tive que marcar outra visita</t>
   </si>
   <si>
@@ -4862,9 +4859,6 @@
   <si>
     <t>Há cerca de 3 meses, estou com dificuldades para conseguir pagar, tanto débito automático quanto boleto, e também para agendamento de visitas e correção de defeito no equipamento. Há quase 2 meses sem funcionar
 Assistência está deixando muito a desejar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financeiro </t>
   </si>
   <si>
     <t>Problemas no faturamento</t>
@@ -53242,13 +53236,13 @@
         <v>46221.760682870372</v>
       </c>
       <c r="E1370" s="4" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="F1370" s="4" t="s">
         <v>1465</v>
       </c>
       <c r="G1370" s="4" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="H1370" s="4" t="s">
         <v>18</v>
@@ -53257,7 +53251,7 @@
         <v>50</v>
       </c>
       <c r="J1370" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1370" s="4" t="s">
         <v>1442</v>
@@ -53283,7 +53277,7 @@
         <v>1465</v>
       </c>
       <c r="G1371" s="4" t="s">
-        <v>1543</v>
+        <v>1542</v>
       </c>
       <c r="H1371" s="4" t="s">
         <v>18</v>
@@ -53292,7 +53286,7 @@
         <v>59</v>
       </c>
       <c r="J1371" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1371" s="4" t="s">
         <v>1441</v>
@@ -53318,7 +53312,7 @@
         <v>1465</v>
       </c>
       <c r="G1372" s="4" t="s">
-        <v>1544</v>
+        <v>1543</v>
       </c>
       <c r="H1372" s="4" t="s">
         <v>13</v>
@@ -53327,7 +53321,7 @@
         <v>26</v>
       </c>
       <c r="J1372" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1372" s="4" t="s">
         <v>1441</v>
@@ -53353,7 +53347,7 @@
         <v>1465</v>
       </c>
       <c r="G1373" s="4" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
       <c r="H1373" s="4" t="s">
         <v>13</v>
@@ -53362,7 +53356,7 @@
         <v>26</v>
       </c>
       <c r="J1373" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1373" s="4" t="s">
         <v>1441</v>
@@ -53388,7 +53382,7 @@
         <v>1465</v>
       </c>
       <c r="G1374" s="4" t="s">
-        <v>1546</v>
+        <v>1545</v>
       </c>
       <c r="H1374" s="4" t="s">
         <v>18</v>
@@ -53397,7 +53391,7 @@
         <v>1010</v>
       </c>
       <c r="J1374" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1374" s="4" t="s">
         <v>1441</v>
@@ -53423,7 +53417,7 @@
         <v>1465</v>
       </c>
       <c r="G1375" s="4" t="s">
-        <v>1547</v>
+        <v>1546</v>
       </c>
       <c r="H1375" s="4" t="s">
         <v>18</v>
@@ -53432,7 +53426,7 @@
         <v>1010</v>
       </c>
       <c r="J1375" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1375" s="4" t="s">
         <v>1442</v>
@@ -53467,7 +53461,7 @@
         <v>32</v>
       </c>
       <c r="J1376" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1376" s="4" t="s">
         <v>1441</v>
@@ -53502,7 +53496,7 @@
         <v>1010</v>
       </c>
       <c r="J1377" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1377" s="4" t="s">
         <v>1442</v>
@@ -53537,7 +53531,7 @@
         <v>81</v>
       </c>
       <c r="J1378" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1378" s="4" t="s">
         <v>1441</v>
@@ -53572,7 +53566,7 @@
         <v>151</v>
       </c>
       <c r="J1379" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1379" s="4" t="s">
         <v>1441</v>
@@ -53607,7 +53601,7 @@
         <v>1010</v>
       </c>
       <c r="J1380" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1380" s="4" t="s">
         <v>1441</v>
@@ -53639,10 +53633,10 @@
         <v>1535</v>
       </c>
       <c r="I1381" s="4" t="s">
-        <v>1536</v>
+        <v>1561</v>
       </c>
       <c r="J1381" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1381" s="4" t="s">
         <v>1441</v>
@@ -53668,7 +53662,7 @@
         <v>1465</v>
       </c>
       <c r="G1382" s="4" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="H1382" s="4" t="s">
         <v>34</v>
@@ -53677,7 +53671,7 @@
         <v>98</v>
       </c>
       <c r="J1382" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1382" s="4" t="s">
         <v>1441</v>
@@ -53703,7 +53697,7 @@
         <v>1465</v>
       </c>
       <c r="G1383" s="4" t="s">
-        <v>1538</v>
+        <v>1537</v>
       </c>
       <c r="H1383" s="4" t="s">
         <v>18</v>
@@ -53712,7 +53706,7 @@
         <v>1010</v>
       </c>
       <c r="J1383" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1383" s="4" t="s">
         <v>1441</v>
@@ -53738,7 +53732,7 @@
         <v>1465</v>
       </c>
       <c r="G1384" s="4" t="s">
-        <v>1539</v>
+        <v>1538</v>
       </c>
       <c r="H1384" s="4" t="s">
         <v>18</v>
@@ -53747,7 +53741,7 @@
         <v>50</v>
       </c>
       <c r="J1384" s="4" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="K1384" s="4" t="s">
         <v>1441</v>
@@ -53773,7 +53767,7 @@
         <v>1465</v>
       </c>
       <c r="G1385" s="4" t="s">
-        <v>1548</v>
+        <v>1547</v>
       </c>
       <c r="H1385" s="4" t="s">
         <v>152</v>
@@ -53808,7 +53802,7 @@
         <v>1465</v>
       </c>
       <c r="G1386" s="4" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="H1386" s="4" t="s">
         <v>34</v>
@@ -53843,7 +53837,7 @@
         <v>1465</v>
       </c>
       <c r="G1387" s="4" t="s">
-        <v>1550</v>
+        <v>1549</v>
       </c>
       <c r="H1387" s="4" t="s">
         <v>18</v>
@@ -53878,7 +53872,7 @@
         <v>1465</v>
       </c>
       <c r="G1388" s="4" t="s">
-        <v>1551</v>
+        <v>1550</v>
       </c>
       <c r="H1388" s="4" t="s">
         <v>18</v>
@@ -53913,13 +53907,13 @@
         <v>1465</v>
       </c>
       <c r="G1389" s="4" t="s">
-        <v>1552</v>
+        <v>1551</v>
       </c>
       <c r="H1389" s="4" t="s">
         <v>80</v>
       </c>
       <c r="I1389" s="4" t="s">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="J1389" s="4" t="s">
         <v>1405</v>
@@ -53948,7 +53942,7 @@
         <v>1465</v>
       </c>
       <c r="G1390" s="4" t="s">
-        <v>1554</v>
+        <v>1553</v>
       </c>
       <c r="H1390" s="4" t="s">
         <v>18</v>
@@ -53983,7 +53977,7 @@
         <v>1465</v>
       </c>
       <c r="G1391" s="4" t="s">
-        <v>1555</v>
+        <v>1554</v>
       </c>
       <c r="H1391" s="4" t="s">
         <v>18</v>
@@ -54018,7 +54012,7 @@
         <v>1465</v>
       </c>
       <c r="G1392" s="4" t="s">
-        <v>1556</v>
+        <v>1555</v>
       </c>
       <c r="H1392" s="4" t="s">
         <v>18</v>
@@ -54038,7 +54032,7 @@
         <v>396</v>
       </c>
       <c r="B1393" s="4" t="s">
-        <v>1557</v>
+        <v>1556</v>
       </c>
       <c r="C1393" s="4">
         <v>106661</v>
@@ -54047,13 +54041,13 @@
         <v>46230.440486111111</v>
       </c>
       <c r="E1393" s="4" t="s">
-        <v>1558</v>
+        <v>1557</v>
       </c>
       <c r="F1393" s="4" t="s">
         <v>1465</v>
       </c>
       <c r="G1393" s="4" t="s">
-        <v>1559</v>
+        <v>1558</v>
       </c>
       <c r="H1393" s="4" t="s">
         <v>18</v>
@@ -54088,7 +54082,7 @@
         <v>1465</v>
       </c>
       <c r="G1394" s="4" t="s">
-        <v>1560</v>
+        <v>1559</v>
       </c>
       <c r="H1394" s="4" t="s">
         <v>18</v>
@@ -54123,13 +54117,13 @@
         <v>1465</v>
       </c>
       <c r="G1395" s="4" t="s">
+        <v>1560</v>
+      </c>
+      <c r="H1395" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="I1395" s="4" t="s">
         <v>1561</v>
-      </c>
-      <c r="H1395" s="4" t="s">
-        <v>1562</v>
-      </c>
-      <c r="I1395" s="4" t="s">
-        <v>1563</v>
       </c>
       <c r="J1395" s="4" t="s">
         <v>1405</v>
@@ -54158,7 +54152,7 @@
         <v>1465</v>
       </c>
       <c r="G1396" s="4" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="H1396" s="4" t="s">
         <v>31</v>
@@ -54193,7 +54187,7 @@
         <v>1465</v>
       </c>
       <c r="G1397" s="4" t="s">
-        <v>1565</v>
+        <v>1563</v>
       </c>
       <c r="H1397" s="4" t="s">
         <v>34</v>
@@ -54222,13 +54216,13 @@
         <v>46232.304594907408</v>
       </c>
       <c r="E1398" s="4" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="F1398" s="4" t="s">
         <v>1465</v>
       </c>
       <c r="G1398" s="4" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="H1398" s="4" t="s">
         <v>18</v>
@@ -54263,13 +54257,13 @@
         <v>1465</v>
       </c>
       <c r="G1399" s="4" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="H1399" s="4" t="s">
-        <v>1562</v>
+        <v>1535</v>
       </c>
       <c r="I1399" s="4" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
       <c r="J1399" s="4" t="s">
         <v>1405</v>
@@ -54298,7 +54292,7 @@
         <v>1465</v>
       </c>
       <c r="G1400" s="4" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="H1400" s="4" t="s">
         <v>34</v>
@@ -54333,13 +54327,13 @@
         <v>1465</v>
       </c>
       <c r="G1401" s="4" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="H1401" s="4" t="s">
         <v>80</v>
       </c>
       <c r="I1401" s="4" t="s">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="J1401" s="4" t="s">
         <v>1405</v>
@@ -54362,13 +54356,13 @@
         <v>46233.38753472222</v>
       </c>
       <c r="E1402" s="4" t="s">
-        <v>1571</v>
+        <v>1569</v>
       </c>
       <c r="F1402" s="4" t="s">
         <v>1465</v>
       </c>
       <c r="G1402" s="4" t="s">
-        <v>1572</v>
+        <v>1570</v>
       </c>
       <c r="H1402" s="4" t="s">
         <v>80</v>
@@ -54403,7 +54397,7 @@
         <v>1465</v>
       </c>
       <c r="G1403" s="4" t="s">
-        <v>1573</v>
+        <v>1571</v>
       </c>
       <c r="H1403" s="4" t="s">
         <v>18</v>
@@ -54438,7 +54432,7 @@
         <v>1465</v>
       </c>
       <c r="G1404" s="4" t="s">
-        <v>1574</v>
+        <v>1572</v>
       </c>
       <c r="H1404" s="4" t="s">
         <v>152</v>
@@ -54473,7 +54467,7 @@
         <v>1465</v>
       </c>
       <c r="G1405" s="4" t="s">
-        <v>1575</v>
+        <v>1573</v>
       </c>
       <c r="H1405" s="4" t="s">
         <v>34</v>
@@ -54508,7 +54502,7 @@
         <v>1465</v>
       </c>
       <c r="G1406" s="4" t="s">
-        <v>1576</v>
+        <v>1574</v>
       </c>
       <c r="H1406" s="4" t="s">
         <v>31</v>
@@ -54543,13 +54537,13 @@
         <v>1465</v>
       </c>
       <c r="G1407" s="4" t="s">
-        <v>1577</v>
+        <v>1575</v>
       </c>
       <c r="H1407" s="4" t="s">
-        <v>1562</v>
+        <v>1535</v>
       </c>
       <c r="I1407" s="4" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
       <c r="J1407" s="4" t="s">
         <v>1405</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 03/08/2026 11:38:33,91
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPSMedalliaequaltricsculligan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="385" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0FAECE6-0F71-4C0C-9851-7CE90029DE8E}"/>
+  <xr:revisionPtr revIDLastSave="409" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59E1D58F-46BA-4B81-BBBF-2A4868A517E9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11259" uniqueCount="1576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11314" uniqueCount="1586">
   <si>
     <t>ID</t>
   </si>
@@ -4918,6 +4918,40 @@
     <t>Desorganização e desrespeito com o consuidor - 1) Sempre paguei a Brastemp corretamente e em debito automático. E me gerou impactos ao trocar de cnpj x meu débito automático e eu, que nunca devi na vida, fiquei com pendência e até hj não consigo mais colocar em débito automático novamente.
 2) Marcaram de vir no Sábado, das 8 às 13h. Desmarquei todos os meus compromissos para recebê-los e além de não virem, nem sequer informaram para que eu pudesse então, resolver outras responsabilidades. 
 3) Reagendei para uma 5af à tarde e me apareceu um técnico aqui antes do dia marcado. Eu estava operada. E depois apareceu um outro técnico no dia marcado, foi quando descobrimos que a ordem de serviço anterior não tinha sido fechada. Ou seja, gerou ineficiência até para o técnico do dia marcado, pois poderia atender outros clientes. .</t>
+  </si>
+  <si>
+    <t>FRQ LAGOS RJ R02</t>
+  </si>
+  <si>
+    <t>FRQ SALVADOR BA R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>FRQ GALEAO SUL RJ R05</t>
+  </si>
+  <si>
+    <t>Péssimo serviço. Desmarcaram sem avisar. Vieram num dia diferente do agendado. E não trocaram o filtro. Na época da Brastemp sempre trocaram. Triste.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A comunicação com a Culligan é horrivel, mando diversos email para o financeiro por exemplo e não temos retorno algum nem por email , nem por nenhum outro meio de comunicação. Em alguns casos temos problemas urgente com os bebedouros e já chegaram a marcar visita com mais de uma mês, e até ? todos ficam sem água? 
+Tenho mais de 50 bebedouros, já pedi a base atualizada, até hoje sem retorno. 
+Difícil demais qualquer tipo de comunicação ou retorno. </t>
+  </si>
+  <si>
+    <t>o serviço ta cada vez pior. Estou bastante descontente. estou com problemas em algumas peças que ha 8 meses espero para troca e nada. estou pensando seriamente em cancelar, pois não esta mais valendo a pena</t>
+  </si>
+  <si>
+    <t>Na última agenda marcada, o técnico não compareceu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nao foi resolvido o problema preciso nova visita  urgente </t>
+  </si>
+  <si>
+    <t>Estou sem filtro a mais de 45 dias, estou pagamento minhas faturas e estou gastando comprando água.
+Isso é uma falta de respeito com o cliente, sou clientes a mais de 12 anos e tenho que passar por isso.
+Chega ser lamentável essa situação.</t>
+  </si>
+  <si>
+    <t>O técnico foi fazer a manutenção semestral e deixou o filtro com um barulho ensurdecedor.</t>
   </si>
 </sst>
 </file>
@@ -4974,7 +5008,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4987,6 +5021,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5290,7 +5327,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1407"/>
+  <dimension ref="A1:K1414"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -54552,6 +54589,248 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1408" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1408" s="4">
+        <v>412</v>
+      </c>
+      <c r="C1408" s="4">
+        <v>92325</v>
+      </c>
+      <c r="D1408" s="2">
+        <v>46234.59043152778</v>
+      </c>
+      <c r="E1408" s="4" t="s">
+        <v>1576</v>
+      </c>
+      <c r="F1408" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1408" s="4" t="s">
+        <v>1579</v>
+      </c>
+      <c r="H1408" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1408" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1408" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1408" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1409" spans="1:11" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1409" s="4">
+        <v>413</v>
+      </c>
+      <c r="B1409" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1409" s="4">
+        <v>108099</v>
+      </c>
+      <c r="D1409" s="2">
+        <v>46234.605979837965</v>
+      </c>
+      <c r="E1409" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1409" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1409" s="5" t="s">
+        <v>1580</v>
+      </c>
+      <c r="H1409" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1409" s="4" t="s">
+        <v>1552</v>
+      </c>
+      <c r="J1409" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1409" s="4" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1410" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1410" s="4">
+        <v>414</v>
+      </c>
+      <c r="B1410" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1410" s="4">
+        <v>87586</v>
+      </c>
+      <c r="D1410" s="2">
+        <v>46234.643638819442</v>
+      </c>
+      <c r="E1410" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1410" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1410" s="4" t="s">
+        <v>1581</v>
+      </c>
+      <c r="H1410" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1410" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1410" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1410" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1411" s="4">
+        <v>415</v>
+      </c>
+      <c r="B1411" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1411" s="4">
+        <v>99308</v>
+      </c>
+      <c r="D1411" s="2">
+        <v>46234.773582997688</v>
+      </c>
+      <c r="E1411" s="4" t="s">
+        <v>1577</v>
+      </c>
+      <c r="F1411" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1411" s="4" t="s">
+        <v>1582</v>
+      </c>
+      <c r="H1411" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1411" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1411" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1411" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1412" s="4">
+        <v>416</v>
+      </c>
+      <c r="B1412" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1412" s="4">
+        <v>103189</v>
+      </c>
+      <c r="D1412" s="2">
+        <v>46234.832082858797</v>
+      </c>
+      <c r="E1412" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1412" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1412" s="4" t="s">
+        <v>1583</v>
+      </c>
+      <c r="H1412" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1412" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1412" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1412" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1413" s="4">
+        <v>417</v>
+      </c>
+      <c r="B1413" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1413" s="4">
+        <v>103176</v>
+      </c>
+      <c r="D1413" s="2">
+        <v>46234.918748553238</v>
+      </c>
+      <c r="E1413" s="4" t="s">
+        <v>1578</v>
+      </c>
+      <c r="F1413" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1413" s="4" t="s">
+        <v>1584</v>
+      </c>
+      <c r="H1413" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1413" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1413" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1413" s="4" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1414" s="4">
+        <v>418</v>
+      </c>
+      <c r="B1414" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1414" s="4">
+        <v>90447</v>
+      </c>
+      <c r="D1414" s="2">
+        <v>46236.780051770831</v>
+      </c>
+      <c r="E1414" s="4" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1414" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G1414" s="4" t="s">
+        <v>1585</v>
+      </c>
+      <c r="H1414" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1414" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1414" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1414" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>